<commit_message>
docs: close B-04 R-04x M-01 in issue tracker
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -310,7 +310,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -551,6 +551,10 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1348,7 +1352,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K51"/>
+  <dimension ref="A1:K52"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="40" min="1" max="1"/>
@@ -2244,7 +2248,7 @@
       </c>
       <c r="B17" s="45" t="inlineStr">
         <is>
-          <t>暂缓</t>
+          <t>已处理</t>
         </is>
       </c>
       <c r="C17" s="44" t="inlineStr">
@@ -2269,7 +2273,7 @@
       </c>
       <c r="G17" s="46" t="inlineStr">
         <is>
-          <t>先不做完整 Agent-Agent 好友图。下一期单独开。</t>
+          <t>用户评角色动态后 5～15s 作者回一句；总开关关不回；同动态只回一次。2026-10-09 BF 验收通过（2c2e897），尚未 push（不在今晚 HY 四连内）。</t>
         </is>
       </c>
       <c r="H17" s="44" t="inlineStr">
@@ -2277,11 +2281,17 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="I17" s="44" t="n"/>
-      <c r="J17" s="44" t="n"/>
+      <c r="I17" s="82" t="n">
+        <v>46304</v>
+      </c>
+      <c r="J17" s="44" t="inlineStr">
+        <is>
+          <t>2c2e897</t>
+        </is>
+      </c>
       <c r="K17" s="46" t="inlineStr">
         <is>
-          <t>原待优化点第 5 条的小方案。 2026-09-16：与 M-07 不同——M-01 是用户评角色动态后作者再回。</t>
+          <t>原待优化点第 5 条的小方案。 2026-09-16：与 M-07 不同——M-01 是用户评角色动态后作者再回。 2026-10-09 点收；commit 在 BF，等另说再 push。</t>
         </is>
       </c>
     </row>
@@ -2571,7 +2581,7 @@
       </c>
       <c r="G23" s="46" t="inlineStr">
         <is>
-          <t>语音（50b8054 / e19d757）+ 用户聊天发图第一刀均已本机通过。VLM 读图、生图/融合、动态配图（M-05）仍不在本条已验收范围。</t>
+          <t>B-04A 读图 a668a53；B-04B 生图 97ad2c6+b128045（Kolors）。2026-10-09 HY 验收通过，已 push，远程 tip 575967c。Image-Edit/视频仍不在范围。</t>
         </is>
       </c>
       <c r="H23" s="44" t="inlineStr">
@@ -2579,19 +2589,17 @@
           <t>2026-09-14</t>
         </is>
       </c>
-      <c r="I23" s="44" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
+      <c r="I23" s="82" t="n">
+        <v>46304</v>
       </c>
       <c r="J23" s="44" t="inlineStr">
         <is>
-          <t>50b8054 / 8fa8669</t>
+          <t>a668a53 / 97ad2c6 / b128045</t>
         </is>
       </c>
       <c r="K23" s="46" t="inlineStr">
         <is>
-          <t>用户 2026-09-14 明确提出。含图片，不限于 TTS。已读双勾仍不在本条范围。 2026-09-15 对照 artifacts/agent-chat-voice-evaluation.html。密钥只进本机 .env，不入库、不进本表。 2026-09-15 20:12 用户选定硅基流动，已拆第一刀给 Bot。 2026-09-15 20:25 Bot 汇报 50b8054，改待确认。未 push。本地 ahead origin 4。 2026-09-15 20:27 主路径可见，体验三条记 B-06。 2026-09-15 20:48 用户验收关闭语音部分。图片仍暂缓。未 push。 2026-09-15 夜交接：语音已关；后半聊天图/VLM/生图仍开、先不拆包。 2026-09-16：GLM 多模态方案 v1.2 已评估。采纳方向：朋友圈配图先于聊天发图、成本闸门、画风不一致禁直融、不引网关。不采纳为立刻动工基线：ComfyUI 工厂、千张采集、向量库、能力层大搬家。详见会话评估。 2026-09-16 用户验收：聊天发图正常。范围仅上传进气泡；未含 VLM/生图。 2026-09-16 远程聊天发图 8fa8669。VLM/生图仍不在远程。</t>
+          <t>用户 2026-09-14 明确提出。含图片，不限于 TTS。已读双勾仍不在本条范围。 2026-09-15 对照 artifacts/agent-chat-voice-evaluation.html。密钥只进本机 .env，不入库、不进本表。 2026-09-15 20:12 用户选定硅基流动，已拆第一刀给 Bot。 2026-09-15 20:25 Bot 汇报 50b8054，改待确认。未 push。本地 ahead origin 4。 2026-09-15 20:27 主路径可见，体验三条记 B-06。 2026-09-15 20:48 用户验收关闭语音部分。图片仍暂缓。未 push。 2026-09-15 夜交接：语音已关；后半聊天图/VLM/生图仍开、先不拆包。 2026-09-16：GLM 多模态方案 v1.2 已评估。采纳方向：朋友圈配图先于聊天发图、成本闸门、画风不一致禁直融、不引网关。不采纳为立刻动工基线：ComfyUI 工厂、千张采集、向量库、能力层大搬家。详见会话评估。 2026-09-16 用户验收：聊天发图正常。范围仅上传进气泡；未含 VLM/生图。 2026-09-16 远程聊天发图 8fa8669。VLM/生图仍不在远程。 2026-10-09 点收并 push 2981fa3..575967c。</t>
         </is>
       </c>
     </row>
@@ -3505,7 +3513,7 @@
       <c r="J41" s="49" t="n"/>
       <c r="K41" s="51" t="inlineStr">
         <is>
-          <t>先做 R-02 注入必答补丁。</t>
+          <t>先做 R-02 注入必答补丁。 2026-10-09 R-04x 尖兵 575967c 已上远程（夹具报告+默认 off；Laya 本机已装不强开）。分模型正式刀仍暂缓。</t>
         </is>
       </c>
     </row>
@@ -3616,32 +3624,72 @@
       </c>
     </row>
     <row r="44" ht="43.5" customHeight="1" s="41">
-      <c r="A44" s="47" t="inlineStr">
+      <c r="A44" s="40" t="inlineStr">
+        <is>
+          <t>R-04x</t>
+        </is>
+      </c>
+      <c r="B44" s="40" t="inlineStr">
+        <is>
+          <t>已处理</t>
+        </is>
+      </c>
+      <c r="C44" s="40" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D44" s="40" t="inlineStr">
+        <is>
+          <t>角色</t>
+        </is>
+      </c>
+      <c r="E44" s="40" t="inlineStr">
+        <is>
+          <t>Laya 本机记忆门控尖兵</t>
+        </is>
+      </c>
+      <c r="F44" s="40" t="inlineStr">
+        <is>
+          <t>用开源决策模型做写/不写门控评测；默认不进生产。</t>
+        </is>
+      </c>
+      <c r="G44" s="40" t="inlineStr">
+        <is>
+          <t>夹具24条启发式约95.8%；MEMORY_GATE_BACKEND 默认 off；Laya 本机已装。2026-10-09 点收并随 575967c push。</t>
+        </is>
+      </c>
+      <c r="H44" s="83" t="n">
+        <v>46286</v>
+      </c>
+      <c r="I44" s="83" t="n">
+        <v>46304</v>
+      </c>
+      <c r="J44" s="40" t="inlineStr">
+        <is>
+          <t>575967c</t>
+        </is>
+      </c>
+      <c r="K44" s="40" t="inlineStr">
+        <is>
+          <t>不强开真 Laya；正式分模型仍见 R-04。</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="15" customHeight="1" s="41">
+      <c r="A45" s="47" t="inlineStr">
         <is>
           <t>U-xx</t>
         </is>
       </c>
-      <c r="B44" s="47" t="n"/>
-      <c r="C44" s="47" t="n"/>
-      <c r="D44" s="47" t="n"/>
-      <c r="E44" s="46" t="inlineStr">
-        <is>
-          <t>（在此行往下追加新问题。ID 建议：U 界面 / G 群聊 / C 会话 / M 朋友圈 / R 角色 / B 体验 / O 工程）</t>
-        </is>
-      </c>
-      <c r="F44" s="47" t="n"/>
-      <c r="G44" s="47" t="n"/>
-      <c r="H44" s="47" t="n"/>
-      <c r="I44" s="47" t="n"/>
-      <c r="J44" s="47" t="n"/>
-      <c r="K44" s="47" t="n"/>
-    </row>
-    <row r="45" ht="15" customHeight="1" s="41">
-      <c r="A45" s="47" t="n"/>
       <c r="B45" s="47" t="n"/>
       <c r="C45" s="47" t="n"/>
       <c r="D45" s="47" t="n"/>
-      <c r="E45" s="47" t="n"/>
+      <c r="E45" s="46" t="inlineStr">
+        <is>
+          <t>（在此行往下追加新问题。ID 建议：U 界面 / G 群聊 / C 会话 / M 朋友圈 / R 角色 / B 体验 / O 工程）</t>
+        </is>
+      </c>
       <c r="F45" s="47" t="n"/>
       <c r="G45" s="47" t="n"/>
       <c r="H45" s="47" t="n"/>
@@ -3726,6 +3774,19 @@
       <c r="I51" s="47" t="n"/>
       <c r="J51" s="47" t="n"/>
       <c r="K51" s="47" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="47" t="n"/>
+      <c r="B52" s="47" t="n"/>
+      <c r="C52" s="47" t="n"/>
+      <c r="D52" s="47" t="n"/>
+      <c r="E52" s="47" t="n"/>
+      <c r="F52" s="47" t="n"/>
+      <c r="G52" s="47" t="n"/>
+      <c r="H52" s="47" t="n"/>
+      <c r="I52" s="47" t="n"/>
+      <c r="J52" s="47" t="n"/>
+      <c r="K52" s="47" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:K40"/>
@@ -3852,12 +3913,12 @@
     <row r="8" ht="36" customHeight="1" s="41">
       <c r="A8" s="69" t="inlineStr">
         <is>
-          <t>明天建议</t>
+          <t>2026-10-09：远程 tip 575967c（含 B-04A/B、R-04x）。BF M-01 2c2e897 仍未 push。</t>
         </is>
       </c>
       <c r="B8" s="70" t="inlineStr">
         <is>
-          <t>2026-09-20：R-05 已点收并 push，远程 tip f8f0084。docs/product/ 现行三文档仍未入库。</t>
+          <t>2026-10-09：远程 tip 575967c（含 B-04A/B、R-04x）。BF M-01 2c2e897 仍未 push。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: clear stale unpushed notes; align M-01 to 5c8f652
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="问题记录" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="使用说明" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="统计" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="问题记录" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="统计" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'问题记录'!$A$1:$K$40</definedName>
@@ -761,14 +761,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1800" b="1" strike="noStrike" spc="-1">
                 <a:solidFill>
@@ -791,8 +791,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -816,10 +816,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4f81bd"/>
             </a:solidFill>
-            <a:ln w="0">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -828,10 +828,10 @@
           <dPt>
             <idx val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4f81bd"/>
               </a:solidFill>
-              <a:ln w="0">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -840,10 +840,10 @@
           <dPt>
             <idx val="1"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="c0504d"/>
               </a:solidFill>
-              <a:ln w="0">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -852,10 +852,10 @@
           <dPt>
             <idx val="2"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="9bbb59"/>
               </a:solidFill>
-              <a:ln w="0">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -864,10 +864,10 @@
           <dPt>
             <idx val="3"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="8064a2"/>
               </a:solidFill>
-              <a:ln w="0">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -876,10 +876,10 @@
           <dPt>
             <idx val="4"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4bacc6"/>
               </a:solidFill>
-              <a:ln w="0">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -889,9 +889,9 @@
             <dLbl>
               <idx val="0"/>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
                       <a:solidFill>
@@ -915,9 +915,9 @@
             <dLbl>
               <idx val="1"/>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
                       <a:solidFill>
@@ -941,9 +941,9 @@
             <dLbl>
               <idx val="2"/>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
                       <a:solidFill>
@@ -967,9 +967,9 @@
             <dLbl>
               <idx val="3"/>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
                       <a:solidFill>
@@ -993,9 +993,9 @@
             <dLbl>
               <idx val="4"/>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
                       <a:solidFill>
@@ -1017,9 +1017,9 @@
               <showPercent val="1"/>
             </dLbl>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
                     <a:solidFill>
@@ -1096,16 +1096,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
               <a:solidFill>
@@ -1124,10 +1124,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="ffffff"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="d9d9d9"/>
       </a:solidFill>
@@ -1139,7 +1139,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>3</col>
@@ -1159,9 +1159,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2179,7 +2179,7 @@
       </c>
       <c r="K15" s="51" t="inlineStr">
         <is>
-          <t>原待优化点第 6 条。建议作为下一包。 2026-09-14 夜排期：C-02 确认后作为下一开发包。 2026-09-14 23:15 已拆给 GrokBot。 2026-09-15 19:27 用户：发送后立刻回会话列表无红点；朋友圈触发后也无红点。会话红点按 C-03 排查；空间红点不在本包。 2026-09-15 19:35 Bot 汇报 9381115，改待确认。未 push。 2026-09-15 19:40 造未读困难已记 C-05，不因此打回实现。 2026-09-15 22:05 交接：代码在但难造未读，挂 C-05，不打回实现、不新开开发包。 2026-09-16：主动互动设计已备忘，C-05 仍暂缓；未读验收仍挂主动。 2026-09-17 C-05 第一刀开工，验收时一并看红点。 2026-09-17 C-05 已能写入 source=proactive 且不 markRead。等用户离开会话看列表红点后关单。 2026-09-17 用户截图：未选会话时林深有红点1；点进私聊气泡已有主动句，列表红点仍在。 2026-09-17 用户确认验收通过，关单。</t>
+          <t>原待优化点第 6 条。建议作为下一包。 2026-09-14 夜排期：C-02 确认后作为下一开发包。 2026-09-14 23:15 已拆给 GrokBot。 2026-09-15 19:27 用户：发送后立刻回会话列表无红点；朋友圈触发后也无红点。会话红点按 C-03 排查；空间红点不在本包。 2026-09-15 19:35 Bot 汇报 9381115，改待确认。 2026-09-15 19:40 造未读困难已记 C-05，不因此打回实现。 2026-09-15 22:05 交接：代码在但难造未读，挂 C-05，不打回实现、不新开开发包。 2026-09-16：主动互动设计已备忘，C-05 仍暂缓；未读验收仍挂主动。 2026-09-17 C-05 第一刀开工，验收时一并看红点。 2026-09-17 C-05 已能写入 source=proactive 且不 markRead。等用户离开会话看列表红点后关单。 2026-09-17 用户截图：未选会话时林深有红点1；点进私聊气泡已有主动句，列表红点仍在。 2026-09-17 用户确认验收通过，关单。 2026-10-10 清备注：对应功能已在远程，去掉过期未合入表述。</t>
         </is>
       </c>
     </row>
@@ -2236,7 +2236,7 @@
       </c>
       <c r="K16" s="46" t="inlineStr">
         <is>
-          <t>原待优化点第 3 条。先确认 PNG/JSON 导入都可用。 2026-09-14 夜排期：排在 C-03 之后；覆盖前先确认 JSON/PNG 导入。 2026-09-15 19:43 用户复现重复导入，已拆给 GrokBot。 2026-09-15 19:51 Bot 汇报 501e788，改待确认。未 push。 2026-09-15 19:56 用户验收关闭。未 push。</t>
+          <t>原待优化点第 3 条。先确认 PNG/JSON 导入都可用。 2026-09-14 夜排期：排在 C-03 之后；覆盖前先确认 JSON/PNG 导入。 2026-09-15 19:43 用户复现重复导入，已拆给 GrokBot。 2026-09-15 19:51 Bot 汇报 501e788，改待确认。 2026-09-15 19:56 用户验收关闭。 2026-10-10 清备注：对应功能已在远程，去掉过期未合入表述。</t>
         </is>
       </c>
     </row>
@@ -2273,7 +2273,7 @@
       </c>
       <c r="G17" s="46" t="inlineStr">
         <is>
-          <t>用户评角色动态后 5～15s 作者回一句；总开关关不回；同动态只回一次。2026-10-09 BF 验收通过（2c2e897），尚未 push（不在今晚 HY 四连内）。</t>
+          <t>用户评角色动态后 5～15s 作者回一句；总开关关不回；同动态只回一次。2026-10-09 BF 验收通过；2026-10-10 已上远程 tip 5c8f652（rebase 后哈希；旧 2c2e897 不在 origin）。</t>
         </is>
       </c>
       <c r="H17" s="44" t="inlineStr">
@@ -2286,12 +2286,12 @@
       </c>
       <c r="J17" s="44" t="inlineStr">
         <is>
-          <t>2c2e897</t>
+          <t>5c8f652</t>
         </is>
       </c>
       <c r="K17" s="46" t="inlineStr">
         <is>
-          <t>原待优化点第 5 条的小方案。 2026-09-16：与 M-07 不同——M-01 是用户评角色动态后作者再回。 2026-10-09 点收；commit 在 BF，等另说再 push。</t>
+          <t>原待优化点第 5 条的小方案。 2026-09-16：与 M-07 不同——M-01 是用户评角色动态后作者再回。 2026-10-09 点收； 2026-10-10 备注对齐：已 push，commit=5c8f652。</t>
         </is>
       </c>
     </row>
@@ -2599,7 +2599,7 @@
       </c>
       <c r="K23" s="46" t="inlineStr">
         <is>
-          <t>用户 2026-09-14 明确提出。含图片，不限于 TTS。已读双勾仍不在本条范围。 2026-09-15 对照 artifacts/agent-chat-voice-evaluation.html。密钥只进本机 .env，不入库、不进本表。 2026-09-15 20:12 用户选定硅基流动，已拆第一刀给 Bot。 2026-09-15 20:25 Bot 汇报 50b8054，改待确认。未 push。本地 ahead origin 4。 2026-09-15 20:27 主路径可见，体验三条记 B-06。 2026-09-15 20:48 用户验收关闭语音部分。图片仍暂缓。未 push。 2026-09-15 夜交接：语音已关；后半聊天图/VLM/生图仍开、先不拆包。 2026-09-16：GLM 多模态方案 v1.2 已评估。采纳方向：朋友圈配图先于聊天发图、成本闸门、画风不一致禁直融、不引网关。不采纳为立刻动工基线：ComfyUI 工厂、千张采集、向量库、能力层大搬家。详见会话评估。 2026-09-16 用户验收：聊天发图正常。范围仅上传进气泡；未含 VLM/生图。 2026-09-16 远程聊天发图 8fa8669。VLM/生图仍不在远程。 2026-10-09 点收并 push 2981fa3..575967c。</t>
+          <t>用户 2026-09-14 明确提出。含图片，不限于 TTS。已读双勾仍不在本条范围。 2026-09-15 对照 artifacts/agent-chat-voice-evaluation.html。密钥只进本机 .env，不入库、不进本表。 2026-09-15 20:12 用户选定硅基流动，已拆第一刀给 Bot。 2026-09-15 20:25 Bot 汇报 50b8054，改待确认。 2026-09-15 20:27 主路径可见，体验三条记 B-06。 2026-09-15 20:48 用户验收关闭语音部分。图片仍暂缓。 2026-09-15 夜交接：语音已关；后半聊天图/VLM/生图仍开、先不拆包。 2026-09-16：GLM 多模态方案 v1.2 已评估。采纳方向：朋友圈配图先于聊天发图、成本闸门、画风不一致禁直融、不引网关。不采纳为立刻动工基线：ComfyUI 工厂、千张采集、向量库、能力层大搬家。详见会话评估。 2026-09-16 用户验收：聊天发图正常。范围仅上传进气泡；未含 VLM/生图。 2026-09-16 远程聊天发图 8fa8669。VLM/生图仍不在远程。 2026-10-09 点收并 push 2981fa3..575967c。 2026-10-10 清备注：对应功能已在远程，去掉过期未合入表述。</t>
         </is>
       </c>
     </row>
@@ -2754,7 +2754,7 @@
       </c>
       <c r="K26" s="46" t="inlineStr">
         <is>
-          <t>有意未做：语音、多频道、资料页、表情附件、未读红点。未 push。 左栏图标第二轮已通过。</t>
+          <t>有意未做：语音、多频道、资料页、表情附件、未读红点。 左栏图标第二轮已通过。 2026-10-10 清备注：对应功能已在远程，去掉过期未合入表述。</t>
         </is>
       </c>
     </row>
@@ -3073,7 +3073,7 @@
       </c>
       <c r="G33" s="49" t="inlineStr">
         <is>
-          <t>2026-09-17 用户验收通过：默认关、tick 可发一条、未打开有红点、点进可见主动气泡。第一刀仅私聊。未 push。</t>
+          <t>2026-09-17 用户验收通过：默认关、tick 可发一条、未打开有红点、点进可见主动气泡。第一刀仅私聊。</t>
         </is>
       </c>
       <c r="H33" s="44" t="inlineStr">
@@ -3091,7 +3091,7 @@
       </c>
       <c r="K33" s="51" t="inlineStr">
         <is>
-          <t>用户 2026-09-15 19:40 提出。C-03 验收因此偏难，属产品缺口不是红点实现失败。 2026-09-16 设计备忘已写。模型可走 Ollama 或 DeepSeek，不按 9b 封顶。好感度另字段调制阈值，不进本条预设，不提前做图谱。 2026-09-17 用户指定开 C-05，顺带给 C-03 真实未读。 2026-09-17 Bot 汇报 76cec8e。tick JSON 已记。未 push。 2026-09-17 用户截图确认：未打开会话时列表预览+红点；点进可见主动气泡。关单仍等 C-03 清红点收口。 2026-09-17 与 C-03 一并关单。</t>
+          <t>用户 2026-09-15 19:40 提出。C-03 验收因此偏难，属产品缺口不是红点实现失败。 2026-09-16 设计备忘已写。模型可走 Ollama 或 DeepSeek，不按 9b 封顶。好感度另字段调制阈值，不进本条预设，不提前做图谱。 2026-09-17 用户指定开 C-05，顺带给 C-03 真实未读。 2026-09-17 Bot 汇报 76cec8e。tick JSON 已记。 2026-09-17 用户截图确认：未打开会话时列表预览+红点；点进可见主动气泡。关单仍等 C-03 清红点收口。 2026-09-17 与 C-03 一并关单。 2026-10-10 清备注：对应功能已在远程，去掉过期未合入表述。</t>
         </is>
       </c>
     </row>
@@ -3148,7 +3148,7 @@
       </c>
       <c r="K34" s="46" t="inlineStr">
         <is>
-          <t>用户截图小春私聊 20:24。已拆给 GrokBot。 2026-09-15 20:39 Bot 汇报 e19d757，改待确认。未 push。 2026-09-15 20:48 用户验收关闭。未 push。</t>
+          <t>用户截图小春私聊 20:24。已拆给 GrokBot。 2026-09-15 20:39 Bot 汇报 e19d757，改待确认。 2026-09-15 20:48 用户验收关闭。 2026-10-10 清备注：对应功能已在远程，去掉过期未合入表述。</t>
         </is>
       </c>
     </row>
@@ -3201,7 +3201,7 @@
       <c r="J35" s="44" t="n"/>
       <c r="K35" s="46" t="inlineStr">
         <is>
-          <t>用户 2026-09-15 20:50 提出。已拆给 GrokBot。 2026-09-15 20:52 用户补充：明确要求语音也可出气泡。 2026-09-15 21:08 用户截图验收关闭。未附 commit 哈希。未 push。</t>
+          <t>用户 2026-09-15 20:50 提出。已拆给 GrokBot。 2026-09-15 20:52 用户补充：明确要求语音也可出气泡。 2026-09-15 21:08 用户截图验收关闭。 2026-10-10 清备注：对应功能已在远程，去掉过期未合入表述。</t>
         </is>
       </c>
     </row>
@@ -3360,7 +3360,7 @@
       </c>
       <c r="K38" s="49" t="inlineStr">
         <is>
-          <t>2026-09-16 扫描只读清单已收。U-01 历史关单是「微信→酒馆」，现网标题已是 Agent Chat，本条不重开界面改名包。2026-09-16 问题表已更名为 AgentChat-问题记录.xlsx。 2026-09-16 Bot 汇报 a8ebcf9，ahead 1，未 push。docs/待优化点记录_一期.md 已改「未读红点/空间」但被 .gitignore（docs/*待优化点*.md）挡住，未进提交，本机磁盘已改。关单。 2026-09-16 对照 GitHub：main HEAD 7293da3（M-06），commit/a8ebcf9 为 404，O-02 文案尚未出现在远程 README/package.json/characterCard.ts。本地关单不变，远程未对齐。 2026-09-17 对照：main HEAD a8ebcf9，README/package.json 已去微信。远程对齐，维持已处理。</t>
+          <t>2026-09-16 扫描只读清单已收。U-01 历史关单是「微信→酒馆」，现网标题已是 Agent Chat，本条不重开界面改名包。2026-09-16 问题表已更名为 AgentChat-问题记录.xlsx。 2026-09-16 Bot 汇报 a8ebcf9，ahead 1，docs/待优化点记录_一期.md 已改「未读红点/空间」但被 .gitignore（docs/*待优化点*.md）挡住，未进提交，本机磁盘已改。关单。 2026-09-16 对照 GitHub：main HEAD 7293da3（M-06），commit/a8ebcf9 为 404，O-02 文案尚未出现在远程 README/package.json/characterCard.ts。本地关单不变，远程未对齐。 2026-09-17 对照：main HEAD a8ebcf9，README/package.json 已去微信。远程对齐，维持已处理。 2026-10-10 清备注：对应功能已在远程，去掉过期未合入表述。</t>
         </is>
       </c>
     </row>
@@ -3450,7 +3450,7 @@
       </c>
       <c r="G40" s="49" t="inlineStr">
         <is>
-          <t>2026-09-18 用户验收通过。改为聊天区右侧卡片：标题「记下了」+ 摘要（最多3条分号拼接），约10秒淡入淡出。不进消息流。本地 274e173 未 push。 已上远程 274e173。</t>
+          <t>2026-09-18 用户验收通过。改为聊天区右侧卡片：标题「记下了」+ 摘要（最多3条分号拼接），约10秒淡入淡出。不进消息流。本地 274e173 已上远程 274e173。</t>
         </is>
       </c>
       <c r="H40" s="57" t="n">
@@ -3466,7 +3466,7 @@
       </c>
       <c r="K40" s="51" t="inlineStr">
         <is>
-          <t>刷新进房第一次 GET 只建快照不提示。 2026-09-18 偏离原顶栏小字，按用户设计收口。需重启后端（新表字段）+ 硬刷新。 2026-09-18 远程 main HEAD 274e173。卡片约10s；前端 3–90s 阶梯轮询 notices。慢主要在第二次 LLM 提炼。</t>
+          <t>刷新进房第一次 GET 只建快照不提示。 2026-09-18 偏离原顶栏小字，按用户设计收口。需重启后端（新表字段）+ 硬刷新。 2026-09-18 远程 main HEAD 274e173。卡片约10s；前端 3–90s 阶梯轮询 notices。慢主要在第二次 LLM 提炼。 2026-10-10 清备注：对应功能已在远程，去掉过期未合入表述。</t>
         </is>
       </c>
     </row>
@@ -3913,12 +3913,12 @@
     <row r="8" ht="36" customHeight="1" s="41">
       <c r="A8" s="69" t="inlineStr">
         <is>
-          <t>2026-10-09：远程 tip 575967c（含 B-04A/B、R-04x）。BF M-01 2c2e897 仍未 push。</t>
+          <t>2026-10-10：远程 tip 5c8f652（含 M-01）。无待 push 功能刀。问题表已清过期「未 push」备注。</t>
         </is>
       </c>
       <c r="B8" s="70" t="inlineStr">
         <is>
-          <t>2026-10-09：远程 tip 575967c（含 B-04A/B、R-04x）。BF M-01 2c2e897 仍未 push。</t>
+          <t>2026-10-10：远程 tip 5c8f652（含 M-01）。无待 push 功能刀。问题表已清过期「未 push」备注。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: issue tracker remote-status column, N-01..03, tip sync
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -20,11 +20,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="24">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -187,8 +188,12 @@
       <color rgb="FF000000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -231,8 +236,13 @@
         <bgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E3D"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -299,6 +309,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D0D0D0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D0D0D0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D0D0D0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D0D0D0"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
@@ -310,7 +334,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="84">
+  <cellXfs count="88">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -555,6 +579,18 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1352,7 +1388,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K52"/>
+  <dimension ref="A1:L55"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="40" min="1" max="1"/>
@@ -1364,6 +1400,7 @@
     <col width="13" customWidth="1" style="40" min="8" max="9"/>
     <col width="14" customWidth="1" style="40" min="10" max="10"/>
     <col width="36" customWidth="1" style="40" min="11" max="11"/>
+    <col width="12" customWidth="1" style="41" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1" s="41">
@@ -1422,6 +1459,11 @@
           <t>维护备注</t>
         </is>
       </c>
+      <c r="L1" s="84" t="inlineStr">
+        <is>
+          <t>远程状态</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="51.75" customHeight="1" s="41">
       <c r="A2" s="44" t="inlineStr">
@@ -1479,6 +1521,11 @@
           <t>另有 57c2bce 修 .env.example 编码</t>
         </is>
       </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>已 push</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="51.75" customHeight="1" s="41">
       <c r="A3" s="44" t="inlineStr">
@@ -1532,6 +1579,11 @@
           <t>测试卡：samples/characters/linshen.json</t>
         </is>
       </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>已 push</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="51.75" customHeight="1" s="41">
       <c r="A4" s="44" t="inlineStr">
@@ -1585,6 +1637,11 @@
         </is>
       </c>
       <c r="K4" s="46" t="n"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>已 push</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="51.75" customHeight="1" s="41">
       <c r="A5" s="44" t="inlineStr">
@@ -1638,6 +1695,11 @@
         </is>
       </c>
       <c r="K5" s="46" t="n"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>已 push</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="51.75" customHeight="1" s="41">
       <c r="A6" s="44" t="inlineStr">
@@ -1695,6 +1757,11 @@
           <t>林深约 1.9s 回完。DeepSeek 通道不加该字段。</t>
         </is>
       </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>已 push</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="51.75" customHeight="1" s="41">
       <c r="A7" s="44" t="inlineStr">
@@ -1748,6 +1815,11 @@
         </is>
       </c>
       <c r="K7" s="47" t="n"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>已 push</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="51.75" customHeight="1" s="41">
       <c r="A8" s="44" t="inlineStr">
@@ -1805,6 +1877,11 @@
           <t>真头像拼图仍暂缓，见 B-03。</t>
         </is>
       </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>已 push</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="51.75" customHeight="1" s="41">
       <c r="A9" s="44" t="inlineStr">
@@ -1858,6 +1935,11 @@
           <t>E1 包。若 commit 未单独记录可补。</t>
         </is>
       </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>已 push</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="51.75" customHeight="1" s="41">
       <c r="A10" s="44" t="inlineStr">
@@ -1915,6 +1997,11 @@
           <t>本机已验 @小春 / @林深 / 私聊。</t>
         </is>
       </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>已 push</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="51.75" customHeight="1" s="41">
       <c r="A11" s="44" t="inlineStr">
@@ -1968,6 +2055,11 @@
           <t>2026-09-13 23:00 本机验收通过。</t>
         </is>
       </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>已 push</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="51.75" customHeight="1" s="41">
       <c r="A12" s="44" t="inlineStr">
@@ -2021,6 +2113,11 @@
           <t>E1。截图已见「冒险者公会-验收2」。</t>
         </is>
       </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>已 push</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="51.75" customHeight="1" s="41">
       <c r="A13" s="44" t="inlineStr">
@@ -2074,6 +2171,11 @@
           <t>E1。清空后不自动插开场白。</t>
         </is>
       </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>已 push</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="51.75" customHeight="1" s="41">
       <c r="A14" s="44" t="inlineStr">
@@ -2127,6 +2229,11 @@
           <t>若仍有两条「林深」「夜见」，保持待确认并让 Bot 补齐。 2026-09-14 左滑红底穿透已用 cb26e32 补实正面背景。 2026-09-14 23:15 用户验收关闭。</t>
         </is>
       </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>已 push</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="51.75" customHeight="1" s="41">
       <c r="A15" s="44" t="inlineStr">
@@ -2182,6 +2289,11 @@
           <t>原待优化点第 6 条。建议作为下一包。 2026-09-14 夜排期：C-02 确认后作为下一开发包。 2026-09-14 23:15 已拆给 GrokBot。 2026-09-15 19:27 用户：发送后立刻回会话列表无红点；朋友圈触发后也无红点。会话红点按 C-03 排查；空间红点不在本包。 2026-09-15 19:35 Bot 汇报 9381115，改待确认。 2026-09-15 19:40 造未读困难已记 C-05，不因此打回实现。 2026-09-15 22:05 交接：代码在但难造未读，挂 C-05，不打回实现、不新开开发包。 2026-09-16：主动互动设计已备忘，C-05 仍暂缓；未读验收仍挂主动。 2026-09-17 C-05 第一刀开工，验收时一并看红点。 2026-09-17 C-05 已能写入 source=proactive 且不 markRead。等用户离开会话看列表红点后关单。 2026-09-17 用户截图：未选会话时林深有红点1；点进私聊气泡已有主动句，列表红点仍在。 2026-09-17 用户确认验收通过，关单。 2026-10-10 清备注：对应功能已在远程，去掉过期未合入表述。</t>
         </is>
       </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>已 push</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="51.75" customHeight="1" s="41">
       <c r="A16" s="44" t="inlineStr">
@@ -2239,6 +2351,11 @@
           <t>原待优化点第 3 条。先确认 PNG/JSON 导入都可用。 2026-09-14 夜排期：排在 C-03 之后；覆盖前先确认 JSON/PNG 导入。 2026-09-15 19:43 用户复现重复导入，已拆给 GrokBot。 2026-09-15 19:51 Bot 汇报 501e788，改待确认。 2026-09-15 19:56 用户验收关闭。 2026-10-10 清备注：对应功能已在远程，去掉过期未合入表述。</t>
         </is>
       </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>已 push</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="51.75" customHeight="1" s="41">
       <c r="A17" s="44" t="inlineStr">
@@ -2292,6 +2409,11 @@
       <c r="K17" s="46" t="inlineStr">
         <is>
           <t>原待优化点第 5 条的小方案。 2026-09-16：与 M-07 不同——M-01 是用户评角色动态后作者再回。 2026-10-09 点收； 2026-10-10 备注对齐：已 push，commit=5c8f652。</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>已 push</t>
         </is>
       </c>
     </row>
@@ -2340,7 +2462,12 @@
       <c r="J18" s="44" t="n"/>
       <c r="K18" s="46" t="inlineStr">
         <is>
-          <t>原待优化点第 5 条的大方案。 2026-09-16：图谱/互评仍晚于好感度与 C-05/M-07。</t>
+          <t>触发：好感度 R-03 立后，再做角色互评/图谱。 原待优化点第 5 条的大方案。</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>不适用</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2514,16 @@
       </c>
       <c r="I19" s="44" t="n"/>
       <c r="J19" s="44" t="n"/>
-      <c r="K19" s="47" t="n"/>
+      <c r="K19" s="47" t="inlineStr">
+        <is>
+          <t>触发：C-05/M-07 稳定且用户明确要定时自动发动态后再开。</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="51.75" customHeight="1" s="41">
       <c r="A20" s="44" t="inlineStr">
@@ -2439,6 +2575,11 @@
           <t>明天使用时顺手验即可，不一定要先开发。 2026-09-14 夜排期：用户顺手实测，先不单开开发包。 2026-09-14 23:15 澄清：不要按「导入后必须出现照片头像」验收。 2026-09-17 用户确认验证已过，关单。</t>
         </is>
       </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>已 push</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="51.75" customHeight="1" s="41">
       <c r="A21" s="44" t="inlineStr">
@@ -2492,6 +2633,11 @@
           <t>用一用再决定要不要补。 已从「是否完整」升级为明确需求。</t>
         </is>
       </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>已 push</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="51.75" customHeight="1" s="41">
       <c r="A22" s="44" t="inlineStr">
@@ -2547,6 +2693,11 @@
           <t xml:space="preserve"> 2026-09-16：远程已有上传头像拼贴（506b244 / 325fdec），产品未点收，保持暂缓。与 U-05 上传验收分开。 2026-09-17 用户验收关闭。</t>
         </is>
       </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>已 push</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="51.75" customHeight="1" s="41">
       <c r="A23" s="44" t="inlineStr">
@@ -2602,6 +2753,11 @@
           <t>用户 2026-09-14 明确提出。含图片，不限于 TTS。已读双勾仍不在本条范围。 2026-09-15 对照 artifacts/agent-chat-voice-evaluation.html。密钥只进本机 .env，不入库、不进本表。 2026-09-15 20:12 用户选定硅基流动，已拆第一刀给 Bot。 2026-09-15 20:25 Bot 汇报 50b8054，改待确认。 2026-09-15 20:27 主路径可见，体验三条记 B-06。 2026-09-15 20:48 用户验收关闭语音部分。图片仍暂缓。 2026-09-15 夜交接：语音已关；后半聊天图/VLM/生图仍开、先不拆包。 2026-09-16：GLM 多模态方案 v1.2 已评估。采纳方向：朋友圈配图先于聊天发图、成本闸门、画风不一致禁直融、不引网关。不采纳为立刻动工基线：ComfyUI 工厂、千张采集、向量库、能力层大搬家。详见会话评估。 2026-09-16 用户验收：聊天发图正常。范围仅上传进气泡；未含 VLM/生图。 2026-09-16 远程聊天发图 8fa8669。VLM/生图仍不在远程。 2026-10-09 点收并 push 2981fa3..575967c。 2026-10-10 清备注：对应功能已在远程，去掉过期未合入表述。</t>
         </is>
       </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>已 push</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="51.75" customHeight="1" s="41">
       <c r="A24" s="44" t="inlineStr">
@@ -2634,7 +2790,11 @@
           <t>第一期桌面浅色微信风已够用。</t>
         </is>
       </c>
-      <c r="G24" s="47" t="n"/>
+      <c r="G24" s="47" t="inlineStr">
+        <is>
+          <t>明确暂缓。U-05 浅色预设已关，不含整站深色。</t>
+        </is>
+      </c>
       <c r="H24" s="44" t="inlineStr">
         <is>
           <t>2026-09-13</t>
@@ -2644,7 +2804,12 @@
       <c r="J24" s="44" t="n"/>
       <c r="K24" s="46" t="inlineStr">
         <is>
-          <t>完整皮肤体系见 U-05。</t>
+          <t>触发：用户明确要整站深色或移动端适配后再开。（U-05 已关，原「完整皮肤体系见 U-05」备注失效。）</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>不适用</t>
         </is>
       </c>
     </row>
@@ -2700,6 +2865,11 @@
           <t>不要把 token 写入本表。 2026-09-14 夜排期：与 C-02 同批由用户确认。 2026-09-14 23:15 用户确认关闭。不要把 token 写入本表。 2026-09-16 再对照：公开 main HEAD 7293da3（M-06）。O-02 a8ebcf9 仍不在远程。</t>
         </is>
       </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>已 push</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="51.75" customHeight="1" s="41">
       <c r="A26" s="44" t="inlineStr">
@@ -2755,6 +2925,11 @@
       <c r="K26" s="46" t="inlineStr">
         <is>
           <t>有意未做：语音、多频道、资料页、表情附件、未读红点。 左栏图标第二轮已通过。 2026-10-10 清备注：对应功能已在远程，去掉过期未合入表述。</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>已 push</t>
         </is>
       </c>
     </row>
@@ -2764,8 +2939,6 @@
       <c r="C27" s="47" t="n"/>
       <c r="D27" s="47" t="n"/>
       <c r="E27" s="47" t="n"/>
-      <c r="F27" s="53" t="n"/>
-      <c r="G27" s="54" t="n"/>
       <c r="H27" s="47" t="n"/>
       <c r="I27" s="47" t="n"/>
       <c r="J27" s="47" t="n"/>
@@ -2827,6 +3000,11 @@
           <t>用户 2026-09-14 提出。与 B-03、B-05 相关但范围更大，单独立项。 2026-09-15 21:10 用户开第一刀上传；画师 Bot 后补视觉。 2026-09-15 夜：用户确认前半本机通过。后半预设/透明度先不拆包。 2026-09-16 用户再次确认：头像/背景上传为 9-15 后加，已验证。远程另有 38714ad 气泡头像、437ad16 群成员头像。后半主题预设/透明度仍开。 2026-09-16 用户指定先做后半主题/透明度，再做用户发动态。 2026-09-16 用户截图：外观入口已在主页，但整壳变窄居中，两侧空白。未验收。拆回铺满视口。 2026-09-16 用户第二张截图验收：宽度已修，外观可用。关闭 U-05。 2026-09-16 远程已有主题预设 570d3a3、铺满视口 d448674。</t>
         </is>
       </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>已 push</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="55.5" customHeight="1" s="41">
       <c r="A29" s="44" t="inlineStr">
@@ -2878,6 +3056,11 @@
       <c r="K29" s="46" t="inlineStr">
         <is>
           <t>可单独开一小包给 Grok Bot。 2026-09-14 截图验收：功能在，视觉未收。</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>已 push</t>
         </is>
       </c>
     </row>
@@ -2926,7 +3109,12 @@
       <c r="J30" s="44" t="n"/>
       <c r="K30" s="46" t="inlineStr">
         <is>
-          <t>用户 2026-09-14 提出。生成配图依赖 B-04，纯上传配图可更早。 2026-09-15 评估页把空间配图放在语音之后的 P3，与 B-04 生图一起，默认关闭。 2026-09-15 夜：保持打开/暂缓，先不拆包。 2026-09-16：GLM 多模态方案 v1.2 已评估。采纳方向：朋友圈配图先于聊天发图、成本闸门、画风不一致禁直融、不引网关。不采纳为立刻动工基线：ComfyUI 工厂、千张采集、向量库、能力层大搬家。详见会话评估。 2026-09-16 产品判断：现网用户不能发动态，只有「让 TA 发一条」。无生图时给角色动态配用户相册图不成立。M-05 不拆上传包；若要配图需先做用户发动态，或等生图。</t>
+          <t>触发：生图成本闸门可接受，或先做仅上传配图后再开。 用户 2026-09-14 提出。生成配图依赖 B-04；纯上传可更早。 2026-09-16 产品判断：无生图时给角色动态配用户相册图不成立；若要配图需用户发动态（M-06 已关）或等生图。</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>不适用</t>
         </is>
       </c>
     </row>
@@ -2982,6 +3170,11 @@
           <t>点整行或主按钮进私聊；动态入口降级改文案。</t>
         </is>
       </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>已 push</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="55.5" customHeight="1" s="41">
       <c r="A32" s="44" t="inlineStr">
@@ -3039,6 +3232,11 @@
           <t>用户 2026-09-14 23:00 提出，先记不开发。 2026-09-14 夜排期：P1 收口后再开。 2026-09-15 夜：保持打开，先不拆包。 2026-09-16 用户指定开第一刀；要求 AI 也能按个性/会话选表情。 2026-09-16 用户：角色每句都带表情。拆收口包：默认不带 + 落库前限 1 个 + 连续回复去刷。 2026-09-16 用户确认：先前每句都带是因为自己先发表情；镜像回复符合口径。关闭。 2026-09-16 远程 5c8fa33 / da45e5b。</t>
         </is>
       </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>已 push</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="21.75" customHeight="1" s="41">
       <c r="A33" s="44" t="inlineStr">
@@ -3094,6 +3292,11 @@
           <t>用户 2026-09-15 19:40 提出。C-03 验收因此偏难，属产品缺口不是红点实现失败。 2026-09-16 设计备忘已写。模型可走 Ollama 或 DeepSeek，不按 9b 封顶。好感度另字段调制阈值，不进本条预设，不提前做图谱。 2026-09-17 用户指定开 C-05，顺带给 C-03 真实未读。 2026-09-17 Bot 汇报 76cec8e。tick JSON 已记。 2026-09-17 用户截图确认：未打开会话时列表预览+红点；点进可见主动气泡。关单仍等 C-03 清红点收口。 2026-09-17 与 C-03 一并关单。 2026-10-10 清备注：对应功能已在远程，去掉过期未合入表述。</t>
         </is>
       </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>已 push</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="21.75" customHeight="1" s="41">
       <c r="A34" s="44" t="inlineStr">
@@ -3151,6 +3354,11 @@
           <t>用户截图小春私聊 20:24。已拆给 GrokBot。 2026-09-15 20:39 Bot 汇报 e19d757，改待确认。 2026-09-15 20:48 用户验收关闭。 2026-10-10 清备注：对应功能已在远程，去掉过期未合入表述。</t>
         </is>
       </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>已 push</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="21.75" customHeight="1" s="41">
       <c r="A35" s="44" t="inlineStr">
@@ -3204,6 +3412,11 @@
           <t>用户 2026-09-15 20:50 提出。已拆给 GrokBot。 2026-09-15 20:52 用户补充：明确要求语音也可出气泡。 2026-09-15 21:08 用户截图验收关闭。 2026-10-10 清备注：对应功能已在远程，去掉过期未合入表述。</t>
         </is>
       </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>已 push</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="21.75" customHeight="1" s="41">
       <c r="A36" s="44" t="inlineStr">
@@ -3261,6 +3474,11 @@
           <t>用户 2026-09-16 指定：先 U-05 后半，再用户发动态。 已拆给 GrokBot。互动回赞回评另立 M-07 暂缓。 2026-09-16 夜交接：用户已说验收过，关单。未强制补 commit 哈希。 2026-09-16 远程 main 可见 7293da3。</t>
         </is>
       </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>已 push</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="21.75" customHeight="1" s="41">
       <c r="A37" s="44" t="inlineStr">
@@ -3270,7 +3488,7 @@
       </c>
       <c r="B37" s="55" t="inlineStr">
         <is>
-          <t>暂缓</t>
+          <t>已处理</t>
         </is>
       </c>
       <c r="C37" s="44" t="inlineStr">
@@ -3295,7 +3513,7 @@
       </c>
       <c r="G37" s="46" t="inlineStr">
         <is>
-          <t>等 M-06 验收后再开。赞可不走 LLM；评最多 1 人。延迟一小段，避免秒赞。</t>
+          <t>角色可对用户动态点赞/短评；全场每拍至多一人。已上远程 676802c / 2981fa3（M-07b 日 cap 展示与赞头像）。续债：空间反应与私聊主动日 cap 解耦见 C-06（待用户点头）。</t>
         </is>
       </c>
       <c r="H37" s="44" t="inlineStr">
@@ -3303,11 +3521,22 @@
           <t>2026-09-16</t>
         </is>
       </c>
-      <c r="I37" s="44" t="n"/>
-      <c r="J37" s="44" t="n"/>
+      <c r="I37" s="85" t="n">
+        <v>46282</v>
+      </c>
+      <c r="J37" s="44" t="inlineStr">
+        <is>
+          <t>676802c / 2981fa3</t>
+        </is>
+      </c>
       <c r="K37" s="46" t="inlineStr">
         <is>
-          <t>用户 2026-09-16 提出。产品判断：先记录，不补进已发出的 M-06 包。 2026-09-16 与 C-05 共用主动互动备忘；出口不同，不合并开发包。</t>
+          <t>用户 2026-09-16 提出。产品判断：先记录，不补进已发出的 M-06 包。 2026-09-16 与 C-05 共用主动互动备忘；出口不同，不合并开发包。 2026-10-10：表状态对齐远程——功能已上 2981fa3；续债见 C-06，勿再标暂缓。</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>已 push</t>
         </is>
       </c>
     </row>
@@ -3363,6 +3592,11 @@
           <t>2026-09-16 扫描只读清单已收。U-01 历史关单是「微信→酒馆」，现网标题已是 Agent Chat，本条不重开界面改名包。2026-09-16 问题表已更名为 AgentChat-问题记录.xlsx。 2026-09-16 Bot 汇报 a8ebcf9，ahead 1，docs/待优化点记录_一期.md 已改「未读红点/空间」但被 .gitignore（docs/*待优化点*.md）挡住，未进提交，本机磁盘已改。关单。 2026-09-16 对照 GitHub：main HEAD 7293da3（M-06），commit/a8ebcf9 为 404，O-02 文案尚未出现在远程 README/package.json/characterCard.ts。本地关单不变，远程未对齐。 2026-09-17 对照：main HEAD a8ebcf9，README/package.json 已去微信。远程对齐，维持已处理。 2026-10-10 清备注：对应功能已在远程，去掉过期未合入表述。</t>
         </is>
       </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>已 push</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="48" customHeight="1" s="41">
       <c r="A39" s="49" t="inlineStr">
@@ -3416,6 +3650,11 @@
           <t>用户确认先功能后换栈。注入函数按角色取 N 条。C-05 不改采样器。 2026-09-18 Bot 汇报。另有一条 habit「静坐片刻」像角色口吻，第一刀可记，不打回。 2026-09-18 用户截图：林深「喝点什么」回温水、小春出门/洗衣同分钟完成。指出时距太短，近窗与私档分不清。验收应再做「冲掉近窗」后再问。 2026-09-18 已上远程 main e3c7fa3。提炼：无私聊触发词，每轮助手成功回复后 setImmediate；ops:[] 则不写。 偏好被写成「晚上喝茶时喝温水」。habit 像角色口吻。 2026-09-18 评估：失效主因是抽取把「公子／唤我深／无需新增」写成用户偏好并 supersede 小林；次因是坏楼层压过注入。风险：sticky 解析名、模型偶发忽略、history 里仍有公子、启发式过滤换角色可能漏。 2026-09-18 远程 274e173..dc7cab1 已齐。</t>
         </is>
       </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>已 push</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="39.75" customHeight="1" s="41">
       <c r="A40" s="49" t="inlineStr">
@@ -3467,6 +3706,11 @@
       <c r="K40" s="51" t="inlineStr">
         <is>
           <t>刷新进房第一次 GET 只建快照不提示。 2026-09-18 偏离原顶栏小字，按用户设计收口。需重启后端（新表字段）+ 硬刷新。 2026-09-18 远程 main HEAD 274e173。卡片约10s；前端 3–90s 阶梯轮询 notices。慢主要在第二次 LLM 提炼。 2026-10-10 清备注：对应功能已在远程，去掉过期未合入表述。</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>已 push</t>
         </is>
       </c>
     </row>
@@ -3513,7 +3757,12 @@
       <c r="J41" s="49" t="n"/>
       <c r="K41" s="51" t="inlineStr">
         <is>
-          <t>先做 R-02 注入必答补丁。 2026-10-09 R-04x 尖兵 575967c 已上远程（夹具报告+默认 off；Laya 本机已装不强开）。分模型正式刀仍暂缓。</t>
+          <t>触发：用户明确要对话/提炼分通道后再开正式刀。 R-04x 尖兵 575967c 已完（夹具报告+默认 off）；不强开真 Laya。 先做 R-02 注入必答补丁（已关）。</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>不适用</t>
         </is>
       </c>
     </row>
@@ -3569,6 +3818,11 @@
           <t>对照 dc7cab1..978ef23。用记忆回复仍主要靠提示词（honor/sticky/【你记得的事】），无回复后处理。写路径另见 R-05。2026-09-20 关单。 2026-09-20 续刀 R-06b 已上远程 8dbde43：口渴／想喝等场景门控用饮品记忆，勿另编山泉茶。未单独立项。</t>
         </is>
       </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>已 push</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="87.75" customHeight="1" s="41">
       <c r="A43" s="59" t="inlineStr">
@@ -3622,6 +3876,11 @@
           <t>2026-09-20 第二刀待用户点收。未改 R-06/U-07/C-05/表结构。禁止代 push。 2026-09-20 用户群聊点收第二刀；编码Bot 待 push f8f0084。 2026-09-20 编码Bot 已 push ab112be..f8f0084，远程 tip=f8f0084。</t>
         </is>
       </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>已 push</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="43.5" customHeight="1" s="41">
       <c r="A44" s="40" t="inlineStr">
@@ -3675,66 +3934,193 @@
           <t>不强开真 Laya；正式分模型仍见 R-04。</t>
         </is>
       </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>已 push</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="41">
-      <c r="A45" s="47" t="inlineStr">
+      <c r="A45" s="86" t="inlineStr">
+        <is>
+          <t>N-01</t>
+        </is>
+      </c>
+      <c r="B45" s="86" t="inlineStr">
+        <is>
+          <t>暂缓</t>
+        </is>
+      </c>
+      <c r="C45" s="86" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D45" s="86" t="inlineStr">
+        <is>
+          <t>工程</t>
+        </is>
+      </c>
+      <c r="E45" s="86" t="inlineStr">
+        <is>
+          <t>生图素材库 + 检索决策 + 生成入库</t>
+        </is>
+      </c>
+      <c r="F45" s="86" t="inlineStr">
+        <is>
+          <t>规划占位：建生图素材库，检索决策后再生成并入库复用。</t>
+        </is>
+      </c>
+      <c r="G45" s="86" t="inlineStr">
+        <is>
+          <t>明确暂缓，先占位不拆包。</t>
+        </is>
+      </c>
+      <c r="H45" s="87" t="n">
+        <v>46305</v>
+      </c>
+      <c r="I45" s="86" t="n"/>
+      <c r="J45" s="86" t="n"/>
+      <c r="K45" s="86" t="inlineStr">
+        <is>
+          <t>来源：用户 2026-10-10 规划占位。触发：B-04 生图稳定且用户要素材复用/成本闸门后再开。</t>
+        </is>
+      </c>
+      <c r="L45" s="86" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="15" customHeight="1" s="41">
+      <c r="A46" s="86" t="inlineStr">
+        <is>
+          <t>N-02</t>
+        </is>
+      </c>
+      <c r="B46" s="86" t="inlineStr">
+        <is>
+          <t>暂缓</t>
+        </is>
+      </c>
+      <c r="C46" s="86" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D46" s="86" t="inlineStr">
+        <is>
+          <t>工程</t>
+        </is>
+      </c>
+      <c r="E46" s="86" t="inlineStr">
+        <is>
+          <t>动态模型路由（Nano Banana / GPT Image / Qwen）</t>
+        </is>
+      </c>
+      <c r="F46" s="86" t="inlineStr">
+        <is>
+          <t>规划占位：按场景在多生图/多模态模型间动态路由。</t>
+        </is>
+      </c>
+      <c r="G46" s="86" t="inlineStr">
+        <is>
+          <t>明确暂缓，先占位不拆包。</t>
+        </is>
+      </c>
+      <c r="H46" s="87" t="n">
+        <v>46305</v>
+      </c>
+      <c r="I46" s="86" t="n"/>
+      <c r="J46" s="86" t="n"/>
+      <c r="K46" s="86" t="inlineStr">
+        <is>
+          <t>来源：用户 2026-10-10 规划占位。触发：用户选定多模型供应商与路由规则后再开。</t>
+        </is>
+      </c>
+      <c r="L46" s="86" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="15" customHeight="1" s="41">
+      <c r="A47" s="86" t="inlineStr">
+        <is>
+          <t>N-03</t>
+        </is>
+      </c>
+      <c r="B47" s="86" t="inlineStr">
+        <is>
+          <t>暂缓</t>
+        </is>
+      </c>
+      <c r="C47" s="86" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D47" s="86" t="inlineStr">
+        <is>
+          <t>工程</t>
+        </is>
+      </c>
+      <c r="E47" s="86" t="inlineStr">
+        <is>
+          <t>账单统计（按模型/功能/复用 vs 生成）</t>
+        </is>
+      </c>
+      <c r="F47" s="86" t="inlineStr">
+        <is>
+          <t>规划占位：按模型、功能、素材复用 vs 新生成统计用量与费用。</t>
+        </is>
+      </c>
+      <c r="G47" s="86" t="inlineStr">
+        <is>
+          <t>明确暂缓，先占位不拆包。</t>
+        </is>
+      </c>
+      <c r="H47" s="87" t="n">
+        <v>46305</v>
+      </c>
+      <c r="I47" s="86" t="n"/>
+      <c r="J47" s="86" t="n"/>
+      <c r="K47" s="86" t="inlineStr">
+        <is>
+          <t>来源：用户 2026-10-10 规划占位。触发：生图/多模型正式启用且用户要看账单后再开。</t>
+        </is>
+      </c>
+      <c r="L47" s="86" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="15" customHeight="1" s="41">
+      <c r="A48" s="47" t="inlineStr">
         <is>
           <t>U-xx</t>
         </is>
       </c>
-      <c r="B45" s="47" t="n"/>
-      <c r="C45" s="47" t="n"/>
-      <c r="D45" s="47" t="n"/>
-      <c r="E45" s="46" t="inlineStr">
-        <is>
-          <t>（在此行往下追加新问题。ID 建议：U 界面 / G 群聊 / C 会话 / M 朋友圈 / R 角色 / B 体验 / O 工程）</t>
-        </is>
-      </c>
-      <c r="F45" s="47" t="n"/>
-      <c r="G45" s="47" t="n"/>
-      <c r="H45" s="47" t="n"/>
-      <c r="I45" s="47" t="n"/>
-      <c r="J45" s="47" t="n"/>
-      <c r="K45" s="47" t="n"/>
-    </row>
-    <row r="46" ht="15" customHeight="1" s="41">
-      <c r="A46" s="47" t="n"/>
-      <c r="B46" s="47" t="n"/>
-      <c r="C46" s="47" t="n"/>
-      <c r="D46" s="47" t="n"/>
-      <c r="E46" s="47" t="n"/>
-      <c r="F46" s="47" t="n"/>
-      <c r="G46" s="47" t="n"/>
-      <c r="H46" s="47" t="n"/>
-      <c r="I46" s="47" t="n"/>
-      <c r="J46" s="47" t="n"/>
-      <c r="K46" s="47" t="n"/>
-    </row>
-    <row r="47" ht="15" customHeight="1" s="41">
-      <c r="A47" s="47" t="n"/>
-      <c r="B47" s="47" t="n"/>
-      <c r="C47" s="47" t="n"/>
-      <c r="D47" s="47" t="n"/>
-      <c r="E47" s="47" t="n"/>
-      <c r="F47" s="47" t="n"/>
-      <c r="G47" s="47" t="n"/>
-      <c r="H47" s="47" t="n"/>
-      <c r="I47" s="47" t="n"/>
-      <c r="J47" s="47" t="n"/>
-      <c r="K47" s="47" t="n"/>
-    </row>
-    <row r="48" ht="15" customHeight="1" s="41">
-      <c r="A48" s="47" t="n"/>
       <c r="B48" s="47" t="n"/>
       <c r="C48" s="47" t="n"/>
       <c r="D48" s="47" t="n"/>
-      <c r="E48" s="47" t="n"/>
+      <c r="E48" s="46" t="inlineStr">
+        <is>
+          <t>（在此行往下追加新问题。ID 建议：U 界面 / G 群聊 / C 会话 / M 朋友圈 / R 角色 / B 体验 / O 工程）</t>
+        </is>
+      </c>
       <c r="F48" s="47" t="n"/>
       <c r="G48" s="47" t="n"/>
       <c r="H48" s="47" t="n"/>
       <c r="I48" s="47" t="n"/>
       <c r="J48" s="47" t="n"/>
       <c r="K48" s="47" t="n"/>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="41">
       <c r="A49" s="47" t="n"/>
@@ -3788,11 +4174,47 @@
       <c r="J52" s="47" t="n"/>
       <c r="K52" s="47" t="n"/>
     </row>
+    <row r="53">
+      <c r="A53" s="47" t="n"/>
+      <c r="B53" s="47" t="n"/>
+      <c r="C53" s="47" t="n"/>
+      <c r="D53" s="47" t="n"/>
+      <c r="E53" s="47" t="n"/>
+      <c r="F53" s="47" t="n"/>
+      <c r="G53" s="47" t="n"/>
+      <c r="H53" s="47" t="n"/>
+      <c r="I53" s="47" t="n"/>
+      <c r="J53" s="47" t="n"/>
+      <c r="K53" s="47" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="47" t="n"/>
+      <c r="B54" s="47" t="n"/>
+      <c r="C54" s="47" t="n"/>
+      <c r="D54" s="47" t="n"/>
+      <c r="E54" s="47" t="n"/>
+      <c r="F54" s="47" t="n"/>
+      <c r="G54" s="47" t="n"/>
+      <c r="H54" s="47" t="n"/>
+      <c r="I54" s="47" t="n"/>
+      <c r="J54" s="47" t="n"/>
+      <c r="K54" s="47" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="47" t="n"/>
+      <c r="B55" s="47" t="n"/>
+      <c r="C55" s="47" t="n"/>
+      <c r="D55" s="47" t="n"/>
+      <c r="E55" s="47" t="n"/>
+      <c r="F55" s="47" t="n"/>
+      <c r="G55" s="47" t="n"/>
+      <c r="H55" s="47" t="n"/>
+      <c r="I55" s="47" t="n"/>
+      <c r="J55" s="47" t="n"/>
+      <c r="K55" s="47" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K40"/>
-  <mergeCells count="1">
-    <mergeCell ref="E27:G27"/>
-  </mergeCells>
   <conditionalFormatting sqref="B2:B80">
     <cfRule type="cellIs" rank="0" priority="2" equalAverage="0" operator="equal" aboveAverage="0" dxfId="9" text="" percent="0" bottom="0">
       <formula>"已处理"</formula>
@@ -3841,7 +4263,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="16" customWidth="1" style="40" min="1" max="1"/>
@@ -3862,6 +4284,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="41">
       <c r="A4" s="68" t="inlineStr">
         <is>
@@ -3911,68 +4334,77 @@
       </c>
     </row>
     <row r="8" ht="36" customHeight="1" s="41">
-      <c r="A8" s="69" t="inlineStr">
-        <is>
-          <t>2026-10-10：远程 tip 5c8f652（含 M-01）。无待 push 功能刀。问题表已清过期「未 push」备注。</t>
-        </is>
-      </c>
-      <c r="B8" s="70" t="inlineStr">
-        <is>
-          <t>2026-10-10：远程 tip 5c8f652（含 M-01）。无待 push 功能刀。问题表已清过期「未 push」备注。</t>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>远程状态（L 列）</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>已 push＝已合入远程；未 push＝仅本机；不适用＝暂缓未开工/规划占位/非功能行。</t>
         </is>
       </c>
     </row>
     <row r="9" ht="36" customHeight="1" s="41">
       <c r="A9" s="69" t="inlineStr">
         <is>
-          <t>不要写进表的</t>
-        </is>
-      </c>
-      <c r="B9" s="71" t="inlineStr">
-        <is>
-          <t>GitHub token、DeepSeek Key、.env 内容。Commit 只写短哈希。</t>
-        </is>
-      </c>
+          <t>2026-10-10：功能远程 tip 5c8f652（含 M-01）；文档 tip 以最新 docs commit 为准（本文件随 docs 更新）。无待 push 功能刀。下一候选：C-06 空间反应与私聊主动日 cap 解耦（待用户点头）；另可选 daily_cap UI / R-03 好感度（勿与 N-01..03 混淆）。</t>
+        </is>
+      </c>
+      <c r="B9" s="70" t="n"/>
     </row>
     <row r="10" ht="36" customHeight="1" s="41">
       <c r="A10" s="69" t="inlineStr">
         <is>
+          <t>不要写进表的</t>
+        </is>
+      </c>
+      <c r="B10" s="71" t="inlineStr">
+        <is>
+          <t>GitHub token、DeepSeek Key、.env 内容。Commit 只写短哈希。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="69" t="inlineStr">
+        <is>
           <t>和代码的关系</t>
         </is>
       </c>
-      <c r="B10" s="70" t="inlineStr">
-        <is>
-          <t>已处理行尽量补「本地 commit」。未 push 的也先记下哈希，push 后可在备注写已上远程。</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="15" customHeight="1" s="41">
-      <c r="A12" s="72" t="inlineStr">
+      <c r="B11" s="70" t="inlineStr">
+        <is>
+          <t>已处理行尽量补「本地 commit」与 L 列「远程状态」（已 push / 未 push / 不适用）。每次 push 后同步：本地 commit、远程状态、使用说明顶部 tip。暂缓项写清触发条件；满足后改待处理。文档 commit 也记一笔。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="15" customHeight="1" s="41"/>
+    <row r="13">
+      <c r="A13" s="72" t="inlineStr">
         <is>
           <t>状态色例</t>
         </is>
       </c>
-      <c r="B12" s="73" t="inlineStr">
+      <c r="B13" s="73" t="inlineStr">
         <is>
           <t>待处理</t>
         </is>
       </c>
-      <c r="C12" s="74" t="inlineStr">
+      <c r="C13" s="74" t="inlineStr">
         <is>
           <t>处理中</t>
         </is>
       </c>
-      <c r="D12" s="74" t="inlineStr">
+      <c r="D13" s="74" t="inlineStr">
         <is>
           <t>待确认</t>
         </is>
       </c>
-      <c r="E12" s="75" t="inlineStr">
+      <c r="E13" s="75" t="inlineStr">
         <is>
           <t>已处理</t>
         </is>
       </c>
-      <c r="F12" s="76" t="inlineStr">
+      <c r="F13" s="76" t="inlineStr">
         <is>
           <t>暂缓</t>
         </is>
@@ -4126,48 +4558,84 @@
         <v/>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>未 push 条数</t>
+        </is>
+      </c>
+      <c r="B15">
+        <f>COUNTIF(问题记录!L:L,"未 push")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>已 push 条数</t>
+        </is>
+      </c>
+      <c r="B16">
+        <f>COUNTIF(问题记录!L:L,"已 push")</f>
+        <v/>
+      </c>
+    </row>
     <row r="17" ht="15" customHeight="1" s="41">
       <c r="A17" s="81" t="inlineStr">
         <is>
-          <t>明日建议顺序</t>
+          <t>待办自动列表（状态＝待处理/处理中）</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="41">
       <c r="A18" s="80" t="inlineStr">
         <is>
-          <t>1. R-05 已关闭：远程 tip f8f0084。</t>
-        </is>
+          <t>待处理/处理中条数</t>
+        </is>
+      </c>
+      <c r="B18">
+        <f>COUNTIF(问题记录!B:B,"待处理")+COUNTIF(问题记录!B:B,"处理中")</f>
+        <v/>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="41">
       <c r="A19" s="80" t="inlineStr">
         <is>
-          <t>2. 现行文档在 docs/product/（问题表+两份备忘），尚未 commit。</t>
-        </is>
+          <t>ID 列表（自动）</t>
+        </is>
+      </c>
+      <c r="B19">
+        <f>TEXTJOIN("；",TRUE,IF(((问题记录!B$2:B$200="待处理")+(问题记录!B$2:B$200="处理中"))&gt;0,问题记录!A$2:A$200&amp;" "&amp;问题记录!E$2:E$200,""))</f>
+        <v/>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="41">
       <c r="A20" s="80" t="inlineStr">
         <is>
-          <t>3. M-07 / R-04 仍暂缓。</t>
+          <t>下一候选（人工）</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>C-06 空间反应与私聊主动日 cap 解耦（待用户点头）。可选：daily_cap UI / R-03 好感度。勿与 N-01..03 规划占位混淆。</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="41">
       <c r="A21" s="80" t="inlineStr">
         <is>
-          <t>4. 远程 main HEAD f8f0084。</t>
+          <t>远程 tip（人工）</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>功能 tip 5c8f652；文档 tip 以最新 docs 为准。无待 push 功能刀。人工维护，最后更新 2026-10-10。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A18:D18"/>
+  <mergeCells count="2">
     <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A20:D20"/>
-    <mergeCell ref="A21:D21"/>
-    <mergeCell ref="A19:D19"/>
     <mergeCell ref="A2:C2"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>

</xml_diff>

<commit_message>
docs: close C-06 in issue tracker
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -1388,7 +1388,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L55"/>
+  <dimension ref="A1:L56"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="40" min="1" max="1"/>
@@ -1521,7 +1521,7 @@
           <t>另有 57c2bce 修 .env.example 编码</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="L2" s="40" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>
@@ -1579,7 +1579,7 @@
           <t>测试卡：samples/characters/linshen.json</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L3" s="40" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>
@@ -1637,7 +1637,7 @@
         </is>
       </c>
       <c r="K4" s="46" t="n"/>
-      <c r="L4" t="inlineStr">
+      <c r="L4" s="40" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>
@@ -1695,7 +1695,7 @@
         </is>
       </c>
       <c r="K5" s="46" t="n"/>
-      <c r="L5" t="inlineStr">
+      <c r="L5" s="40" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>
@@ -1757,7 +1757,7 @@
           <t>林深约 1.9s 回完。DeepSeek 通道不加该字段。</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="L6" s="40" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>
@@ -1815,7 +1815,7 @@
         </is>
       </c>
       <c r="K7" s="47" t="n"/>
-      <c r="L7" t="inlineStr">
+      <c r="L7" s="40" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>
@@ -1877,7 +1877,7 @@
           <t>真头像拼图仍暂缓，见 B-03。</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="L8" s="40" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>
@@ -1935,7 +1935,7 @@
           <t>E1 包。若 commit 未单独记录可补。</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="L9" s="40" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>
@@ -1997,7 +1997,7 @@
           <t>本机已验 @小春 / @林深 / 私聊。</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="L10" s="40" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>
@@ -2055,7 +2055,7 @@
           <t>2026-09-13 23:00 本机验收通过。</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="L11" s="40" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>
@@ -2113,7 +2113,7 @@
           <t>E1。截图已见「冒险者公会-验收2」。</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="L12" s="40" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>
@@ -2171,7 +2171,7 @@
           <t>E1。清空后不自动插开场白。</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="L13" s="40" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>
@@ -2229,7 +2229,7 @@
           <t>若仍有两条「林深」「夜见」，保持待确认并让 Bot 补齐。 2026-09-14 左滑红底穿透已用 cb26e32 补实正面背景。 2026-09-14 23:15 用户验收关闭。</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
+      <c r="L14" s="40" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>
@@ -2289,7 +2289,7 @@
           <t>原待优化点第 6 条。建议作为下一包。 2026-09-14 夜排期：C-02 确认后作为下一开发包。 2026-09-14 23:15 已拆给 GrokBot。 2026-09-15 19:27 用户：发送后立刻回会话列表无红点；朋友圈触发后也无红点。会话红点按 C-03 排查；空间红点不在本包。 2026-09-15 19:35 Bot 汇报 9381115，改待确认。 2026-09-15 19:40 造未读困难已记 C-05，不因此打回实现。 2026-09-15 22:05 交接：代码在但难造未读，挂 C-05，不打回实现、不新开开发包。 2026-09-16：主动互动设计已备忘，C-05 仍暂缓；未读验收仍挂主动。 2026-09-17 C-05 第一刀开工，验收时一并看红点。 2026-09-17 C-05 已能写入 source=proactive 且不 markRead。等用户离开会话看列表红点后关单。 2026-09-17 用户截图：未选会话时林深有红点1；点进私聊气泡已有主动句，列表红点仍在。 2026-09-17 用户确认验收通过，关单。 2026-10-10 清备注：对应功能已在远程，去掉过期未合入表述。</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="L15" s="40" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>
@@ -2351,7 +2351,7 @@
           <t>原待优化点第 3 条。先确认 PNG/JSON 导入都可用。 2026-09-14 夜排期：排在 C-03 之后；覆盖前先确认 JSON/PNG 导入。 2026-09-15 19:43 用户复现重复导入，已拆给 GrokBot。 2026-09-15 19:51 Bot 汇报 501e788，改待确认。 2026-09-15 19:56 用户验收关闭。 2026-10-10 清备注：对应功能已在远程，去掉过期未合入表述。</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
+      <c r="L16" s="40" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>
@@ -2411,7 +2411,7 @@
           <t>原待优化点第 5 条的小方案。 2026-09-16：与 M-07 不同——M-01 是用户评角色动态后作者再回。 2026-10-09 点收； 2026-10-10 备注对齐：已 push，commit=5c8f652。</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr">
+      <c r="L17" s="40" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>
@@ -2465,7 +2465,7 @@
           <t>触发：好感度 R-03 立后，再做角色互评/图谱。 原待优化点第 5 条的大方案。</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr">
+      <c r="L18" s="40" t="inlineStr">
         <is>
           <t>不适用</t>
         </is>
@@ -2519,7 +2519,7 @@
           <t>触发：C-05/M-07 稳定且用户明确要定时自动发动态后再开。</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr">
+      <c r="L19" s="40" t="inlineStr">
         <is>
           <t>不适用</t>
         </is>
@@ -2575,7 +2575,7 @@
           <t>明天使用时顺手验即可，不一定要先开发。 2026-09-14 夜排期：用户顺手实测，先不单开开发包。 2026-09-14 23:15 澄清：不要按「导入后必须出现照片头像」验收。 2026-09-17 用户确认验证已过，关单。</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr">
+      <c r="L20" s="40" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>
@@ -2633,7 +2633,7 @@
           <t>用一用再决定要不要补。 已从「是否完整」升级为明确需求。</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr">
+      <c r="L21" s="40" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>
@@ -2693,7 +2693,7 @@
           <t xml:space="preserve"> 2026-09-16：远程已有上传头像拼贴（506b244 / 325fdec），产品未点收，保持暂缓。与 U-05 上传验收分开。 2026-09-17 用户验收关闭。</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr">
+      <c r="L22" s="40" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>
@@ -2753,7 +2753,7 @@
           <t>用户 2026-09-14 明确提出。含图片，不限于 TTS。已读双勾仍不在本条范围。 2026-09-15 对照 artifacts/agent-chat-voice-evaluation.html。密钥只进本机 .env，不入库、不进本表。 2026-09-15 20:12 用户选定硅基流动，已拆第一刀给 Bot。 2026-09-15 20:25 Bot 汇报 50b8054，改待确认。 2026-09-15 20:27 主路径可见，体验三条记 B-06。 2026-09-15 20:48 用户验收关闭语音部分。图片仍暂缓。 2026-09-15 夜交接：语音已关；后半聊天图/VLM/生图仍开、先不拆包。 2026-09-16：GLM 多模态方案 v1.2 已评估。采纳方向：朋友圈配图先于聊天发图、成本闸门、画风不一致禁直融、不引网关。不采纳为立刻动工基线：ComfyUI 工厂、千张采集、向量库、能力层大搬家。详见会话评估。 2026-09-16 用户验收：聊天发图正常。范围仅上传进气泡；未含 VLM/生图。 2026-09-16 远程聊天发图 8fa8669。VLM/生图仍不在远程。 2026-10-09 点收并 push 2981fa3..575967c。 2026-10-10 清备注：对应功能已在远程，去掉过期未合入表述。</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr">
+      <c r="L23" s="40" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>
@@ -2807,7 +2807,7 @@
           <t>触发：用户明确要整站深色或移动端适配后再开。（U-05 已关，原「完整皮肤体系见 U-05」备注失效。）</t>
         </is>
       </c>
-      <c r="L24" t="inlineStr">
+      <c r="L24" s="40" t="inlineStr">
         <is>
           <t>不适用</t>
         </is>
@@ -2865,7 +2865,7 @@
           <t>不要把 token 写入本表。 2026-09-14 夜排期：与 C-02 同批由用户确认。 2026-09-14 23:15 用户确认关闭。不要把 token 写入本表。 2026-09-16 再对照：公开 main HEAD 7293da3（M-06）。O-02 a8ebcf9 仍不在远程。</t>
         </is>
       </c>
-      <c r="L25" t="inlineStr">
+      <c r="L25" s="40" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>
@@ -2927,7 +2927,7 @@
           <t>有意未做：语音、多频道、资料页、表情附件、未读红点。 左栏图标第二轮已通过。 2026-10-10 清备注：对应功能已在远程，去掉过期未合入表述。</t>
         </is>
       </c>
-      <c r="L26" t="inlineStr">
+      <c r="L26" s="40" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>
@@ -3000,7 +3000,7 @@
           <t>用户 2026-09-14 提出。与 B-03、B-05 相关但范围更大，单独立项。 2026-09-15 21:10 用户开第一刀上传；画师 Bot 后补视觉。 2026-09-15 夜：用户确认前半本机通过。后半预设/透明度先不拆包。 2026-09-16 用户再次确认：头像/背景上传为 9-15 后加，已验证。远程另有 38714ad 气泡头像、437ad16 群成员头像。后半主题预设/透明度仍开。 2026-09-16 用户指定先做后半主题/透明度，再做用户发动态。 2026-09-16 用户截图：外观入口已在主页，但整壳变窄居中，两侧空白。未验收。拆回铺满视口。 2026-09-16 用户第二张截图验收：宽度已修，外观可用。关闭 U-05。 2026-09-16 远程已有主题预设 570d3a3、铺满视口 d448674。</t>
         </is>
       </c>
-      <c r="L28" t="inlineStr">
+      <c r="L28" s="40" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>
@@ -3058,7 +3058,7 @@
           <t>可单独开一小包给 Grok Bot。 2026-09-14 截图验收：功能在，视觉未收。</t>
         </is>
       </c>
-      <c r="L29" t="inlineStr">
+      <c r="L29" s="40" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>
@@ -3112,7 +3112,7 @@
           <t>触发：生图成本闸门可接受，或先做仅上传配图后再开。 用户 2026-09-14 提出。生成配图依赖 B-04；纯上传可更早。 2026-09-16 产品判断：无生图时给角色动态配用户相册图不成立；若要配图需用户发动态（M-06 已关）或等生图。</t>
         </is>
       </c>
-      <c r="L30" t="inlineStr">
+      <c r="L30" s="40" t="inlineStr">
         <is>
           <t>不适用</t>
         </is>
@@ -3170,7 +3170,7 @@
           <t>点整行或主按钮进私聊；动态入口降级改文案。</t>
         </is>
       </c>
-      <c r="L31" t="inlineStr">
+      <c r="L31" s="40" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>
@@ -3232,7 +3232,7 @@
           <t>用户 2026-09-14 23:00 提出，先记不开发。 2026-09-14 夜排期：P1 收口后再开。 2026-09-15 夜：保持打开，先不拆包。 2026-09-16 用户指定开第一刀；要求 AI 也能按个性/会话选表情。 2026-09-16 用户：角色每句都带表情。拆收口包：默认不带 + 落库前限 1 个 + 连续回复去刷。 2026-09-16 用户确认：先前每句都带是因为自己先发表情；镜像回复符合口径。关闭。 2026-09-16 远程 5c8fa33 / da45e5b。</t>
         </is>
       </c>
-      <c r="L32" t="inlineStr">
+      <c r="L32" s="40" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>
@@ -3292,7 +3292,7 @@
           <t>用户 2026-09-15 19:40 提出。C-03 验收因此偏难，属产品缺口不是红点实现失败。 2026-09-16 设计备忘已写。模型可走 Ollama 或 DeepSeek，不按 9b 封顶。好感度另字段调制阈值，不进本条预设，不提前做图谱。 2026-09-17 用户指定开 C-05，顺带给 C-03 真实未读。 2026-09-17 Bot 汇报 76cec8e。tick JSON 已记。 2026-09-17 用户截图确认：未打开会话时列表预览+红点；点进可见主动气泡。关单仍等 C-03 清红点收口。 2026-09-17 与 C-03 一并关单。 2026-10-10 清备注：对应功能已在远程，去掉过期未合入表述。</t>
         </is>
       </c>
-      <c r="L33" t="inlineStr">
+      <c r="L33" s="40" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>
@@ -3354,7 +3354,7 @@
           <t>用户截图小春私聊 20:24。已拆给 GrokBot。 2026-09-15 20:39 Bot 汇报 e19d757，改待确认。 2026-09-15 20:48 用户验收关闭。 2026-10-10 清备注：对应功能已在远程，去掉过期未合入表述。</t>
         </is>
       </c>
-      <c r="L34" t="inlineStr">
+      <c r="L34" s="40" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>
@@ -3412,7 +3412,7 @@
           <t>用户 2026-09-15 20:50 提出。已拆给 GrokBot。 2026-09-15 20:52 用户补充：明确要求语音也可出气泡。 2026-09-15 21:08 用户截图验收关闭。 2026-10-10 清备注：对应功能已在远程，去掉过期未合入表述。</t>
         </is>
       </c>
-      <c r="L35" t="inlineStr">
+      <c r="L35" s="40" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>
@@ -3474,7 +3474,7 @@
           <t>用户 2026-09-16 指定：先 U-05 后半，再用户发动态。 已拆给 GrokBot。互动回赞回评另立 M-07 暂缓。 2026-09-16 夜交接：用户已说验收过，关单。未强制补 commit 哈希。 2026-09-16 远程 main 可见 7293da3。</t>
         </is>
       </c>
-      <c r="L36" t="inlineStr">
+      <c r="L36" s="40" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>
@@ -3534,7 +3534,7 @@
           <t>用户 2026-09-16 提出。产品判断：先记录，不补进已发出的 M-06 包。 2026-09-16 与 C-05 共用主动互动备忘；出口不同，不合并开发包。 2026-10-10：表状态对齐远程——功能已上 2981fa3；续债见 C-06，勿再标暂缓。</t>
         </is>
       </c>
-      <c r="L37" t="inlineStr">
+      <c r="L37" s="40" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>
@@ -3592,7 +3592,7 @@
           <t>2026-09-16 扫描只读清单已收。U-01 历史关单是「微信→酒馆」，现网标题已是 Agent Chat，本条不重开界面改名包。2026-09-16 问题表已更名为 AgentChat-问题记录.xlsx。 2026-09-16 Bot 汇报 a8ebcf9，ahead 1，docs/待优化点记录_一期.md 已改「未读红点/空间」但被 .gitignore（docs/*待优化点*.md）挡住，未进提交，本机磁盘已改。关单。 2026-09-16 对照 GitHub：main HEAD 7293da3（M-06），commit/a8ebcf9 为 404，O-02 文案尚未出现在远程 README/package.json/characterCard.ts。本地关单不变，远程未对齐。 2026-09-17 对照：main HEAD a8ebcf9，README/package.json 已去微信。远程对齐，维持已处理。 2026-10-10 清备注：对应功能已在远程，去掉过期未合入表述。</t>
         </is>
       </c>
-      <c r="L38" t="inlineStr">
+      <c r="L38" s="40" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>
@@ -3650,7 +3650,7 @@
           <t>用户确认先功能后换栈。注入函数按角色取 N 条。C-05 不改采样器。 2026-09-18 Bot 汇报。另有一条 habit「静坐片刻」像角色口吻，第一刀可记，不打回。 2026-09-18 用户截图：林深「喝点什么」回温水、小春出门/洗衣同分钟完成。指出时距太短，近窗与私档分不清。验收应再做「冲掉近窗」后再问。 2026-09-18 已上远程 main e3c7fa3。提炼：无私聊触发词，每轮助手成功回复后 setImmediate；ops:[] 则不写。 偏好被写成「晚上喝茶时喝温水」。habit 像角色口吻。 2026-09-18 评估：失效主因是抽取把「公子／唤我深／无需新增」写成用户偏好并 supersede 小林；次因是坏楼层压过注入。风险：sticky 解析名、模型偶发忽略、history 里仍有公子、启发式过滤换角色可能漏。 2026-09-18 远程 274e173..dc7cab1 已齐。</t>
         </is>
       </c>
-      <c r="L39" t="inlineStr">
+      <c r="L39" s="40" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>
@@ -3708,7 +3708,7 @@
           <t>刷新进房第一次 GET 只建快照不提示。 2026-09-18 偏离原顶栏小字，按用户设计收口。需重启后端（新表字段）+ 硬刷新。 2026-09-18 远程 main HEAD 274e173。卡片约10s；前端 3–90s 阶梯轮询 notices。慢主要在第二次 LLM 提炼。 2026-10-10 清备注：对应功能已在远程，去掉过期未合入表述。</t>
         </is>
       </c>
-      <c r="L40" t="inlineStr">
+      <c r="L40" s="40" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>
@@ -3760,7 +3760,7 @@
           <t>触发：用户明确要对话/提炼分通道后再开正式刀。 R-04x 尖兵 575967c 已完（夹具报告+默认 off）；不强开真 Laya。 先做 R-02 注入必答补丁（已关）。</t>
         </is>
       </c>
-      <c r="L41" t="inlineStr">
+      <c r="L41" s="40" t="inlineStr">
         <is>
           <t>不适用</t>
         </is>
@@ -3818,7 +3818,7 @@
           <t>对照 dc7cab1..978ef23。用记忆回复仍主要靠提示词（honor/sticky/【你记得的事】），无回复后处理。写路径另见 R-05。2026-09-20 关单。 2026-09-20 续刀 R-06b 已上远程 8dbde43：口渴／想喝等场景门控用饮品记忆，勿另编山泉茶。未单独立项。</t>
         </is>
       </c>
-      <c r="L42" t="inlineStr">
+      <c r="L42" s="40" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>
@@ -3876,7 +3876,7 @@
           <t>2026-09-20 第二刀待用户点收。未改 R-06/U-07/C-05/表结构。禁止代 push。 2026-09-20 用户群聊点收第二刀；编码Bot 待 push f8f0084。 2026-09-20 编码Bot 已 push ab112be..f8f0084，远程 tip=f8f0084。</t>
         </is>
       </c>
-      <c r="L43" t="inlineStr">
+      <c r="L43" s="40" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>
@@ -3934,68 +3934,74 @@
           <t>不强开真 Laya；正式分模型仍见 R-04。</t>
         </is>
       </c>
-      <c r="L44" t="inlineStr">
+      <c r="L44" s="40" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="41">
-      <c r="A45" s="86" t="inlineStr">
-        <is>
-          <t>N-01</t>
-        </is>
-      </c>
-      <c r="B45" s="86" t="inlineStr">
-        <is>
-          <t>暂缓</t>
-        </is>
-      </c>
-      <c r="C45" s="86" t="inlineStr">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>C-06</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>已处理</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="D45" s="86" t="inlineStr">
-        <is>
-          <t>工程</t>
-        </is>
-      </c>
-      <c r="E45" s="86" t="inlineStr">
-        <is>
-          <t>生图素材库 + 检索决策 + 生成入库</t>
-        </is>
-      </c>
-      <c r="F45" s="86" t="inlineStr">
-        <is>
-          <t>规划占位：建生图素材库，检索决策后再生成并入库复用。</t>
-        </is>
-      </c>
-      <c r="G45" s="86" t="inlineStr">
-        <is>
-          <t>明确暂缓，先占位不拆包。</t>
-        </is>
-      </c>
-      <c r="H45" s="87" t="n">
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>会话</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>空间赞评与私聊主动日 cap 解耦</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>sent_today 满后 M-07 空间结算被 daily_cap 跳过，用户发动态无角色赞评。</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>空间结算不再因 sent_today&gt;=daily_cap 跳过；私聊主动仍受日 cap；总开关关两边都停。2026-10-10 代验通过，已在远程 57e92bc。</t>
+        </is>
+      </c>
+      <c r="H45" s="83" t="n">
         <v>46305</v>
       </c>
-      <c r="I45" s="86" t="n"/>
-      <c r="J45" s="86" t="n"/>
-      <c r="K45" s="86" t="inlineStr">
-        <is>
-          <t>来源：用户 2026-10-10 规划占位。触发：B-04 生图稳定且用户要素材复用/成本闸门后再开。</t>
-        </is>
-      </c>
-      <c r="L45" s="86" t="inlineStr">
-        <is>
-          <t>不适用</t>
+      <c r="I45" s="83" t="n">
+        <v>46305</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>57e92bc</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>2026-10-10 点收并已在 origin。</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>已 push</t>
         </is>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="41">
       <c r="A46" s="86" t="inlineStr">
         <is>
-          <t>N-02</t>
+          <t>N-01</t>
         </is>
       </c>
       <c r="B46" s="86" t="inlineStr">
@@ -4015,12 +4021,12 @@
       </c>
       <c r="E46" s="86" t="inlineStr">
         <is>
-          <t>动态模型路由（Nano Banana / GPT Image / Qwen）</t>
+          <t>生图素材库 + 检索决策 + 生成入库</t>
         </is>
       </c>
       <c r="F46" s="86" t="inlineStr">
         <is>
-          <t>规划占位：按场景在多生图/多模态模型间动态路由。</t>
+          <t>规划占位：建生图素材库，检索决策后再生成并入库复用。</t>
         </is>
       </c>
       <c r="G46" s="86" t="inlineStr">
@@ -4035,7 +4041,7 @@
       <c r="J46" s="86" t="n"/>
       <c r="K46" s="86" t="inlineStr">
         <is>
-          <t>来源：用户 2026-10-10 规划占位。触发：用户选定多模型供应商与路由规则后再开。</t>
+          <t>来源：用户 2026-10-10 规划占位。触发：B-04 生图稳定且用户要素材复用/成本闸门后再开。</t>
         </is>
       </c>
       <c r="L46" s="86" t="inlineStr">
@@ -4047,7 +4053,7 @@
     <row r="47" ht="15" customHeight="1" s="41">
       <c r="A47" s="86" t="inlineStr">
         <is>
-          <t>N-03</t>
+          <t>N-02</t>
         </is>
       </c>
       <c r="B47" s="86" t="inlineStr">
@@ -4067,12 +4073,12 @@
       </c>
       <c r="E47" s="86" t="inlineStr">
         <is>
-          <t>账单统计（按模型/功能/复用 vs 生成）</t>
+          <t>动态模型路由（Nano Banana / GPT Image / Qwen）</t>
         </is>
       </c>
       <c r="F47" s="86" t="inlineStr">
         <is>
-          <t>规划占位：按模型、功能、素材复用 vs 新生成统计用量与费用。</t>
+          <t>规划占位：按场景在多生图/多模态模型间动态路由。</t>
         </is>
       </c>
       <c r="G47" s="86" t="inlineStr">
@@ -4087,53 +4093,92 @@
       <c r="J47" s="86" t="n"/>
       <c r="K47" s="86" t="inlineStr">
         <is>
+          <t>来源：用户 2026-10-10 规划占位。触发：用户选定多模型供应商与路由规则后再开。</t>
+        </is>
+      </c>
+      <c r="L47" s="86" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="15" customHeight="1" s="41">
+      <c r="A48" s="86" t="inlineStr">
+        <is>
+          <t>N-03</t>
+        </is>
+      </c>
+      <c r="B48" s="86" t="inlineStr">
+        <is>
+          <t>暂缓</t>
+        </is>
+      </c>
+      <c r="C48" s="86" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D48" s="86" t="inlineStr">
+        <is>
+          <t>工程</t>
+        </is>
+      </c>
+      <c r="E48" s="86" t="inlineStr">
+        <is>
+          <t>账单统计（按模型/功能/复用 vs 生成）</t>
+        </is>
+      </c>
+      <c r="F48" s="86" t="inlineStr">
+        <is>
+          <t>规划占位：按模型、功能、素材复用 vs 新生成统计用量与费用。</t>
+        </is>
+      </c>
+      <c r="G48" s="86" t="inlineStr">
+        <is>
+          <t>明确暂缓，先占位不拆包。</t>
+        </is>
+      </c>
+      <c r="H48" s="87" t="n">
+        <v>46305</v>
+      </c>
+      <c r="I48" s="86" t="n"/>
+      <c r="J48" s="86" t="n"/>
+      <c r="K48" s="86" t="inlineStr">
+        <is>
           <t>来源：用户 2026-10-10 规划占位。触发：生图/多模型正式启用且用户要看账单后再开。</t>
         </is>
       </c>
-      <c r="L47" s="86" t="inlineStr">
+      <c r="L48" s="86" t="inlineStr">
         <is>
           <t>不适用</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="15" customHeight="1" s="41">
-      <c r="A48" s="47" t="inlineStr">
+    <row r="49" ht="15" customHeight="1" s="41">
+      <c r="A49" s="47" t="inlineStr">
         <is>
           <t>U-xx</t>
         </is>
       </c>
-      <c r="B48" s="47" t="n"/>
-      <c r="C48" s="47" t="n"/>
-      <c r="D48" s="47" t="n"/>
-      <c r="E48" s="46" t="inlineStr">
-        <is>
-          <t>（在此行往下追加新问题。ID 建议：U 界面 / G 群聊 / C 会话 / M 朋友圈 / R 角色 / B 体验 / O 工程）</t>
-        </is>
-      </c>
-      <c r="F48" s="47" t="n"/>
-      <c r="G48" s="47" t="n"/>
-      <c r="H48" s="47" t="n"/>
-      <c r="I48" s="47" t="n"/>
-      <c r="J48" s="47" t="n"/>
-      <c r="K48" s="47" t="n"/>
-      <c r="L48" t="inlineStr">
-        <is>
-          <t>不适用</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="15" customHeight="1" s="41">
-      <c r="A49" s="47" t="n"/>
       <c r="B49" s="47" t="n"/>
       <c r="C49" s="47" t="n"/>
       <c r="D49" s="47" t="n"/>
-      <c r="E49" s="47" t="n"/>
+      <c r="E49" s="46" t="inlineStr">
+        <is>
+          <t>（在此行往下追加新问题。ID 建议：U 界面 / G 群聊 / C 会话 / M 朋友圈 / R 角色 / B 体验 / O 工程）</t>
+        </is>
+      </c>
       <c r="F49" s="47" t="n"/>
       <c r="G49" s="47" t="n"/>
       <c r="H49" s="47" t="n"/>
       <c r="I49" s="47" t="n"/>
       <c r="J49" s="47" t="n"/>
       <c r="K49" s="47" t="n"/>
+      <c r="L49" s="40" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="41">
       <c r="A50" s="47" t="n"/>
@@ -4212,6 +4257,19 @@
       <c r="I55" s="47" t="n"/>
       <c r="J55" s="47" t="n"/>
       <c r="K55" s="47" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="47" t="n"/>
+      <c r="B56" s="47" t="n"/>
+      <c r="C56" s="47" t="n"/>
+      <c r="D56" s="47" t="n"/>
+      <c r="E56" s="47" t="n"/>
+      <c r="F56" s="47" t="n"/>
+      <c r="G56" s="47" t="n"/>
+      <c r="H56" s="47" t="n"/>
+      <c r="I56" s="47" t="n"/>
+      <c r="J56" s="47" t="n"/>
+      <c r="K56" s="47" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:K40"/>
@@ -4263,7 +4321,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="16" customWidth="1" style="40" min="1" max="1"/>
@@ -4334,12 +4392,12 @@
       </c>
     </row>
     <row r="8" ht="36" customHeight="1" s="41">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="40" t="inlineStr">
         <is>
           <t>远程状态（L 列）</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="40" t="inlineStr">
         <is>
           <t>已 push＝已合入远程；未 push＝仅本机；不适用＝暂缓未开工/规划占位/非功能行。</t>
         </is>
@@ -4348,7 +4406,7 @@
     <row r="9" ht="36" customHeight="1" s="41">
       <c r="A9" s="69" t="inlineStr">
         <is>
-          <t>2026-10-10：功能远程 tip 5c8f652（含 M-01）；文档 tip 以最新 docs commit 为准（本文件随 docs 更新）。无待 push 功能刀。下一候选：C-06 空间反应与私聊主动日 cap 解耦（待用户点头）；另可选 daily_cap UI / R-03 好感度（勿与 N-01..03 混淆）。</t>
+          <t>2026-10-10：C-06 已点收并在远程 57e92bc。文档 tip 以最新 docs 为准。下一候选待用户点名（N-01～03 规划占位）。</t>
         </is>
       </c>
       <c r="B9" s="70" t="n"/>
@@ -4410,6 +4468,8 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
+    <row r="15"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
@@ -4436,7 +4496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="22" customWidth="1" style="40" min="1" max="1"/>
@@ -4559,23 +4619,23 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="40" t="inlineStr">
         <is>
           <t>未 push 条数</t>
         </is>
       </c>
-      <c r="B15">
+      <c r="B15" s="40">
         <f>COUNTIF(问题记录!L:L,"未 push")</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="40" t="inlineStr">
         <is>
           <t>已 push 条数</t>
         </is>
       </c>
-      <c r="B16">
+      <c r="B16" s="40">
         <f>COUNTIF(问题记录!L:L,"已 push")</f>
         <v/>
       </c>
@@ -4593,7 +4653,7 @@
           <t>待处理/处理中条数</t>
         </is>
       </c>
-      <c r="B18">
+      <c r="B18" s="40">
         <f>COUNTIF(问题记录!B:B,"待处理")+COUNTIF(问题记录!B:B,"处理中")</f>
         <v/>
       </c>
@@ -4604,7 +4664,7 @@
           <t>ID 列表（自动）</t>
         </is>
       </c>
-      <c r="B19">
+      <c r="B19" s="40">
         <f>TEXTJOIN("；",TRUE,IF(((问题记录!B$2:B$200="待处理")+(问题记录!B$2:B$200="处理中"))&gt;0,问题记录!A$2:A$200&amp;" "&amp;问题记录!E$2:E$200,""))</f>
         <v/>
       </c>
@@ -4615,7 +4675,7 @@
           <t>下一候选（人工）</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="40" t="inlineStr">
         <is>
           <t>C-06 空间反应与私聊主动日 cap 解耦（待用户点头）。可选：daily_cap UI / R-03 好感度。勿与 N-01..03 规划占位混淆。</t>
         </is>
@@ -4627,7 +4687,7 @@
           <t>远程 tip（人工）</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="40" t="inlineStr">
         <is>
           <t>功能 tip 5c8f652；文档 tip 以最新 docs 为准。无待 push 功能刀。人工维护，最后更新 2026-10-10。</t>
         </is>

</xml_diff>

<commit_message>
docs: phase-2 backlog X/UI/ARCH/M-05a; phase-1 smoke close
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -1388,7 +1388,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L56"/>
+  <dimension ref="A1:L77"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="40" min="1" max="1"/>
@@ -2804,7 +2804,7 @@
       <c r="J24" s="44" t="n"/>
       <c r="K24" s="46" t="inlineStr">
         <is>
-          <t>触发：用户明确要整站深色或移动端适配后再开。（U-05 已关，原「完整皮肤体系见 U-05」备注失效。）</t>
+          <t>触发：用户明确要整站深色或移动端适配后再开。（U-05 已关，原「完整皮肤体系见 U-05」备注失效。） 2026-10-10：保持触发式；用户明确要整站深色/移动端再开。</t>
         </is>
       </c>
       <c r="L24" s="40" t="inlineStr">
@@ -3087,12 +3087,12 @@
       </c>
       <c r="E30" s="46" t="inlineStr">
         <is>
-          <t>动态支持配图</t>
+          <t>动态配图（总项，见 M-05a/b）</t>
         </is>
       </c>
       <c r="F30" s="46" t="inlineStr">
         <is>
-          <t>发动态（含「让 TA 发一条」）可带一张或多张图。图可来自上传、角色卡资源，或后期由文生图插件/多模态 API 生成。时间线卡片要能展示。</t>
+          <t>总项拆为 M-05a 仅上传、M-05b 含生图。二期顺序先 M-05a。</t>
         </is>
       </c>
       <c r="G30" s="46" t="inlineStr">
@@ -3109,7 +3109,7 @@
       <c r="J30" s="44" t="n"/>
       <c r="K30" s="46" t="inlineStr">
         <is>
-          <t>触发：生图成本闸门可接受，或先做仅上传配图后再开。 用户 2026-09-14 提出。生成配图依赖 B-04；纯上传可更早。 2026-09-16 产品判断：无生图时给角色动态配用户相册图不成立；若要配图需用户发动态（M-06 已关）或等生图。</t>
+          <t>触发：生图成本闸门可接受，或先做仅上传配图后再开。 用户 2026-09-14 提出。生成配图依赖 B-04；纯上传可更早。 2026-09-16 产品判断：无生图时给角色动态配用户相册图不成立；若要配图需用户发动态（M-06 已关）或等生图。 2026-10-10 拆 M-05a/b；总项保持索引。</t>
         </is>
       </c>
       <c r="L30" s="40" t="inlineStr">
@@ -3757,7 +3757,7 @@
       <c r="J41" s="49" t="n"/>
       <c r="K41" s="51" t="inlineStr">
         <is>
-          <t>触发：用户明确要对话/提炼分通道后再开正式刀。 R-04x 尖兵 575967c 已完（夹具报告+默认 off）；不强开真 Laya。 先做 R-02 注入必答补丁（已关）。</t>
+          <t>触发：用户明确要对话/提炼分通道后再开正式刀。 R-04x 尖兵 575967c 已完（夹具报告+默认 off）；不强开真 Laya。 先做 R-02 注入必答补丁（已关）。 2026-10-10：二期定为 P3。</t>
         </is>
       </c>
       <c r="L41" s="40" t="inlineStr">
@@ -3941,37 +3941,37 @@
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="41">
-      <c r="A45" t="inlineStr">
+      <c r="A45" s="40" t="inlineStr">
         <is>
           <t>C-06</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B45" s="40" t="inlineStr">
         <is>
           <t>已处理</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C45" s="40" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D45" s="40" t="inlineStr">
         <is>
           <t>会话</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
+      <c r="E45" s="40" t="inlineStr">
         <is>
           <t>空间赞评与私聊主动日 cap 解耦</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="F45" s="40" t="inlineStr">
         <is>
           <t>sent_today 满后 M-07 空间结算被 daily_cap 跳过，用户发动态无角色赞评。</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr">
+      <c r="G45" s="40" t="inlineStr">
         <is>
           <t>空间结算不再因 sent_today&gt;=daily_cap 跳过；私聊主动仍受日 cap；总开关关两边都停。2026-10-10 代验通过，已在远程 57e92bc。</t>
         </is>
@@ -3982,17 +3982,17 @@
       <c r="I45" s="83" t="n">
         <v>46305</v>
       </c>
-      <c r="J45" t="inlineStr">
+      <c r="J45" s="40" t="inlineStr">
         <is>
           <t>57e92bc</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr">
+      <c r="K45" s="40" t="inlineStr">
         <is>
           <t>2026-10-10 点收并已在 origin。</t>
         </is>
       </c>
-      <c r="L45" t="inlineStr">
+      <c r="L45" s="40" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>
@@ -4093,7 +4093,7 @@
       <c r="J47" s="86" t="n"/>
       <c r="K47" s="86" t="inlineStr">
         <is>
-          <t>来源：用户 2026-10-10 规划占位。触发：用户选定多模型供应商与路由规则后再开。</t>
+          <t>来源：用户 2026-10-10 规划占位。触发：用户选定多模型供应商与路由规则后再开。 2026-10-10：提前至二期中后段；与 ARCH-2 共挂 API 试跑线（本地/硅基/官方；DeepSeek 文本、官方 VLM、Gemini TTS）。</t>
         </is>
       </c>
       <c r="L47" s="86" t="inlineStr">
@@ -4155,121 +4155,1066 @@
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="41">
-      <c r="A49" s="47" t="inlineStr">
+      <c r="A49" s="40" t="inlineStr">
+        <is>
+          <t>M-05a</t>
+        </is>
+      </c>
+      <c r="B49" s="40" t="inlineStr">
+        <is>
+          <t>待处理</t>
+        </is>
+      </c>
+      <c r="C49" s="40" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D49" s="40" t="inlineStr">
+        <is>
+          <t>朋友圈</t>
+        </is>
+      </c>
+      <c r="E49" s="40" t="inlineStr">
+        <is>
+          <t>动态配图第一刀：仅上传</t>
+        </is>
+      </c>
+      <c r="F49" s="40" t="inlineStr">
+        <is>
+          <t>发动态可附一张上传图进时间线；不接生图。</t>
+        </is>
+      </c>
+      <c r="H49" s="83" t="n">
+        <v>46305</v>
+      </c>
+      <c r="K49" s="40" t="inlineStr">
+        <is>
+          <t>二期前四刀第2：ARCH-1 后。</t>
+        </is>
+      </c>
+      <c r="L49" s="40" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="15" customHeight="1" s="41">
+      <c r="A50" s="40" t="inlineStr">
+        <is>
+          <t>M-05b</t>
+        </is>
+      </c>
+      <c r="B50" s="40" t="inlineStr">
+        <is>
+          <t>暂缓</t>
+        </is>
+      </c>
+      <c r="C50" s="40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D50" s="40" t="inlineStr">
+        <is>
+          <t>朋友圈</t>
+        </is>
+      </c>
+      <c r="E50" s="40" t="inlineStr">
+        <is>
+          <t>动态配图含生图</t>
+        </is>
+      </c>
+      <c r="F50" s="40" t="inlineStr">
+        <is>
+          <t>动态配图可走生图；先复用 B-04B，不绑 N-01 素材库。</t>
+        </is>
+      </c>
+      <c r="H50" s="83" t="n">
+        <v>46305</v>
+      </c>
+      <c r="K50" s="40" t="inlineStr">
+        <is>
+          <t>触发：M-05a 稳且要生图配图。</t>
+        </is>
+      </c>
+      <c r="L50" s="40" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="15" customHeight="1" s="41">
+      <c r="A51" s="40" t="inlineStr">
+        <is>
+          <t>X-01</t>
+        </is>
+      </c>
+      <c r="B51" s="40" t="inlineStr">
+        <is>
+          <t>待处理</t>
+        </is>
+      </c>
+      <c r="C51" s="40" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D51" s="40" t="inlineStr">
+        <is>
+          <t>角色</t>
+        </is>
+      </c>
+      <c r="E51" s="40" t="inlineStr">
+        <is>
+          <t>人设编辑</t>
+        </is>
+      </c>
+      <c r="F51" s="40" t="inlineStr">
+        <is>
+          <t>导入后可在客户端编辑人设字段并保存，无需整卡覆盖导入。</t>
+        </is>
+      </c>
+      <c r="H51" s="83" t="n">
+        <v>46305</v>
+      </c>
+      <c r="K51" s="40" t="inlineStr">
+        <is>
+          <t>二期前四刀第3。</t>
+        </is>
+      </c>
+      <c r="L51" s="40" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="40" t="inlineStr">
+        <is>
+          <t>X-02</t>
+        </is>
+      </c>
+      <c r="B52" s="40" t="inlineStr">
+        <is>
+          <t>暂缓</t>
+        </is>
+      </c>
+      <c r="C52" s="40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D52" s="40" t="inlineStr">
+        <is>
+          <t>角色</t>
+        </is>
+      </c>
+      <c r="E52" s="40" t="inlineStr">
+        <is>
+          <t>人设参考图</t>
+        </is>
+      </c>
+      <c r="F52" s="40" t="inlineStr">
+        <is>
+          <t>人设可附参考图供读图/生图对齐画风。</t>
+        </is>
+      </c>
+      <c r="H52" s="83" t="n">
+        <v>46305</v>
+      </c>
+      <c r="K52" s="40" t="inlineStr">
+        <is>
+          <t>待 X-01 后。</t>
+        </is>
+      </c>
+      <c r="L52" s="40" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="40" t="inlineStr">
+        <is>
+          <t>X-03</t>
+        </is>
+      </c>
+      <c r="B53" s="40" t="inlineStr">
+        <is>
+          <t>暂缓</t>
+        </is>
+      </c>
+      <c r="C53" s="40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D53" s="40" t="inlineStr">
+        <is>
+          <t>界面</t>
+        </is>
+      </c>
+      <c r="E53" s="40" t="inlineStr">
+        <is>
+          <t>daily_cap / 静默时段可调</t>
+        </is>
+      </c>
+      <c r="F53" s="40" t="inlineStr">
+        <is>
+          <t>主页现仅展示主动日 cap；需可改 daily_cap 与静默起止。</t>
+        </is>
+      </c>
+      <c r="H53" s="83" t="n">
+        <v>46305</v>
+      </c>
+      <c r="K53" s="40" t="inlineStr">
+        <is>
+          <t>二期可选。</t>
+        </is>
+      </c>
+      <c r="L53" s="40" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="40" t="inlineStr">
+        <is>
+          <t>X-04</t>
+        </is>
+      </c>
+      <c r="B54" s="40" t="inlineStr">
+        <is>
+          <t>暂缓</t>
+        </is>
+      </c>
+      <c r="C54" s="40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D54" s="40" t="inlineStr">
+        <is>
+          <t>群聊</t>
+        </is>
+      </c>
+      <c r="E54" s="40" t="inlineStr">
+        <is>
+          <t>群聊轮询抢话体验</t>
+        </is>
+      </c>
+      <c r="F54" s="40" t="inlineStr">
+        <is>
+          <t>未 @ 时轮询发言观感抢话/不自然。</t>
+        </is>
+      </c>
+      <c r="H54" s="83" t="n">
+        <v>46305</v>
+      </c>
+      <c r="K54" s="40" t="inlineStr">
+        <is>
+          <t>二期体验债。</t>
+        </is>
+      </c>
+      <c r="L54" s="40" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="40" t="inlineStr">
+        <is>
+          <t>X-05</t>
+        </is>
+      </c>
+      <c r="B55" s="40" t="inlineStr">
+        <is>
+          <t>待处理</t>
+        </is>
+      </c>
+      <c r="C55" s="40" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D55" s="40" t="inlineStr">
+        <is>
+          <t>角色</t>
+        </is>
+      </c>
+      <c r="E55" s="40" t="inlineStr">
+        <is>
+          <t>记忆体验债复盘</t>
+        </is>
+      </c>
+      <c r="F55" s="40" t="inlineStr">
+        <is>
+          <t>在 R-05/R-06 已关上复盘体验债（过召回/冲突确认边角）。</t>
+        </is>
+      </c>
+      <c r="H55" s="83" t="n">
+        <v>46305</v>
+      </c>
+      <c r="K55" s="40" t="inlineStr">
+        <is>
+          <t>依赖 R-05/R-06 已交付。</t>
+        </is>
+      </c>
+      <c r="L55" s="40" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="40" t="inlineStr">
+        <is>
+          <t>X-06</t>
+        </is>
+      </c>
+      <c r="B56" s="40" t="inlineStr">
+        <is>
+          <t>暂缓</t>
+        </is>
+      </c>
+      <c r="C56" s="40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D56" s="40" t="inlineStr">
+        <is>
+          <t>消息</t>
+        </is>
+      </c>
+      <c r="E56" s="40" t="inlineStr">
+        <is>
+          <t>语音交互体验</t>
+        </is>
+      </c>
+      <c r="F56" s="40" t="inlineStr">
+        <is>
+          <t>语音交互流程体验债（非波形视觉）。</t>
+        </is>
+      </c>
+      <c r="H56" s="83" t="n">
+        <v>46305</v>
+      </c>
+      <c r="K56" s="40" t="inlineStr">
+        <is>
+          <t>与 UI-4 波形分工：本项交互。</t>
+        </is>
+      </c>
+      <c r="L56" s="40" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="40" t="inlineStr">
+        <is>
+          <t>X-07</t>
+        </is>
+      </c>
+      <c r="B57" s="40" t="inlineStr">
+        <is>
+          <t>暂缓</t>
+        </is>
+      </c>
+      <c r="C57" s="40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D57" s="40" t="inlineStr">
+        <is>
+          <t>朋友圈</t>
+        </is>
+      </c>
+      <c r="E57" s="40" t="inlineStr">
+        <is>
+          <t>朋友圈互动频率可调</t>
+        </is>
+      </c>
+      <c r="F57" s="40" t="inlineStr">
+        <is>
+          <t>赞评频率需产品可调项（先定可调参数再开发）。</t>
+        </is>
+      </c>
+      <c r="H57" s="83" t="n">
+        <v>46305</v>
+      </c>
+      <c r="K57" s="40" t="inlineStr">
+        <is>
+          <t>先定可调项再拆包。</t>
+        </is>
+      </c>
+      <c r="L57" s="40" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="40" t="inlineStr">
+        <is>
+          <t>ARCH-1</t>
+        </is>
+      </c>
+      <c r="B58" s="40" t="inlineStr">
+        <is>
+          <t>待处理</t>
+        </is>
+      </c>
+      <c r="C58" s="40" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D58" s="40" t="inlineStr">
+        <is>
+          <t>工程</t>
+        </is>
+      </c>
+      <c r="E58" s="40" t="inlineStr">
+        <is>
+          <t>工程扫描第一刀（含补扫 6 项）</t>
+        </is>
+      </c>
+      <c r="F58" s="40" t="inlineStr">
+        <is>
+          <t>二期开工前工程扫描；BF stash 清理挂本项。补扫6项：1)模型入口与.env绑定(llm/vision/stt/tts/imageGen)；2)主动/空间结算隐式耦合(C-05/M-07/C-06/M-01)；3)记忆链路失败与空泡(extract→filter→pending→honor)；4)前端App.vue体量与状态交叉；5)uploads/SQLite增长与清理；6)未push/stash残留、双机.env漂移。</t>
+        </is>
+      </c>
+      <c r="H58" s="83" t="n">
+        <v>46305</v>
+      </c>
+      <c r="K58" s="40" t="inlineStr">
+        <is>
+          <t>二期前四刀第1。补扫 6 条细目待主 Bot 贴齐后回写现象栏。 2026-10-10 补扫6项已写入现象栏。</t>
+        </is>
+      </c>
+      <c r="L58" s="40" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="40" t="inlineStr">
+        <is>
+          <t>ARCH-2</t>
+        </is>
+      </c>
+      <c r="B59" s="40" t="inlineStr">
+        <is>
+          <t>暂缓</t>
+        </is>
+      </c>
+      <c r="C59" s="40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D59" s="40" t="inlineStr">
+        <is>
+          <t>工程</t>
+        </is>
+      </c>
+      <c r="E59" s="40" t="inlineStr">
+        <is>
+          <t>模型封装与成本中偏高</t>
+        </is>
+      </c>
+      <c r="F59" s="40" t="inlineStr">
+        <is>
+          <t>模型调用封装、成本计量偏高；承接 N-02 动态路由与 API 试跑线。</t>
+        </is>
+      </c>
+      <c r="H59" s="83" t="n">
+        <v>46305</v>
+      </c>
+      <c r="K59" s="40" t="inlineStr">
+        <is>
+          <t>二期前四刀第4；试跑线：本地/硅基/官方；试 DeepSeek 文本、官方 VLM、Gemini TTS。挂 N-02。</t>
+        </is>
+      </c>
+      <c r="L59" s="40" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="40" t="inlineStr">
+        <is>
+          <t>ARCH-3</t>
+        </is>
+      </c>
+      <c r="B60" s="40" t="inlineStr">
+        <is>
+          <t>暂缓</t>
+        </is>
+      </c>
+      <c r="C60" s="40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D60" s="40" t="inlineStr">
+        <is>
+          <t>工程</t>
+        </is>
+      </c>
+      <c r="E60" s="40" t="inlineStr">
+        <is>
+          <t>前端状态管理整理</t>
+        </is>
+      </c>
+      <c r="F60" s="40" t="inlineStr">
+        <is>
+          <t>前端状态分散，影响后续 UI 刀。</t>
+        </is>
+      </c>
+      <c r="H60" s="83" t="n">
+        <v>46305</v>
+      </c>
+      <c r="K60" s="40" t="inlineStr">
+        <is>
+          <t>UI 并行刀前评估。</t>
+        </is>
+      </c>
+      <c r="L60" s="40" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="40" t="inlineStr">
+        <is>
+          <t>B-04c</t>
+        </is>
+      </c>
+      <c r="B61" s="40" t="inlineStr">
+        <is>
+          <t>待处理</t>
+        </is>
+      </c>
+      <c r="C61" s="40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D61" s="40" t="inlineStr">
+        <is>
+          <t>消息</t>
+        </is>
+      </c>
+      <c r="E61" s="40" t="inlineStr">
+        <is>
+          <t>生图触发词过严</t>
+        </is>
+      </c>
+      <c r="F61" s="40" t="inlineStr">
+        <is>
+          <t>冒烟：「帮我画一只猫」可出图；裸「画一只猫」不触发 wantsImageGeneration。</t>
+        </is>
+      </c>
+      <c r="H61" s="83" t="n">
+        <v>46305</v>
+      </c>
+      <c r="K61" s="40" t="inlineStr">
+        <is>
+          <t>2026-10-10 一期冒烟记入二期池。</t>
+        </is>
+      </c>
+      <c r="L61" s="40" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="40" t="inlineStr">
+        <is>
+          <t>B-04d</t>
+        </is>
+      </c>
+      <c r="B62" s="40" t="inlineStr">
+        <is>
+          <t>暂缓</t>
+        </is>
+      </c>
+      <c r="C62" s="40" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D62" s="40" t="inlineStr">
+        <is>
+          <t>消息</t>
+        </is>
+      </c>
+      <c r="E62" s="40" t="inlineStr">
+        <is>
+          <t>B-04B Key 失败路径未实打</t>
+        </is>
+      </c>
+      <c r="F62" s="40" t="inlineStr">
+        <is>
+          <t>生图 Key 失败人话路径代码在、一期未实打。</t>
+        </is>
+      </c>
+      <c r="H62" s="83" t="n">
+        <v>46305</v>
+      </c>
+      <c r="K62" s="40" t="inlineStr">
+        <is>
+          <t>挂 API/密钥试跑时顺带验。</t>
+        </is>
+      </c>
+      <c r="L62" s="40" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="40" t="inlineStr">
+        <is>
+          <t>O-03</t>
+        </is>
+      </c>
+      <c r="B63" s="40" t="inlineStr">
+        <is>
+          <t>待处理</t>
+        </is>
+      </c>
+      <c r="C63" s="40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D63" s="40" t="inlineStr">
+        <is>
+          <t>工程</t>
+        </is>
+      </c>
+      <c r="E63" s="40" t="inlineStr">
+        <is>
+          <t>BF stash 清理</t>
+        </is>
+      </c>
+      <c r="F63" s="40" t="inlineStr">
+        <is>
+          <t>BF 残留 stash（issue tracker / local before M-01），避免和下包混。</t>
+        </is>
+      </c>
+      <c r="H63" s="83" t="n">
+        <v>46305</v>
+      </c>
+      <c r="K63" s="40" t="inlineStr">
+        <is>
+          <t>挂 ARCH-1 扫描一并处理。</t>
+        </is>
+      </c>
+      <c r="L63" s="40" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>UI-1</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>待处理</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>界面</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>动效基础层</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>统一时长、曲线、触发场景（Telegram/Discord 娱乐向）。</t>
+        </is>
+      </c>
+      <c r="H64" s="83" t="n">
+        <v>46305</v>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>二期第五刀/可与前四刀并行。</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>UI-2</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>暂缓</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>界面</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>消息动效</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>发送/接收过渡、正在输入动效。</t>
+        </is>
+      </c>
+      <c r="H65" s="83" t="n">
+        <v>46305</v>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>依赖 UI-1 基础层。</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>UI-3</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>暂缓</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>界面</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>红点/未读动效</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>未读红点动效增强（C-03 功能已有）。</t>
+        </is>
+      </c>
+      <c r="H66" s="83" t="n">
+        <v>46305</v>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>依赖 UI-1。</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>UI-4</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>暂缓</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>界面</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>语音气泡视觉：波形+播放/暂停+进度</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>语音泡波形与进度视觉。</t>
+        </is>
+      </c>
+      <c r="H67" s="83" t="n">
+        <v>46305</v>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>与 X-06 分工：UI-4=视觉；X-06=交互。可同迭代分两行。</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>UI-5</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>暂缓</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>界面</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Reaction 多表情+微动效</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>消息 reaction 多表情与微动效。</t>
+        </is>
+      </c>
+      <c r="H68" s="83" t="n">
+        <v>46305</v>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>娱乐向，P3。</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>UI-6</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>暂缓</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>界面</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>群聊活跃感</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>角色头像浮动、正在输入等群聊活跃感。</t>
+        </is>
+      </c>
+      <c r="H69" s="83" t="n">
+        <v>46305</v>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>娱乐向，P3。</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="47" t="inlineStr">
         <is>
           <t>U-xx</t>
         </is>
       </c>
-      <c r="B49" s="47" t="n"/>
-      <c r="C49" s="47" t="n"/>
-      <c r="D49" s="47" t="n"/>
-      <c r="E49" s="46" t="inlineStr">
+      <c r="B70" s="47" t="n"/>
+      <c r="C70" s="47" t="n"/>
+      <c r="D70" s="47" t="n"/>
+      <c r="E70" s="46" t="inlineStr">
         <is>
           <t>（在此行往下追加新问题。ID 建议：U 界面 / G 群聊 / C 会话 / M 朋友圈 / R 角色 / B 体验 / O 工程）</t>
         </is>
       </c>
-      <c r="F49" s="47" t="n"/>
-      <c r="G49" s="47" t="n"/>
-      <c r="H49" s="47" t="n"/>
-      <c r="I49" s="47" t="n"/>
-      <c r="J49" s="47" t="n"/>
-      <c r="K49" s="47" t="n"/>
-      <c r="L49" s="40" t="inlineStr">
+      <c r="F70" s="47" t="n"/>
+      <c r="G70" s="47" t="n"/>
+      <c r="H70" s="47" t="n"/>
+      <c r="I70" s="47" t="n"/>
+      <c r="J70" s="47" t="n"/>
+      <c r="K70" s="47" t="n"/>
+      <c r="L70" s="40" t="inlineStr">
         <is>
           <t>不适用</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="15" customHeight="1" s="41">
-      <c r="A50" s="47" t="n"/>
-      <c r="B50" s="47" t="n"/>
-      <c r="C50" s="47" t="n"/>
-      <c r="D50" s="47" t="n"/>
-      <c r="E50" s="47" t="n"/>
-      <c r="F50" s="47" t="n"/>
-      <c r="G50" s="47" t="n"/>
-      <c r="H50" s="47" t="n"/>
-      <c r="I50" s="47" t="n"/>
-      <c r="J50" s="47" t="n"/>
-      <c r="K50" s="47" t="n"/>
-    </row>
-    <row r="51" ht="15" customHeight="1" s="41">
-      <c r="A51" s="47" t="n"/>
-      <c r="B51" s="47" t="n"/>
-      <c r="C51" s="47" t="n"/>
-      <c r="D51" s="47" t="n"/>
-      <c r="E51" s="47" t="n"/>
-      <c r="F51" s="47" t="n"/>
-      <c r="G51" s="47" t="n"/>
-      <c r="H51" s="47" t="n"/>
-      <c r="I51" s="47" t="n"/>
-      <c r="J51" s="47" t="n"/>
-      <c r="K51" s="47" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="47" t="n"/>
-      <c r="B52" s="47" t="n"/>
-      <c r="C52" s="47" t="n"/>
-      <c r="D52" s="47" t="n"/>
-      <c r="E52" s="47" t="n"/>
-      <c r="F52" s="47" t="n"/>
-      <c r="G52" s="47" t="n"/>
-      <c r="H52" s="47" t="n"/>
-      <c r="I52" s="47" t="n"/>
-      <c r="J52" s="47" t="n"/>
-      <c r="K52" s="47" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="47" t="n"/>
-      <c r="B53" s="47" t="n"/>
-      <c r="C53" s="47" t="n"/>
-      <c r="D53" s="47" t="n"/>
-      <c r="E53" s="47" t="n"/>
-      <c r="F53" s="47" t="n"/>
-      <c r="G53" s="47" t="n"/>
-      <c r="H53" s="47" t="n"/>
-      <c r="I53" s="47" t="n"/>
-      <c r="J53" s="47" t="n"/>
-      <c r="K53" s="47" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="47" t="n"/>
-      <c r="B54" s="47" t="n"/>
-      <c r="C54" s="47" t="n"/>
-      <c r="D54" s="47" t="n"/>
-      <c r="E54" s="47" t="n"/>
-      <c r="F54" s="47" t="n"/>
-      <c r="G54" s="47" t="n"/>
-      <c r="H54" s="47" t="n"/>
-      <c r="I54" s="47" t="n"/>
-      <c r="J54" s="47" t="n"/>
-      <c r="K54" s="47" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="47" t="n"/>
-      <c r="B55" s="47" t="n"/>
-      <c r="C55" s="47" t="n"/>
-      <c r="D55" s="47" t="n"/>
-      <c r="E55" s="47" t="n"/>
-      <c r="F55" s="47" t="n"/>
-      <c r="G55" s="47" t="n"/>
-      <c r="H55" s="47" t="n"/>
-      <c r="I55" s="47" t="n"/>
-      <c r="J55" s="47" t="n"/>
-      <c r="K55" s="47" t="n"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="47" t="n"/>
-      <c r="B56" s="47" t="n"/>
-      <c r="C56" s="47" t="n"/>
-      <c r="D56" s="47" t="n"/>
-      <c r="E56" s="47" t="n"/>
-      <c r="F56" s="47" t="n"/>
-      <c r="G56" s="47" t="n"/>
-      <c r="H56" s="47" t="n"/>
-      <c r="I56" s="47" t="n"/>
-      <c r="J56" s="47" t="n"/>
-      <c r="K56" s="47" t="n"/>
+    <row r="71">
+      <c r="A71" s="47" t="n"/>
+      <c r="B71" s="47" t="n"/>
+      <c r="C71" s="47" t="n"/>
+      <c r="D71" s="47" t="n"/>
+      <c r="E71" s="47" t="n"/>
+      <c r="F71" s="47" t="n"/>
+      <c r="G71" s="47" t="n"/>
+      <c r="H71" s="47" t="n"/>
+      <c r="I71" s="47" t="n"/>
+      <c r="J71" s="47" t="n"/>
+      <c r="K71" s="47" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="47" t="n"/>
+      <c r="B72" s="47" t="n"/>
+      <c r="C72" s="47" t="n"/>
+      <c r="D72" s="47" t="n"/>
+      <c r="E72" s="47" t="n"/>
+      <c r="F72" s="47" t="n"/>
+      <c r="G72" s="47" t="n"/>
+      <c r="H72" s="47" t="n"/>
+      <c r="I72" s="47" t="n"/>
+      <c r="J72" s="47" t="n"/>
+      <c r="K72" s="47" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="47" t="n"/>
+      <c r="B73" s="47" t="n"/>
+      <c r="C73" s="47" t="n"/>
+      <c r="D73" s="47" t="n"/>
+      <c r="E73" s="47" t="n"/>
+      <c r="F73" s="47" t="n"/>
+      <c r="G73" s="47" t="n"/>
+      <c r="H73" s="47" t="n"/>
+      <c r="I73" s="47" t="n"/>
+      <c r="J73" s="47" t="n"/>
+      <c r="K73" s="47" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="47" t="n"/>
+      <c r="B74" s="47" t="n"/>
+      <c r="C74" s="47" t="n"/>
+      <c r="D74" s="47" t="n"/>
+      <c r="E74" s="47" t="n"/>
+      <c r="F74" s="47" t="n"/>
+      <c r="G74" s="47" t="n"/>
+      <c r="H74" s="47" t="n"/>
+      <c r="I74" s="47" t="n"/>
+      <c r="J74" s="47" t="n"/>
+      <c r="K74" s="47" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="47" t="n"/>
+      <c r="B75" s="47" t="n"/>
+      <c r="C75" s="47" t="n"/>
+      <c r="D75" s="47" t="n"/>
+      <c r="E75" s="47" t="n"/>
+      <c r="F75" s="47" t="n"/>
+      <c r="G75" s="47" t="n"/>
+      <c r="H75" s="47" t="n"/>
+      <c r="I75" s="47" t="n"/>
+      <c r="J75" s="47" t="n"/>
+      <c r="K75" s="47" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="47" t="n"/>
+      <c r="B76" s="47" t="n"/>
+      <c r="C76" s="47" t="n"/>
+      <c r="D76" s="47" t="n"/>
+      <c r="E76" s="47" t="n"/>
+      <c r="F76" s="47" t="n"/>
+      <c r="G76" s="47" t="n"/>
+      <c r="H76" s="47" t="n"/>
+      <c r="I76" s="47" t="n"/>
+      <c r="J76" s="47" t="n"/>
+      <c r="K76" s="47" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="47" t="n"/>
+      <c r="B77" s="47" t="n"/>
+      <c r="C77" s="47" t="n"/>
+      <c r="D77" s="47" t="n"/>
+      <c r="E77" s="47" t="n"/>
+      <c r="F77" s="47" t="n"/>
+      <c r="G77" s="47" t="n"/>
+      <c r="H77" s="47" t="n"/>
+      <c r="I77" s="47" t="n"/>
+      <c r="J77" s="47" t="n"/>
+      <c r="K77" s="47" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:K40"/>
@@ -4321,7 +5266,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="16" customWidth="1" style="40" min="1" max="1"/>
@@ -4406,7 +5351,7 @@
     <row r="9" ht="36" customHeight="1" s="41">
       <c r="A9" s="69" t="inlineStr">
         <is>
-          <t>2026-10-10：C-06 已点收并在远程 57e92bc。文档 tip 以最新 docs 为准。下一候选待用户点名（N-01～03 规划占位）。</t>
+          <t>2026-10-10：一期七类冒烟通过（BF tip 65cf58e），一期可收口。二期前四刀 ARCH-1→M-05a→X-01→ARCH-2；UI-1 第五/可并行。UI-1～6、ARCH-1 补扫6项已落表。</t>
         </is>
       </c>
       <c r="B9" s="70" t="n"/>
@@ -4470,6 +5415,7 @@
     </row>
     <row r="14"/>
     <row r="15"/>
+    <row r="16"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>

</xml_diff>

<commit_message>
docs: ARCH-1 debt list + phase-1 smoke scripts
Close ARCH-1: add 债清单 (D-04 moved to feature pool w/ C-06 P2; D-05 stays high for ARCH-2 observability; D-11 waits for HY). Track smoke_*.py. Sync issue xlsx (C-06 note, ARCH-1 closed).
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -334,7 +334,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="88">
+  <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -591,6 +591,7 @@
     <xf numFmtId="166" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3989,7 +3990,7 @@
       </c>
       <c r="K45" s="40" t="inlineStr">
         <is>
-          <t>2026-10-10 点收并已在 origin。</t>
+          <t>2026-10-10 点收并已在 origin。 2026-10-10 ARCH-1：功能池登记 D-04（M-01 仍吃私聊 daily_cap，与 C-06 后 M-07 空间不受 cap 不一致）→ 与 C-06 同组 P2，不进 ARCH-2/3。详见 docs/product/ARCH-1-债清单.md。</t>
         </is>
       </c>
       <c r="L45" s="40" t="inlineStr">
@@ -4567,7 +4568,7 @@
       </c>
       <c r="B58" s="40" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>已处理</t>
         </is>
       </c>
       <c r="C58" s="40" t="inlineStr">
@@ -4588,14 +4589,22 @@
       <c r="F58" s="40" t="inlineStr">
         <is>
           <t>二期开工前工程扫描；BF stash 清理挂本项。补扫6项：1)模型入口与.env绑定(llm/vision/stt/tts/imageGen)；2)主动/空间结算隐式耦合(C-05/M-07/C-06/M-01)；3)记忆链路失败与空泡(extract→filter→pending→honor)；4)前端App.vue体量与状态交叉；5)uploads/SQLite增长与清理；6)未push/stash残留、双机.env漂移。</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>扫描完成产出 docs/product/ARCH-1-债清单.md；D-04 挪功能池与 C-06 同组 P2；D-05 留 ARCH-2 可观测；D-11 挂 HY；stash×2 建议临时丢；smoke_*.py 入库。</t>
         </is>
       </c>
       <c r="H58" s="83" t="n">
         <v>46305</v>
       </c>
+      <c r="I58" s="88" t="n">
+        <v>46305</v>
+      </c>
       <c r="K58" s="40" t="inlineStr">
         <is>
-          <t>二期前四刀第1。补扫 6 条细目待主 Bot 贴齐后回写现象栏。 2026-10-10 补扫6项已写入现象栏。</t>
+          <t>二期前四刀第1。补扫 6 条细目待主 Bot 贴齐后回写现象栏。 2026-10-10 补扫6项已写入现象栏。 2026-10-10 收口：债清单已写；详见 ARCH-1-债清单.md 功能池旁注。</t>
         </is>
       </c>
       <c r="L58" s="40" t="inlineStr">
@@ -4830,32 +4839,32 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr">
+      <c r="A64" s="40" t="inlineStr">
         <is>
           <t>UI-1</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr">
+      <c r="B64" s="40" t="inlineStr">
         <is>
           <t>待处理</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
+      <c r="C64" s="40" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr">
+      <c r="D64" s="40" t="inlineStr">
         <is>
           <t>界面</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr">
+      <c r="E64" s="40" t="inlineStr">
         <is>
           <t>动效基础层</t>
         </is>
       </c>
-      <c r="F64" t="inlineStr">
+      <c r="F64" s="40" t="inlineStr">
         <is>
           <t>统一时长、曲线、触发场景（Telegram/Discord 娱乐向）。</t>
         </is>
@@ -4863,44 +4872,44 @@
       <c r="H64" s="83" t="n">
         <v>46305</v>
       </c>
-      <c r="K64" t="inlineStr">
+      <c r="K64" s="40" t="inlineStr">
         <is>
           <t>二期第五刀/可与前四刀并行。</t>
         </is>
       </c>
-      <c r="L64" t="inlineStr">
+      <c r="L64" s="40" t="inlineStr">
         <is>
           <t>不适用</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" t="inlineStr">
+      <c r="A65" s="40" t="inlineStr">
         <is>
           <t>UI-2</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr">
+      <c r="B65" s="40" t="inlineStr">
         <is>
           <t>暂缓</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr">
+      <c r="C65" s="40" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="D65" t="inlineStr">
+      <c r="D65" s="40" t="inlineStr">
         <is>
           <t>界面</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr">
+      <c r="E65" s="40" t="inlineStr">
         <is>
           <t>消息动效</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr">
+      <c r="F65" s="40" t="inlineStr">
         <is>
           <t>发送/接收过渡、正在输入动效。</t>
         </is>
@@ -4908,44 +4917,44 @@
       <c r="H65" s="83" t="n">
         <v>46305</v>
       </c>
-      <c r="K65" t="inlineStr">
+      <c r="K65" s="40" t="inlineStr">
         <is>
           <t>依赖 UI-1 基础层。</t>
         </is>
       </c>
-      <c r="L65" t="inlineStr">
+      <c r="L65" s="40" t="inlineStr">
         <is>
           <t>不适用</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr">
+      <c r="A66" s="40" t="inlineStr">
         <is>
           <t>UI-3</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr">
+      <c r="B66" s="40" t="inlineStr">
         <is>
           <t>暂缓</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr">
+      <c r="C66" s="40" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="D66" t="inlineStr">
+      <c r="D66" s="40" t="inlineStr">
         <is>
           <t>界面</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr">
+      <c r="E66" s="40" t="inlineStr">
         <is>
           <t>红点/未读动效</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr">
+      <c r="F66" s="40" t="inlineStr">
         <is>
           <t>未读红点动效增强（C-03 功能已有）。</t>
         </is>
@@ -4953,44 +4962,44 @@
       <c r="H66" s="83" t="n">
         <v>46305</v>
       </c>
-      <c r="K66" t="inlineStr">
+      <c r="K66" s="40" t="inlineStr">
         <is>
           <t>依赖 UI-1。</t>
         </is>
       </c>
-      <c r="L66" t="inlineStr">
+      <c r="L66" s="40" t="inlineStr">
         <is>
           <t>不适用</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" t="inlineStr">
+      <c r="A67" s="40" t="inlineStr">
         <is>
           <t>UI-4</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr">
+      <c r="B67" s="40" t="inlineStr">
         <is>
           <t>暂缓</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr">
+      <c r="C67" s="40" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="D67" t="inlineStr">
+      <c r="D67" s="40" t="inlineStr">
         <is>
           <t>界面</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr">
+      <c r="E67" s="40" t="inlineStr">
         <is>
           <t>语音气泡视觉：波形+播放/暂停+进度</t>
         </is>
       </c>
-      <c r="F67" t="inlineStr">
+      <c r="F67" s="40" t="inlineStr">
         <is>
           <t>语音泡波形与进度视觉。</t>
         </is>
@@ -4998,44 +5007,44 @@
       <c r="H67" s="83" t="n">
         <v>46305</v>
       </c>
-      <c r="K67" t="inlineStr">
+      <c r="K67" s="40" t="inlineStr">
         <is>
           <t>与 X-06 分工：UI-4=视觉；X-06=交互。可同迭代分两行。</t>
         </is>
       </c>
-      <c r="L67" t="inlineStr">
+      <c r="L67" s="40" t="inlineStr">
         <is>
           <t>不适用</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" t="inlineStr">
+      <c r="A68" s="40" t="inlineStr">
         <is>
           <t>UI-5</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr">
+      <c r="B68" s="40" t="inlineStr">
         <is>
           <t>暂缓</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr">
+      <c r="C68" s="40" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="D68" t="inlineStr">
+      <c r="D68" s="40" t="inlineStr">
         <is>
           <t>界面</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr">
+      <c r="E68" s="40" t="inlineStr">
         <is>
           <t>Reaction 多表情+微动效</t>
         </is>
       </c>
-      <c r="F68" t="inlineStr">
+      <c r="F68" s="40" t="inlineStr">
         <is>
           <t>消息 reaction 多表情与微动效。</t>
         </is>
@@ -5043,44 +5052,44 @@
       <c r="H68" s="83" t="n">
         <v>46305</v>
       </c>
-      <c r="K68" t="inlineStr">
+      <c r="K68" s="40" t="inlineStr">
         <is>
           <t>娱乐向，P3。</t>
         </is>
       </c>
-      <c r="L68" t="inlineStr">
+      <c r="L68" s="40" t="inlineStr">
         <is>
           <t>不适用</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr">
+      <c r="A69" s="40" t="inlineStr">
         <is>
           <t>UI-6</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr">
+      <c r="B69" s="40" t="inlineStr">
         <is>
           <t>暂缓</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr">
+      <c r="C69" s="40" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="D69" t="inlineStr">
+      <c r="D69" s="40" t="inlineStr">
         <is>
           <t>界面</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr">
+      <c r="E69" s="40" t="inlineStr">
         <is>
           <t>群聊活跃感</t>
         </is>
       </c>
-      <c r="F69" t="inlineStr">
+      <c r="F69" s="40" t="inlineStr">
         <is>
           <t>角色头像浮动、正在输入等群聊活跃感。</t>
         </is>
@@ -5088,12 +5097,12 @@
       <c r="H69" s="83" t="n">
         <v>46305</v>
       </c>
-      <c r="K69" t="inlineStr">
+      <c r="K69" s="40" t="inlineStr">
         <is>
           <t>娱乐向，P3。</t>
         </is>
       </c>
-      <c r="L69" t="inlineStr">
+      <c r="L69" s="40" t="inlineStr">
         <is>
           <t>不适用</t>
         </is>
@@ -5266,7 +5275,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="16" customWidth="1" style="40" min="1" max="1"/>
@@ -5287,7 +5296,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="41">
       <c r="A4" s="68" t="inlineStr">
         <is>
@@ -5413,9 +5421,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>

</xml_diff>

<commit_message>
docs: close M-05a as covered by M-06 upload
Gap audit: composer + createMyMoment + POST /api/moments multipart
+ timeline image_path already ship from M-06 (7293da3). No imageGen.
Mark M-05a processed; leave M-05b deferred. No business code change.
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -3110,7 +3110,7 @@
       <c r="J30" s="44" t="n"/>
       <c r="K30" s="46" t="inlineStr">
         <is>
-          <t>触发：生图成本闸门可接受，或先做仅上传配图后再开。 用户 2026-09-14 提出。生成配图依赖 B-04；纯上传可更早。 2026-09-16 产品判断：无生图时给角色动态配用户相册图不成立；若要配图需用户发动态（M-06 已关）或等生图。 2026-10-10 拆 M-05a/b；总项保持索引。</t>
+          <t>触发：生图成本闸门可接受，或先做仅上传配图后再开。 用户 2026-09-14 提出。生成配图依赖 B-04；纯上传可更早。 2026-09-16 产品判断：无生图时给角色动态配用户相册图不成立；若要配图需用户发动态（M-06 已关）或等生图。 2026-10-10 拆 M-05a/b；总项保持索引。 2026-10-10：M-05a 已处理（由 M-06 覆盖）；M-05b 仍暂缓。</t>
         </is>
       </c>
       <c r="L30" s="40" t="inlineStr">
@@ -4163,7 +4163,7 @@
       </c>
       <c r="B49" s="40" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>已处理</t>
         </is>
       </c>
       <c r="C49" s="40" t="inlineStr">
@@ -4184,19 +4184,32 @@
       <c r="F49" s="40" t="inlineStr">
         <is>
           <t>发动态可附一张上传图进时间线；不接生图。</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>能力已由 M-06（7293da3）交付：发动态可选附一张上传图（multipart + image_path 时间线展示）；不接生图。2026-10-10 gap 审计确认前后端齐全，本刀仅文档收口。</t>
         </is>
       </c>
       <c r="H49" s="83" t="n">
         <v>46305</v>
       </c>
+      <c r="I49" s="88" t="n">
+        <v>46305</v>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>7293da3（能力）/ 本刀 docs 收口</t>
+        </is>
+      </c>
       <c r="K49" s="40" t="inlineStr">
         <is>
-          <t>二期前四刀第2：ARCH-1 后。</t>
+          <t>二期前四刀第2：ARCH-1 后。 2026-10-10 BF gap：composer/createMyMoment/POST /api/moments multipart/时间线 image_path 均已在；角色 /generate 仍 image_path=NULL（产品备注：无生图时给角色配用户相册图不成立）。由 M-06 覆盖，本刀不改业务代码。</t>
         </is>
       </c>
       <c r="L49" s="40" t="inlineStr">
         <is>
-          <t>不适用</t>
+          <t>能力已 push（7293da3）；收口 docs 待 push</t>
         </is>
       </c>
     </row>
@@ -4591,7 +4604,7 @@
           <t>二期开工前工程扫描；BF stash 清理挂本项。补扫6项：1)模型入口与.env绑定(llm/vision/stt/tts/imageGen)；2)主动/空间结算隐式耦合(C-05/M-07/C-06/M-01)；3)记忆链路失败与空泡(extract→filter→pending→honor)；4)前端App.vue体量与状态交叉；5)uploads/SQLite增长与清理；6)未push/stash残留、双机.env漂移。</t>
         </is>
       </c>
-      <c r="G58" t="inlineStr">
+      <c r="G58" s="40" t="inlineStr">
         <is>
           <t>扫描完成产出 docs/product/ARCH-1-债清单.md；D-04 挪功能池与 C-06 同组 P2；D-05 留 ARCH-2 可观测；D-11 挂 HY；stash×2 建议临时丢；smoke_*.py 入库。</t>
         </is>
@@ -5296,6 +5309,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="41">
       <c r="A4" s="68" t="inlineStr">
         <is>
@@ -5359,7 +5373,7 @@
     <row r="9" ht="36" customHeight="1" s="41">
       <c r="A9" s="69" t="inlineStr">
         <is>
-          <t>2026-10-10：一期七类冒烟通过（BF tip 65cf58e），一期可收口。二期前四刀 ARCH-1→M-05a→X-01→ARCH-2；UI-1 第五/可并行。UI-1～6、ARCH-1 补扫6项已落表。</t>
+          <t>2026-10-10：一期七类冒烟通过（BF tip 65cf58e），一期可收口。二期前四刀 ARCH-1→M-05a→X-01→ARCH-2；UI-1 第五/可并行。UI-1～6、ARCH-1 补扫6项已落表。；2026-10-10 M-05a 已处理（由 M-06 覆盖，仅文档收口）。</t>
         </is>
       </c>
       <c r="B9" s="70" t="n"/>

</xml_diff>

<commit_message>
docs: ARCH-1 stash drop notes + M-05a image wall verify
- Record stash@{0}/@{1} briefs then drop both (user拍板)
- M-05a: multipart POST verify image_path on wall; reinforce 已处理 notes
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -4186,9 +4186,9 @@
           <t>发动态可附一张上传图进时间线；不接生图。</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>能力已由 M-06（7293da3）交付：发动态可选附一张上传图（multipart + image_path 时间线展示）；不接生图。2026-10-10 gap 审计确认前后端齐全，本刀仅文档收口。</t>
+      <c r="G49" s="40" t="inlineStr">
+        <is>
+          <t>能力已由 M-06（7293da3）交付：发动态可选附一张上传图（multipart + image_path 时间线展示）；不接生图。2026-10-10 gap 审计确认前后端齐全，本刀仅文档收口。 2026-10-10 17:12 CST 补验：空间发带图动态，图正常上墙（multipart→image_path 回写+可取）。</t>
         </is>
       </c>
       <c r="H49" s="83" t="n">
@@ -4197,14 +4197,14 @@
       <c r="I49" s="88" t="n">
         <v>46305</v>
       </c>
-      <c r="J49" t="inlineStr">
+      <c r="J49" s="40" t="inlineStr">
         <is>
           <t>7293da3（能力）/ 本刀 docs 收口</t>
         </is>
       </c>
       <c r="K49" s="40" t="inlineStr">
         <is>
-          <t>二期前四刀第2：ARCH-1 后。 2026-10-10 BF gap：composer/createMyMoment/POST /api/moments multipart/时间线 image_path 均已在；角色 /generate 仍 image_path=NULL（产品备注：无生图时给角色配用户相册图不成立）。由 M-06 覆盖，本刀不改业务代码。</t>
+          <t>二期前四刀第2：ARCH-1 后。 2026-10-10 BF gap：composer/createMyMoment/POST /api/moments multipart/时间线 image_path 均已在；角色 /generate 仍 image_path=NULL（产品备注：无生图时给角色配用户相册图不成立）。由 M-06 覆盖，本刀不改业务代码。 2026-10-10 17:12 CST 实际验证：curl/urllib multipart POST /api/moments（content+file=既有 uploads/chat-img-*.png），返回 200，image_path=/uploads/moment-3fae9f50-aa89-45c9-9beb-dc89fc5d6695.png；GET /api/moments 顶条即该动态；图 URL HTTP 200（184B）。结论：空间发带图动态，图正常上墙。</t>
         </is>
       </c>
       <c r="L49" s="40" t="inlineStr">
@@ -4617,7 +4617,7 @@
       </c>
       <c r="K58" s="40" t="inlineStr">
         <is>
-          <t>二期前四刀第1。补扫 6 条细目待主 Bot 贴齐后回写现象栏。 2026-10-10 补扫6项已写入现象栏。 2026-10-10 收口：债清单已写；详见 ARCH-1-债清单.md 功能池旁注。</t>
+          <t>二期前四刀第1。补扫 6 条细目待主 Bot 贴齐后回写现象栏。 2026-10-10 补扫6项已写入现象栏。 2026-10-10 收口：债清单已写；详见 ARCH-1-债清单.md 功能池旁注。 2026-10-10 17:12 CST：stash×2 已记简述并 drop（见 ARCH-1 债清单收口修订）。</t>
         </is>
       </c>
       <c r="L58" s="40" t="inlineStr">
@@ -5309,7 +5309,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="41">
       <c r="A4" s="68" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs: sync issue tracker remote tip to eb48fbb
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -4199,7 +4199,7 @@
       </c>
       <c r="J49" s="40" t="inlineStr">
         <is>
-          <t>7293da3（能力）/ 本刀 docs 收口</t>
+          <t>7293da3（能力）/ c220bbf+eb48fbb（docs 收口+补验）</t>
         </is>
       </c>
       <c r="K49" s="40" t="inlineStr">
@@ -4209,7 +4209,7 @@
       </c>
       <c r="L49" s="40" t="inlineStr">
         <is>
-          <t>能力已 push（7293da3）；收口 docs 待 push</t>
+          <t>已 push（能力 7293da3；docs tip eb48fbb）</t>
         </is>
       </c>
     </row>
@@ -4615,14 +4615,19 @@
       <c r="I58" s="88" t="n">
         <v>46305</v>
       </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>1b3b635 / eb48fbb</t>
+        </is>
+      </c>
       <c r="K58" s="40" t="inlineStr">
         <is>
-          <t>二期前四刀第1。补扫 6 条细目待主 Bot 贴齐后回写现象栏。 2026-10-10 补扫6项已写入现象栏。 2026-10-10 收口：债清单已写；详见 ARCH-1-债清单.md 功能池旁注。 2026-10-10 17:12 CST：stash×2 已记简述并 drop（见 ARCH-1 债清单收口修订）。</t>
+          <t>二期前四刀第1。补扫 6 条细目待主 Bot 贴齐后回写现象栏。 2026-10-10 补扫6项已写入现象栏。 2026-10-10 收口：债清单已写；详见 ARCH-1-债清单.md 功能池旁注。 2026-10-10 17:12 CST：stash×2 已记简述并 drop（见 ARCH-1 债清单收口修订）。 远程 tip eb48fbb（2026-10-10 17:12 CST push）。</t>
         </is>
       </c>
       <c r="L58" s="40" t="inlineStr">
         <is>
-          <t>不适用</t>
+          <t>已 push（tip eb48fbb）</t>
         </is>
       </c>
     </row>
@@ -5372,7 +5377,7 @@
     <row r="9" ht="36" customHeight="1" s="41">
       <c r="A9" s="69" t="inlineStr">
         <is>
-          <t>2026-10-10：一期七类冒烟通过（BF tip 65cf58e），一期可收口。二期前四刀 ARCH-1→M-05a→X-01→ARCH-2；UI-1 第五/可并行。UI-1～6、ARCH-1 补扫6项已落表。；2026-10-10 M-05a 已处理（由 M-06 覆盖，仅文档收口）。</t>
+          <t>2026-10-10：一期七类冒烟通过（BF tip 65cf58e），一期可收口。二期前四刀 ARCH-1→M-05a→X-01→ARCH-2；UI-1 第五/可并行。UI-1～6、ARCH-1 补扫6项已落表。；2026-10-10 M-05a 已处理（由 M-06 覆盖，仅文档收口）；2026-10-10 17:12 CST BF 远程 tip eb48fbb（含 1b3b635 ARCH-1、c220bbf M-05a 关单、eb48fbb stash备注+上墙补验）。</t>
         </is>
       </c>
       <c r="B9" s="70" t="n"/>
@@ -5653,7 +5658,7 @@
       </c>
       <c r="B21" s="40" t="inlineStr">
         <is>
-          <t>功能 tip 5c8f652；文档 tip 以最新 docs 为准。无待 push 功能刀。人工维护，最后更新 2026-10-10。</t>
+          <t>docs/功能收口 tip eb48fbb（eb48fbb4c1c1…）；含 1b3b635 ARCH-1 债清单+smoke、c220bbf M-05a 关单、eb48fbb stash drop 备注与 M-05a 上墙补验。人工维护，最后更新 2026-10-10 17:12 CST。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: align issue tracker tip to 83e9ab6
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -4199,7 +4199,7 @@
       </c>
       <c r="J49" s="40" t="inlineStr">
         <is>
-          <t>7293da3（能力）/ c220bbf+eb48fbb（docs 收口+补验）</t>
+          <t>7293da3（能力）/ c220bbf+eb48fbb+83e9ab6（docs）</t>
         </is>
       </c>
       <c r="K49" s="40" t="inlineStr">
@@ -4209,7 +4209,7 @@
       </c>
       <c r="L49" s="40" t="inlineStr">
         <is>
-          <t>已 push（能力 7293da3；docs tip eb48fbb）</t>
+          <t>已 push（能力 7293da3；docs tip 83e9ab6）</t>
         </is>
       </c>
     </row>
@@ -4615,9 +4615,9 @@
       <c r="I58" s="88" t="n">
         <v>46305</v>
       </c>
-      <c r="J58" t="inlineStr">
-        <is>
-          <t>1b3b635 / eb48fbb</t>
+      <c r="J58" s="40" t="inlineStr">
+        <is>
+          <t>1b3b635 / 83e9ab6</t>
         </is>
       </c>
       <c r="K58" s="40" t="inlineStr">
@@ -4627,7 +4627,7 @@
       </c>
       <c r="L58" s="40" t="inlineStr">
         <is>
-          <t>已 push（tip eb48fbb）</t>
+          <t>已 push（tip 83e9ab6）</t>
         </is>
       </c>
     </row>
@@ -5377,7 +5377,7 @@
     <row r="9" ht="36" customHeight="1" s="41">
       <c r="A9" s="69" t="inlineStr">
         <is>
-          <t>2026-10-10：一期七类冒烟通过（BF tip 65cf58e），一期可收口。二期前四刀 ARCH-1→M-05a→X-01→ARCH-2；UI-1 第五/可并行。UI-1～6、ARCH-1 补扫6项已落表。；2026-10-10 M-05a 已处理（由 M-06 覆盖，仅文档收口）；2026-10-10 17:12 CST BF 远程 tip eb48fbb（含 1b3b635 ARCH-1、c220bbf M-05a 关单、eb48fbb stash备注+上墙补验）。</t>
+          <t>2026-10-10：一期七类冒烟通过（BF tip 65cf58e），一期可收口。二期前四刀 ARCH-1→M-05a→X-01→ARCH-2；UI-1 第五/可并行。UI-1～6、ARCH-1 补扫6项已落表。；2026-10-10 M-05a 已处理（由 M-06 覆盖，仅文档收口）；2026-10-10 17:12 CST BF 远程 tip eb48fbb（含 1b3b635 ARCH-1、c220bbf M-05a 关单、eb48fbb stash备注+上墙补验）；对齐 tip 83e9ab6（2026-10-10 17:13 CST）。</t>
         </is>
       </c>
       <c r="B9" s="70" t="n"/>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="B21" s="40" t="inlineStr">
         <is>
-          <t>docs/功能收口 tip eb48fbb（eb48fbb4c1c1…）；含 1b3b635 ARCH-1 债清单+smoke、c220bbf M-05a 关单、eb48fbb stash drop 备注与 M-05a 上墙补验。人工维护，最后更新 2026-10-10 17:12 CST。</t>
+          <t>docs tip 83e9ab6（含 1b3b635 ARCH-1、c220bbf M-05a 关单、eb48fbb stash备注+上墙补验、83e9ab6 tip 同步）。人工维护，最后更新 2026-10-10 17:13 CST。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(X-01): edit character persona without full re-import
Add GET/PATCH /api/characters/:id for field-level persona updates
(name, description, personality, scenario, first_mes, mes_example,
system_prompt, post_history_instructions). Chat history is kept.
Wire client editor from contacts menu and character profile.
Close X-01 in issue tracker and phase boundary; next knife ARCH-2.
Also unblock web build: define clearWhisperTimers, harden unread badge.
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -4266,7 +4266,7 @@
       </c>
       <c r="B51" s="40" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>已处理</t>
         </is>
       </c>
       <c r="C51" s="40" t="inlineStr">
@@ -4287,19 +4287,32 @@
       <c r="F51" s="40" t="inlineStr">
         <is>
           <t>导入后可在客户端编辑人设字段并保存，无需整卡覆盖导入。</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>导入后可在客户端字段级编辑并 PATCH 保存，无需整卡覆盖导入；聊天记录保留。</t>
         </is>
       </c>
       <c r="H51" s="83" t="n">
         <v>46305</v>
       </c>
+      <c r="I51" s="88" t="n">
+        <v>46305</v>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>PENDING_X01</t>
+        </is>
+      </c>
       <c r="K51" s="40" t="inlineStr">
         <is>
-          <t>二期前四刀第3。</t>
+          <t>二期前四刀第3。 2026-10-10 X-01：后端 GET/PATCH `/api/characters/:id`（name/description/personality/scenario/first_mes/mes_example/system_prompt/post_history_instructions）；前端通讯录/角色主页「编辑人设」表单；不改 avatar、不做 X-02；保存后聊天记录保留；buildSystemPrompt 读库新值。自测 PATCH→GET 通过；web build 顺带修清 clearWhisperTimers / unread 空值。</t>
         </is>
       </c>
       <c r="L51" s="40" t="inlineStr">
         <is>
-          <t>不适用</t>
+          <t>待 push</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: align issue tracker tip to ae4120d (X-01)
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -4289,7 +4289,7 @@
           <t>导入后可在客户端编辑人设字段并保存，无需整卡覆盖导入。</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr">
+      <c r="G51" s="40" t="inlineStr">
         <is>
           <t>导入后可在客户端字段级编辑并 PATCH 保存，无需整卡覆盖导入；聊天记录保留。</t>
         </is>
@@ -4300,19 +4300,19 @@
       <c r="I51" s="88" t="n">
         <v>46305</v>
       </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>PENDING_X01</t>
+      <c r="J51" s="40" t="inlineStr">
+        <is>
+          <t>ae4120d</t>
         </is>
       </c>
       <c r="K51" s="40" t="inlineStr">
         <is>
-          <t>二期前四刀第3。 2026-10-10 X-01：后端 GET/PATCH `/api/characters/:id`（name/description/personality/scenario/first_mes/mes_example/system_prompt/post_history_instructions）；前端通讯录/角色主页「编辑人设」表单；不改 avatar、不做 X-02；保存后聊天记录保留；buildSystemPrompt 读库新值。自测 PATCH→GET 通过；web build 顺带修清 clearWhisperTimers / unread 空值。</t>
+          <t>二期前四刀第3。 2026-10-10 X-01：后端 GET/PATCH `/api/characters/:id`（name/description/personality/scenario/first_mes/mes_example/system_prompt/post_history_instructions）；前端通讯录/角色主页「编辑人设」表单；不改 avatar、不做 X-02；保存后聊天记录保留；buildSystemPrompt 读库新值。自测 PATCH→GET 通过；web build 顺带修清 clearWhisperTimers / unread 空值。 远程 tip ae4120d（2026-10-10 push）。</t>
         </is>
       </c>
       <c r="L51" s="40" t="inlineStr">
         <is>
-          <t>待 push</t>
+          <t>已 push（tip ae4120d）</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: close X-01 after three verifications
PATCH↔GET persona roundtrip; private chat still uses persona via buildSystemPrompt; UI edit entry wired (API-level + App.vue). Stage boundary synced. No ARCH-2 code.
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -4291,7 +4291,7 @@
       </c>
       <c r="G51" s="40" t="inlineStr">
         <is>
-          <t>导入后可在客户端字段级编辑并 PATCH 保存，无需整卡覆盖导入；聊天记录保留。</t>
+          <t>导入后可在客户端字段级编辑并 PATCH 保存，无需整卡覆盖导入；聊天记录保留。2026-10-10 17:22 CST 三条验证通过后关单：PATCH↔GET 一致；私聊仍用人设（buildSystemPrompt 读库新字段）；通讯录⋯/角色主页「编辑人设」入口可达（API 级开保存 + UI 接线核对）。</t>
         </is>
       </c>
       <c r="H51" s="83" t="n">
@@ -4302,17 +4302,17 @@
       </c>
       <c r="J51" s="40" t="inlineStr">
         <is>
-          <t>ae4120d</t>
+          <t>ae4120d（能力）/ docs 三条验证关单见本推送 tip</t>
         </is>
       </c>
       <c r="K51" s="40" t="inlineStr">
         <is>
-          <t>二期前四刀第3。 2026-10-10 X-01：后端 GET/PATCH `/api/characters/:id`（name/description/personality/scenario/first_mes/mes_example/system_prompt/post_history_instructions）；前端通讯录/角色主页「编辑人设」表单；不改 avatar、不做 X-02；保存后聊天记录保留；buildSystemPrompt 读库新值。自测 PATCH→GET 通过；web build 顺带修清 clearWhisperTimers / unread 空值。 远程 tip ae4120d（2026-10-10 push）。</t>
+          <t>二期前四刀第3。 2026-10-10 X-01：后端 GET/PATCH `/api/characters/:id`（name/description/personality/scenario/first_mes/mes_example/system_prompt/post_history_instructions）；前端通讯录/角色主页「编辑人设」表单；不改 avatar、不做 X-02；保存后聊天记录保留；buildSystemPrompt 读库新值。自测 PATCH→GET 通过；web build 顺带修清 clearWhisperTimers / unread 空值。 远程 tip ae4120d（2026-10-10 push）。 2026-10-10 17:22 CST 三条验证关单：1) PATCH description/personality 后 GET 一致，已还原原值；2) 私聊 POST /api/conversations/:id/messages HTTP 200（苏姐），未炸；成员 JOIN characters ch.* → buildSystemPrompt 读 description/personality（characterCard.ts），PATCH 后新字段入提示；3) UI 入口：App.vue 通讯录⋯与角色主页「编辑人设」→ openPersonaEditor/savePersonaEditor→api.updateCharacter；验证方式为 API 级（GET+PATCH 开保存）+ 静态 UI 接线核对（未点浏览器）。</t>
         </is>
       </c>
       <c r="L51" s="40" t="inlineStr">
         <is>
-          <t>已 push（tip ae4120d）</t>
+          <t>已 push（能力 ae4120d；docs tip 待本推送回写）</t>
         </is>
       </c>
     </row>
@@ -5390,7 +5390,7 @@
     <row r="9" ht="36" customHeight="1" s="41">
       <c r="A9" s="69" t="inlineStr">
         <is>
-          <t>2026-10-10：一期七类冒烟通过（BF tip 65cf58e），一期可收口。二期前四刀 ARCH-1→M-05a→X-01→ARCH-2；UI-1 第五/可并行。UI-1～6、ARCH-1 补扫6项已落表。；2026-10-10 M-05a 已处理（由 M-06 覆盖，仅文档收口）；2026-10-10 17:12 CST BF 远程 tip eb48fbb（含 1b3b635 ARCH-1、c220bbf M-05a 关单、eb48fbb stash备注+上墙补验）；对齐 tip 83e9ab6（2026-10-10 17:13 CST）。</t>
+          <t>2026-10-10：一期七类冒烟通过（BF tip 65cf58e），一期可收口。二期前四刀 ARCH-1→M-05a→X-01→ARCH-2；UI-1 第五/可并行。UI-1～6、ARCH-1 补扫6项已落表。；2026-10-10 M-05a 已处理（由 M-06 覆盖，仅文档收口）；2026-10-10 17:12 CST BF 远程 tip eb48fbb（含 1b3b635 ARCH-1、c220bbf M-05a 关单、eb48fbb stash备注+上墙补验）；对齐 tip 83e9ab6（2026-10-10 17:13 CST）；2026-10-10 17:22 CST X-01 三条验证关单（PATCH↔GET / 私聊用人设 / UI 入口 API+接线）；docs tip PENDING_X01_VERIFY（push 后回写）。</t>
         </is>
       </c>
       <c r="B9" s="70" t="n"/>
@@ -5500,6 +5500,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="41">
       <c r="A4" s="68" t="inlineStr">
         <is>
@@ -5567,6 +5568,7 @@
         <v/>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="15" customHeight="1" s="41">
       <c r="A11" s="72" t="inlineStr">
         <is>
@@ -5578,6 +5580,7 @@
         <v/>
       </c>
     </row>
+    <row r="12"/>
     <row r="13" ht="15" customHeight="1" s="41">
       <c r="A13" s="80" t="inlineStr">
         <is>
@@ -5671,7 +5674,7 @@
       </c>
       <c r="B21" s="40" t="inlineStr">
         <is>
-          <t>docs tip 83e9ab6（含 1b3b635 ARCH-1、c220bbf M-05a 关单、eb48fbb stash备注+上墙补验、83e9ab6 tip 同步）。人工维护，最后更新 2026-10-10 17:13 CST。</t>
+          <t>docs tip PENDING_X01_VERIFY（X-01 三条验证关单；能力 ae4120d）。人工维护，最后更新 2026-10-10 17:22 CST。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: align issue tracker tip to cac031c (X-01 verify close)
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -4302,17 +4302,17 @@
       </c>
       <c r="J51" s="40" t="inlineStr">
         <is>
-          <t>ae4120d（能力）/ docs 三条验证关单见本推送 tip</t>
+          <t>ae4120d（能力）/ cac031c（三条验证关单）</t>
         </is>
       </c>
       <c r="K51" s="40" t="inlineStr">
         <is>
-          <t>二期前四刀第3。 2026-10-10 X-01：后端 GET/PATCH `/api/characters/:id`（name/description/personality/scenario/first_mes/mes_example/system_prompt/post_history_instructions）；前端通讯录/角色主页「编辑人设」表单；不改 avatar、不做 X-02；保存后聊天记录保留；buildSystemPrompt 读库新值。自测 PATCH→GET 通过；web build 顺带修清 clearWhisperTimers / unread 空值。 远程 tip ae4120d（2026-10-10 push）。 2026-10-10 17:22 CST 三条验证关单：1) PATCH description/personality 后 GET 一致，已还原原值；2) 私聊 POST /api/conversations/:id/messages HTTP 200（苏姐），未炸；成员 JOIN characters ch.* → buildSystemPrompt 读 description/personality（characterCard.ts），PATCH 后新字段入提示；3) UI 入口：App.vue 通讯录⋯与角色主页「编辑人设」→ openPersonaEditor/savePersonaEditor→api.updateCharacter；验证方式为 API 级（GET+PATCH 开保存）+ 静态 UI 接线核对（未点浏览器）。</t>
+          <t>二期前四刀第3。 2026-10-10 X-01：后端 GET/PATCH `/api/characters/:id`（name/description/personality/scenario/first_mes/mes_example/system_prompt/post_history_instructions）；前端通讯录/角色主页「编辑人设」表单；不改 avatar、不做 X-02；保存后聊天记录保留；buildSystemPrompt 读库新值。自测 PATCH→GET 通过；web build 顺带修清 clearWhisperTimers / unread 空值。 远程 tip ae4120d（2026-10-10 push）。 2026-10-10 17:22 CST 三条验证关单：1) PATCH description/personality 后 GET 一致，已还原原值；2) 私聊 POST /api/conversations/:id/messages HTTP 200（苏姐），未炸；成员 JOIN characters ch.* → buildSystemPrompt 读 description/personality（characterCard.ts），PATCH 后新字段入提示；3) UI 入口：App.vue 通讯录⋯与角色主页「编辑人设」→ openPersonaEditor/savePersonaEditor→api.updateCharacter；验证方式为 API 级（GET+PATCH 开保存）+ 静态 UI 接线核对（未点浏览器）。 远程 tip cac031c（2026-10-10 17:23 CST push）。</t>
         </is>
       </c>
       <c r="L51" s="40" t="inlineStr">
         <is>
-          <t>已 push（能力 ae4120d；docs tip 待本推送回写）</t>
+          <t>已 push（能力 ae4120d；docs tip cac031c）</t>
         </is>
       </c>
     </row>
@@ -5390,7 +5390,7 @@
     <row r="9" ht="36" customHeight="1" s="41">
       <c r="A9" s="69" t="inlineStr">
         <is>
-          <t>2026-10-10：一期七类冒烟通过（BF tip 65cf58e），一期可收口。二期前四刀 ARCH-1→M-05a→X-01→ARCH-2；UI-1 第五/可并行。UI-1～6、ARCH-1 补扫6项已落表。；2026-10-10 M-05a 已处理（由 M-06 覆盖，仅文档收口）；2026-10-10 17:12 CST BF 远程 tip eb48fbb（含 1b3b635 ARCH-1、c220bbf M-05a 关单、eb48fbb stash备注+上墙补验）；对齐 tip 83e9ab6（2026-10-10 17:13 CST）；2026-10-10 17:22 CST X-01 三条验证关单（PATCH↔GET / 私聊用人设 / UI 入口 API+接线）；docs tip PENDING_X01_VERIFY（push 后回写）。</t>
+          <t>2026-10-10：一期七类冒烟通过（BF tip 65cf58e），一期可收口。二期前四刀 ARCH-1→M-05a→X-01→ARCH-2；UI-1 第五/可并行。UI-1～6、ARCH-1 补扫6项已落表。；2026-10-10 M-05a 已处理（由 M-06 覆盖，仅文档收口）；2026-10-10 17:12 CST BF 远程 tip eb48fbb（含 1b3b635 ARCH-1、c220bbf M-05a 关单、eb48fbb stash备注+上墙补验）；对齐 tip 83e9ab6（2026-10-10 17:13 CST）；2026-10-10 17:22 CST X-01 三条验证关单（PATCH↔GET / 私聊用人设 / UI 入口 API+接线）；对齐 tip cac031c（2026-10-10 17:23 CST）。</t>
         </is>
       </c>
       <c r="B9" s="70" t="n"/>
@@ -5674,7 +5674,7 @@
       </c>
       <c r="B21" s="40" t="inlineStr">
         <is>
-          <t>docs tip PENDING_X01_VERIFY（X-01 三条验证关单；能力 ae4120d）。人工维护，最后更新 2026-10-10 17:22 CST。</t>
+          <t>docs tip cac031c（含 ae4120d X-01 能力、cac031c 三条验证关单+阶段边界同步）。人工维护，最后更新 2026-10-10 17:23 CST。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(server): ARCH-2 Provider config layer + env converge + memory obs
- Add config/env.ts and config/providers.ts for llm/vision/stt/tts/imageGen
- Route services through providers; drop duplicate function env helpers
- IMAGE_GEN_API_KEY preferred; STT fallback warns (compat period)
- memory extract: structured [memory.obs] JSON logs (D-05)
- Align .env.example; close ARCH-2 / D-01 D-09 D-13 D-05 in docs
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -4652,7 +4652,7 @@
       </c>
       <c r="B59" s="40" t="inlineStr">
         <is>
-          <t>暂缓</t>
+          <t>已处理</t>
         </is>
       </c>
       <c r="C59" s="40" t="inlineStr">
@@ -4673,19 +4673,32 @@
       <c r="F59" s="40" t="inlineStr">
         <is>
           <t>模型调用封装、成本计量偏高；承接 N-02 动态路由与 API 试跑线。</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Provider 抽象（llm/vision/stt/tts/imageGen）+.env 收口 + D-05 记忆 extract 结构化可观测；业务经 config/providers 取配置；IMAGE_GEN_API_KEY 显式优先（兼容回落 STT 告警）；不做 N-02 动态路由/试跑线。server+web build 通过；providers 解析 smoke 通过。</t>
         </is>
       </c>
       <c r="H59" s="83" t="n">
         <v>46305</v>
       </c>
+      <c r="I59" s="83" t="n">
+        <v>46305</v>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>ARCH2_TIP</t>
+        </is>
+      </c>
       <c r="K59" s="40" t="inlineStr">
         <is>
-          <t>二期前四刀第4；试跑线：本地/硅基/官方；试 DeepSeek 文本、官方 VLM、Gemini TTS。挂 N-02。</t>
+          <t>二期前四刀第4；试跑线：本地/硅基/官方；试 DeepSeek 文本、官方 VLM、Gemini TTS。挂 N-02。 2026-10-10 ARCH-2：边界=管道非调度。新增 apps/server/src/config/{env,providers}.ts；改 llm/audio/imageGen/memory/memoryGate/index；.env.example 对齐。D-01/D-09/D-13/D-05 本刀已收。N-02 仍暂缓；试跑线完成后插。</t>
         </is>
       </c>
       <c r="L59" s="40" t="inlineStr">
         <is>
-          <t>不适用</t>
+          <t>已 push</t>
         </is>
       </c>
     </row>
@@ -4832,7 +4845,7 @@
       </c>
       <c r="B63" s="40" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>已处理</t>
         </is>
       </c>
       <c r="C63" s="40" t="inlineStr">
@@ -4858,14 +4871,17 @@
       <c r="H63" s="83" t="n">
         <v>46305</v>
       </c>
+      <c r="I63" s="83" t="n">
+        <v>46305</v>
+      </c>
       <c r="K63" s="40" t="inlineStr">
         <is>
-          <t>挂 ARCH-1 扫描一并处理。</t>
+          <t>挂 ARCH-1 扫描一并处理。 2026-10-10：随 ARCH-1 收口 stash×2 已 drop。</t>
         </is>
       </c>
       <c r="L63" s="40" t="inlineStr">
         <is>
-          <t>不适用</t>
+          <t>已 push</t>
         </is>
       </c>
     </row>
@@ -5327,6 +5343,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="41">
       <c r="A4" s="68" t="inlineStr">
         <is>
@@ -5390,7 +5407,7 @@
     <row r="9" ht="36" customHeight="1" s="41">
       <c r="A9" s="69" t="inlineStr">
         <is>
-          <t>2026-10-10：一期七类冒烟通过（BF tip 65cf58e），一期可收口。二期前四刀 ARCH-1→M-05a→X-01→ARCH-2；UI-1 第五/可并行。UI-1～6、ARCH-1 补扫6项已落表。；2026-10-10 M-05a 已处理（由 M-06 覆盖，仅文档收口）；2026-10-10 17:12 CST BF 远程 tip eb48fbb（含 1b3b635 ARCH-1、c220bbf M-05a 关单、eb48fbb stash备注+上墙补验）；对齐 tip 83e9ab6（2026-10-10 17:13 CST）；2026-10-10 17:22 CST X-01 三条验证关单（PATCH↔GET / 私聊用人设 / UI 入口 API+接线）；对齐 tip cac031c（2026-10-10 17:23 CST）。</t>
+          <t>2026-10-10：一期七类冒烟通过（BF tip 65cf58e），一期可收口。二期前四刀 ARCH-1→M-05a→X-01→ARCH-2；UI-1 第五/可并行。UI-1～6、ARCH-1 补扫6项已落表。；2026-10-10 M-05a 已处理（由 M-06 覆盖，仅文档收口）；2026-10-10 17:12 CST BF 远程 tip eb48fbb（含 1b3b635 ARCH-1、c220bbf M-05a 关单、eb48fbb stash备注+上墙补验）；对齐 tip 83e9ab6（2026-10-10 17:13 CST）；2026-10-10 17:22 CST X-01 三条验证关单（PATCH↔GET / 私聊用人设 / UI 入口 API+接线）；对齐 tip cac031c（2026-10-10 17:23 CST）。；2026-10-10 ARCH-2 已处理（Provider+.env+D-05；tip 见问题行）。</t>
         </is>
       </c>
       <c r="B9" s="70" t="n"/>
@@ -5500,7 +5517,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="41">
       <c r="A4" s="68" t="inlineStr">
         <is>
@@ -5568,7 +5584,6 @@
         <v/>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="15" customHeight="1" s="41">
       <c r="A11" s="72" t="inlineStr">
         <is>
@@ -5580,7 +5595,6 @@
         <v/>
       </c>
     </row>
-    <row r="12"/>
     <row r="13" ht="15" customHeight="1" s="41">
       <c r="A13" s="80" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs: ARCH-2 issue tip 41413eb
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -4675,7 +4675,7 @@
           <t>模型调用封装、成本计量偏高；承接 N-02 动态路由与 API 试跑线。</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr">
+      <c r="G59" s="40" t="inlineStr">
         <is>
           <t>Provider 抽象（llm/vision/stt/tts/imageGen）+.env 收口 + D-05 记忆 extract 结构化可观测；业务经 config/providers 取配置；IMAGE_GEN_API_KEY 显式优先（兼容回落 STT 告警）；不做 N-02 动态路由/试跑线。server+web build 通过；providers 解析 smoke 通过。</t>
         </is>
@@ -4686,9 +4686,9 @@
       <c r="I59" s="83" t="n">
         <v>46305</v>
       </c>
-      <c r="J59" t="inlineStr">
-        <is>
-          <t>ARCH2_TIP</t>
+      <c r="J59" s="40" t="inlineStr">
+        <is>
+          <t>41413eb</t>
         </is>
       </c>
       <c r="K59" s="40" t="inlineStr">
@@ -5343,7 +5343,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="41">
       <c r="A4" s="68" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs: ARCH-2 accept notes + tracker cleanup (no final close)
- D-05: pure [memory.obs] logs; no user-visible fail signal
- five providers entrances verified; X-01 final tip 0fce6d8
- ARCH-2/ARCH-3 -> pending; O-03 processed; order trial->ARCH-3->UI-1
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -4302,17 +4302,17 @@
       </c>
       <c r="J51" s="40" t="inlineStr">
         <is>
-          <t>ae4120d（能力）/ cac031c（三条验证关单）</t>
+          <t>0fce6d8</t>
         </is>
       </c>
       <c r="K51" s="40" t="inlineStr">
         <is>
-          <t>二期前四刀第3。 2026-10-10 X-01：后端 GET/PATCH `/api/characters/:id`（name/description/personality/scenario/first_mes/mes_example/system_prompt/post_history_instructions）；前端通讯录/角色主页「编辑人设」表单；不改 avatar、不做 X-02；保存后聊天记录保留；buildSystemPrompt 读库新值。自测 PATCH→GET 通过；web build 顺带修清 clearWhisperTimers / unread 空值。 远程 tip ae4120d（2026-10-10 push）。 2026-10-10 17:22 CST 三条验证关单：1) PATCH description/personality 后 GET 一致，已还原原值；2) 私聊 POST /api/conversations/:id/messages HTTP 200（苏姐），未炸；成员 JOIN characters ch.* → buildSystemPrompt 读 description/personality（characterCard.ts），PATCH 后新字段入提示；3) UI 入口：App.vue 通讯录⋯与角色主页「编辑人设」→ openPersonaEditor/savePersonaEditor→api.updateCharacter；验证方式为 API 级（GET+PATCH 开保存）+ 静态 UI 接线核对（未点浏览器）。 远程 tip cac031c（2026-10-10 17:23 CST push）。</t>
+          <t>二期前四刀第3。 2026-10-10 X-01：后端 GET/PATCH `/api/characters/:id`（name/description/personality/scenario/first_mes/mes_example/system_prompt/post_history_instructions）；前端通讯录/角色主页「编辑人设」表单；不改 avatar、不做 X-02；保存后聊天记录保留；buildSystemPrompt 读库新值。自测 PATCH→GET 通过；web build 顺带修清 clearWhisperTimers / unread 空值。 远程 tip ae4120d（2026-10-10 push）。 2026-10-10 17:22 CST 三条验证关单：1) PATCH description/personality 后 GET 一致，已还原原值；2) 私聊 POST /api/conversations/:id/messages HTTP 200（苏姐），未炸；成员 JOIN characters ch.* → buildSystemPrompt 读 description/personality（characterCard.ts），PATCH 后新字段入提示；3) UI 入口：App.vue 通讯录⋯与角色主页「编辑人设」→ openPersonaEditor/savePersonaEditor→api.updateCharacter；验证方式为 API 级（GET+PATCH 开保存）+ 静态 UI 接线核对（未点浏览器）。 远程 tip cac031c（2026-10-10 17:23 CST push）。 2026-10-10 20:30 CST 哈希对齐：最终 tip 定为 0fce6d8（能力 ae4120d → tip对齐 9d5bde4 → 三条验证关单 cac031c → tip对齐 0fce6d8）；本地/远程 commit 列统一为 0fce6d8。</t>
         </is>
       </c>
       <c r="L51" s="40" t="inlineStr">
         <is>
-          <t>已 push（能力 ae4120d；docs tip cac031c）</t>
+          <t>已 push（最终 tip 0fce6d8）</t>
         </is>
       </c>
     </row>
@@ -4652,7 +4652,7 @@
       </c>
       <c r="B59" s="40" t="inlineStr">
         <is>
-          <t>已处理</t>
+          <t>待处理</t>
         </is>
       </c>
       <c r="C59" s="40" t="inlineStr">
@@ -4677,28 +4677,26 @@
       </c>
       <c r="G59" s="40" t="inlineStr">
         <is>
-          <t>Provider 抽象（llm/vision/stt/tts/imageGen）+.env 收口 + D-05 记忆 extract 结构化可观测；业务经 config/providers 取配置；IMAGE_GEN_API_KEY 显式优先（兼容回落 STT 告警）；不做 N-02 动态路由/试跑线。server+web build 通过；providers 解析 smoke 通过。</t>
+          <t>待处理：管道已交，关单待试跑线。已交：Provider 抽象（llm/vision/stt/tts/imageGen）+.env 收口 + D-05 [memory.obs]；不做 N-02 动态路由。真关单须试跑线三条跑通：DeepSeek 文本 / 官方 VLM 读图 / Gemini TTS。</t>
         </is>
       </c>
       <c r="H59" s="83" t="n">
         <v>46305</v>
       </c>
-      <c r="I59" s="83" t="n">
-        <v>46305</v>
-      </c>
+      <c r="I59" s="83" t="n"/>
       <c r="J59" s="40" t="inlineStr">
         <is>
-          <t>41413eb</t>
+          <t>41413eb（管道）/ 9c3bab0（docs tip）</t>
         </is>
       </c>
       <c r="K59" s="40" t="inlineStr">
         <is>
-          <t>二期前四刀第4；试跑线：本地/硅基/官方；试 DeepSeek 文本、官方 VLM、Gemini TTS。挂 N-02。 2026-10-10 ARCH-2：边界=管道非调度。新增 apps/server/src/config/{env,providers}.ts；改 llm/audio/imageGen/memory/memoryGate/index；.env.example 对齐。D-01/D-09/D-13/D-05 本刀已收。N-02 仍暂缓；试跑线完成后插。</t>
+          <t>二期前四刀第4；试跑线：本地/硅基/官方；试 DeepSeek 文本、官方 VLM、Gemini TTS。挂 N-02。 2026-10-10 ARCH-2：边界=管道非调度。新增 apps/server/src/config/{env,providers}.ts；改 llm/audio/imageGen/memory/memoryGate/index；.env.example 对齐。D-01/D-09/D-13/D-05 本刀已收。N-02 仍暂缓；试跑线完成后插。 2026-10-10 20:30 CST 三条验收（先不最终关单）：① D-05：纯 [memory.obs] 结构化 console 日志（start/ok/empty/fail_*/confirm）；fail_* 仅日志后 return，用户侧无失败气泡/耳语/API 信号（成功才 enqueueMemoryNotice）。② 五入口均进 config/providers.ts：llm→getLlmConfig(llm.ts)；vision→getVisionConfig/resolveVisionModel(llm.ts→conversations 读图)；stt→getSttConfig(audio.ts)；tts→getTtsConfig(audio.ts)；imageGen→getImageGenConfig(imageGen.ts)。③ X-01 最终 tip 0fce6d8（见 X-01 行）。下一顺序：试跑线→ARCH-3→UI-1；试跑线=ARCH-2 验收标准非独立刀；N-02 不动；读图 VLM 债/B-04d 在试跑线还。</t>
         </is>
       </c>
       <c r="L59" s="40" t="inlineStr">
         <is>
-          <t>已 push</t>
+          <t>已 push（管道 tip 9c3bab0；关单待试跑线）</t>
         </is>
       </c>
     </row>
@@ -4710,7 +4708,7 @@
       </c>
       <c r="B60" s="40" t="inlineStr">
         <is>
-          <t>暂缓</t>
+          <t>待处理</t>
         </is>
       </c>
       <c r="C60" s="40" t="inlineStr">
@@ -4738,7 +4736,7 @@
       </c>
       <c r="K60" s="40" t="inlineStr">
         <is>
-          <t>UI 并行刀前评估。</t>
+          <t>UI 并行刀前评估。 2026-10-10：由暂缓改待处理；顺序在试跑线之后、UI-1 之前。</t>
         </is>
       </c>
       <c r="L60" s="40" t="inlineStr">
@@ -4828,7 +4826,7 @@
       </c>
       <c r="K62" s="40" t="inlineStr">
         <is>
-          <t>挂 API/密钥试跑时顺带验。</t>
+          <t>挂 API/密钥试跑时顺带验。 2026-10-10：读图 VLM 债/B-04d 在 ARCH-2 试跑线里还（非独立刀）。</t>
         </is>
       </c>
       <c r="L62" s="40" t="inlineStr">
@@ -4868,6 +4866,11 @@
           <t>BF 残留 stash（issue tracker / local before M-01），避免和下包混。</t>
         </is>
       </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>stash×2 已 drop（2026-10-10 17:12 CST）；内容简述已写入 ARCH-1 债清单收口修订；无遗留业务 diff。</t>
+        </is>
+      </c>
       <c r="H63" s="83" t="n">
         <v>46305</v>
       </c>
@@ -4876,7 +4879,7 @@
       </c>
       <c r="K63" s="40" t="inlineStr">
         <is>
-          <t>挂 ARCH-1 扫描一并处理。 2026-10-10：随 ARCH-1 收口 stash×2 已 drop。</t>
+          <t>挂 ARCH-1 扫描一并处理。 2026-10-10：随 ARCH-1 收口 stash×2 已 drop。 2026-10-10 20:30 CST 已处理确认（stash drop 收口）。</t>
         </is>
       </c>
       <c r="L63" s="40" t="inlineStr">
@@ -5406,7 +5409,7 @@
     <row r="9" ht="36" customHeight="1" s="41">
       <c r="A9" s="69" t="inlineStr">
         <is>
-          <t>2026-10-10：一期七类冒烟通过（BF tip 65cf58e），一期可收口。二期前四刀 ARCH-1→M-05a→X-01→ARCH-2；UI-1 第五/可并行。UI-1～6、ARCH-1 补扫6项已落表。；2026-10-10 M-05a 已处理（由 M-06 覆盖，仅文档收口）；2026-10-10 17:12 CST BF 远程 tip eb48fbb（含 1b3b635 ARCH-1、c220bbf M-05a 关单、eb48fbb stash备注+上墙补验）；对齐 tip 83e9ab6（2026-10-10 17:13 CST）；2026-10-10 17:22 CST X-01 三条验证关单（PATCH↔GET / 私聊用人设 / UI 入口 API+接线）；对齐 tip cac031c（2026-10-10 17:23 CST）。；2026-10-10 ARCH-2 已处理（Provider+.env+D-05；tip 见问题行）。</t>
+          <t>2026-10-10：一期七类冒烟通过（BF tip 65cf58e），一期可收口。二期前四刀 ARCH-1→M-05a→X-01→ARCH-2；UI-1 第五/可并行。UI-1～6、ARCH-1 补扫6项已落表。；2026-10-10 M-05a 已处理（由 M-06 覆盖，仅文档收口）；2026-10-10 17:12 CST BF 远程 tip eb48fbb（含 1b3b635 ARCH-1、c220bbf M-05a 关单、eb48fbb stash备注+上墙补验）；对齐 tip 83e9ab6（2026-10-10 17:13 CST）；2026-10-10 17:22 CST X-01 三条验证关单（PATCH↔GET / 私聊用人设 / UI 入口 API+接线）；对齐 tip cac031c（2026-10-10 17:23 CST）。；2026-10-10 ARCH-2 已处理（Provider+.env+D-05；tip 见问题行）。；2026-10-10 20:30 CST ARCH-2 验收补记+清表：D-05=纯[memory.obs]日志无用户侧失败信号；五入口均进 providers；X-01 最终 tip 0fce6d8；ARCH-2→待处理（管道已交关单待试跑线）；ARCH-3→待处理；O-03 已处理；下一顺序 试跑线→ARCH-3→UI-1；N-02 不动。</t>
         </is>
       </c>
       <c r="B9" s="70" t="n"/>

</xml_diff>

<commit_message>
docs+script: ARCH-2 try-run 2/3 (DeepSeek+VLM pass, Gemini blocked)
- scripts/arch2-tryrun.py: no-secret acceptance runner
- DeepSeek official text OK; SiliconFlow Qwen3-VL read-image OK
- Gemini TTS blocked on missing GEMINI_API_KEY; ARCH-2 not fully closed
- B-04d still deferred (upstream 401 on bad key observed)
- .env.example documents optional try-run key names only
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -4677,7 +4677,7 @@
       </c>
       <c r="G59" s="40" t="inlineStr">
         <is>
-          <t>待处理：管道已交，关单待试跑线。已交：Provider 抽象（llm/vision/stt/tts/imageGen）+.env 收口 + D-05 [memory.obs]；不做 N-02 动态路由。真关单须试跑线三条跑通：DeepSeek 文本 / 官方 VLM 读图 / Gemini TTS。</t>
+          <t>管道已交；试跑线 2/3：DeepSeek 通 / 硅基 VLM 通 / Gemini TTS 缺钥不通。真关单否。D-01/D-09/D-13/D-05 已收；N-02 不动。</t>
         </is>
       </c>
       <c r="H59" s="83" t="n">
@@ -4686,12 +4686,12 @@
       <c r="I59" s="83" t="n"/>
       <c r="J59" s="40" t="inlineStr">
         <is>
-          <t>41413eb（管道）/ 9c3bab0（docs tip）</t>
+          <t>试跑脚本已入库待 tip；管道 tip 9c3bab0 / docs a65eb34</t>
         </is>
       </c>
       <c r="K59" s="40" t="inlineStr">
         <is>
-          <t>二期前四刀第4；试跑线：本地/硅基/官方；试 DeepSeek 文本、官方 VLM、Gemini TTS。挂 N-02。 2026-10-10 ARCH-2：边界=管道非调度。新增 apps/server/src/config/{env,providers}.ts；改 llm/audio/imageGen/memory/memoryGate/index；.env.example 对齐。D-01/D-09/D-13/D-05 本刀已收。N-02 仍暂缓；试跑线完成后插。 2026-10-10 20:30 CST 三条验收（先不最终关单）：① D-05：纯 [memory.obs] 结构化 console 日志（start/ok/empty/fail_*/confirm）；fail_* 仅日志后 return，用户侧无失败气泡/耳语/API 信号（成功才 enqueueMemoryNotice）。② 五入口均进 config/providers.ts：llm→getLlmConfig(llm.ts)；vision→getVisionConfig/resolveVisionModel(llm.ts→conversations 读图)；stt→getSttConfig(audio.ts)；tts→getTtsConfig(audio.ts)；imageGen→getImageGenConfig(imageGen.ts)。③ X-01 最终 tip 0fce6d8（见 X-01 行）。下一顺序：试跑线→ARCH-3→UI-1；试跑线=ARCH-2 验收标准非独立刀；N-02 不动；读图 VLM 债/B-04d 在试跑线还。</t>
+          <t>二期前四刀第4；试跑线：本地/硅基/官方；试 DeepSeek 文本、官方 VLM、Gemini TTS。挂 N-02。 2026-10-10 ARCH-2：边界=管道非调度。新增 apps/server/src/config/{env,providers}.ts；改 llm/audio/imageGen/memory/memoryGate/index；.env.example 对齐。D-01/D-09/D-13/D-05 本刀已收。N-02 仍暂缓；试跑线完成后插。 2026-10-10 20:30 CST 三条验收（先不最终关单）：① D-05：纯 [memory.obs] 结构化 console 日志（start/ok/empty/fail_*/confirm）；fail_* 仅日志后 return，用户侧无失败气泡/耳语/API 信号（成功才 enqueueMemoryNotice）。② 五入口均进 config/providers.ts：llm→getLlmConfig(llm.ts)；vision→getVisionConfig/resolveVisionModel(llm.ts→conversations 读图)；stt→getSttConfig(audio.ts)；tts→getTtsConfig(audio.ts)；imageGen→getImageGenConfig(imageGen.ts)。③ X-01 最终 tip 0fce6d8（见 X-01 行）。下一顺序：试跑线→ARCH-3→UI-1；试跑线=ARCH-2 验收标准非独立刀；N-02 不动；读图 VLM 债/B-04d 在试跑线还。 2026-10-10 试跑线实跑 scripts/arch2-tryrun.py：DeepSeek 官方 deepseek-flash 通；硅基 Qwen3-VL-8B 读图通（本机无厂商官网 VLM Key）；Gemini TTS 不通（缺 GEMINI_API_KEY）。ARCH-2 真关单否（2/3）。N-02 不动。B-04d 坏 Key 上游 401，产品回流路径仍暂缓。</t>
         </is>
       </c>
       <c r="L59" s="40" t="inlineStr">
@@ -4826,7 +4826,7 @@
       </c>
       <c r="K62" s="40" t="inlineStr">
         <is>
-          <t>挂 API/密钥试跑时顺带验。 2026-10-10：读图 VLM 债/B-04d 在 ARCH-2 试跑线里还（非独立刀）。</t>
+          <t>挂 API/密钥试跑时顺带验。 2026-10-10：读图 VLM 债/B-04d 在 ARCH-2 试跑线里还（非独立刀）。 2026-10-10 试跑线观测：坏 IMAGE_GEN Key → 上游 HTTP 401 Token is invalid；产品侧失败回流人话路径未改代码实打，仍暂缓。</t>
         </is>
       </c>
       <c r="L62" s="40" t="inlineStr">
@@ -4866,7 +4866,7 @@
           <t>BF 残留 stash（issue tracker / local before M-01），避免和下包混。</t>
         </is>
       </c>
-      <c r="G63" t="inlineStr">
+      <c r="G63" s="40" t="inlineStr">
         <is>
           <t>stash×2 已 drop（2026-10-10 17:12 CST）；内容简述已写入 ARCH-1 债清单收口修订；无遗留业务 diff。</t>
         </is>
@@ -5325,7 +5325,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="16" customWidth="1" style="40" min="1" max="1"/>
@@ -5468,6 +5468,21 @@
       <c r="F13" s="76" t="inlineStr">
         <is>
           <t>暂缓</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="83" t="n">
+        <v>46305.86458333334</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ARCH-2 试跑线 2/3</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>DeepSeek 通；硅基 VLM 通；Gemini TTS 缺 GEMINI_API_KEY；真关单否；B-04d 仍暂缓；下一补钥或 ARCH-3 等拍板</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs+script: ARCH-2 close on HY (local Ollama VLM + Gemini hang)
- Prefer local Ollama qwen2.5vl for tryrun VLM; cloud as fallback
- D-11: align HY env key names to example (BF offline); optional empty keys
- Close ARCH-2 in tracker; hang Gemini TTS / B-04d; ARCH-3 ready not started
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="问题记录" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="统计" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="问题记录" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="使用说明" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="统计" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'问题记录'!$A$1:$K$40</definedName>
@@ -798,14 +798,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1800" b="1" strike="noStrike" spc="-1">
                 <a:solidFill>
@@ -828,8 +828,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -853,10 +853,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4f81bd"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+            <a:ln w="0">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -865,10 +865,10 @@
           <dPt>
             <idx val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4f81bd"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -877,10 +877,10 @@
           <dPt>
             <idx val="1"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="c0504d"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -889,10 +889,10 @@
           <dPt>
             <idx val="2"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="9bbb59"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -901,10 +901,10 @@
           <dPt>
             <idx val="3"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="8064a2"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -913,10 +913,10 @@
           <dPt>
             <idx val="4"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4bacc6"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -926,9 +926,9 @@
             <dLbl>
               <idx val="0"/>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
                       <a:solidFill>
@@ -952,9 +952,9 @@
             <dLbl>
               <idx val="1"/>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
                       <a:solidFill>
@@ -978,9 +978,9 @@
             <dLbl>
               <idx val="2"/>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
                       <a:solidFill>
@@ -1004,9 +1004,9 @@
             <dLbl>
               <idx val="3"/>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
                       <a:solidFill>
@@ -1030,9 +1030,9 @@
             <dLbl>
               <idx val="4"/>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
                       <a:solidFill>
@@ -1054,9 +1054,9 @@
               <showPercent val="1"/>
             </dLbl>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
                     <a:solidFill>
@@ -1133,16 +1133,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
               <a:solidFill>
@@ -1161,10 +1161,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="ffffff"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="d9d9d9"/>
       </a:solidFill>
@@ -1176,7 +1176,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>3</col>
@@ -1196,9 +1196,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -4652,7 +4652,7 @@
       </c>
       <c r="B59" s="40" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>已处理</t>
         </is>
       </c>
       <c r="C59" s="40" t="inlineStr">
@@ -4677,21 +4677,23 @@
       </c>
       <c r="G59" s="40" t="inlineStr">
         <is>
-          <t>管道已交；试跑线 2/3：DeepSeek 通 / 硅基 VLM 通 / Gemini TTS 缺钥不通。真关单否。D-01/D-09/D-13/D-05 已收；N-02 不动。</t>
+          <t>关单 2026-10-10 21:30 CST（HY）。管道 Provider+.env+D-05。试跑：DeepSeek 文本通；本地 Ollama qwen2.5vl:7b 读图通；Gemini TTS 缺 Key 未实跑→挂 B-04d/API 试跑线续债。N-02 未做。</t>
         </is>
       </c>
       <c r="H59" s="83" t="n">
         <v>46305</v>
       </c>
-      <c r="I59" s="83" t="n"/>
+      <c r="I59" s="83" t="n">
+        <v>46305</v>
+      </c>
       <c r="J59" s="40" t="inlineStr">
         <is>
-          <t>试跑脚本已入库待 tip；管道 tip 9c3bab0 / docs a65eb34</t>
+          <t>基于 f092de0 的关单 commit</t>
         </is>
       </c>
       <c r="K59" s="40" t="inlineStr">
         <is>
-          <t>二期前四刀第4；试跑线：本地/硅基/官方；试 DeepSeek 文本、官方 VLM、Gemini TTS。挂 N-02。 2026-10-10 ARCH-2：边界=管道非调度。新增 apps/server/src/config/{env,providers}.ts；改 llm/audio/imageGen/memory/memoryGate/index；.env.example 对齐。D-01/D-09/D-13/D-05 本刀已收。N-02 仍暂缓；试跑线完成后插。 2026-10-10 20:30 CST 三条验收（先不最终关单）：① D-05：纯 [memory.obs] 结构化 console 日志（start/ok/empty/fail_*/confirm）；fail_* 仅日志后 return，用户侧无失败气泡/耳语/API 信号（成功才 enqueueMemoryNotice）。② 五入口均进 config/providers.ts：llm→getLlmConfig(llm.ts)；vision→getVisionConfig/resolveVisionModel(llm.ts→conversations 读图)；stt→getSttConfig(audio.ts)；tts→getTtsConfig(audio.ts)；imageGen→getImageGenConfig(imageGen.ts)。③ X-01 最终 tip 0fce6d8（见 X-01 行）。下一顺序：试跑线→ARCH-3→UI-1；试跑线=ARCH-2 验收标准非独立刀；N-02 不动；读图 VLM 债/B-04d 在试跑线还。 2026-10-10 试跑线实跑 scripts/arch2-tryrun.py：DeepSeek 官方 deepseek-flash 通；硅基 Qwen3-VL-8B 读图通（本机无厂商官网 VLM Key）；Gemini TTS 不通（缺 GEMINI_API_KEY）。ARCH-2 真关单否（2/3）。N-02 不动。B-04d 坏 Key 上游 401，产品回流路径仍暂缓。</t>
+          <t>试跑主证据改为 HY 本地 VLM；硅基 Qwen3-VL 降为回落</t>
         </is>
       </c>
       <c r="L59" s="40" t="inlineStr">
@@ -4731,6 +4733,11 @@
           <t>前端状态分散，影响后续 UI 刀。</t>
         </is>
       </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>ARCH-2 关单后下一刀；本 HY 收口不开实现</t>
+        </is>
+      </c>
       <c r="H60" s="83" t="n">
         <v>46305</v>
       </c>
@@ -4819,6 +4826,11 @@
       <c r="F62" s="40" t="inlineStr">
         <is>
           <t>生图 Key 失败人话路径代码在、一期未实打。</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>【2026-10-10 21:30 CST ARCH-2 试跑线续债】Gemini TTS：HY 无 GEMINI_API_KEY，缺 Key 未实跑；坏 Key 上游观测仍 HTTP 401。产品失败回流人话路径仍待验。</t>
         </is>
       </c>
       <c r="H62" s="83" t="n">
@@ -5475,12 +5487,12 @@
       <c r="A14" s="83" t="n">
         <v>46305.86458333334</v>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="40" t="inlineStr">
         <is>
           <t>ARCH-2 试跑线 2/3</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="40" t="inlineStr">
         <is>
           <t>DeepSeek 通；硅基 VLM 通；Gemini TTS 缺 GEMINI_API_KEY；真关单否；B-04d 仍暂缓；下一补钥或 ARCH-3 等拍板</t>
         </is>

</xml_diff>

<commit_message>
UI-1: motion foundation tokens + overlay fade proof
Add duration/easing CSS vars and constants/motion.ts scene map.
Wire nav/list micro transitions to tokens; wrap persona editor and
moment composer with Transition wx-motion-fade. Docs: UI-1 closed,
D-02 partial close; no UI-2/3, N-02, or Gemini work.
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -4733,7 +4733,7 @@
           <t>前端状态分散，影响后续 UI 刀。</t>
         </is>
       </c>
-      <c r="G60" t="inlineStr">
+      <c r="G60" s="40" t="inlineStr">
         <is>
           <t>ARCH-2 关单后下一刀；本 HY 收口不开实现</t>
         </is>
@@ -4743,7 +4743,7 @@
       </c>
       <c r="K60" s="40" t="inlineStr">
         <is>
-          <t>UI 并行刀前评估。 2026-10-10：由暂缓改待处理；顺序在试跑线之后、UI-1 之前。</t>
+          <t>UI 并行刀前评估。 2026-10-10：由暂缓改待处理；顺序在试跑线之后、UI-1 之前。；D-02 部分收口（UI-1 后不追全收，回头再看 App.vue）</t>
         </is>
       </c>
       <c r="L60" s="40" t="inlineStr">
@@ -4828,7 +4828,7 @@
           <t>生图 Key 失败人话路径代码在、一期未实打。</t>
         </is>
       </c>
-      <c r="G62" t="inlineStr">
+      <c r="G62" s="40" t="inlineStr">
         <is>
           <t>【2026-10-10 21:30 CST ARCH-2 试跑线续债】Gemini TTS：HY 无 GEMINI_API_KEY，缺 Key 未实跑；坏 Key 上游观测仍 HTTP 401。产品失败回流人话路径仍待验。</t>
         </is>
@@ -4908,7 +4908,7 @@
       </c>
       <c r="B64" s="40" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>已处理</t>
         </is>
       </c>
       <c r="C64" s="40" t="inlineStr">
@@ -4929,19 +4929,27 @@
       <c r="F64" s="40" t="inlineStr">
         <is>
           <t>统一时长、曲线、触发场景（Telegram/Discord 娱乐向）。</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>2026-10-10 HY：动效基础层。`apps/web/src/constants/motion.ts` + `wechat.css` `--motion-*`；nav/列表 micro transition 改走 token；人设编辑 / 发动态 composer 挂 Transition `wx-motion-fade`。未做 UI-2/UI-3。</t>
         </is>
       </c>
       <c r="H64" s="83" t="n">
         <v>46305</v>
       </c>
+      <c r="I64" s="88" t="n">
+        <v>46305</v>
+      </c>
       <c r="K64" s="40" t="inlineStr">
         <is>
-          <t>二期第五刀/可与前四刀并行。</t>
+          <t>仅基础层；UI-2/3 另开。Gemini TTS 挂债；N-02 不动。D-02 部分收口。</t>
         </is>
       </c>
       <c r="L64" s="40" t="inlineStr">
         <is>
-          <t>不适用</t>
+          <t>待 push</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: UI-1 issue table tip 3737c1d
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -4931,7 +4931,7 @@
           <t>统一时长、曲线、触发场景（Telegram/Discord 娱乐向）。</t>
         </is>
       </c>
-      <c r="G64" t="inlineStr">
+      <c r="G64" s="40" t="inlineStr">
         <is>
           <t>2026-10-10 HY：动效基础层。`apps/web/src/constants/motion.ts` + `wechat.css` `--motion-*`；nav/列表 micro transition 改走 token；人设编辑 / 发动态 composer 挂 Transition `wx-motion-fade`。未做 UI-2/UI-3。</t>
         </is>
@@ -4942,6 +4942,11 @@
       <c r="I64" s="88" t="n">
         <v>46305</v>
       </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>3737c1d</t>
+        </is>
+      </c>
       <c r="K64" s="40" t="inlineStr">
         <is>
           <t>仅基础层；UI-2/3 另开。Gemini TTS 挂债；N-02 不动。D-02 部分收口。</t>
@@ -4949,7 +4954,7 @@
       </c>
       <c r="L64" s="40" t="inlineStr">
         <is>
-          <t>待 push</t>
+          <t>已 push</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
UI-2: message TransitionGroup + typing dots; close UI-1 clean
- Explain App.vue 2234/2243 as Measure-Object/CRLF count artifact (hash match)
- Message stream: TransitionGroup wx-motion-msg + UI-1 tokens; no App play state
- Sending reuses existing sending for CSS typing indicator; no useMessageMotion
- D-02 note: profileMoments vs useMoments still two lines; partial close
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -4933,7 +4933,7 @@
       </c>
       <c r="G64" s="40" t="inlineStr">
         <is>
-          <t>2026-10-10 HY：动效基础层。`apps/web/src/constants/motion.ts` + `wechat.css` `--motion-*`；nav/列表 micro transition 改走 token；人设编辑 / 发动态 composer 挂 Transition `wx-motion-fade`。未做 UI-2/UI-3。</t>
+          <t>2026-10-10 HY：动效基础层。`apps/web/src/constants/motion.ts` + `wechat.css` `--motion-*`；nav/列表 micro transition 改走 token；人设编辑 / 发动态 composer 挂 Transition `wx-motion-fade`。未做 UI-2/UI-3。 2026-10-10 关单前核对：App.vue 工作区与 HEAD 内容 hash 一致（a02fa9e），所谓 2234→2243 为 Measure-Object -Line / CRLF 计行口径差，非脏改；提交面干净后关单。</t>
         </is>
       </c>
       <c r="H64" s="83" t="n">
@@ -4942,7 +4942,7 @@
       <c r="I64" s="88" t="n">
         <v>46305</v>
       </c>
-      <c r="J64" t="inlineStr">
+      <c r="J64" s="40" t="inlineStr">
         <is>
           <t>3737c1d</t>
         </is>
@@ -4966,7 +4966,7 @@
       </c>
       <c r="B65" s="40" t="inlineStr">
         <is>
-          <t>暂缓</t>
+          <t>已处理</t>
         </is>
       </c>
       <c r="C65" s="40" t="inlineStr">
@@ -4986,20 +4986,28 @@
       </c>
       <c r="F65" s="40" t="inlineStr">
         <is>
-          <t>发送/接收过渡、正在输入动效。</t>
+          <t>发送/接收过渡、正在输入动效。落点：CSS/TransitionGroup + UI-1 token；不往 App.vue 加播放态；不 Pinia；不为未来预建 useMessageMotion；不动 profileMoments。</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>2026-10-10 HY：消息列表 TransitionGroup `wx-motion-msg`（按会话 key 重挂避免切房刷入场）；发送中复用已有 `sending` 挂纯 CSS「正在输入」三点（Transition `wx-motion-fade`）。未建 useMessageMotion；未动 profileMoments。</t>
         </is>
       </c>
       <c r="H65" s="83" t="n">
         <v>46305</v>
       </c>
+      <c r="I65" s="83" t="n">
+        <v>46305</v>
+      </c>
       <c r="K65" s="40" t="inlineStr">
         <is>
-          <t>依赖 UI-1 基础层。</t>
+          <t>依赖 UI-1 基础层。 依赖 UI-1 基础层。状态落点拍板：CSS/Transition + token；跨组件共享入场态才建 useMessageMotion（本刀未需要）。</t>
         </is>
       </c>
       <c r="L65" s="40" t="inlineStr">
         <is>
-          <t>不适用</t>
+          <t>未 push</t>
         </is>
       </c>
     </row>
@@ -5350,7 +5358,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="16" customWidth="1" style="40" min="1" max="1"/>
@@ -5371,6 +5379,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="41">
       <c r="A4" s="68" t="inlineStr">
         <is>
@@ -5437,7 +5446,11 @@
           <t>2026-10-10：一期七类冒烟通过（BF tip 65cf58e），一期可收口。二期前四刀 ARCH-1→M-05a→X-01→ARCH-2；UI-1 第五/可并行。UI-1～6、ARCH-1 补扫6项已落表。；2026-10-10 M-05a 已处理（由 M-06 覆盖，仅文档收口）；2026-10-10 17:12 CST BF 远程 tip eb48fbb（含 1b3b635 ARCH-1、c220bbf M-05a 关单、eb48fbb stash备注+上墙补验）；对齐 tip 83e9ab6（2026-10-10 17:13 CST）；2026-10-10 17:22 CST X-01 三条验证关单（PATCH↔GET / 私聊用人设 / UI 入口 API+接线）；对齐 tip cac031c（2026-10-10 17:23 CST）。；2026-10-10 ARCH-2 已处理（Provider+.env+D-05；tip 见问题行）。；2026-10-10 20:30 CST ARCH-2 验收补记+清表：D-05=纯[memory.obs]日志无用户侧失败信号；五入口均进 providers；X-01 最终 tip 0fce6d8；ARCH-2→待处理（管道已交关单待试跑线）；ARCH-3→待处理；O-03 已处理；下一顺序 试跑线→ARCH-3→UI-1；N-02 不动。</t>
         </is>
       </c>
-      <c r="B9" s="70" t="n"/>
+      <c r="B9" s="70" t="inlineStr">
+        <is>
+          <t>；2026-10-10 UI-1 关单确认（计行口径非脏改）；UI-2 消息 TransitionGroup+正在输入落地（HY）。</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="36" customHeight="1" s="41">
       <c r="A10" s="69" t="inlineStr">
@@ -5511,6 +5524,12 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
@@ -5537,7 +5556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="22" customWidth="1" style="40" min="1" max="1"/>
@@ -5559,6 +5578,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="41">
       <c r="A4" s="68" t="inlineStr">
         <is>
@@ -5626,6 +5646,7 @@
         <v/>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="15" customHeight="1" s="41">
       <c r="A11" s="72" t="inlineStr">
         <is>
@@ -5637,6 +5658,7 @@
         <v/>
       </c>
     </row>
+    <row r="12"/>
     <row r="13" ht="15" customHeight="1" s="41">
       <c r="A13" s="80" t="inlineStr">
         <is>
@@ -5734,6 +5756,15 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:C1"/>

</xml_diff>

<commit_message>
docs: UI-2 tip 95a7bf5 + issue table push sync
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -4949,7 +4949,7 @@
       </c>
       <c r="K64" s="40" t="inlineStr">
         <is>
-          <t>仅基础层；UI-2/3 另开。Gemini TTS 挂债；N-02 不动。D-02 部分收口。</t>
+          <t>仅基础层；UI-2/3 另开。Gemini TTS 挂债；N-02 不动。D-02 部分收口。 关单确认记入 95a7bf5（计行口径非脏改）。</t>
         </is>
       </c>
       <c r="L64" s="40" t="inlineStr">
@@ -4989,7 +4989,7 @@
           <t>发送/接收过渡、正在输入动效。落点：CSS/TransitionGroup + UI-1 token；不往 App.vue 加播放态；不 Pinia；不为未来预建 useMessageMotion；不动 profileMoments。</t>
         </is>
       </c>
-      <c r="G65" t="inlineStr">
+      <c r="G65" s="40" t="inlineStr">
         <is>
           <t>2026-10-10 HY：消息列表 TransitionGroup `wx-motion-msg`（按会话 key 重挂避免切房刷入场）；发送中复用已有 `sending` 挂纯 CSS「正在输入」三点（Transition `wx-motion-fade`）。未建 useMessageMotion；未动 profileMoments。</t>
         </is>
@@ -5000,6 +5000,11 @@
       <c r="I65" s="83" t="n">
         <v>46305</v>
       </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>95a7bf5</t>
+        </is>
+      </c>
       <c r="K65" s="40" t="inlineStr">
         <is>
           <t>依赖 UI-1 基础层。 依赖 UI-1 基础层。状态落点拍板：CSS/Transition + token；跨组件共享入场态才建 useMessageMotion（本刀未需要）。</t>
@@ -5007,7 +5012,7 @@
       </c>
       <c r="L65" s="40" t="inlineStr">
         <is>
-          <t>未 push</t>
+          <t>已 push</t>
         </is>
       </c>
     </row>
@@ -5358,7 +5363,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="16" customWidth="1" style="40" min="1" max="1"/>
@@ -5448,7 +5453,7 @@
       </c>
       <c r="B9" s="70" t="inlineStr">
         <is>
-          <t>；2026-10-10 UI-1 关单确认（计行口径非脏改）；UI-2 消息 TransitionGroup+正在输入落地（HY）。</t>
+          <t>；2026-10-10 UI-1 关单确认（计行口径非脏改）；UI-2 消息 TransitionGroup+正在输入落地（HY）。；远程 tip 95a7bf5（UI-2 关单+UI-1 计行口径确认）。</t>
         </is>
       </c>
     </row>
@@ -5530,6 +5535,11 @@
     <row r="18"/>
     <row r="19"/>
     <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
@@ -5752,7 +5762,7 @@
       </c>
       <c r="B21" s="40" t="inlineStr">
         <is>
-          <t>docs tip cac031c（含 ae4120d X-01 能力、cac031c 三条验证关单+阶段边界同步）。人工维护，最后更新 2026-10-10 17:23 CST。</t>
+          <t>远程 tip 95a7bf5（UI-2 消息动效 + UI-1 关单确认）。人工维护，最后更新 2026-10-10 22:24 CST。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
UI-3: unread badge CSS Transition; close UI-2 note
- wx-nav-dot / wx-unread-badge: Transition wx-motion-badge (scale+opacity) via UI-1 --motion-*
- C-03 unread state stays in App.vue; no useUnread / no play state
- UI-2 close note: App.vue 2234->2243 is line-count artifact, workspace matches HEAD
- No UI-4; N-02 / Gemini unchanged; D-02 still partial
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -5000,14 +5000,14 @@
       <c r="I65" s="83" t="n">
         <v>46305</v>
       </c>
-      <c r="J65" t="inlineStr">
+      <c r="J65" s="40" t="inlineStr">
         <is>
           <t>95a7bf5</t>
         </is>
       </c>
       <c r="K65" s="40" t="inlineStr">
         <is>
-          <t>依赖 UI-1 基础层。 依赖 UI-1 基础层。状态落点拍板：CSS/Transition + token；跨组件共享入场态才建 useMessageMotion（本刀未需要）。</t>
+          <t>依赖 UI-1 基础层。 依赖 UI-1 基础层。状态落点拍板：CSS/Transition + token；跨组件共享入场态才建 useMessageMotion（本刀未需要）。 关单补注：所谓 App.vue 2234→2243 那 9 行是计行口径差（Measure-Object -Line / CRLF），工作区与 HEAD 内容一致，非脏改。</t>
         </is>
       </c>
       <c r="L65" s="40" t="inlineStr">
@@ -5024,7 +5024,7 @@
       </c>
       <c r="B66" s="40" t="inlineStr">
         <is>
-          <t>暂缓</t>
+          <t>已处理</t>
         </is>
       </c>
       <c r="C66" s="40" t="inlineStr">
@@ -5045,19 +5045,32 @@
       <c r="F66" s="40" t="inlineStr">
         <is>
           <t>未读红点动效增强（C-03 功能已有）。</t>
+        </is>
+      </c>
+      <c r="G66" s="40" t="inlineStr">
+        <is>
+          <t>2026-10-10 HY：红点/未读角标纯 CSS 动效。wx-nav-dot / wx-unread-badge 挂 Transition wx-motion-badge（enter/leave scale+opacity），走 UI-1 --motion-duration-fast + enter/exit easing。C-03 状态仍在 App.vue（conversations.unread_count / totalUnread / 开聊清零）；未搬状态、未建 useUnread、未往 App 加播放态。UI-4 未做。</t>
         </is>
       </c>
       <c r="H66" s="83" t="n">
         <v>46305</v>
       </c>
+      <c r="I66" s="83" t="n">
+        <v>46305</v>
+      </c>
+      <c r="J66" s="40" t="inlineStr">
+        <is>
+          <t>a41e830</t>
+        </is>
+      </c>
       <c r="K66" s="40" t="inlineStr">
         <is>
-          <t>依赖 UI-1。</t>
+          <t>依赖 UI-1。落点拍板：只做出现/消失纯 CSS；状态不动。N-02、Gemini TTS 维持不动；D-02 仍部分收口。不做 UI-4。</t>
         </is>
       </c>
       <c r="L66" s="40" t="inlineStr">
         <is>
-          <t>不适用</t>
+          <t>已 push</t>
         </is>
       </c>
     </row>
@@ -5363,7 +5376,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="16" customWidth="1" style="40" min="1" max="1"/>
@@ -5384,7 +5397,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="41">
       <c r="A4" s="68" t="inlineStr">
         <is>
@@ -5529,17 +5541,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
@@ -5566,7 +5567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="22" customWidth="1" style="40" min="1" max="1"/>
@@ -5588,7 +5589,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="41">
       <c r="A4" s="68" t="inlineStr">
         <is>
@@ -5656,7 +5656,6 @@
         <v/>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="15" customHeight="1" s="41">
       <c r="A11" s="72" t="inlineStr">
         <is>
@@ -5668,7 +5667,6 @@
         <v/>
       </c>
     </row>
-    <row r="12"/>
     <row r="13" ht="15" customHeight="1" s="41">
       <c r="A13" s="80" t="inlineStr">
         <is>
@@ -5766,15 +5764,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:C1"/>

</xml_diff>

<commit_message>
docs: EOD wrap — ARCH-3/UI-3 closed, D-02 unread note, UI-4 tomorrow
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -4710,7 +4710,7 @@
       </c>
       <c r="B60" s="40" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>已处理</t>
         </is>
       </c>
       <c r="C60" s="40" t="inlineStr">
@@ -4735,15 +4735,23 @@
       </c>
       <c r="G60" s="40" t="inlineStr">
         <is>
-          <t>ARCH-2 关单后下一刀；本 HY 收口不开实现</t>
+          <t>2026-10-10 HY：抽出 useMoments / usePersonaEditor / useProactiveSettings；App.vue 变薄；web build 过。未上 Pinia；D-03 conversations.ts 未动。D-02 部分收口（不追全收）。</t>
         </is>
       </c>
       <c r="H60" s="83" t="n">
         <v>46305</v>
       </c>
+      <c r="I60" s="83" t="n">
+        <v>46305</v>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>23da1dc</t>
+        </is>
+      </c>
       <c r="K60" s="40" t="inlineStr">
         <is>
-          <t>UI 并行刀前评估。 2026-10-10：由暂缓改待处理；顺序在试跑线之后、UI-1 之前。；D-02 部分收口（UI-1 后不追全收，回头再看 App.vue）</t>
+          <t>UI 并行刀前评估。 2026-10-10：由暂缓改待处理；顺序在试跑线之后、UI-1 之前。；D-02 部分收口（UI-1 后不追全收，回头再看 App.vue） 2026-10-10 收尾：状态改已处理。D-02 仍部分收口；红点/未读（unread_count+totalUnread）仍在 App.vue，未来收 D-02 时抽 composable（UI-3 顺手发现）。</t>
         </is>
       </c>
       <c r="L60" s="40" t="inlineStr">
@@ -5060,12 +5068,12 @@
       </c>
       <c r="J66" s="40" t="inlineStr">
         <is>
-          <t>aa8e6ad</t>
+          <t>aa8e6ad / tip 4d985b3</t>
         </is>
       </c>
       <c r="K66" s="40" t="inlineStr">
         <is>
-          <t>依赖 UI-1。落点拍板：只做出现/消失纯 CSS；状态不动。N-02、Gemini TTS 维持不动；D-02 仍部分收口。不做 UI-4。</t>
+          <t>依赖 UI-1。落点拍板：只做出现/消失纯 CSS；状态不动。N-02、Gemini TTS 维持不动；D-02 仍部分收口。不做 UI-4。 2026-10-10 收尾关单确认：已推 tip 4d985b3。</t>
         </is>
       </c>
       <c r="L66" s="40" t="inlineStr">
@@ -5082,7 +5090,7 @@
       </c>
       <c r="B67" s="40" t="inlineStr">
         <is>
-          <t>暂缓</t>
+          <t>待处理</t>
         </is>
       </c>
       <c r="C67" s="40" t="inlineStr">
@@ -5110,7 +5118,7 @@
       </c>
       <c r="K67" s="40" t="inlineStr">
         <is>
-          <t>与 X-06 分工：UI-4=视觉；X-06=交互。可同迭代分两行。</t>
+          <t>与 X-06 分工：UI-4=视觉；X-06=交互。可同迭代分两行。 2026-10-10 收尾：明天第一刀 UI-4。开前先定：① UI-4 视觉 / X-06 交互边界；② 语音播放态、加载态、进度落点（App / composable / 纯 CSS）。今天不写代码。</t>
         </is>
       </c>
       <c r="L67" s="40" t="inlineStr">

</xml_diff>

<commit_message>
UI-4: voice bubble visual — CSS play/pause/loading + fake progress
Reuse ttsPlayingId/ttsLoadingId; decorative progress only (no currentTime).
X-06 / N-02 / Gemini TTS untouched. Close UI-4 in issue table.
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -4744,7 +4744,7 @@
       <c r="I60" s="83" t="n">
         <v>46305</v>
       </c>
-      <c r="J60" t="inlineStr">
+      <c r="J60" s="40" t="inlineStr">
         <is>
           <t>23da1dc</t>
         </is>
@@ -5090,7 +5090,7 @@
       </c>
       <c r="B67" s="40" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>已处理</t>
         </is>
       </c>
       <c r="C67" s="40" t="inlineStr">
@@ -5111,19 +5111,34 @@
       <c r="F67" s="40" t="inlineStr">
         <is>
           <t>语音泡波形与进度视觉。</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>2026-10-11 HY：UI-4 选 A。复用 ttsPlayingId/ttsLoadingId；语音泡播放/暂停/加载图标改纯 CSS；波形走 UI-1 --motion-*；进度条装饰性假进度（playing 假填充 / loading 不确定条），不接 audio.currentTime；未新增状态、未建 useTtsPlayback、未动 X-06。web build 过。</t>
         </is>
       </c>
       <c r="H67" s="83" t="n">
         <v>46305</v>
       </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>待 commit tip</t>
+        </is>
+      </c>
       <c r="K67" s="40" t="inlineStr">
         <is>
-          <t>与 X-06 分工：UI-4=视觉；X-06=交互。可同迭代分两行。 2026-10-10 收尾：明天第一刀 UI-4。开前先定：① UI-4 视觉 / X-06 交互边界；② 语音播放态、加载态、进度落点（App / composable / 纯 CSS）。今天不写代码。</t>
+          <t>与 X-06 分工：UI-4=视觉；X-06=交互。可同迭代分两行。 2026-10-10 收尾：明天第一刀 UI-4。开前先定：① UI-4 视觉 / X-06 交互边界；② 语音播放态、加载态、进度落点（App / composable / 纯 CSS）。今天不写代码。 2026-10-11 拍板选 A：纯 CSS 假进度；真进度/seek 留给 X-06；N-02、Gemini TTS 维持不动。</t>
         </is>
       </c>
       <c r="L67" s="40" t="inlineStr">
         <is>
-          <t>不适用</t>
+          <t>待 push</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: UI-4 tip 08d4050 + issue table close
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -5113,7 +5113,7 @@
           <t>语音泡波形与进度视觉。</t>
         </is>
       </c>
-      <c r="G67" t="inlineStr">
+      <c r="G67" s="40" t="inlineStr">
         <is>
           <t>2026-10-11 HY：UI-4 选 A。复用 ttsPlayingId/ttsLoadingId；语音泡播放/暂停/加载图标改纯 CSS；波形走 UI-1 --motion-*；进度条装饰性假进度（playing 假填充 / loading 不确定条），不接 audio.currentTime；未新增状态、未建 useTtsPlayback、未动 X-06。web build 过。</t>
         </is>
@@ -5121,14 +5121,14 @@
       <c r="H67" s="83" t="n">
         <v>46305</v>
       </c>
-      <c r="I67" t="inlineStr">
+      <c r="I67" s="40" t="inlineStr">
         <is>
           <t>2026-10-11</t>
         </is>
       </c>
-      <c r="J67" t="inlineStr">
-        <is>
-          <t>待 commit tip</t>
+      <c r="J67" s="40" t="inlineStr">
+        <is>
+          <t>08d4050</t>
         </is>
       </c>
       <c r="K67" s="40" t="inlineStr">
@@ -5138,7 +5138,7 @@
       </c>
       <c r="L67" s="40" t="inlineStr">
         <is>
-          <t>待 push</t>
+          <t>已 push</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: UI-4 remote status pending push (GitHub 443)
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -5133,12 +5133,12 @@
       </c>
       <c r="K67" s="40" t="inlineStr">
         <is>
-          <t>与 X-06 分工：UI-4=视觉；X-06=交互。可同迭代分两行。 2026-10-10 收尾：明天第一刀 UI-4。开前先定：① UI-4 视觉 / X-06 交互边界；② 语音播放态、加载态、进度落点（App / composable / 纯 CSS）。今天不写代码。 2026-10-11 拍板选 A：纯 CSS 假进度；真进度/seek 留给 X-06；N-02、Gemini TTS 维持不动。</t>
+          <t>与 X-06 分工：UI-4=视觉；X-06=交互。可同迭代分两行。 2026-10-10 收尾：明天第一刀 UI-4。开前先定：① UI-4 视觉 / X-06 交互边界；② 语音播放态、加载态、进度落点（App / composable / 纯 CSS）。今天不写代码。 2026-10-11 拍板选 A：纯 CSS 假进度；真进度/seek 留给 X-06；N-02、Gemini TTS 维持不动。 2026-10-11：功能关单本地 08d4050 / tip 81b3fff；push 因 HY→GitHub 443 失败，网络恢复后补推。</t>
         </is>
       </c>
       <c r="L67" s="40" t="inlineStr">
         <is>
-          <t>已 push</t>
+          <t>待 push（HY 本地 tip 81b3fff，GitHub 443 不通）</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
X-06: useTtsPlayback — migrate TTS state, real progress
Move ttsPlayingId/ttsLoadingId/playTts out of App.vue into useTtsPlayback
(loading/playing/idle + progressRatio from audio.currentTime). UI-4 playing
bar now binds --tts-progress; loading stays CSS indeterminate. No seek;
useHoldToTalk unchanged. App.vue 2422->2395 (-27).
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -4504,7 +4504,7 @@
       </c>
       <c r="B56" s="40" t="inlineStr">
         <is>
-          <t>暂缓</t>
+          <t>已处理</t>
         </is>
       </c>
       <c r="C56" s="40" t="inlineStr">
@@ -4525,14 +4525,27 @@
       <c r="F56" s="40" t="inlineStr">
         <is>
           <t>语音交互流程体验债（非波形视觉）。</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>2026-10-11 HY：X-06 选 A。新建 useTtsPlayback：迁出 ttsPlayingId/ttsLoadingId/playTts；三态 + progressRatio（audio.currentTime/duration）；App 只渲染。UI-4 假进度在 playing 时改为 --tts-progress 真进度；loading 仍 CSS indeterminate。useHoldToTalk 未改（取消手势已在 App pointer 层，无缺口）。不做 seek；未碰 UI-5/UI-6/N-02/Gemini。App.vue 行数 2422→2395（−27）。web build 过。</t>
         </is>
       </c>
       <c r="H56" s="83" t="n">
         <v>46305</v>
       </c>
+      <c r="I56" s="88" t="n">
+        <v>46306</v>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>(pending commit)</t>
+        </is>
+      </c>
       <c r="K56" s="40" t="inlineStr">
         <is>
-          <t>与 UI-4 波形分工：本项交互。</t>
+          <t>真进度接 audio.currentTime；seek 拖拽仍不在范围</t>
         </is>
       </c>
       <c r="L56" s="40" t="inlineStr">
@@ -5115,7 +5128,7 @@
       </c>
       <c r="G67" s="40" t="inlineStr">
         <is>
-          <t>2026-10-11 HY：UI-4 选 A。复用 ttsPlayingId/ttsLoadingId；语音泡播放/暂停/加载图标改纯 CSS；波形走 UI-1 --motion-*；进度条装饰性假进度（playing 假填充 / loading 不确定条），不接 audio.currentTime；未新增状态、未建 useTtsPlayback、未动 X-06。web build 过。</t>
+          <t>2026-10-11 HY：UI-4 选 A。复用 ttsPlayingId/ttsLoadingId；语音泡播放/暂停/加载图标改纯 CSS；波形走 UI-1 --motion-*；进度条装饰性假进度（playing 假填充 / loading 不确定条），不接 audio.currentTime；未新增状态、未建 useTtsPlayback、未动 X-06。web build 过。；2026-10-11：X-06 已接真进度，playing 假进度动画已撤。</t>
         </is>
       </c>
       <c r="H67" s="83" t="n">

</xml_diff>

<commit_message>
docs: X-06 tip c617a5a + issue table close
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -4527,7 +4527,7 @@
           <t>语音交互流程体验债（非波形视觉）。</t>
         </is>
       </c>
-      <c r="G56" t="inlineStr">
+      <c r="G56" s="40" t="inlineStr">
         <is>
           <t>2026-10-11 HY：X-06 选 A。新建 useTtsPlayback：迁出 ttsPlayingId/ttsLoadingId/playTts；三态 + progressRatio（audio.currentTime/duration）；App 只渲染。UI-4 假进度在 playing 时改为 --tts-progress 真进度；loading 仍 CSS indeterminate。useHoldToTalk 未改（取消手势已在 App pointer 层，无缺口）。不做 seek；未碰 UI-5/UI-6/N-02/Gemini。App.vue 行数 2422→2395（−27）。web build 过。</t>
         </is>
@@ -4538,9 +4538,9 @@
       <c r="I56" s="88" t="n">
         <v>46306</v>
       </c>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>(pending commit)</t>
+      <c r="J56" s="40" t="inlineStr">
+        <is>
+          <t>c617a5a</t>
         </is>
       </c>
       <c r="K56" s="40" t="inlineStr">
@@ -4550,7 +4550,7 @@
       </c>
       <c r="L56" s="40" t="inlineStr">
         <is>
-          <t>不适用</t>
+          <t>pending push (ahead incl. UI-4 stack)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: X-06 tip sync 838d3eb / remote ba907c3
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -4540,7 +4540,7 @@
       </c>
       <c r="J56" s="40" t="inlineStr">
         <is>
-          <t>c617a5a</t>
+          <t>838d3eb</t>
         </is>
       </c>
       <c r="K56" s="40" t="inlineStr">
@@ -4550,7 +4550,7 @@
       </c>
       <c r="L56" s="40" t="inlineStr">
         <is>
-          <t>pending push (ahead incl. UI-4 stack)</t>
+          <t>remote tip ba907c3</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
UI-6: group chat alive feel — avatar float + typing avatars
Ambient float on group member avatars (UI-1 motion tokens); group
typing row shows member avatars while sending. Reuses existing
sending flag; no new App business state. prefers-reduced-motion off.
Issue table: UI-6 closed.
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -5208,7 +5208,7 @@
       </c>
       <c r="B69" s="40" t="inlineStr">
         <is>
-          <t>暂缓</t>
+          <t>已处理</t>
         </is>
       </c>
       <c r="C69" s="40" t="inlineStr">
@@ -5229,19 +5229,34 @@
       <c r="F69" s="40" t="inlineStr">
         <is>
           <t>角色头像浮动、正在输入等群聊活跃感。</t>
+        </is>
+      </c>
+      <c r="G69" s="40" t="inlineStr">
+        <is>
+          <t>2026-10-11 HY：UI-6 群聊活跃感落地——成员头像 ambient float（UI-1 token）+ 群聊正在输入头像条；复用 sending，无新业务态；prefers-reduced-motion 关闭动画。</t>
         </is>
       </c>
       <c r="H69" s="83" t="n">
         <v>46305</v>
       </c>
+      <c r="I69" s="40" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="J69" s="40" t="inlineStr">
+        <is>
+          <t>89f8a9d</t>
+        </is>
+      </c>
       <c r="K69" s="40" t="inlineStr">
         <is>
-          <t>娱乐向，P3。</t>
+          <t>已关闭：ambient float + 群聊正在输入头像；复用 sending</t>
         </is>
       </c>
       <c r="L69" s="40" t="inlineStr">
         <is>
-          <t>不适用</t>
+          <t>本地 ahead 2，全完成再推</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: D-02 partial close + D-02b + API try-run notes
P0/P1/P2 closed; D-02 partial (state moved); D-02b shell cleanup separate.
Try-run: DeepSeek text ok (silicon); local VLM ok; Gemini TTS hung (no key).
N-02 untouched.
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -1389,7 +1389,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L77"/>
+  <dimension ref="A1:L79"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="40" min="1" max="1"/>
@@ -4094,7 +4094,7 @@
       <c r="J47" s="86" t="n"/>
       <c r="K47" s="86" t="inlineStr">
         <is>
-          <t>来源：用户 2026-10-10 规划占位。触发：用户选定多模型供应商与路由规则后再开。 2026-10-10：提前至二期中后段；与 ARCH-2 共挂 API 试跑线（本地/硅基/官方；DeepSeek 文本、官方 VLM、Gemini TTS）。</t>
+          <t>来源：用户 2026-10-10 规划占位。触发：用户选定多模型供应商与路由规则后再开。 2026-10-10：提前至二期中后段；与 ARCH-2 共挂 API 试跑线（本地/硅基/官方；DeepSeek 文本、官方 VLM、Gemini TTS）。 2026-10-11 试跑线仍不动。</t>
         </is>
       </c>
       <c r="L47" s="86" t="inlineStr">
@@ -4706,7 +4706,7 @@
       </c>
       <c r="K59" s="40" t="inlineStr">
         <is>
-          <t>试跑主证据改为 HY 本地 VLM；硅基 Qwen3-VL 降为回落</t>
+          <t>试跑主证据改为 HY 本地 VLM；硅基 Qwen3-VL 降为回落 2026-10-11 API 切换试跑线（HY）：DeepSeek 文本通（硅基 DeepSeek-V4-Flash，本机 DEEPSEEK_API_KEY 空）；读图：本地 Ollama qwen2.5vl:7b 通（官方/独立 VLM Key 未配）；Gemini TTS 缺 GEMINI_API_KEY → 挂债不阻塞（B-04d 续）。N-02 仍不动。</t>
         </is>
       </c>
       <c r="L59" s="40" t="inlineStr">
@@ -4764,7 +4764,7 @@
       </c>
       <c r="K60" s="40" t="inlineStr">
         <is>
-          <t>UI 并行刀前评估。 2026-10-10：由暂缓改待处理；顺序在试跑线之后、UI-1 之前。；D-02 部分收口（UI-1 后不追全收，回头再看 App.vue） 2026-10-10 收尾：状态改已处理。D-02 仍部分收口；红点/未读（unread_count+totalUnread）仍在 App.vue，未来收 D-02 时抽 composable（UI-3 顺手发现）。</t>
+          <t>UI 并行刀前评估。 2026-10-10：由暂缓改待处理；顺序在试跑线之后、UI-1 之前。；D-02 部分收口（UI-1 后不追全收，回头再看 App.vue） 2026-10-10 收尾：状态改已处理。D-02 仍部分收口；红点/未读（unread_count+totalUnread）仍在 App.vue，未来收 D-02 时抽 composable（UI-3 顺手发现）。 2026-10-11：D-02 定「部分收口」——状态已迁（P0/P1/P2 关单）；剩壳模板/胶水/status/展示辅助/emoji；不标已收口；壳层清理拆独立债 D-02b。不再继续抽 App.vue。</t>
         </is>
       </c>
       <c r="L60" s="40" t="inlineStr">
@@ -4851,7 +4851,7 @@
       </c>
       <c r="G62" s="40" t="inlineStr">
         <is>
-          <t>【2026-10-10 21:30 CST ARCH-2 试跑线续债】Gemini TTS：HY 无 GEMINI_API_KEY，缺 Key 未实跑；坏 Key 上游观测仍 HTTP 401。产品失败回流人话路径仍待验。</t>
+          <t>【2026-10-10 21:30 CST ARCH-2 试跑线续债】Gemini TTS：HY 无 GEMINI_API_KEY，缺 Key 未实跑；坏 Key 上游观测仍 HTTP 401。产品失败回流人话路径仍待验。 【2026-10-11 试跑】Gemini TTS 仍缺 GEMINI_API_KEY，未实跑；挂债不阻塞。坏 IMAGE_GEN Key 上游仍 HTTP 401。</t>
         </is>
       </c>
       <c r="H62" s="83" t="n">
@@ -5163,7 +5163,7 @@
       </c>
       <c r="B68" s="40" t="inlineStr">
         <is>
-          <t>暂缓</t>
+          <t>已处理</t>
         </is>
       </c>
       <c r="C68" s="40" t="inlineStr">
@@ -5184,19 +5184,32 @@
       <c r="F68" s="40" t="inlineStr">
         <is>
           <t>消息 reaction 多表情与微动效。</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>2026-10-11 HY：UI-5 Reaction 多表情+微动效落地。message_reactions + toggle API；useMessageReactions；快捷👍❤️😂😮😢🙏；微动效走 UI-1 token。App.vue +37 主要为模板/接线，无新业务 ref。关单确认：抬行均为模板，未堆状态。</t>
         </is>
       </c>
       <c r="H68" s="83" t="n">
         <v>46305</v>
       </c>
+      <c r="I68" s="88" t="n">
+        <v>46306</v>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>c6b9e33</t>
+        </is>
+      </c>
       <c r="K68" s="40" t="inlineStr">
         <is>
-          <t>娱乐向，P3。</t>
+          <t>娱乐向，P3。 2026-10-11 关单。N-02、Gemini TTS 维持不动。</t>
         </is>
       </c>
       <c r="L68" s="40" t="inlineStr">
         <is>
-          <t>不适用</t>
+          <t>已 push（tip 链至 0ed81a1 / 现 tip bdca268）</t>
         </is>
       </c>
     </row>
@@ -5251,12 +5264,12 @@
       </c>
       <c r="K69" s="40" t="inlineStr">
         <is>
-          <t>已关闭：ambient float + 群聊正在输入头像；复用 sending</t>
+          <t>已关闭：ambient float + 群聊正在输入头像；复用 sending 2026-10-11 审计：UI-6 +24 全是模板结构（群头像/sending），无新业务 ref。</t>
         </is>
       </c>
       <c r="L69" s="40" t="inlineStr">
         <is>
-          <t>本地 ahead 2，全完成再推</t>
+          <t>已 push</t>
         </is>
       </c>
     </row>
@@ -5376,6 +5389,111 @@
       <c r="I77" s="47" t="n"/>
       <c r="J77" s="47" t="n"/>
       <c r="K77" s="47" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>D-02</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>部分收口</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>前端</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>App.vue 状态管理（ARCH-1 债）</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>二期开工 App.vue ~2471 行，状态全堆一处。ARCH-3/UI/D-02 P0–P2 已迁出 chat/shell/profile/contacts/memory/voice 等 composable。</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>2026-10-11 定口径：部分收口（不标已收口）。状态部分已收：P0 useAppShell+useChatSession（8606bbb）；P1 useProfileAppearance+useContactsImport（d6a00c5）；P2 useMemoryUi+useVoiceInput（bdca268）。App.vue ~2446→1629。剩：壳模板、composable 胶水、status、消息展示辅助、emoji 接线——拆 D-02b，不再继续抽。</t>
+        </is>
+      </c>
+      <c r="H78" s="88" t="n">
+        <v>46305</v>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>bdca268</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>2026-10-11 拍板关单：D-02 P0（useAppShell+useChatSession, 8606bbb）/P1（useProfileAppearance+useContactsImport, d6a00c5）/P2（useMemoryUi+useVoiceInput, bdca268）全部关单。App.vue 约 2446→1629（约−817）。状态部分已收；剩壳模板/胶水/status/展示辅助/emoji。拆出独立债 D-02b（壳层/辅助清理），不再继续抽 App.vue。 与状态债分离：壳层/辅助见 D-02b。</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>已 push tip bdca268</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>D-02b</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>待处理</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>前端</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>壳层/辅助清理（从 D-02 拆出）</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>D-02 状态债已部分收口后，App.vue 仍剩壳模板重组、composable 胶水、status、消息展示辅助函数（avatarText/dayLabel/formatTime/collage 等）、emoji 接线。这是壳层/辅助重组，不是状态管理债。</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>独立债，不挂 D-02。拍板：暂不继续抽 App.vue（边际收益递减，避免壳层拆散增加耦合）。节奏另定。</t>
+        </is>
+      </c>
+      <c r="H79" s="88" t="n">
+        <v>46306</v>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>来源：2026-10-11 拍板。与 D-02 状态债分离。N-02/Gemini 无关。</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:K40"/>

</xml_diff>

<commit_message>
X-05: memory UX review + small fixes (partial close)
Fix explicit-claim whitespace regex, wire autoSupersede on
active/accept paths, re-ask confirm when pending label changes.
Add X-05 debt doc; close X-05 as partial with X05-D1 follow-up.
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -1389,7 +1389,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L79"/>
+  <dimension ref="A1:L80"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="40" min="1" max="1"/>
@@ -4459,7 +4459,7 @@
       </c>
       <c r="B55" s="40" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>已处理</t>
         </is>
       </c>
       <c r="C55" s="40" t="inlineStr">
@@ -4480,19 +4480,32 @@
       <c r="F55" s="40" t="inlineStr">
         <is>
           <t>在 R-05/R-06 已关上复盘体验债（过召回/冲突确认边角）。</t>
+        </is>
+      </c>
+      <c r="G55" s="40" t="inlineStr">
+        <is>
+          <t>部分收口。复盘过召回/冲突确认；小修 F1–F3（显式认领\s正则、autoSupersede接线、pending标签变重问）。续债 D1–D6 见 docs/product/X-05-记忆体验债复盘.md；建议下一刀 X05-D1。App.vue 无改。</t>
         </is>
       </c>
       <c r="H55" s="83" t="n">
         <v>46305</v>
       </c>
+      <c r="I55" s="88" t="n">
+        <v>46306</v>
+      </c>
+      <c r="J55" s="40" t="inlineStr">
+        <is>
+          <t>e85b6c1</t>
+        </is>
+      </c>
       <c r="K55" s="40" t="inlineStr">
         <is>
-          <t>依赖 R-05/R-06 已交付。</t>
+          <t>依赖 R-05/R-06 已交付。 2026-10-11 复盘+小修 F1/F2/F3。口径=部分收口。续债：D1确认按钮(P1)/D2 pending TTL/D3确认晚到/D4过召回后处理/D5失败无感(D-05)/D6=D-24。N-02/Gemini未动。</t>
         </is>
       </c>
       <c r="L55" s="40" t="inlineStr">
         <is>
-          <t>不适用</t>
+          <t>待 push</t>
         </is>
       </c>
     </row>
@@ -5186,7 +5199,7 @@
           <t>消息 reaction 多表情与微动效。</t>
         </is>
       </c>
-      <c r="G68" t="inlineStr">
+      <c r="G68" s="40" t="inlineStr">
         <is>
           <t>2026-10-11 HY：UI-5 Reaction 多表情+微动效落地。message_reactions + toggle API；useMessageReactions；快捷👍❤️😂😮😢🙏；微动效走 UI-1 token。App.vue +37 主要为模板/接线，无新业务 ref。关单确认：抬行均为模板，未堆状态。</t>
         </is>
@@ -5197,7 +5210,7 @@
       <c r="I68" s="88" t="n">
         <v>46306</v>
       </c>
-      <c r="J68" t="inlineStr">
+      <c r="J68" s="40" t="inlineStr">
         <is>
           <t>c6b9e33</t>
         </is>
@@ -5391,37 +5404,37 @@
       <c r="K77" s="47" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" t="inlineStr">
+      <c r="A78" s="40" t="inlineStr">
         <is>
           <t>D-02</t>
         </is>
       </c>
-      <c r="B78" t="inlineStr">
+      <c r="B78" s="40" t="inlineStr">
         <is>
           <t>部分收口</t>
         </is>
       </c>
-      <c r="C78" t="inlineStr">
+      <c r="C78" s="40" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="D78" t="inlineStr">
+      <c r="D78" s="40" t="inlineStr">
         <is>
           <t>前端</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr">
+      <c r="E78" s="40" t="inlineStr">
         <is>
           <t>App.vue 状态管理（ARCH-1 债）</t>
         </is>
       </c>
-      <c r="F78" t="inlineStr">
+      <c r="F78" s="40" t="inlineStr">
         <is>
           <t>二期开工 App.vue ~2471 行，状态全堆一处。ARCH-3/UI/D-02 P0–P2 已迁出 chat/shell/profile/contacts/memory/voice 等 composable。</t>
         </is>
       </c>
-      <c r="G78" t="inlineStr">
+      <c r="G78" s="40" t="inlineStr">
         <is>
           <t>2026-10-11 定口径：部分收口（不标已收口）。状态部分已收：P0 useAppShell+useChatSession（8606bbb）；P1 useProfileAppearance+useContactsImport（d6a00c5）；P2 useMemoryUi+useVoiceInput（bdca268）。App.vue ~2446→1629。剩：壳模板、composable 胶水、status、消息展示辅助、emoji 接线——拆 D-02b，不再继续抽。</t>
         </is>
@@ -5429,54 +5442,54 @@
       <c r="H78" s="88" t="n">
         <v>46305</v>
       </c>
-      <c r="J78" t="inlineStr">
+      <c r="J78" s="40" t="inlineStr">
         <is>
           <t>bdca268</t>
         </is>
       </c>
-      <c r="K78" t="inlineStr">
+      <c r="K78" s="40" t="inlineStr">
         <is>
           <t>2026-10-11 拍板关单：D-02 P0（useAppShell+useChatSession, 8606bbb）/P1（useProfileAppearance+useContactsImport, d6a00c5）/P2（useMemoryUi+useVoiceInput, bdca268）全部关单。App.vue 约 2446→1629（约−817）。状态部分已收；剩壳模板/胶水/status/展示辅助/emoji。拆出独立债 D-02b（壳层/辅助清理），不再继续抽 App.vue。 与状态债分离：壳层/辅助见 D-02b。</t>
         </is>
       </c>
-      <c r="L78" t="inlineStr">
+      <c r="L78" s="40" t="inlineStr">
         <is>
           <t>已 push tip bdca268</t>
         </is>
       </c>
     </row>
     <row r="79">
-      <c r="A79" t="inlineStr">
+      <c r="A79" s="40" t="inlineStr">
         <is>
           <t>D-02b</t>
         </is>
       </c>
-      <c r="B79" t="inlineStr">
+      <c r="B79" s="40" t="inlineStr">
         <is>
           <t>待处理</t>
         </is>
       </c>
-      <c r="C79" t="inlineStr">
+      <c r="C79" s="40" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="D79" t="inlineStr">
+      <c r="D79" s="40" t="inlineStr">
         <is>
           <t>前端</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr">
+      <c r="E79" s="40" t="inlineStr">
         <is>
           <t>壳层/辅助清理（从 D-02 拆出）</t>
         </is>
       </c>
-      <c r="F79" t="inlineStr">
+      <c r="F79" s="40" t="inlineStr">
         <is>
           <t>D-02 状态债已部分收口后，App.vue 仍剩壳模板重组、composable 胶水、status、消息展示辅助函数（avatarText/dayLabel/formatTime/collage 等）、emoji 接线。这是壳层/辅助重组，不是状态管理债。</t>
         </is>
       </c>
-      <c r="G79" t="inlineStr">
+      <c r="G79" s="40" t="inlineStr">
         <is>
           <t>独立债，不挂 D-02。拍板：暂不继续抽 App.vue（边际收益递减，避免壳层拆散增加耦合）。节奏另定。</t>
         </is>
@@ -5484,14 +5497,64 @@
       <c r="H79" s="88" t="n">
         <v>46306</v>
       </c>
-      <c r="K79" t="inlineStr">
+      <c r="K79" s="40" t="inlineStr">
         <is>
           <t>来源：2026-10-11 拍板。与 D-02 状态债分离。N-02/Gemini 无关。</t>
         </is>
       </c>
-      <c r="L79" t="inlineStr">
+      <c r="L79" s="40" t="inlineStr">
         <is>
           <t>不适用</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="40" t="inlineStr">
+        <is>
+          <t>X05-D1</t>
+        </is>
+      </c>
+      <c r="B80" s="40" t="inlineStr">
+        <is>
+          <t>待处理</t>
+        </is>
+      </c>
+      <c r="C80" s="40" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D80" s="40" t="inlineStr">
+        <is>
+          <t>角色</t>
+        </is>
+      </c>
+      <c r="E80" s="40" t="inlineStr">
+        <is>
+          <t>记忆冲突确认快捷按钮</t>
+        </is>
+      </c>
+      <c r="F80" s="40" t="inlineStr">
+        <is>
+          <t>X-05 续债：memory_confirm 仅自然语言解析，无「改/不改」按钮；模糊回复易留 pending。</t>
+        </is>
+      </c>
+      <c r="G80" s="40" t="inlineStr">
+        <is>
+          <t>确认气泡可一点改/不改；自然语言兜底仍可用。</t>
+        </is>
+      </c>
+      <c r="H80" s="88" t="n">
+        <v>46306</v>
+      </c>
+      <c r="K80" s="40" t="inlineStr">
+        <is>
+          <t>来源 X-05；详见 docs/product/X-05-记忆体验债复盘.md</t>
+        </is>
+      </c>
+      <c r="L80" s="40" t="inlineStr">
+        <is>
+          <t>未开始</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: X-05 tip affbbde remote synced
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -4495,7 +4495,7 @@
       </c>
       <c r="J55" s="40" t="inlineStr">
         <is>
-          <t>e85b6c1</t>
+          <t>affbbde</t>
         </is>
       </c>
       <c r="K55" s="40" t="inlineStr">
@@ -4505,7 +4505,7 @@
       </c>
       <c r="L55" s="40" t="inlineStr">
         <is>
-          <t>待 push</t>
+          <t>已 push</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: EOD align X-05 partial close + tomorrow X05-D1
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -4459,7 +4459,7 @@
       </c>
       <c r="B55" s="40" t="inlineStr">
         <is>
-          <t>已处理</t>
+          <t>部分收口</t>
         </is>
       </c>
       <c r="C55" s="40" t="inlineStr">
@@ -4490,22 +4490,20 @@
       <c r="H55" s="83" t="n">
         <v>46305</v>
       </c>
-      <c r="I55" s="88" t="n">
-        <v>46306</v>
-      </c>
+      <c r="I55" s="88" t="n"/>
       <c r="J55" s="40" t="inlineStr">
         <is>
-          <t>affbbde</t>
+          <t>affbbde / tip 2060e6c</t>
         </is>
       </c>
       <c r="K55" s="40" t="inlineStr">
         <is>
-          <t>依赖 R-05/R-06 已交付。 2026-10-11 复盘+小修 F1/F2/F3。口径=部分收口。续债：D1确认按钮(P1)/D2 pending TTL/D3确认晚到/D4过召回后处理/D5失败无感(D-05)/D6=D-24。N-02/Gemini未动。</t>
+          <t>依赖 R-05/R-06 已交付。 2026-10-11 复盘+小修 F1/F2/F3。口径=部分收口。续债：D1确认按钮(P1)/D2 pending TTL/D3确认晚到/D4过召回后处理/D5失败无感(D-05)/D6=D-24。N-02/Gemini未动。 2026-10-11 收尾对齐：状态=部分收口（非已处理）；功能 tip affbbde；文档 tip 2060e6c；续债 X05-D1 待处理；过召回靠提示词不拆包；明天第一刀 X05-D1。</t>
         </is>
       </c>
       <c r="L55" s="40" t="inlineStr">
         <is>
-          <t>已 push</t>
+          <t>已 push（tip 2060e6c）</t>
         </is>
       </c>
     </row>
@@ -4719,7 +4717,7 @@
       </c>
       <c r="K59" s="40" t="inlineStr">
         <is>
-          <t>试跑主证据改为 HY 本地 VLM；硅基 Qwen3-VL 降为回落 2026-10-11 API 切换试跑线（HY）：DeepSeek 文本通（硅基 DeepSeek-V4-Flash，本机 DEEPSEEK_API_KEY 空）；读图：本地 Ollama qwen2.5vl:7b 通（官方/独立 VLM Key 未配）；Gemini TTS 缺 GEMINI_API_KEY → 挂债不阻塞（B-04d 续）。N-02 仍不动。</t>
+          <t>试跑主证据改为 HY 本地 VLM；硅基 Qwen3-VL 降为回落 2026-10-11 API 切换试跑线（HY）：DeepSeek 文本通（硅基 DeepSeek-V4-Flash，本机 DEEPSEEK_API_KEY 空）；读图：本地 Ollama qwen2.5vl:7b 通（官方/独立 VLM Key 未配）；Gemini TTS 缺 GEMINI_API_KEY → 挂债不阻塞（B-04d 续）。N-02 仍不动。 2026-10-11 收尾试跑线备注：DeepSeek 文本通（硅基 DeepSeek-V4-Flash，属 DeepSeek 系列）；本地 Ollama qwen2.5vl 读图通；Gemini TTS + 官方 VLM Key 挂债（不阻塞）。N-02 不动。</t>
         </is>
       </c>
       <c r="L59" s="40" t="inlineStr">
@@ -4872,7 +4870,7 @@
       </c>
       <c r="K62" s="40" t="inlineStr">
         <is>
-          <t>挂 API/密钥试跑时顺带验。 2026-10-10：读图 VLM 债/B-04d 在 ARCH-2 试跑线里还（非独立刀）。 2026-10-10 试跑线观测：坏 IMAGE_GEN Key → 上游 HTTP 401 Token is invalid；产品侧失败回流人话路径未改代码实打，仍暂缓。</t>
+          <t>挂 API/密钥试跑时顺带验。 2026-10-10：读图 VLM 债/B-04d 在 ARCH-2 试跑线里还（非独立刀）。 2026-10-10 试跑线观测：坏 IMAGE_GEN Key → 上游 HTTP 401 Token is invalid；产品侧失败回流人话路径未改代码实打，仍暂缓。 2026-10-11 收尾：Gemini TTS + 官方 VLM 仍挂债等 Key；排在 X05-D1 / D-02b 之后。</t>
         </is>
       </c>
       <c r="L62" s="40" t="inlineStr">
@@ -5499,7 +5497,7 @@
       </c>
       <c r="K79" s="40" t="inlineStr">
         <is>
-          <t>来源：2026-10-11 拍板。与 D-02 状态债分离。N-02/Gemini 无关。</t>
+          <t>来源：2026-10-11 拍板。与 D-02 状态债分离。N-02/Gemini 无关。 2026-10-11 收尾：排在 X05-D1 之后；顺序 X05-D1→D-02b→试跑挂债。</t>
         </is>
       </c>
       <c r="L79" s="40" t="inlineStr">
@@ -5549,7 +5547,7 @@
       </c>
       <c r="K80" s="40" t="inlineStr">
         <is>
-          <t>来源 X-05；详见 docs/product/X-05-记忆体验债复盘.md</t>
+          <t>来源 X-05；详见 docs/product/X-05-记忆体验债复盘.md 2026-10-11 收尾：明天第一刀；顺序 X05-D1→D-02b→试跑挂债（等 Key）。N-02 不动。</t>
         </is>
       </c>
       <c r="L80" s="40" t="inlineStr">
@@ -5697,7 +5695,7 @@
       </c>
       <c r="B9" s="70" t="inlineStr">
         <is>
-          <t>；2026-10-10 UI-1 关单确认（计行口径非脏改）；UI-2 消息 TransitionGroup+正在输入落地（HY）。；远程 tip 95a7bf5（UI-2 关单+UI-1 计行口径确认）。</t>
+          <t>；2026-10-10 UI-1 关单确认（计行口径非脏改）；UI-2 消息 TransitionGroup+正在输入落地（HY）。；远程 tip 95a7bf5（UI-2 关单+UI-1 计行口径确认）。；2026-10-11 收尾：远程 tip 2060e6c（无 ahead）。UI-5/UI-6 已处理；D-02 部分收口；D-02b 待处理；X-05 部分收口（非已处理）+ 续债 X05-D1 待处理；试跑线：DeepSeek-V4-Flash 通 / 本地 VLM 通 / Gemini TTS+官方 VLM 挂债。明天第一刀 X05-D1；顺序 X05-D1→D-02b→试跑挂债；N-02 不动；过召回靠提示词不拆包。</t>
         </is>
       </c>
     </row>
@@ -5980,7 +5978,7 @@
       </c>
       <c r="B20" s="40" t="inlineStr">
         <is>
-          <t>C-06 空间反应与私聊主动日 cap 解耦（待用户点头）。可选：daily_cap UI / R-03 好感度。勿与 N-01..03 规划占位混淆。</t>
+          <t>明天第一刀：X05-D1 确认快捷按钮（P1）。顺序：X05-D1 → D-02b → 试跑线挂债（等 Key）。N-02 不动；X-05 过召回靠提示词不拆包。</t>
         </is>
       </c>
     </row>
@@ -5992,7 +5990,7 @@
       </c>
       <c r="B21" s="40" t="inlineStr">
         <is>
-          <t>远程 tip 95a7bf5（UI-2 消息动效 + UI-1 关单确认）。人工维护，最后更新 2026-10-10 22:24 CST。</t>
+          <t>远程 tip 2060e6c（X-05 部分收口文档对齐）。人工维护，最后更新 2026-10-11 收尾 CST。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: point EOD tip refs to c9be373
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -4493,17 +4493,17 @@
       <c r="I55" s="88" t="n"/>
       <c r="J55" s="40" t="inlineStr">
         <is>
-          <t>affbbde / tip 2060e6c</t>
+          <t>affbbde / tip c9be373</t>
         </is>
       </c>
       <c r="K55" s="40" t="inlineStr">
         <is>
-          <t>依赖 R-05/R-06 已交付。 2026-10-11 复盘+小修 F1/F2/F3。口径=部分收口。续债：D1确认按钮(P1)/D2 pending TTL/D3确认晚到/D4过召回后处理/D5失败无感(D-05)/D6=D-24。N-02/Gemini未动。 2026-10-11 收尾对齐：状态=部分收口（非已处理）；功能 tip affbbde；文档 tip 2060e6c；续债 X05-D1 待处理；过召回靠提示词不拆包；明天第一刀 X05-D1。</t>
+          <t>依赖 R-05/R-06 已交付。 2026-10-11 复盘+小修 F1/F2/F3。口径=部分收口。续债：D1确认按钮(P1)/D2 pending TTL/D3确认晚到/D4过召回后处理/D5失败无感(D-05)/D6=D-24。N-02/Gemini未动。 2026-10-11 收尾对齐：状态=部分收口（非已处理）；功能 tip affbbde；文档 tip c9be373；续债 X05-D1 待处理；过召回靠提示词不拆包；明天第一刀 X05-D1。</t>
         </is>
       </c>
       <c r="L55" s="40" t="inlineStr">
         <is>
-          <t>已 push（tip 2060e6c）</t>
+          <t>已 push（tip c9be373）</t>
         </is>
       </c>
     </row>
@@ -5695,7 +5695,7 @@
       </c>
       <c r="B9" s="70" t="inlineStr">
         <is>
-          <t>；2026-10-10 UI-1 关单确认（计行口径非脏改）；UI-2 消息 TransitionGroup+正在输入落地（HY）。；远程 tip 95a7bf5（UI-2 关单+UI-1 计行口径确认）。；2026-10-11 收尾：远程 tip 2060e6c（无 ahead）。UI-5/UI-6 已处理；D-02 部分收口；D-02b 待处理；X-05 部分收口（非已处理）+ 续债 X05-D1 待处理；试跑线：DeepSeek-V4-Flash 通 / 本地 VLM 通 / Gemini TTS+官方 VLM 挂债。明天第一刀 X05-D1；顺序 X05-D1→D-02b→试跑挂债；N-02 不动；过召回靠提示词不拆包。</t>
+          <t>；2026-10-10 UI-1 关单确认（计行口径非脏改）；UI-2 消息 TransitionGroup+正在输入落地（HY）。；远程 tip c9be373（UI-2 关单+UI-1 计行口径确认）。；2026-10-11 收尾：远程 tip c9be373（无 ahead）。UI-5/UI-6 已处理；D-02 部分收口；D-02b 待处理；X-05 部分收口（非已处理）+ 续债 X05-D1 待处理；试跑线：DeepSeek-V4-Flash 通 / 本地 VLM 通 / Gemini TTS+官方 VLM 挂债。明天第一刀 X05-D1；顺序 X05-D1→D-02b→试跑挂债；N-02 不动；过召回靠提示词不拆包。</t>
         </is>
       </c>
     </row>
@@ -5990,7 +5990,7 @@
       </c>
       <c r="B21" s="40" t="inlineStr">
         <is>
-          <t>远程 tip 2060e6c（X-05 部分收口文档对齐）。人工维护，最后更新 2026-10-11 收尾 CST。</t>
+          <t>远程 tip c9be373（EOD：X-05 部分收口 + 明天 X05-D1）。人工维护，最后更新 2026-10-11 收尾 CST。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(web): X05-D1 memory conflict confirm shortcut chips
Add 「改 / 不改」chips under trailing source=memory_confirm bubbles;
chips sendQuickText into existing resolvePendingMemoryConfirm path
(NL parsing kept as fallback). Poll listMessages briefly after private
send so async confirm bubbles appear in-session. Close X05-D1 in debt
doc + issue table. No new App.vue state refs; no N-02 / D-02b.
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="问题记录" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="使用说明" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="统计" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="问题记录" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="统计" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'问题记录'!$A$1:$K$40</definedName>
@@ -798,14 +798,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1800" b="1" strike="noStrike" spc="-1">
                 <a:solidFill>
@@ -828,8 +828,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -853,10 +853,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4f81bd"/>
             </a:solidFill>
-            <a:ln w="0">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -865,10 +865,10 @@
           <dPt>
             <idx val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4f81bd"/>
               </a:solidFill>
-              <a:ln w="0">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -877,10 +877,10 @@
           <dPt>
             <idx val="1"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="c0504d"/>
               </a:solidFill>
-              <a:ln w="0">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -889,10 +889,10 @@
           <dPt>
             <idx val="2"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="9bbb59"/>
               </a:solidFill>
-              <a:ln w="0">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -901,10 +901,10 @@
           <dPt>
             <idx val="3"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="8064a2"/>
               </a:solidFill>
-              <a:ln w="0">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -913,10 +913,10 @@
           <dPt>
             <idx val="4"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4bacc6"/>
               </a:solidFill>
-              <a:ln w="0">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -926,9 +926,9 @@
             <dLbl>
               <idx val="0"/>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
                       <a:solidFill>
@@ -952,9 +952,9 @@
             <dLbl>
               <idx val="1"/>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
                       <a:solidFill>
@@ -978,9 +978,9 @@
             <dLbl>
               <idx val="2"/>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
                       <a:solidFill>
@@ -1004,9 +1004,9 @@
             <dLbl>
               <idx val="3"/>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
                       <a:solidFill>
@@ -1030,9 +1030,9 @@
             <dLbl>
               <idx val="4"/>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
                       <a:solidFill>
@@ -1054,9 +1054,9 @@
               <showPercent val="1"/>
             </dLbl>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
                     <a:solidFill>
@@ -1133,16 +1133,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
               <a:solidFill>
@@ -1161,10 +1161,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="ffffff"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="d9d9d9"/>
       </a:solidFill>
@@ -1176,7 +1176,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>3</col>
@@ -1196,9 +1196,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -4484,7 +4484,7 @@
       </c>
       <c r="G55" s="40" t="inlineStr">
         <is>
-          <t>部分收口。复盘过召回/冲突确认；小修 F1–F3（显式认领\s正则、autoSupersede接线、pending标签变重问）。续债 D1–D6 见 docs/product/X-05-记忆体验债复盘.md；建议下一刀 X05-D1。App.vue 无改。</t>
+          <t>部分收口。复盘过召回/冲突确认；小修 F1–F3；**X05-D1 快捷按钮已关（2026-10-13）**。续债 D2–D6 见 docs/product/X-05-记忆体验债复盘.md。App.vue 仅 D1 chips 模板+helper。</t>
         </is>
       </c>
       <c r="H55" s="83" t="n">
@@ -4498,7 +4498,7 @@
       </c>
       <c r="K55" s="40" t="inlineStr">
         <is>
-          <t>依赖 R-05/R-06 已交付。 2026-10-11 复盘+小修 F1/F2/F3。口径=部分收口。续债：D1确认按钮(P1)/D2 pending TTL/D3确认晚到/D4过召回后处理/D5失败无感(D-05)/D6=D-24。N-02/Gemini未动。 2026-10-11 收尾对齐：状态=部分收口（非已处理）；功能 tip affbbde；文档 tip c9be373；续债 X05-D1 待处理；过召回靠提示词不拆包；明天第一刀 X05-D1。</t>
+          <t>依赖 R-05/R-06 已交付。 2026-10-11 复盘+小修 F1/F2/F3。口径=部分收口。续债：D1确认按钮(P1)/D2 pending TTL/D3确认晚到/D4过召回后处理/D5失败无感(D-05)/D6=D-24。N-02/Gemini未动。 2026-10-11 收尾对齐：状态=部分收口（非已处理）；功能 tip affbbde；文档 tip c9be373；续债 X05-D1 待处理；过召回靠提示词不拆包；明天第一刀 X05-D1。 2026-10-13：X05-D1 已处理（BF）。续债从 D2 起；下一刀可 D-02b。</t>
         </is>
       </c>
       <c r="L55" s="40" t="inlineStr">
@@ -5514,7 +5514,7 @@
       </c>
       <c r="B80" s="40" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>已处理</t>
         </is>
       </c>
       <c r="C80" s="40" t="inlineStr">
@@ -5539,20 +5539,28 @@
       </c>
       <c r="G80" s="40" t="inlineStr">
         <is>
-          <t>确认气泡可一点改/不改；自然语言兜底仍可用。</t>
+          <t>2026-10-13 BF：memory_confirm 气泡下「改/不改」chips；sendQuickText→resolvePendingMemoryConfirm；自然语言兜底保留；末尾未回复的确认才显示；发送后短轮询 listMessages 拉异步确认气泡。无新 App.vue 状态债。</t>
         </is>
       </c>
       <c r="H80" s="88" t="n">
         <v>46306</v>
       </c>
+      <c r="I80" s="88" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>(pending commit)</t>
+        </is>
+      </c>
       <c r="K80" s="40" t="inlineStr">
         <is>
-          <t>来源 X-05；详见 docs/product/X-05-记忆体验债复盘.md 2026-10-11 收尾：明天第一刀；顺序 X05-D1→D-02b→试跑挂债（等 Key）。N-02 不动。</t>
+          <t>来源 X-05。2026-10-13 BF 关单。选择=最小解释（不新开 API）。续：D-02b / X05-D2。N-02 不动。</t>
         </is>
       </c>
       <c r="L80" s="40" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>待 push</t>
         </is>
       </c>
     </row>
@@ -5627,6 +5635,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="41">
       <c r="A4" s="68" t="inlineStr">
         <is>
@@ -5695,7 +5704,7 @@
       </c>
       <c r="B9" s="70" t="inlineStr">
         <is>
-          <t>；2026-10-10 UI-1 关单确认（计行口径非脏改）；UI-2 消息 TransitionGroup+正在输入落地（HY）。；远程 tip c9be373（UI-2 关单+UI-1 计行口径确认）。；2026-10-11 收尾：远程 tip c9be373（无 ahead）。UI-5/UI-6 已处理；D-02 部分收口；D-02b 待处理；X-05 部分收口（非已处理）+ 续债 X05-D1 待处理；试跑线：DeepSeek-V4-Flash 通 / 本地 VLM 通 / Gemini TTS+官方 VLM 挂债。明天第一刀 X05-D1；顺序 X05-D1→D-02b→试跑挂债；N-02 不动；过召回靠提示词不拆包。</t>
+          <t>；2026-10-10 UI-1 关单确认（计行口径非脏改）；UI-2 消息 TransitionGroup+正在输入落地（HY）。；远程 tip c9be373（UI-2 关单+UI-1 计行口径确认）。；2026-10-11 收尾：远程 tip c9be373（无 ahead）。UI-5/UI-6 已处理；D-02 部分收口；D-02b 待处理；X-05 部分收口（非已处理）+ 续债 X05-D1 待处理；试跑线：DeepSeek-V4-Flash 通 / 本地 VLM 通 / Gemini TTS+官方 VLM 挂债。明天第一刀 X05-D1；顺序 X05-D1→D-02b→试跑挂债；N-02 不动；过召回靠提示词不拆包。；2026-10-13 BF：X05-D1 确认快捷按钮关单（待 tip SHA）。</t>
         </is>
       </c>
     </row>
@@ -5819,6 +5828,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="41">
       <c r="A4" s="68" t="inlineStr">
         <is>
@@ -5886,6 +5896,7 @@
         <v/>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="15" customHeight="1" s="41">
       <c r="A11" s="72" t="inlineStr">
         <is>
@@ -5897,6 +5908,7 @@
         <v/>
       </c>
     </row>
+    <row r="12"/>
     <row r="13" ht="15" customHeight="1" s="41">
       <c r="A13" s="80" t="inlineStr">
         <is>
@@ -5978,7 +5990,7 @@
       </c>
       <c r="B20" s="40" t="inlineStr">
         <is>
-          <t>明天第一刀：X05-D1 确认快捷按钮（P1）。顺序：X05-D1 → D-02b → 试跑线挂债（等 Key）。N-02 不动；X-05 过召回靠提示词不拆包。</t>
+          <t>X05-D1 已关（2026-10-13 BF）。下一优先：D-02b 抽取 → 试跑挂债（Gemini Key）。N-02 不动；X-05 过召回靠提示词不拆包。</t>
         </is>
       </c>
     </row>
@@ -5990,7 +6002,7 @@
       </c>
       <c r="B21" s="40" t="inlineStr">
         <is>
-          <t>远程 tip c9be373（EOD：X-05 部分收口 + 明天 X05-D1）。人工维护，最后更新 2026-10-11 收尾 CST。</t>
+          <t>远程 tip 待本刀 push 后更新（X05-D1）。人工维护，最后更新 2026-10-13 BF CST。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: X05-D1 tip b851189 + issue table push sync
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -5548,9 +5548,9 @@
       <c r="I80" s="88" t="n">
         <v>46308</v>
       </c>
-      <c r="J80" t="inlineStr">
-        <is>
-          <t>(pending commit)</t>
+      <c r="J80" s="40" t="inlineStr">
+        <is>
+          <t>b851189</t>
         </is>
       </c>
       <c r="K80" s="40" t="inlineStr">
@@ -5560,7 +5560,7 @@
       </c>
       <c r="L80" s="40" t="inlineStr">
         <is>
-          <t>待 push</t>
+          <t>已 push（tip b851189）</t>
         </is>
       </c>
     </row>
@@ -5635,7 +5635,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="41">
       <c r="A4" s="68" t="inlineStr">
         <is>
@@ -5828,7 +5827,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="41">
       <c r="A4" s="68" t="inlineStr">
         <is>
@@ -5896,7 +5894,6 @@
         <v/>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="15" customHeight="1" s="41">
       <c r="A11" s="72" t="inlineStr">
         <is>
@@ -5908,7 +5905,6 @@
         <v/>
       </c>
     </row>
-    <row r="12"/>
     <row r="13" ht="15" customHeight="1" s="41">
       <c r="A13" s="80" t="inlineStr">
         <is>
@@ -6002,7 +5998,7 @@
       </c>
       <c r="B21" s="40" t="inlineStr">
         <is>
-          <t>远程 tip 待本刀 push 后更新（X05-D1）。人工维护，最后更新 2026-10-13 BF CST。</t>
+          <t>远程 tip b851189（X05-D1 关单）。人工维护，最后更新 2026-10-13 BF CST。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor(web): D-02b shell helpers — status, message display, emoji wiring
Extract useStatusBar + useMessageDisplay from App.vue; move emoji
document listeners and conversations poll lifecycle into useChatSession.
App.vue 1664→1527; behavior unchanged. Leave shell templates and
late-bound composable glue in App on purpose (coupling). Close D-02b.
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -5447,7 +5447,7 @@
       </c>
       <c r="K78" s="40" t="inlineStr">
         <is>
-          <t>2026-10-11 拍板关单：D-02 P0（useAppShell+useChatSession, 8606bbb）/P1（useProfileAppearance+useContactsImport, d6a00c5）/P2（useMemoryUi+useVoiceInput, bdca268）全部关单。App.vue 约 2446→1629（约−817）。状态部分已收；剩壳模板/胶水/status/展示辅助/emoji。拆出独立债 D-02b（壳层/辅助清理），不再继续抽 App.vue。 与状态债分离：壳层/辅助见 D-02b。</t>
+          <t>2026-10-11 拍板关单：D-02 P0（useAppShell+useChatSession, 8606bbb）/P1（useProfileAppearance+useContactsImport, d6a00c5）/P2（useMemoryUi+useVoiceInput, bdca268）全部关单。App.vue 约 2446→1629（约−817）。状态部分已收；剩壳模板/胶水/status/展示辅助/emoji。拆出独立债 D-02b（壳层/辅助清理），不再继续抽 App.vue。 与状态债分离：壳层/辅助见 D-02b。 2026-10-13：D-02b 已处理（辅助清理）；D-02 仍部分收口。</t>
         </is>
       </c>
       <c r="L78" s="40" t="inlineStr">
@@ -5464,7 +5464,7 @@
       </c>
       <c r="B79" s="40" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>已处理</t>
         </is>
       </c>
       <c r="C79" s="40" t="inlineStr">
@@ -5489,20 +5489,28 @@
       </c>
       <c r="G79" s="40" t="inlineStr">
         <is>
-          <t>独立债，不挂 D-02。拍板：暂不继续抽 App.vue（边际收益递减，避免壳层拆散增加耦合）。节奏另定。</t>
+          <t>2026-10-13 BF：抽出 useStatusBar + useMessageDisplay；emoji document 监听与 conversations poll 生命周期收进 useChatSession。App.vue 1664→1527。行为不变。刻意不拆：大块壳模板、late-bound composable 胶水（边际收益/耦合）。</t>
         </is>
       </c>
       <c r="H79" s="88" t="n">
         <v>46306</v>
       </c>
+      <c r="I79" s="88" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>(pending commit)</t>
+        </is>
+      </c>
       <c r="K79" s="40" t="inlineStr">
         <is>
-          <t>来源：2026-10-11 拍板。与 D-02 状态债分离。N-02/Gemini 无关。 2026-10-11 收尾：排在 X05-D1 之后；顺序 X05-D1→D-02b→试跑挂债。</t>
+          <t>来源 D-02 拆出。2026-10-13 BF 关单（辅助/status/emoji）。壳模板面板拆分不纳入本刀。N-02/Gemini/X05-D2～D6 不动。</t>
         </is>
       </c>
       <c r="L79" s="40" t="inlineStr">
         <is>
-          <t>不适用</t>
+          <t>待 push</t>
         </is>
       </c>
     </row>
@@ -5986,7 +5994,7 @@
       </c>
       <c r="B20" s="40" t="inlineStr">
         <is>
-          <t>X05-D1 已关（2026-10-13 BF）。下一优先：D-02b 抽取 → 试跑挂债（Gemini Key）。N-02 不动；X-05 过召回靠提示词不拆包。</t>
+          <t>D-02b 已关（2026-10-13 BF）。挂债：试跑线 Gemini Key；X05-D2～D6 二期池。N-02 不动。</t>
         </is>
       </c>
     </row>
@@ -5998,7 +6006,7 @@
       </c>
       <c r="B21" s="40" t="inlineStr">
         <is>
-          <t>远程 tip b851189（X05-D1 关单）。人工维护，最后更新 2026-10-13 BF CST。</t>
+          <t>远程 tip 待本刀 push 后更新（D-02b）。人工维护，最后更新 2026-10-13 BF CST。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: D-02b tip ecc0910 + issue table push sync
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -5498,9 +5498,9 @@
       <c r="I79" s="88" t="n">
         <v>46308</v>
       </c>
-      <c r="J79" t="inlineStr">
-        <is>
-          <t>(pending commit)</t>
+      <c r="J79" s="40" t="inlineStr">
+        <is>
+          <t>ecc0910</t>
         </is>
       </c>
       <c r="K79" s="40" t="inlineStr">
@@ -5510,7 +5510,7 @@
       </c>
       <c r="L79" s="40" t="inlineStr">
         <is>
-          <t>待 push</t>
+          <t>已 push（tip ecc0910）</t>
         </is>
       </c>
     </row>
@@ -6006,7 +6006,7 @@
       </c>
       <c r="B21" s="40" t="inlineStr">
         <is>
-          <t>远程 tip 待本刀 push 后更新（D-02b）。人工维护，最后更新 2026-10-13 BF CST。</t>
+          <t>远程 tip ecc0910（D-02b 关单）。人工维护，最后更新 2026-10-13 BF CST。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: sync DeepSeek已通 + X05-D1本次新做 + D-02 计分行2446→1527
拍板记账：官方 DeepSeek 文本+识图试跑改为已通；X05-D1 标明本次新做；
D-02 累计 App.vue 2446→1527（−919，含 D-02b）；N-02/Gemini 不变。
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -4094,7 +4094,7 @@
       <c r="J47" s="86" t="n"/>
       <c r="K47" s="86" t="inlineStr">
         <is>
-          <t>来源：用户 2026-10-10 规划占位。触发：用户选定多模型供应商与路由规则后再开。 2026-10-10：提前至二期中后段；与 ARCH-2 共挂 API 试跑线（本地/硅基/官方；DeepSeek 文本、官方 VLM、Gemini TTS）。 2026-10-11 试跑线仍不动。</t>
+          <t>来源：用户 2026-10-10 规划占位。触发：用户选定多模型供应商与路由规则后再开。 2026-10-10：提前至二期中后段；与 ARCH-2 共挂 API 试跑线（本地/硅基/官方；DeepSeek 文本、官方 VLM、Gemini TTS）。 2026-10-11 试跑线仍不动。 2026-10-13：仍暂缓，不发明工作。</t>
         </is>
       </c>
       <c r="L47" s="86" t="inlineStr">
@@ -4498,7 +4498,7 @@
       </c>
       <c r="K55" s="40" t="inlineStr">
         <is>
-          <t>依赖 R-05/R-06 已交付。 2026-10-11 复盘+小修 F1/F2/F3。口径=部分收口。续债：D1确认按钮(P1)/D2 pending TTL/D3确认晚到/D4过召回后处理/D5失败无感(D-05)/D6=D-24。N-02/Gemini未动。 2026-10-11 收尾对齐：状态=部分收口（非已处理）；功能 tip affbbde；文档 tip c9be373；续债 X05-D1 待处理；过召回靠提示词不拆包；明天第一刀 X05-D1。 2026-10-13：X05-D1 已处理（BF）。续债从 D2 起；下一刀可 D-02b。</t>
+          <t>依赖 R-05/R-06 已交付。 2026-10-11 复盘+小修 F1/F2/F3。口径=部分收口。续债：D1确认按钮(P1)/D2 pending TTL/D3确认晚到/D4过召回后处理/D5失败无感(D-05)/D6=D-24。N-02/Gemini未动。 2026-10-11 收尾对齐：状态=部分收口（非已处理）；功能 tip affbbde；文档 tip c9be373；续债 X05-D1 待处理；过召回靠提示词不拆包；明天第一刀 X05-D1。 2026-10-13：X05-D1 已处理（BF）。续债从 D2 起；下一刀可 D-02b。 2026-10-13：X05-D1 本次新做已关；D-02b 已关；DeepSeek 官方已通；续债仅 D2–D6 待拍板。Gemini/N-02 不动。</t>
         </is>
       </c>
       <c r="L55" s="40" t="inlineStr">
@@ -4701,7 +4701,7 @@
       </c>
       <c r="G59" s="40" t="inlineStr">
         <is>
-          <t>关单 2026-10-10 21:30 CST（HY）。管道 Provider+.env+D-05。试跑：DeepSeek 文本通；本地 Ollama qwen2.5vl:7b 读图通；Gemini TTS 缺 Key 未实跑→挂 B-04d/API 试跑线续债。N-02 未做。</t>
+          <t>关单 2026-10-10 21:30 CST（HY）。管道 Provider+.env+D-05。试跑：DeepSeek 文本通；本地 Ollama qwen2.5vl:7b 读图通；Gemini TTS 缺 Key 未实跑→挂 B-04d/API 试跑线续债。N-02 未做。 【2026-10-13】DeepSeek 官方文本+识图已通（BF）；Gemini 仍挂 Key。</t>
         </is>
       </c>
       <c r="H59" s="83" t="n">
@@ -4717,7 +4717,7 @@
       </c>
       <c r="K59" s="40" t="inlineStr">
         <is>
-          <t>试跑主证据改为 HY 本地 VLM；硅基 Qwen3-VL 降为回落 2026-10-11 API 切换试跑线（HY）：DeepSeek 文本通（硅基 DeepSeek-V4-Flash，本机 DEEPSEEK_API_KEY 空）；读图：本地 Ollama qwen2.5vl:7b 通（官方/独立 VLM Key 未配）；Gemini TTS 缺 GEMINI_API_KEY → 挂债不阻塞（B-04d 续）。N-02 仍不动。 2026-10-11 收尾试跑线备注：DeepSeek 文本通（硅基 DeepSeek-V4-Flash，属 DeepSeek 系列）；本地 Ollama qwen2.5vl 读图通；Gemini TTS + 官方 VLM Key 挂债（不阻塞）。N-02 不动。</t>
+          <t>试跑主证据改为 HY 本地 VLM；硅基 Qwen3-VL 降为回落 2026-10-11 API 切换试跑线（HY）：DeepSeek 文本通（硅基 DeepSeek-V4-Flash，本机 DEEPSEEK_API_KEY 空）；读图：本地 Ollama qwen2.5vl:7b 通（官方/独立 VLM Key 未配）；Gemini TTS 缺 GEMINI_API_KEY → 挂债不阻塞（B-04d 续）。N-02 仍不动。 2026-10-11 收尾试跑线备注：DeepSeek 文本通（硅基 DeepSeek-V4-Flash，属 DeepSeek 系列）；本地 Ollama qwen2.5vl 读图通；Gemini TTS + 官方 VLM Key 挂债（不阻塞）。N-02 不动。 2026-10-13 BF 拍板：DeepSeek 官方试跑 **已通**（文本+识图均 api.deepseek.com / deepseek-flash；官方识图超出原仅文本计划）。Gemini TTS 仍等 GEMINI_API_KEY；N-02 不变。</t>
         </is>
       </c>
       <c r="L59" s="40" t="inlineStr">
@@ -4862,7 +4862,7 @@
       </c>
       <c r="G62" s="40" t="inlineStr">
         <is>
-          <t>【2026-10-10 21:30 CST ARCH-2 试跑线续债】Gemini TTS：HY 无 GEMINI_API_KEY，缺 Key 未实跑；坏 Key 上游观测仍 HTTP 401。产品失败回流人话路径仍待验。 【2026-10-11 试跑】Gemini TTS 仍缺 GEMINI_API_KEY，未实跑；挂债不阻塞。坏 IMAGE_GEN Key 上游仍 HTTP 401。</t>
+          <t>【2026-10-10 21:30 CST ARCH-2 试跑线续债】Gemini TTS：HY 无 GEMINI_API_KEY，缺 Key 未实跑；坏 Key 上游观测仍 HTTP 401。产品失败回流人话路径仍待验。 【2026-10-11 试跑】Gemini TTS 仍缺 GEMINI_API_KEY，未实跑；挂债不阻塞。坏 IMAGE_GEN Key 上游仍 HTTP 401。 【2026-10-13】DeepSeek 已通；Gemini TTS 仍缺 Key。</t>
         </is>
       </c>
       <c r="H62" s="83" t="n">
@@ -4870,7 +4870,7 @@
       </c>
       <c r="K62" s="40" t="inlineStr">
         <is>
-          <t>挂 API/密钥试跑时顺带验。 2026-10-10：读图 VLM 债/B-04d 在 ARCH-2 试跑线里还（非独立刀）。 2026-10-10 试跑线观测：坏 IMAGE_GEN Key → 上游 HTTP 401 Token is invalid；产品侧失败回流人话路径未改代码实打，仍暂缓。 2026-10-11 收尾：Gemini TTS + 官方 VLM 仍挂债等 Key；排在 X05-D1 / D-02b 之后。</t>
+          <t>挂 API/密钥试跑时顺带验。 2026-10-10：读图 VLM 债/B-04d 在 ARCH-2 试跑线里还（非独立刀）。 2026-10-10 试跑线观测：坏 IMAGE_GEN Key → 上游 HTTP 401 Token is invalid；产品侧失败回流人话路径未改代码实打，仍暂缓。 2026-10-11 收尾：Gemini TTS + 官方 VLM 仍挂债等 Key；排在 X05-D1 / D-02b 之后。 2026-10-13：DeepSeek 官方文本+识图已通，不再算试跑挂债；本条续挂 **Gemini TTS 等 Key** + 生图失败人话路径。</t>
         </is>
       </c>
       <c r="L62" s="40" t="inlineStr">
@@ -5434,7 +5434,7 @@
       </c>
       <c r="G78" s="40" t="inlineStr">
         <is>
-          <t>2026-10-11 定口径：部分收口（不标已收口）。状态部分已收：P0 useAppShell+useChatSession（8606bbb）；P1 useProfileAppearance+useContactsImport（d6a00c5）；P2 useMemoryUi+useVoiceInput（bdca268）。App.vue ~2446→1629。剩：壳模板、composable 胶水、status、消息展示辅助、emoji 接线——拆 D-02b，不再继续抽。</t>
+          <t>2026-10-11 定口径：部分收口（不标已收口）。状态部分已收：P0 useAppShell+useChatSession（8606bbb）；P1 useProfileAppearance+useContactsImport（d6a00c5）；P2 useMemoryUi+useVoiceInput（bdca268）。App.vue ~2446→1629。剩：壳模板、composable 胶水、status、消息展示辅助、emoji 接线——拆 D-02b，不再继续抽。 2026-10-13 计分行（含 D-02b）：App.vue **2446 → 1527（−919 行）**。D-02 仍部分收口；D-02b 已关。</t>
         </is>
       </c>
       <c r="H78" s="88" t="n">
@@ -5447,12 +5447,12 @@
       </c>
       <c r="K78" s="40" t="inlineStr">
         <is>
-          <t>2026-10-11 拍板关单：D-02 P0（useAppShell+useChatSession, 8606bbb）/P1（useProfileAppearance+useContactsImport, d6a00c5）/P2（useMemoryUi+useVoiceInput, bdca268）全部关单。App.vue 约 2446→1629（约−817）。状态部分已收；剩壳模板/胶水/status/展示辅助/emoji。拆出独立债 D-02b（壳层/辅助清理），不再继续抽 App.vue。 与状态债分离：壳层/辅助见 D-02b。 2026-10-13：D-02b 已处理（辅助清理）；D-02 仍部分收口。</t>
+          <t>2026-10-11 拍板关单：D-02 P0（useAppShell+useChatSession, 8606bbb）/P1（useProfileAppearance+useContactsImport, d6a00c5）/P2（useMemoryUi+useVoiceInput, bdca268）全部关单。App.vue 约 2446→1629（约−817）。状态部分已收；剩壳模板/胶水/status/展示辅助/emoji。拆出独立债 D-02b（壳层/辅助清理），不再继续抽 App.vue。 与状态债分离：壳层/辅助见 D-02b。 2026-10-13：D-02b 已处理（辅助清理）；D-02 仍部分收口。 2026-10-13 计分行（含 D-02b）：App.vue **2446 → 1527（−919 行）**。D-02 仍部分收口；D-02b 已关。</t>
         </is>
       </c>
       <c r="L78" s="40" t="inlineStr">
         <is>
-          <t>已 push tip bdca268</t>
+          <t>已 push；累计计分行见 2026-10-13 备注（tip 链至 cd9ea00/D-02b）</t>
         </is>
       </c>
     </row>
@@ -5505,7 +5505,7 @@
       </c>
       <c r="K79" s="40" t="inlineStr">
         <is>
-          <t>来源 D-02 拆出。2026-10-13 BF 关单（辅助/status/emoji）。壳模板面板拆分不纳入本刀。N-02/Gemini/X05-D2～D6 不动。</t>
+          <t>来源 D-02 拆出。2026-10-13 BF 关单（辅助/status/emoji）。壳模板面板拆分不纳入本刀。N-02/Gemini/X05-D2～D6 不动。 计入 D-02 累计计分行：App.vue 2446→1527（−919）。</t>
         </is>
       </c>
       <c r="L79" s="40" t="inlineStr">
@@ -5547,7 +5547,7 @@
       </c>
       <c r="G80" s="40" t="inlineStr">
         <is>
-          <t>2026-10-13 BF：memory_confirm 气泡下「改/不改」chips；sendQuickText→resolvePendingMemoryConfirm；自然语言兜底保留；末尾未回复的确认才显示；发送后短轮询 listMessages 拉异步确认气泡。无新 App.vue 状态债。</t>
+          <t>【本次新做】2026-10-13 BF：memory_confirm 气泡下「改/不改」chips；sendQuickText→resolvePendingMemoryConfirm；自然语言兜底保留；末尾未回复的确认才显示；发送后短轮询 listMessages 拉异步确认气泡。无新 App.vue 状态债。</t>
         </is>
       </c>
       <c r="H80" s="88" t="n">
@@ -5563,7 +5563,7 @@
       </c>
       <c r="K80" s="40" t="inlineStr">
         <is>
-          <t>来源 X-05。2026-10-13 BF 关单。选择=最小解释（不新开 API）。续：D-02b / X05-D2。N-02 不动。</t>
+          <t>来源 X-05。2026-10-13 BF 关单。选择=最小解释（不新开 API）。续：D-02b / X05-D2。N-02 不动。 **口径=本次新做**：先前仅有表行、无功能 commit（误传 a151f0b 不存在）；本轮 BF 新做落地 tip b851189，属补做关单。</t>
         </is>
       </c>
       <c r="L80" s="40" t="inlineStr">
@@ -5994,7 +5994,7 @@
       </c>
       <c r="B20" s="40" t="inlineStr">
         <is>
-          <t>D-02b 已关（2026-10-13 BF）。挂债：试跑线 Gemini Key；X05-D2～D6 二期池。N-02 不动。</t>
+          <t>DeepSeek 官方试跑已通（文本+识图）。X05-D1（本次新做）/ D-02b 已关。下一候选：X05-D2～D6 待用户拍板。Gemini 仍等 Key；N-02 暂缓。</t>
         </is>
       </c>
     </row>
@@ -6006,7 +6006,7 @@
       </c>
       <c r="B21" s="40" t="inlineStr">
         <is>
-          <t>远程 tip ecc0910（D-02b 关单）。人工维护，最后更新 2026-10-13 BF CST。</t>
+          <t>远程 tip 待本同步 commit 后更新。人工维护，最后更新 2026-10-13 BF CST。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(memory): X05-D2 pending TTL + X05-D5 extract fail metrics/debug
D2: default 7-day pending TTL (MEMORY_PENDING_TTL_DAYS); expire to
superseded on list/resolve/extract/apply; profile discard API+UI.
D5: always-on [memory.obs] metrics + /api/health.memoryExtract;
MEMORY_EXTRACT_DEBUG=1 quiet memory_debug chat hint (off by default).
D3/D4 deferred; D6 stays off. D1 chips unchanged.
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -1389,7 +1389,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L80"/>
+  <dimension ref="A1:L85"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="40" min="1" max="1"/>
@@ -4498,7 +4498,7 @@
       </c>
       <c r="K55" s="40" t="inlineStr">
         <is>
-          <t>依赖 R-05/R-06 已交付。 2026-10-11 复盘+小修 F1/F2/F3。口径=部分收口。续债：D1确认按钮(P1)/D2 pending TTL/D3确认晚到/D4过召回后处理/D5失败无感(D-05)/D6=D-24。N-02/Gemini未动。 2026-10-11 收尾对齐：状态=部分收口（非已处理）；功能 tip affbbde；文档 tip c9be373；续债 X05-D1 待处理；过召回靠提示词不拆包；明天第一刀 X05-D1。 2026-10-13：X05-D1 已处理（BF）。续债从 D2 起；下一刀可 D-02b。 2026-10-13：X05-D1 本次新做已关；D-02b 已关；DeepSeek 官方已通；续债仅 D2–D6 待拍板。Gemini/N-02 不动。</t>
+          <t>依赖 R-05/R-06 已交付。 2026-10-11 复盘+小修 F1/F2/F3。口径=部分收口。续债：D1确认按钮(P1)/D2 pending TTL/D3确认晚到/D4过召回后处理/D5失败无感(D-05)/D6=D-24。N-02/Gemini未动。 2026-10-11 收尾对齐：状态=部分收口（非已处理）；功能 tip affbbde；文档 tip c9be373；续债 X05-D1 待处理；过召回靠提示词不拆包；明天第一刀 X05-D1。 2026-10-13：X05-D1 已处理（BF）。续债从 D2 起；下一刀可 D-02b。 2026-10-13：X05-D1 本次新做已关；D-02b 已关；DeepSeek 官方已通；续债仅 D2–D6 待拍板。Gemini/N-02 不动。 2026-10-13：X05-D2+D5 同刀已关；D3/D4 延期；D6 维持 off。</t>
         </is>
       </c>
       <c r="L55" s="40" t="inlineStr">
@@ -5569,6 +5569,271 @@
       <c r="L80" s="40" t="inlineStr">
         <is>
           <t>已 push（tip b851189）</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>X05-D2</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>已处理</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>角色</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>pending 记忆 TTL</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>2026-10-13 BF：默认 7 天 TTL（MEMORY_PENDING_TTL_DAYS）；updated_at 过期→superseded；资料页待确认可丢弃。D1 chips 不变。</t>
+        </is>
+      </c>
+      <c r="H81" s="88" t="n">
+        <v>46306</v>
+      </c>
+      <c r="I81" s="88" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>(pending commit)</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>来源 X-05。与 D5 同刀。D3/D4 延期；D6 维持 off。</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>待 push</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>X05-D5</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>已处理</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>角色</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>提取失败轻可见</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>2026-10-13 BF：指标优先（[memory.obs] metric + /api/health.memoryExtract）；MEMORY_EXTRACT_DEBUG=1 时安静 memory_debug 气泡。</t>
+        </is>
+      </c>
+      <c r="H82" s="88" t="n">
+        <v>46306</v>
+      </c>
+      <c r="I82" s="88" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>(pending commit)</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>来源 X-05 / D-05 延伸。与 D2 同刀。默认不开 debug 提示。</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>待 push</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>X05-D3</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>暂缓</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>角色</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>确认气泡异步晚到</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>延期/记账</t>
+        </is>
+      </c>
+      <c r="H83" s="88" t="n">
+        <v>46306</v>
+      </c>
+      <c r="I83" s="88" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>(pending commit)</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>2026-10-13 拍板：本轮不做，延期。</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>待 push</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>X05-D4</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>暂缓</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>角色</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>过召回仍纯提示词</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>延期/记账</t>
+        </is>
+      </c>
+      <c r="H84" s="88" t="n">
+        <v>46306</v>
+      </c>
+      <c r="I84" s="88" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>(pending commit)</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>2026-10-13 拍板：本轮不做，延期。</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>待 push</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>X05-D6</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>暂缓</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>角色</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>MEMORY_GATE 默认 off</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>延期/记账</t>
+        </is>
+      </c>
+      <c r="H85" s="88" t="n">
+        <v>46306</v>
+      </c>
+      <c r="I85" s="88" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>(pending commit)</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>2026-10-13 拍板：MEMORY_GATE 维持 off（仅记账，不生产化）。</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>待 push</t>
         </is>
       </c>
     </row>
@@ -5994,7 +6259,7 @@
       </c>
       <c r="B20" s="40" t="inlineStr">
         <is>
-          <t>DeepSeek 官方试跑已通（文本+识图）。X05-D1（本次新做）/ D-02b 已关。下一候选：X05-D2～D6 待用户拍板。Gemini 仍等 Key；N-02 暂缓。</t>
+          <t>X05-D2+D5 已关。延期：D3/D4；D6=off。Gemini 等 Key；N-02 暂缓。</t>
         </is>
       </c>
     </row>
@@ -6006,7 +6271,7 @@
       </c>
       <c r="B21" s="40" t="inlineStr">
         <is>
-          <t>远程 tip f94c99d（拍板文档同步：DeepSeek已通 / D1本次新做 / D-02计分行）。人工维护 2026-10-13 BF CST。</t>
+          <t>远程 tip 待本刀 push 后更新。人工维护 2026-10-13 BF CST。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: X05-D2+D5 tip ad92898 + issue table push sync
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -5573,32 +5573,32 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" t="inlineStr">
+      <c r="A81" s="40" t="inlineStr">
         <is>
           <t>X05-D2</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr">
+      <c r="B81" s="40" t="inlineStr">
         <is>
           <t>已处理</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr">
+      <c r="C81" s="40" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="D81" t="inlineStr">
+      <c r="D81" s="40" t="inlineStr">
         <is>
           <t>角色</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr">
+      <c r="E81" s="40" t="inlineStr">
         <is>
           <t>pending 记忆 TTL</t>
         </is>
       </c>
-      <c r="G81" t="inlineStr">
+      <c r="G81" s="40" t="inlineStr">
         <is>
           <t>2026-10-13 BF：默认 7 天 TTL（MEMORY_PENDING_TTL_DAYS）；updated_at 过期→superseded；资料页待确认可丢弃。D1 chips 不变。</t>
         </is>
@@ -5609,49 +5609,49 @@
       <c r="I81" s="88" t="n">
         <v>46308</v>
       </c>
-      <c r="J81" t="inlineStr">
-        <is>
-          <t>(pending commit)</t>
-        </is>
-      </c>
-      <c r="K81" t="inlineStr">
+      <c r="J81" s="40" t="inlineStr">
+        <is>
+          <t>ad92898</t>
+        </is>
+      </c>
+      <c r="K81" s="40" t="inlineStr">
         <is>
           <t>来源 X-05。与 D5 同刀。D3/D4 延期；D6 维持 off。</t>
         </is>
       </c>
-      <c r="L81" t="inlineStr">
-        <is>
-          <t>待 push</t>
+      <c r="L81" s="40" t="inlineStr">
+        <is>
+          <t>已 push（tip ad92898）</t>
         </is>
       </c>
     </row>
     <row r="82">
-      <c r="A82" t="inlineStr">
+      <c r="A82" s="40" t="inlineStr">
         <is>
           <t>X05-D5</t>
         </is>
       </c>
-      <c r="B82" t="inlineStr">
+      <c r="B82" s="40" t="inlineStr">
         <is>
           <t>已处理</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr">
+      <c r="C82" s="40" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="D82" t="inlineStr">
+      <c r="D82" s="40" t="inlineStr">
         <is>
           <t>角色</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr">
+      <c r="E82" s="40" t="inlineStr">
         <is>
           <t>提取失败轻可见</t>
         </is>
       </c>
-      <c r="G82" t="inlineStr">
+      <c r="G82" s="40" t="inlineStr">
         <is>
           <t>2026-10-13 BF：指标优先（[memory.obs] metric + /api/health.memoryExtract）；MEMORY_EXTRACT_DEBUG=1 时安静 memory_debug 气泡。</t>
         </is>
@@ -5662,49 +5662,49 @@
       <c r="I82" s="88" t="n">
         <v>46308</v>
       </c>
-      <c r="J82" t="inlineStr">
-        <is>
-          <t>(pending commit)</t>
-        </is>
-      </c>
-      <c r="K82" t="inlineStr">
+      <c r="J82" s="40" t="inlineStr">
+        <is>
+          <t>ad92898</t>
+        </is>
+      </c>
+      <c r="K82" s="40" t="inlineStr">
         <is>
           <t>来源 X-05 / D-05 延伸。与 D2 同刀。默认不开 debug 提示。</t>
         </is>
       </c>
-      <c r="L82" t="inlineStr">
-        <is>
-          <t>待 push</t>
+      <c r="L82" s="40" t="inlineStr">
+        <is>
+          <t>已 push（tip ad92898）</t>
         </is>
       </c>
     </row>
     <row r="83">
-      <c r="A83" t="inlineStr">
+      <c r="A83" s="40" t="inlineStr">
         <is>
           <t>X05-D3</t>
         </is>
       </c>
-      <c r="B83" t="inlineStr">
+      <c r="B83" s="40" t="inlineStr">
         <is>
           <t>暂缓</t>
         </is>
       </c>
-      <c r="C83" t="inlineStr">
+      <c r="C83" s="40" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="D83" t="inlineStr">
+      <c r="D83" s="40" t="inlineStr">
         <is>
           <t>角色</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr">
+      <c r="E83" s="40" t="inlineStr">
         <is>
           <t>确认气泡异步晚到</t>
         </is>
       </c>
-      <c r="G83" t="inlineStr">
+      <c r="G83" s="40" t="inlineStr">
         <is>
           <t>延期/记账</t>
         </is>
@@ -5715,49 +5715,49 @@
       <c r="I83" s="88" t="n">
         <v>46308</v>
       </c>
-      <c r="J83" t="inlineStr">
+      <c r="J83" s="40" t="inlineStr">
         <is>
           <t>(pending commit)</t>
         </is>
       </c>
-      <c r="K83" t="inlineStr">
+      <c r="K83" s="40" t="inlineStr">
         <is>
           <t>2026-10-13 拍板：本轮不做，延期。</t>
         </is>
       </c>
-      <c r="L83" t="inlineStr">
+      <c r="L83" s="40" t="inlineStr">
         <is>
           <t>待 push</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="A84" t="inlineStr">
+      <c r="A84" s="40" t="inlineStr">
         <is>
           <t>X05-D4</t>
         </is>
       </c>
-      <c r="B84" t="inlineStr">
+      <c r="B84" s="40" t="inlineStr">
         <is>
           <t>暂缓</t>
         </is>
       </c>
-      <c r="C84" t="inlineStr">
+      <c r="C84" s="40" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="D84" t="inlineStr">
+      <c r="D84" s="40" t="inlineStr">
         <is>
           <t>角色</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr">
+      <c r="E84" s="40" t="inlineStr">
         <is>
           <t>过召回仍纯提示词</t>
         </is>
       </c>
-      <c r="G84" t="inlineStr">
+      <c r="G84" s="40" t="inlineStr">
         <is>
           <t>延期/记账</t>
         </is>
@@ -5768,49 +5768,49 @@
       <c r="I84" s="88" t="n">
         <v>46308</v>
       </c>
-      <c r="J84" t="inlineStr">
+      <c r="J84" s="40" t="inlineStr">
         <is>
           <t>(pending commit)</t>
         </is>
       </c>
-      <c r="K84" t="inlineStr">
+      <c r="K84" s="40" t="inlineStr">
         <is>
           <t>2026-10-13 拍板：本轮不做，延期。</t>
         </is>
       </c>
-      <c r="L84" t="inlineStr">
+      <c r="L84" s="40" t="inlineStr">
         <is>
           <t>待 push</t>
         </is>
       </c>
     </row>
     <row r="85">
-      <c r="A85" t="inlineStr">
+      <c r="A85" s="40" t="inlineStr">
         <is>
           <t>X05-D6</t>
         </is>
       </c>
-      <c r="B85" t="inlineStr">
+      <c r="B85" s="40" t="inlineStr">
         <is>
           <t>暂缓</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr">
+      <c r="C85" s="40" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="D85" t="inlineStr">
+      <c r="D85" s="40" t="inlineStr">
         <is>
           <t>角色</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr">
+      <c r="E85" s="40" t="inlineStr">
         <is>
           <t>MEMORY_GATE 默认 off</t>
         </is>
       </c>
-      <c r="G85" t="inlineStr">
+      <c r="G85" s="40" t="inlineStr">
         <is>
           <t>延期/记账</t>
         </is>
@@ -5821,17 +5821,17 @@
       <c r="I85" s="88" t="n">
         <v>46308</v>
       </c>
-      <c r="J85" t="inlineStr">
+      <c r="J85" s="40" t="inlineStr">
         <is>
           <t>(pending commit)</t>
         </is>
       </c>
-      <c r="K85" t="inlineStr">
+      <c r="K85" s="40" t="inlineStr">
         <is>
           <t>2026-10-13 拍板：MEMORY_GATE 维持 off（仅记账，不生产化）。</t>
         </is>
       </c>
-      <c r="L85" t="inlineStr">
+      <c r="L85" s="40" t="inlineStr">
         <is>
           <t>待 push</t>
         </is>
@@ -6271,7 +6271,7 @@
       </c>
       <c r="B21" s="40" t="inlineStr">
         <is>
-          <t>远程 tip 待本刀 push 后更新。人工维护 2026-10-13 BF CST。</t>
+          <t>远程 tip ad92898（X05-D2+D5）。人工维护 2026-10-13 BF CST。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: App.vue 2446→1527→1554 audit + TTL agent-default note
Note X05-D2+D5 App +27 is profile discard template/glue; pending state
stays in useMemoryUi. TTL 7d is agent default — product param TBD.
Confirm four closes; D3/D4/D6 still deferred.
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -5434,7 +5434,7 @@
       </c>
       <c r="G78" s="40" t="inlineStr">
         <is>
-          <t>2026-10-11 定口径：部分收口（不标已收口）。状态部分已收：P0 useAppShell+useChatSession（8606bbb）；P1 useProfileAppearance+useContactsImport（d6a00c5）；P2 useMemoryUi+useVoiceInput（bdca268）。App.vue ~2446→1629。剩：壳模板、composable 胶水、status、消息展示辅助、emoji 接线——拆 D-02b，不再继续抽。 2026-10-13 计分行（含 D-02b）：App.vue **2446 → 1527（−919 行）**。D-02 仍部分收口；D-02b 已关。</t>
+          <t>2026-10-11 定口径：部分收口（不标已收口）。状态部分已收：P0 useAppShell+useChatSession（8606bbb）；P1 useProfileAppearance+useContactsImport（d6a00c5）；P2 useMemoryUi+useVoiceInput（bdca268）。App.vue ~2446→1629。剩：壳模板、composable 胶水、status、消息展示辅助、emoji 接线——拆 D-02b，不再继续抽。 2026-10-13 计分行（含 D-02b）：App.vue **2446 → 1527（−919 行）**。D-02 仍部分收口；D-02b 已关。 2026-10-13 计分行续：App.vue **2446 → 1527（D-02b）→ 1554（X05-D2+D5）**。D2+D5 +27=资料页丢弃模板+胶水；pending 状态在 useMemoryUi，非 App 新业务 ref。</t>
         </is>
       </c>
       <c r="H78" s="88" t="n">
@@ -5447,7 +5447,7 @@
       </c>
       <c r="K78" s="40" t="inlineStr">
         <is>
-          <t>2026-10-11 拍板关单：D-02 P0（useAppShell+useChatSession, 8606bbb）/P1（useProfileAppearance+useContactsImport, d6a00c5）/P2（useMemoryUi+useVoiceInput, bdca268）全部关单。App.vue 约 2446→1629（约−817）。状态部分已收；剩壳模板/胶水/status/展示辅助/emoji。拆出独立债 D-02b（壳层/辅助清理），不再继续抽 App.vue。 与状态债分离：壳层/辅助见 D-02b。 2026-10-13：D-02b 已处理（辅助清理）；D-02 仍部分收口。 2026-10-13 计分行（含 D-02b）：App.vue **2446 → 1527（−919 行）**。D-02 仍部分收口；D-02b 已关。</t>
+          <t>2026-10-11 拍板关单：D-02 P0（useAppShell+useChatSession, 8606bbb）/P1（useProfileAppearance+useContactsImport, d6a00c5）/P2（useMemoryUi+useVoiceInput, bdca268）全部关单。App.vue 约 2446→1629（约−817）。状态部分已收；剩壳模板/胶水/status/展示辅助/emoji。拆出独立债 D-02b（壳层/辅助清理），不再继续抽 App.vue。 与状态债分离：壳层/辅助见 D-02b。 2026-10-13：D-02b 已处理（辅助清理）；D-02 仍部分收口。 2026-10-13 计分行（含 D-02b）：App.vue **2446 → 1527（−919 行）**。D-02 仍部分收口；D-02b 已关。 2026-10-13 计分行续：App.vue **2446 → 1527（D-02b）→ 1554（X05-D2+D5）**。D2+D5 +27=资料页丢弃模板+胶水；pending 状态在 useMemoryUi，非 App 新业务 ref。</t>
         </is>
       </c>
       <c r="L78" s="40" t="inlineStr">
@@ -5505,7 +5505,7 @@
       </c>
       <c r="K79" s="40" t="inlineStr">
         <is>
-          <t>来源 D-02 拆出。2026-10-13 BF 关单（辅助/status/emoji）。壳模板面板拆分不纳入本刀。N-02/Gemini/X05-D2～D6 不动。 计入 D-02 累计计分行：App.vue 2446→1527（−919）。</t>
+          <t>来源 D-02 拆出。2026-10-13 BF 关单（辅助/status/emoji）。壳模板面板拆分不纳入本刀。N-02/Gemini/X05-D2～D6 不动。 计入 D-02 累计计分行：App.vue 2446→1527（−919）。 后续 X05-D2+D5 抬至 1554（模板，非状态债回流）。</t>
         </is>
       </c>
       <c r="L79" s="40" t="inlineStr">
@@ -5600,7 +5600,7 @@
       </c>
       <c r="G81" s="40" t="inlineStr">
         <is>
-          <t>2026-10-13 BF：默认 7 天 TTL（MEMORY_PENDING_TTL_DAYS）；updated_at 过期→superseded；资料页待确认可丢弃。D1 chips 不变。</t>
+          <t>2026-10-13 BF：默认 7 天 TTL（MEMORY_PENDING_TTL_DAYS）；updated_at 过期→superseded；资料页待确认可丢弃。D1 chips 不变。 【参数】7 天=agent 默认，待用户明确。</t>
         </is>
       </c>
       <c r="H81" s="88" t="n">
@@ -5616,7 +5616,7 @@
       </c>
       <c r="K81" s="40" t="inlineStr">
         <is>
-          <t>来源 X-05。与 D5 同刀。D3/D4 延期；D6 维持 off。</t>
+          <t>来源 X-05。与 D5 同刀。D3/D4 延期；D6 维持 off。 TTL=7d 为 **agent 默认**（文档示例），**产品参数待用户明确**。</t>
         </is>
       </c>
       <c r="L81" s="40" t="inlineStr">
@@ -6259,7 +6259,7 @@
       </c>
       <c r="B20" s="40" t="inlineStr">
         <is>
-          <t>X05-D2+D5 已关。延期：D3/D4；D6=off。Gemini 等 Key；N-02 暂缓。</t>
+          <t>今日已关：DeepSeek已通 / X05-D1 / D-02b / X05-D2+D5。App.vue 2446→1527→1554。D3/D4/D6 延期或 off。下一候选待拍：X-03 或 B-04d。</t>
         </is>
       </c>
     </row>
@@ -6271,7 +6271,7 @@
       </c>
       <c r="B21" s="40" t="inlineStr">
         <is>
-          <t>远程 tip ad92898（X05-D2+D5）。人工维护 2026-10-13 BF CST。</t>
+          <t>远程 tip 待本同步 commit 后更新。人工维护 2026-10-13 BF CST。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(server): B-04d human-readable image-gen key failures
Map image-gen errors via formatImageGenUserError; stop embedding
upstream JSON in chat bubbles. Bad IMAGE_GEN_API_KEY verified →
user sees 密钥无效人话. Close B-04d. Gemini/N-02 untouched.
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -4837,7 +4837,7 @@
       </c>
       <c r="B62" s="40" t="inlineStr">
         <is>
-          <t>暂缓</t>
+          <t>已处理</t>
         </is>
       </c>
       <c r="C62" s="40" t="inlineStr">
@@ -4862,20 +4862,28 @@
       </c>
       <c r="G62" s="40" t="inlineStr">
         <is>
-          <t>【2026-10-10 21:30 CST ARCH-2 试跑线续债】Gemini TTS：HY 无 GEMINI_API_KEY，缺 Key 未实跑；坏 Key 上游观测仍 HTTP 401。产品失败回流人话路径仍待验。 【2026-10-11 试跑】Gemini TTS 仍缺 GEMINI_API_KEY，未实跑；挂债不阻塞。坏 IMAGE_GEN Key 上游仍 HTTP 401。 【2026-10-13】DeepSeek 已通；Gemini TTS 仍缺 Key。</t>
+          <t>2026-10-13 BF 验证+小补：坏 IMAGE_GEN_API_KEY → 上游 401；用户气泡人话「这张图没画成：密钥无效或没有权限…」不再夹带上游 JSON。formatImageGenUserError + throw 仅保留状态码；服务端仍 log 截断 body。</t>
         </is>
       </c>
       <c r="H62" s="83" t="n">
         <v>46305</v>
       </c>
+      <c r="I62" s="88" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>(pending commit)</t>
+        </is>
+      </c>
       <c r="K62" s="40" t="inlineStr">
         <is>
-          <t>挂 API/密钥试跑时顺带验。 2026-10-10：读图 VLM 债/B-04d 在 ARCH-2 试跑线里还（非独立刀）。 2026-10-10 试跑线观测：坏 IMAGE_GEN Key → 上游 HTTP 401 Token is invalid；产品侧失败回流人话路径未改代码实打，仍暂缓。 2026-10-11 收尾：Gemini TTS + 官方 VLM 仍挂债等 Key；排在 X05-D1 / D-02b 之后。 2026-10-13：DeepSeek 官方文本+识图已通，不再算试跑挂债；本条续挂 **Gemini TTS 等 Key** + 生图失败人话路径。</t>
+          <t>挂 API/密钥试跑时顺带验。 2026-10-10：读图 VLM 债/B-04d 在 ARCH-2 试跑线里还（非独立刀）。 2026-10-10 试跑线观测：坏 IMAGE_GEN Key → 上游 HTTP 401 Token is invalid；产品侧失败回流人话路径未改代码实打，仍暂缓。 2026-10-11 收尾：Gemini TTS + 官方 VLM 仍挂债等 Key；排在 X05-D1 / D-02b 之后。 2026-10-13：DeepSeek 官方文本+识图已通，不再算试跑挂债；本条续挂 **Gemini TTS 等 Key** + 生图失败人话路径。 2026-10-13：B-04d 关单（验证失败路径+开发去 JSON）。Gemini TTS 仍等 Key，不在本条。 N-02 不动。生图 Key=IMAGE_GEN_*（硅基），非 DeepSeek 文本键。</t>
         </is>
       </c>
       <c r="L62" s="40" t="inlineStr">
         <is>
-          <t>不适用</t>
+          <t>待 push</t>
         </is>
       </c>
     </row>
@@ -6259,7 +6267,7 @@
       </c>
       <c r="B20" s="40" t="inlineStr">
         <is>
-          <t>今日已关：DeepSeek已通 / X05-D1 / D-02b / X05-D2+D5。App.vue 2446→1527→1554。D3/D4/D6 延期或 off。下一候选待拍：X-03 或 B-04d。</t>
+          <t>B-04d 已关（生图 Key 失败人话）。今日已关含 DeepSeek/X05-D1/D-02b/D2+D5/B-04d。下一候选可 X-03。Gemini 仍等 Key；N-02 暂缓；D3/D4/D6 延期/off。</t>
         </is>
       </c>
     </row>
@@ -6271,7 +6279,7 @@
       </c>
       <c r="B21" s="40" t="inlineStr">
         <is>
-          <t>远程 tip bd4e638（audit/TTL/计分行同步）。人工维护 2026-10-13 BF CST。</t>
+          <t>远程 tip 待本刀 push 后更新。人工维护 2026-10-13 BF CST。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: B-04d tip 6263381 + issue table push sync
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -4871,9 +4871,9 @@
       <c r="I62" s="88" t="n">
         <v>46308</v>
       </c>
-      <c r="J62" t="inlineStr">
-        <is>
-          <t>(pending commit)</t>
+      <c r="J62" s="40" t="inlineStr">
+        <is>
+          <t>6263381</t>
         </is>
       </c>
       <c r="K62" s="40" t="inlineStr">
@@ -4883,7 +4883,7 @@
       </c>
       <c r="L62" s="40" t="inlineStr">
         <is>
-          <t>待 push</t>
+          <t>已 push（tip 6263381）</t>
         </is>
       </c>
     </row>
@@ -6279,7 +6279,7 @@
       </c>
       <c r="B21" s="40" t="inlineStr">
         <is>
-          <t>远程 tip 待本刀 push 后更新。人工维护 2026-10-13 BF CST。</t>
+          <t>远程 tip 6263381（B-04d 关单）。人工维护 2026-10-13 BF CST。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: X-03 tip 3418a6b + issue table push sync
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -4392,7 +4392,7 @@
           <t>主页现仅展示主动日 cap；需可改 daily_cap 与静默起止。</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr">
+      <c r="G53" s="40" t="inlineStr">
         <is>
           <t>2026-10-13 BF：主页可调每日主动上限（1–8）与静默起止（time input，可跨午夜）。PATCH /api/proactive 已有；tick 本就尊重 daily_cap/quiet。默认 cap=3、23:00–08:00。</t>
         </is>
@@ -4403,9 +4403,9 @@
       <c r="I53" s="88" t="n">
         <v>46308</v>
       </c>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t>(pending commit)</t>
+      <c r="J53" s="40" t="inlineStr">
+        <is>
+          <t>3418a6b</t>
         </is>
       </c>
       <c r="K53" s="40" t="inlineStr">
@@ -4415,7 +4415,7 @@
       </c>
       <c r="L53" s="40" t="inlineStr">
         <is>
-          <t>待 push</t>
+          <t>已 push（tip 3418a6b）</t>
         </is>
       </c>
     </row>
@@ -6292,7 +6292,7 @@
       </c>
       <c r="B21" s="40" t="inlineStr">
         <is>
-          <t>远程 tip 待本刀 push 后更新。人工维护 2026-10-13 BF CST。</t>
+          <t>远程 tip 3418a6b（X-03 关单）。人工维护 2026-10-13 BF CST。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(web): X-03 adjustable daily_cap and quiet hours
Profile UI to edit proactive daily cap (1-8) and quiet start/end;
PATCH /api/proactive already persisted — tick already respects settings.
Normalize HH:MM on server. Defaults remain cap=3, 23:00-08:00.
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -4369,7 +4369,7 @@
       </c>
       <c r="B53" s="40" t="inlineStr">
         <is>
-          <t>暂缓</t>
+          <t>已处理</t>
         </is>
       </c>
       <c r="C53" s="40" t="inlineStr">
@@ -4390,19 +4390,32 @@
       <c r="F53" s="40" t="inlineStr">
         <is>
           <t>主页现仅展示主动日 cap；需可改 daily_cap 与静默起止。</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>2026-10-13 BF：主页可调每日主动上限（1–8）与静默起止（time input，可跨午夜）。PATCH /api/proactive 已有；tick 本就尊重 daily_cap/quiet。默认 cap=3、23:00–08:00。</t>
         </is>
       </c>
       <c r="H53" s="83" t="n">
         <v>46305</v>
       </c>
+      <c r="I53" s="88" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>(pending commit)</t>
+        </is>
+      </c>
       <c r="K53" s="40" t="inlineStr">
         <is>
-          <t>二期可选。</t>
+          <t>二期可选。 2026-10-13 关单。与 C-06/D-04 同组主动线；N-02/Gemini/X05-D3～D6 不动。 App.vue 仅模板+接线，逻辑在 useProactiveSettings。</t>
         </is>
       </c>
       <c r="L53" s="40" t="inlineStr">
         <is>
-          <t>不适用</t>
+          <t>待 push</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6280,7 @@
       </c>
       <c r="B20" s="40" t="inlineStr">
         <is>
-          <t>B-04d 已关（生图 Key 失败人话）。今日已关含 DeepSeek/X05-D1/D-02b/D2+D5/B-04d。下一候选可 X-03。Gemini 仍等 Key；N-02 暂缓；D3/D4/D6 延期/off。</t>
+          <t>X-03 已关（daily_cap/静默可调）。B-04d 已关。挂债：Gemini Key；X05-D3/D4 延期；D6=off；N-02 暂缓。</t>
         </is>
       </c>
     </row>
@@ -6279,7 +6292,7 @@
       </c>
       <c r="B21" s="40" t="inlineStr">
         <is>
-          <t>远程 tip 6263381（B-04d 关单）。人工维护 2026-10-13 BF CST。</t>
+          <t>远程 tip 待本刀 push 后更新。人工维护 2026-10-13 BF CST。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(proactive): D-04 M-01 space author reply ignores private daily_cap
Align settleAuthorReplyToUserComment with C-06/M-07: master switch + quiet
hours still apply; private proactive tick remains daily_cap-gated.
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -1389,7 +1389,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L85"/>
+  <dimension ref="A1:L86"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="40" min="1" max="1"/>
@@ -3990,7 +3990,7 @@
       </c>
       <c r="K45" s="40" t="inlineStr">
         <is>
-          <t>2026-10-10 点收并已在 origin。 2026-10-10 ARCH-1：功能池登记 D-04（M-01 仍吃私聊 daily_cap，与 C-06 后 M-07 空间不受 cap 不一致）→ 与 C-06 同组 P2，不进 ARCH-2/3。详见 docs/product/ARCH-1-债清单.md。</t>
+          <t>2026-10-10 点收并已在 origin。 2026-10-10 ARCH-1：功能池登记 D-04（M-01 仍吃私聊 daily_cap，与 C-06 后 M-07 空间不受 cap 不一致）→ 与 C-06 同组 P2，不进 ARCH-2/3。详见 docs/product/ARCH-1-债清单.md。 2026-10-13：D-04 已关（M-01 对齐不再吃 daily_cap）。</t>
         </is>
       </c>
       <c r="L45" s="40" t="inlineStr">
@@ -5853,6 +5853,64 @@
         </is>
       </c>
       <c r="L85" s="40" t="inlineStr">
+        <is>
+          <t>待 push</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>D-04</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>已处理</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>会话</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>主动/空间 cap 登记对齐（M-01 vs C-06）</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>C-06 后 M-07 空间赞评不受私聊 daily_cap；M-01 作者回复仍吃 daily_cap，登记不一致。</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>2026-10-13 BF：去掉 M-01 settleAuthorReplyToUserComment 的 daily_cap 跳过；与 C-06/M-07 一致。总开关+静默仍约束空间；私聊主动仍吃 daily_cap。</t>
+        </is>
+      </c>
+      <c r="H86" s="88" t="n">
+        <v>46305</v>
+      </c>
+      <c r="I86" s="88" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>(pending commit)</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>来源 ARCH-1 功能池 / C-06 遗留。N-02/Gemini/X05-D3～D6 不动。 备注：TTL 7d、静默 23:00–08:00 产品参数待明确；D-11 双机 .env、D-22 smoke_*.py 仍在 ARCH-1 池。</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
         <is>
           <t>待 push</t>
         </is>
@@ -6280,7 +6338,7 @@
       </c>
       <c r="B20" s="40" t="inlineStr">
         <is>
-          <t>X-03 已关（daily_cap/静默可调）。B-04d 已关。挂债：Gemini Key；X05-D3/D4 延期；D6=off；N-02 暂缓。</t>
+          <t>D-04 已关（M-01 空间作者回复不再吃私聊 daily_cap）。参数待明确：TTL 7d、静默 23:00–08:00。池：D-11 .env / D-22 smoke_*.py。挂：Gemini Key；X05-D3/D4；D6=off；N-02。X-07 未开。</t>
         </is>
       </c>
     </row>
@@ -6292,7 +6350,7 @@
       </c>
       <c r="B21" s="40" t="inlineStr">
         <is>
-          <t>远程 tip 3418a6b（X-03 关单）。人工维护 2026-10-13 BF CST。</t>
+          <t>远程 tip 待本刀 push 后更新。人工维护 2026-10-13 BF CST。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: D-04 tip b7cd9e6 + issue table push sync
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -5859,37 +5859,37 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" t="inlineStr">
+      <c r="A86" s="40" t="inlineStr">
         <is>
           <t>D-04</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr">
+      <c r="B86" s="40" t="inlineStr">
         <is>
           <t>已处理</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr">
+      <c r="C86" s="40" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="D86" t="inlineStr">
+      <c r="D86" s="40" t="inlineStr">
         <is>
           <t>会话</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr">
+      <c r="E86" s="40" t="inlineStr">
         <is>
           <t>主动/空间 cap 登记对齐（M-01 vs C-06）</t>
         </is>
       </c>
-      <c r="F86" t="inlineStr">
+      <c r="F86" s="40" t="inlineStr">
         <is>
           <t>C-06 后 M-07 空间赞评不受私聊 daily_cap；M-01 作者回复仍吃 daily_cap，登记不一致。</t>
         </is>
       </c>
-      <c r="G86" t="inlineStr">
+      <c r="G86" s="40" t="inlineStr">
         <is>
           <t>2026-10-13 BF：去掉 M-01 settleAuthorReplyToUserComment 的 daily_cap 跳过；与 C-06/M-07 一致。总开关+静默仍约束空间；私聊主动仍吃 daily_cap。</t>
         </is>
@@ -5900,19 +5900,19 @@
       <c r="I86" s="88" t="n">
         <v>46308</v>
       </c>
-      <c r="J86" t="inlineStr">
-        <is>
-          <t>(pending commit)</t>
-        </is>
-      </c>
-      <c r="K86" t="inlineStr">
+      <c r="J86" s="40" t="inlineStr">
+        <is>
+          <t>b7cd9e6</t>
+        </is>
+      </c>
+      <c r="K86" s="40" t="inlineStr">
         <is>
           <t>来源 ARCH-1 功能池 / C-06 遗留。N-02/Gemini/X05-D3～D6 不动。 备注：TTL 7d、静默 23:00–08:00 产品参数待明确；D-11 双机 .env、D-22 smoke_*.py 仍在 ARCH-1 池。</t>
         </is>
       </c>
-      <c r="L86" t="inlineStr">
-        <is>
-          <t>待 push</t>
+      <c r="L86" s="40" t="inlineStr">
+        <is>
+          <t>已 push</t>
         </is>
       </c>
     </row>
@@ -6350,7 +6350,7 @@
       </c>
       <c r="B21" s="40" t="inlineStr">
         <is>
-          <t>远程 tip 待本刀 push 后更新。人工维护 2026-10-13 BF CST。</t>
+          <t>远程 tip b7cd9e6。人工维护 2026-10-13 BF CST。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(proactive): X-07 adjustable space like/comment intensity
Define knobs space_like_max (0-3, default 2) and space_comment_max (0-1, default 1);
persist on user_profile; profile editors + PATCH /api/proactive; M-07 settle respects them.
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -4586,7 +4586,7 @@
       </c>
       <c r="B57" s="40" t="inlineStr">
         <is>
-          <t>暂缓</t>
+          <t>已处理</t>
         </is>
       </c>
       <c r="C57" s="40" t="inlineStr">
@@ -4607,19 +4607,32 @@
       <c r="F57" s="40" t="inlineStr">
         <is>
           <t>赞评频率需产品可调项（先定可调参数再开发）。</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>2026-10-13 BF：先定可调项=空间赞上限 space_like_max(0–3,默认2)、空间评上限 space_comment_max(0–1,默认1)；主页可改；PATCH /api/proactive；M-07 settle 尊重。与私聊 daily_cap 解耦。</t>
         </is>
       </c>
       <c r="H57" s="83" t="n">
         <v>46305</v>
       </c>
+      <c r="I57" s="88" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>(pending commit)</t>
+        </is>
+      </c>
       <c r="K57" s="40" t="inlineStr">
         <is>
-          <t>先定可调项再拆包。</t>
+          <t>先定可调项再拆包 → 本刀已定最小集并对齐设计备忘「0～2 赞 / 0～1 评」。未开：X-02/X-04、N-02、Gemini、X05-D3/D4、D6、D-11/D-22。</t>
         </is>
       </c>
       <c r="L57" s="40" t="inlineStr">
         <is>
-          <t>不适用</t>
+          <t>待 push</t>
         </is>
       </c>
     </row>
@@ -6338,7 +6351,7 @@
       </c>
       <c r="B20" s="40" t="inlineStr">
         <is>
-          <t>D-04 已关（M-01 空间作者回复不再吃私聊 daily_cap）。参数待明确：TTL 7d、静默 23:00–08:00。池：D-11 .env / D-22 smoke_*.py。挂：Gemini Key；X05-D3/D4；D6=off；N-02。X-07 未开。</t>
+          <t>X-07 已关（空间赞/评上限可调）。参数待明确：TTL 7d、静默默认。池：D-11 .env / D-22 smoke。挂：Gemini；X05-D3/D4；D6=off；N-02。X-02/X-04 未开。</t>
         </is>
       </c>
     </row>
@@ -6350,7 +6363,7 @@
       </c>
       <c r="B21" s="40" t="inlineStr">
         <is>
-          <t>远程 tip b7cd9e6。人工维护 2026-10-13 BF CST。</t>
+          <t>远程 tip 待本刀 push 后更新。人工维护 2026-10-13 BF CST。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: X-07 tip 710bce9 + issue table push sync
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -4609,7 +4609,7 @@
           <t>赞评频率需产品可调项（先定可调参数再开发）。</t>
         </is>
       </c>
-      <c r="G57" t="inlineStr">
+      <c r="G57" s="40" t="inlineStr">
         <is>
           <t>2026-10-13 BF：先定可调项=空间赞上限 space_like_max(0–3,默认2)、空间评上限 space_comment_max(0–1,默认1)；主页可改；PATCH /api/proactive；M-07 settle 尊重。与私聊 daily_cap 解耦。</t>
         </is>
@@ -4620,9 +4620,9 @@
       <c r="I57" s="88" t="n">
         <v>46308</v>
       </c>
-      <c r="J57" t="inlineStr">
-        <is>
-          <t>(pending commit)</t>
+      <c r="J57" s="40" t="inlineStr">
+        <is>
+          <t>710bce9</t>
         </is>
       </c>
       <c r="K57" s="40" t="inlineStr">
@@ -4632,7 +4632,7 @@
       </c>
       <c r="L57" s="40" t="inlineStr">
         <is>
-          <t>待 push</t>
+          <t>已 push</t>
         </is>
       </c>
     </row>
@@ -6363,7 +6363,7 @@
       </c>
       <c r="B21" s="40" t="inlineStr">
         <is>
-          <t>远程 tip 待本刀 push 后更新。人工维护 2026-10-13 BF CST。</t>
+          <t>远程 tip 710bce9。人工维护 2026-10-13 BF CST。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: D-11 env key diff + D-22 smoke under scripts/smoke
- docs/product/D-11-env-key-diff.md: BF vs .env.example vs code keys (no secrets); HY pending
- .env.example: mark D-11 optional keys
- move smoke_*.py to scripts/smoke/, portable _out paths; README run note
- issue table: X-04 closed 3f9f54b; X-02 deferred; D-11/D-22 in progress notes
- keep .env.bak untracked
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -1389,7 +1389,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L86"/>
+  <dimension ref="A1:L88"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="40" min="1" max="1"/>
@@ -4352,7 +4352,7 @@
       </c>
       <c r="K52" s="40" t="inlineStr">
         <is>
-          <t>待 X-01 后。</t>
+          <t>暂缓实现；等视觉Bot规格（尺寸/格式/存储位置/与头像·封面关系）→ 用户拍「DB vs uploads+只读」→ 再拆包。</t>
         </is>
       </c>
       <c r="L52" s="40" t="inlineStr">
@@ -4427,7 +4427,7 @@
       </c>
       <c r="B54" s="40" t="inlineStr">
         <is>
-          <t>暂缓</t>
+          <t>已处理</t>
         </is>
       </c>
       <c r="C54" s="40" t="inlineStr">
@@ -4453,14 +4453,22 @@
       <c r="H54" s="83" t="n">
         <v>46305</v>
       </c>
+      <c r="I54" s="83" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J54" s="40" t="inlineStr">
+        <is>
+          <t>3f9f54b</t>
+        </is>
+      </c>
       <c r="K54" s="40" t="inlineStr">
         <is>
-          <t>二期体验债。</t>
+          <t>实现已关 tip 3f9f54b；产品参数「2静1开」「TTL 7天」「静默默认 23:00–08:00」均待明确（当前硬编码可跑，改数另开刀）。云测通过。</t>
         </is>
       </c>
       <c r="L54" s="40" t="inlineStr">
         <is>
-          <t>不适用</t>
+          <t>已 push</t>
         </is>
       </c>
     </row>
@@ -5924,6 +5932,102 @@
         </is>
       </c>
       <c r="L86" s="40" t="inlineStr">
+        <is>
+          <t>已 push</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="40" t="inlineStr">
+        <is>
+          <t>D-11</t>
+        </is>
+      </c>
+      <c r="B87" s="40" t="inlineStr">
+        <is>
+          <t>已处理</t>
+        </is>
+      </c>
+      <c r="C87" s="40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D87" s="40" t="inlineStr">
+        <is>
+          <t>工程债</t>
+        </is>
+      </c>
+      <c r="E87" s="40" t="inlineStr">
+        <is>
+          <t>双机 .env 键名 diff</t>
+        </is>
+      </c>
+      <c r="H87" s="83" t="n">
+        <v>46308</v>
+      </c>
+      <c r="I87" s="83" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>6aa334d</t>
+        </is>
+      </c>
+      <c r="K87" s="40" t="inlineStr">
+        <is>
+          <t>双机 .env 键名 diff：见 docs/product/D-11-env-key-diff.md（仅键名）；HY 键名待运维回填；.env.example 已标 D-11 可选键。</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>已 push</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="40" t="inlineStr">
+        <is>
+          <t>D-22</t>
+        </is>
+      </c>
+      <c r="B88" s="40" t="inlineStr">
+        <is>
+          <t>已处理</t>
+        </is>
+      </c>
+      <c r="C88" s="40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D88" s="40" t="inlineStr">
+        <is>
+          <t>工程债</t>
+        </is>
+      </c>
+      <c r="E88" s="40" t="inlineStr">
+        <is>
+          <t>smoke_*.py 入库</t>
+        </is>
+      </c>
+      <c r="H88" s="83" t="n">
+        <v>46308</v>
+      </c>
+      <c r="I88" s="83" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>6aa334d</t>
+        </is>
+      </c>
+      <c r="K88" s="40" t="inlineStr">
+        <is>
+          <t>smoke_*.py 收至 scripts/smoke/（去本机绝对路径）；跑法见 scripts/smoke/README.md；.env.bak 仍不入库；产物 scripts/smoke/_out/ gitignore。</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>
@@ -6170,7 +6274,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="22" customWidth="1" style="40" min="1" max="1"/>
@@ -6364,6 +6468,13 @@
       <c r="B21" s="40" t="inlineStr">
         <is>
           <t>远程 tip 710bce9。人工维护 2026-10-13 BF CST。</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-10-13 X-04关3f9f54b；D-11/D-22关6aa334d；X-02暂缓等视觉；HY键名待运维</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: D-11/D-22 tip bccadb9 + issue table push sync
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -5969,9 +5969,9 @@
       <c r="I87" s="83" t="n">
         <v>46308</v>
       </c>
-      <c r="J87" t="inlineStr">
-        <is>
-          <t>6aa334d</t>
+      <c r="J87" s="40" t="inlineStr">
+        <is>
+          <t>bccadb9</t>
         </is>
       </c>
       <c r="K87" s="40" t="inlineStr">
@@ -5979,7 +5979,7 @@
           <t>双机 .env 键名 diff：见 docs/product/D-11-env-key-diff.md（仅键名）；HY 键名待运维回填；.env.example 已标 D-11 可选键。</t>
         </is>
       </c>
-      <c r="L87" t="inlineStr">
+      <c r="L87" s="40" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>
@@ -6017,9 +6017,9 @@
       <c r="I88" s="83" t="n">
         <v>46308</v>
       </c>
-      <c r="J88" t="inlineStr">
-        <is>
-          <t>6aa334d</t>
+      <c r="J88" s="40" t="inlineStr">
+        <is>
+          <t>bccadb9</t>
         </is>
       </c>
       <c r="K88" s="40" t="inlineStr">
@@ -6027,7 +6027,7 @@
           <t>smoke_*.py 收至 scripts/smoke/（去本机绝对路径）；跑法见 scripts/smoke/README.md；.env.bak 仍不入库；产物 scripts/smoke/_out/ gitignore。</t>
         </is>
       </c>
-      <c r="L88" t="inlineStr">
+      <c r="L88" s="40" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>
@@ -6296,6 +6296,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="41">
       <c r="A4" s="68" t="inlineStr">
         <is>
@@ -6363,6 +6364,7 @@
         <v/>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="15" customHeight="1" s="41">
       <c r="A11" s="72" t="inlineStr">
         <is>
@@ -6374,6 +6376,7 @@
         <v/>
       </c>
     </row>
+    <row r="12"/>
     <row r="13" ht="15" customHeight="1" s="41">
       <c r="A13" s="80" t="inlineStr">
         <is>
@@ -6472,9 +6475,9 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>2026-10-13 X-04关3f9f54b；D-11/D-22关6aa334d；X-02暂缓等视觉；HY键名待运维</t>
+      <c r="A22" s="40" t="inlineStr">
+        <is>
+          <t>2026-10-13 X-04关3f9f54b；D-11/D-22关bccadb9；X-02暂缓等视觉；HY键名待运维</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(x-02): character ref images uploads+path (1-3, 1024)
- character_ref_images table; uploads/char-refs/<id>/; DB path+order only
- sharp center-crop 1024; jpeg/webp (png->jpeg); <=2MB human errors
- profile API list/upload/delete; avatar/cover untouched
- character profile thumbs UI; App.vue 1655 lines
- issue table: D-22 full close; D-11 partial (HY pending)
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -4324,7 +4324,7 @@
       </c>
       <c r="B52" s="40" t="inlineStr">
         <is>
-          <t>暂缓</t>
+          <t>处理中</t>
         </is>
       </c>
       <c r="C52" s="40" t="inlineStr">
@@ -4352,7 +4352,7 @@
       </c>
       <c r="K52" s="40" t="inlineStr">
         <is>
-          <t>暂缓实现；等视觉Bot规格（尺寸/格式/存储位置/与头像·封面关系）→ 用户拍「DB vs uploads+只读」→ 再拆包。</t>
+          <t>开做：1024方/jpeg·webp≤2MB/1～3张/uploads+path；参考图≠头像≠封面。实现 tip 待报。</t>
         </is>
       </c>
       <c r="L52" s="40" t="inlineStr">
@@ -5945,7 +5945,7 @@
       </c>
       <c r="B87" s="40" t="inlineStr">
         <is>
-          <t>已处理</t>
+          <t>部分关单</t>
         </is>
       </c>
       <c r="C87" s="40" t="inlineStr">
@@ -5966,9 +5966,7 @@
       <c r="H87" s="83" t="n">
         <v>46308</v>
       </c>
-      <c r="I87" s="83" t="n">
-        <v>46308</v>
-      </c>
+      <c r="I87" s="83" t="n"/>
       <c r="J87" s="40" t="inlineStr">
         <is>
           <t>bccadb9</t>
@@ -5976,12 +5974,12 @@
       </c>
       <c r="K87" s="40" t="inlineStr">
         <is>
-          <t>双机 .env 键名 diff：见 docs/product/D-11-env-key-diff.md（仅键名）；HY 键名待运维回填；.env.example 已标 D-11 可选键。</t>
+          <t>部分关：BF↔.env.example↔代码键名见 docs/product/D-11-env-key-diff.md（bccadb9）；HY 仍离线，键名待运维上线后补；不能全关。</t>
         </is>
       </c>
       <c r="L87" s="40" t="inlineStr">
         <is>
-          <t>已 push</t>
+          <t>BF已push/HY待补</t>
         </is>
       </c>
     </row>
@@ -6024,7 +6022,7 @@
       </c>
       <c r="K88" s="40" t="inlineStr">
         <is>
-          <t>smoke_*.py 收至 scripts/smoke/（去本机绝对路径）；跑法见 scripts/smoke/README.md；.env.bak 仍不入库；产物 scripts/smoke/_out/ gitignore。</t>
+          <t>全关 tip bccadb9：smoke_*.py 迁入 scripts/smoke/（去绝对路径，README 跑法）；根目录旧脚本已删；.env.bak 仍不入库；产物 scripts/smoke/_out/ gitignore。</t>
         </is>
       </c>
       <c r="L88" s="40" t="inlineStr">
@@ -6274,7 +6272,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="22" customWidth="1" style="40" min="1" max="1"/>
@@ -6296,7 +6294,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="41">
       <c r="A4" s="68" t="inlineStr">
         <is>
@@ -6364,7 +6361,6 @@
         <v/>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="15" customHeight="1" s="41">
       <c r="A11" s="72" t="inlineStr">
         <is>
@@ -6376,7 +6372,6 @@
         <v/>
       </c>
     </row>
-    <row r="12"/>
     <row r="13" ht="15" customHeight="1" s="41">
       <c r="A13" s="80" t="inlineStr">
         <is>
@@ -6478,6 +6473,13 @@
       <c r="A22" s="40" t="inlineStr">
         <is>
           <t>2026-10-13 X-04关3f9f54b；D-11/D-22关bccadb9；X-02暂缓等视觉；HY键名待运维</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-10-13 D-22全关 bccadb9；D-11部分关（HY待补）；X-02开做 uploads+path</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: X-02 tip 6eed178 + issue table; D-11/D-22 notes
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -4324,7 +4324,7 @@
       </c>
       <c r="B52" s="40" t="inlineStr">
         <is>
-          <t>处理中</t>
+          <t>已处理</t>
         </is>
       </c>
       <c r="C52" s="40" t="inlineStr">
@@ -4350,14 +4350,22 @@
       <c r="H52" s="83" t="n">
         <v>46305</v>
       </c>
+      <c r="I52" s="83" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>6eed178</t>
+        </is>
+      </c>
       <c r="K52" s="40" t="inlineStr">
         <is>
-          <t>开做：1024方/jpeg·webp≤2MB/1～3张/uploads+path；参考图≠头像≠封面。实现 tip 待报。</t>
+          <t>已实现 tip 6eed178：uploads/char-refs + DB path；1024方 jpeg/webp≤2MB；1～3张（满则替最旧）；角色页缩略图上传/删；气泡头像仍用 avatar_path。App.vue 1655 行。待云测关单。</t>
         </is>
       </c>
       <c r="L52" s="40" t="inlineStr">
         <is>
-          <t>不适用</t>
+          <t>已 push</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6485,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="40" t="inlineStr">
         <is>
           <t>2026-10-13 D-22全关 bccadb9；D-11部分关（HY待补）；X-02开做 uploads+path</t>
         </is>

</xml_diff>

<commit_message>
docs: D-11 full close — HY env key names (no secrets)
Fill HY section in D-11-env-key-diff.md; mark issue D-11 fully closed.
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -4353,7 +4353,7 @@
       <c r="I52" s="83" t="n">
         <v>46308</v>
       </c>
-      <c r="J52" t="inlineStr">
+      <c r="J52" s="40" t="inlineStr">
         <is>
           <t>6eed178</t>
         </is>
@@ -5953,7 +5953,7 @@
       </c>
       <c r="B87" s="40" t="inlineStr">
         <is>
-          <t>部分关单</t>
+          <t>已处理</t>
         </is>
       </c>
       <c r="C87" s="40" t="inlineStr">
@@ -5974,7 +5974,9 @@
       <c r="H87" s="83" t="n">
         <v>46308</v>
       </c>
-      <c r="I87" s="83" t="n"/>
+      <c r="I87" s="83" t="n">
+        <v>46308</v>
+      </c>
       <c r="J87" s="40" t="inlineStr">
         <is>
           <t>bccadb9</t>
@@ -5982,12 +5984,12 @@
       </c>
       <c r="K87" s="40" t="inlineStr">
         <is>
-          <t>部分关：BF↔.env.example↔代码键名见 docs/product/D-11-env-key-diff.md（bccadb9）；HY 仍离线，键名待运维上线后补；不能全关。</t>
+          <t>全关：BF+HY 键名均已写入 docs/product/D-11-env-key-diff.md（无密钥）；差异见文内 BF vs HY 表（HOST 仅 BF；OLLAMA_MODELS/LAYA_*/DeepSeek·Gemini·Google 占位仅 HY）。</t>
         </is>
       </c>
       <c r="L87" s="40" t="inlineStr">
         <is>
-          <t>BF已push/HY待补</t>
+          <t>已 push</t>
         </is>
       </c>
     </row>
@@ -6280,7 +6282,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="22" customWidth="1" style="40" min="1" max="1"/>
@@ -6488,6 +6490,13 @@
       <c r="A23" s="40" t="inlineStr">
         <is>
           <t>2026-10-13 D-22全关 bccadb9；D-11部分关（HY待补）；X-02开做 uploads+path</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-10-13 D-11 全关（HY 键名已补）</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: D-11 tip sync
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -5979,7 +5979,7 @@
       </c>
       <c r="J87" s="40" t="inlineStr">
         <is>
-          <t>bccadb9</t>
+          <t>0a153f5</t>
         </is>
       </c>
       <c r="K87" s="40" t="inlineStr">
@@ -6494,7 +6494,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="40" t="inlineStr">
         <is>
           <t>2026-10-13 D-11 全关（HY 键名已补）</t>
         </is>

</xml_diff>

<commit_message>
docs: EOD 2026-10-13 table sync — App.vue trend, X-06 UI-4 close
X-04 App.vue=1620; X-02/X-06/X-07/D-11/D-22 closed notes; params TBD;
next eval M-05b.
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -4249,7 +4249,7 @@
       </c>
       <c r="K50" s="40" t="inlineStr">
         <is>
-          <t>触发：M-05a 稳且要生图配图。</t>
+          <t>触发：M-05a 稳且要生图配图。；下一优先评估（X-07 已关后）；N-02/Gemini/X05-D3·D4·D6 不动。</t>
         </is>
       </c>
       <c r="L50" s="40" t="inlineStr">
@@ -4360,7 +4360,7 @@
       </c>
       <c r="K52" s="40" t="inlineStr">
         <is>
-          <t>已实现 tip 6eed178：uploads/char-refs + DB path；1024方 jpeg/webp≤2MB；1～3张（满则替最旧）；角色页缩略图上传/删；气泡头像仍用 avatar_path。App.vue 1655 行。待云测关单。</t>
+          <t>已关 tip 6eed178（云测+产品验收通过）：uploads+path、1～3 张、超限人话拒、头像/封面/气泡未动。App.vue=1655 行。</t>
         </is>
       </c>
       <c r="L52" s="40" t="inlineStr">
@@ -4471,7 +4471,7 @@
       </c>
       <c r="K54" s="40" t="inlineStr">
         <is>
-          <t>实现已关 tip 3f9f54b；产品参数「2静1开」「TTL 7天」「静默默认 23:00–08:00」均待明确（当前硬编码可跑，改数另开刀）。云测通过。</t>
+          <t>已关 tip 3f9f54b；X-04 后 App.vue=1620 行。产品参数「2静1开」「TTL 7天」「静默默认 23:00–08:00」均待明确（硬编码可跑，改数另开刀）。</t>
         </is>
       </c>
       <c r="L54" s="40" t="inlineStr">
@@ -4576,21 +4576,21 @@
         <v>46305</v>
       </c>
       <c r="I56" s="88" t="n">
-        <v>46306</v>
+        <v>46308</v>
       </c>
       <c r="J56" s="40" t="inlineStr">
         <is>
-          <t>838d3eb</t>
+          <t>c0b46e1</t>
         </is>
       </c>
       <c r="K56" s="40" t="inlineStr">
         <is>
-          <t>真进度接 audio.currentTime；seek 拖拽仍不在范围</t>
+          <t>随 UI-4 收口：tip c0b46e1（语音气泡 play/pause/loading + 进度）；后续 X-06 useTtsPlayback 真进度 tip 838d3eb 已在主线。</t>
         </is>
       </c>
       <c r="L56" s="40" t="inlineStr">
         <is>
-          <t>remote tip ba907c3</t>
+          <t>已 push</t>
         </is>
       </c>
     </row>
@@ -4638,12 +4638,12 @@
       </c>
       <c r="J57" s="40" t="inlineStr">
         <is>
-          <t>710bce9</t>
+          <t>eb0bb54</t>
         </is>
       </c>
       <c r="K57" s="40" t="inlineStr">
         <is>
-          <t>先定可调项再拆包 → 本刀已定最小集并对齐设计备忘「0～2 赞 / 0～1 评」。未开：X-02/X-04、N-02、Gemini、X05-D3/D4、D6、D-11/D-22。</t>
+          <t>先定可调项再拆包 → 本刀已定最小集并对齐设计备忘「0～2 赞 / 0～1 评」。未开：X-02/X-04、N-02、Gemini、X05-D3/D4、D6、D-11/D-22。；已关 tip eb0bb54（feat 710bce9）；空间赞/评上限可调，不碰 daily_cap/总开关。</t>
         </is>
       </c>
       <c r="L57" s="40" t="inlineStr">
@@ -5497,7 +5497,7 @@
       </c>
       <c r="K78" s="40" t="inlineStr">
         <is>
-          <t>2026-10-11 拍板关单：D-02 P0（useAppShell+useChatSession, 8606bbb）/P1（useProfileAppearance+useContactsImport, d6a00c5）/P2（useMemoryUi+useVoiceInput, bdca268）全部关单。App.vue 约 2446→1629（约−817）。状态部分已收；剩壳模板/胶水/status/展示辅助/emoji。拆出独立债 D-02b（壳层/辅助清理），不再继续抽 App.vue。 与状态债分离：壳层/辅助见 D-02b。 2026-10-13：D-02b 已处理（辅助清理）；D-02 仍部分收口。 2026-10-13 计分行（含 D-02b）：App.vue **2446 → 1527（−919 行）**。D-02 仍部分收口；D-02b 已关。 2026-10-13 计分行续：App.vue **2446 → 1527（D-02b）→ 1554（X05-D2+D5）**。D2+D5 +27=资料页丢弃模板+胶水；pending 状态在 useMemoryUi，非 App 新业务 ref。</t>
+          <t>2026-10-11 拍板关单：D-02 P0（useAppShell+useChatSession, 8606bbb）/P1（useProfileAppearance+useContactsImport, d6a00c5）/P2（useMemoryUi+useVoiceInput, bdca268）全部关单。App.vue 约 2446→1629（约−817）。状态部分已收；剩壳模板/胶水/status/展示辅助/emoji。拆出独立债 D-02b（壳层/辅助清理），不再继续抽 App.vue。 与状态债分离：壳层/辅助见 D-02b。 2026-10-13：D-02b 已处理（辅助清理）；D-02 仍部分收口。 2026-10-13 计分行（含 D-02b）：App.vue **2446 → 1527（−919 行）**。D-02 仍部分收口；D-02b 已关。 2026-10-13 计分行续：App.vue **2446 → 1527（D-02b）→ 1554（X05-D2+D5）**。D2+D5 +27=资料页丢弃模板+胶水；pending 状态在 useMemoryUi，非 App 新业务 ref。；App.vue 趋势：2446→1527（D-02b）→1554（D2+D5）→1590（X-03）→1620（X-04）→1655（X-02）；1527 后为功能 UI 模板抬回，非 D-02 回涨。现 tip App.vue=1655。</t>
         </is>
       </c>
       <c r="L78" s="40" t="inlineStr">
@@ -5555,7 +5555,7 @@
       </c>
       <c r="K79" s="40" t="inlineStr">
         <is>
-          <t>来源 D-02 拆出。2026-10-13 BF 关单（辅助/status/emoji）。壳模板面板拆分不纳入本刀。N-02/Gemini/X05-D2～D6 不动。 计入 D-02 累计计分行：App.vue 2446→1527（−919）。 后续 X05-D2+D5 抬至 1554（模板，非状态债回流）。</t>
+          <t>App.vue 趋势：2446→1527（D-02b）→1554（D2+D5）→1590（X-03）→1620（X-04）→1655（X-02）；1527 后为功能 UI 模板抬回，非 D-02 回涨。现 tip App.vue=1655。</t>
         </is>
       </c>
       <c r="L79" s="40" t="inlineStr">
@@ -5984,7 +5984,7 @@
       </c>
       <c r="K87" s="40" t="inlineStr">
         <is>
-          <t>全关：BF+HY 键名均已写入 docs/product/D-11-env-key-diff.md（无密钥）；差异见文内 BF vs HY 表（HOST 仅 BF；OLLAMA_MODELS/LAYA_*/DeepSeek·Gemini·Google 占位仅 HY）。</t>
+          <t>全关 tip 0a153f5（表同步 3d18db9）：BF+HY 键名均入 D-11-env-key-diff.md，无密钥明文。</t>
         </is>
       </c>
       <c r="L87" s="40" t="inlineStr">
@@ -6032,7 +6032,7 @@
       </c>
       <c r="K88" s="40" t="inlineStr">
         <is>
-          <t>全关 tip bccadb9：smoke_*.py 迁入 scripts/smoke/（去绝对路径，README 跑法）；根目录旧脚本已删；.env.bak 仍不入库；产物 scripts/smoke/_out/ gitignore。</t>
+          <t>全关 tip bccadb9：smoke_*.py → scripts/smoke/；.env.bak 不入库。</t>
         </is>
       </c>
       <c r="L88" s="40" t="inlineStr">
@@ -6282,7 +6282,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="22" customWidth="1" style="40" min="1" max="1"/>
@@ -6497,6 +6497,13 @@
       <c r="A24" s="40" t="inlineStr">
         <is>
           <t>2026-10-13 D-11 全关（HY 键名已补）</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-10-13 EOD：tip 3d18db9 ahead0；X-02/6eed178 X-04/3f9f54b(App1620) X-06/c0b46e1 X-07/eb0bb54 D-11/0a153f5 D-22/bccadb9 均已关；App.vue 2446→1527→1554→1590→1620(X-04)→1655(X-02)；参数待明确 TTL7d/静默23-08/2静1开；下一评 M-05b</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: M-05b tip 78d4e38
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -2396,7 +2396,7 @@
       </c>
       <c r="H17" s="44" t="inlineStr">
         <is>
-          <t>2332424</t>
+          <t>78d4e38</t>
         </is>
       </c>
       <c r="I17" s="82" t="n">
@@ -2738,7 +2738,7 @@
       </c>
       <c r="H23" s="44" t="inlineStr">
         <is>
-          <t>2332424</t>
+          <t>78d4e38</t>
         </is>
       </c>
       <c r="I23" s="82" t="n">
@@ -3863,7 +3863,7 @@
       </c>
       <c r="H43" s="62" t="inlineStr">
         <is>
-          <t>2332424</t>
+          <t>78d4e38</t>
         </is>
       </c>
       <c r="I43" s="65" t="n">
@@ -3881,7 +3881,7 @@
       </c>
       <c r="L43" s="40" t="inlineStr">
         <is>
-          <t>2332424</t>
+          <t>78d4e38</t>
         </is>
       </c>
     </row>
@@ -4252,9 +4252,9 @@
       <c r="I50" s="83" t="n">
         <v>46309</v>
       </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>(push tip)</t>
+      <c r="J50" s="40" t="inlineStr">
+        <is>
+          <t>78d4e38</t>
         </is>
       </c>
       <c r="K50" s="40" t="inlineStr">
@@ -4322,7 +4322,7 @@
       </c>
       <c r="L51" s="40" t="inlineStr">
         <is>
-          <t>2332424</t>
+          <t>78d4e38</t>
         </is>
       </c>
     </row>
@@ -4716,7 +4716,7 @@
       </c>
       <c r="L58" s="40" t="inlineStr">
         <is>
-          <t>2332424</t>
+          <t>78d4e38</t>
         </is>
       </c>
     </row>
@@ -6191,7 +6191,7 @@
       </c>
       <c r="B9" s="70" t="inlineStr">
         <is>
-          <t>2332424</t>
+          <t>78d4e38</t>
         </is>
       </c>
     </row>
@@ -6489,7 +6489,7 @@
       </c>
       <c r="B21" s="40" t="inlineStr">
         <is>
-          <t>2332424</t>
+          <t>78d4e38</t>
         </is>
       </c>
     </row>
@@ -6525,6 +6525,11 @@
       <c r="A26" s="40" t="inlineStr">
         <is>
           <t>2026-10-13 补记：远程 tip（人工）=2332424；待明确：TTL 7天、静默 23:00–08:00、X-07 赞/评上限（及表上已有的 2静1开）；下一候选 M-05b；N-02/Gemini/X05 残债不动。</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>78d4e38</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(B-04c): widen image-gen trigger for 画一只猫
Expand wantsImageGeneration / buildImagePrompt classifiers (只/条/匹…).
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -3073,7 +3073,7 @@
       </c>
       <c r="B30" s="52" t="inlineStr">
         <is>
-          <t>暂缓</t>
+          <t>已处理</t>
         </is>
       </c>
       <c r="C30" s="44" t="inlineStr">
@@ -3115,7 +3115,7 @@
       </c>
       <c r="L30" s="40" t="inlineStr">
         <is>
-          <t>不适用</t>
+          <t>已 push</t>
         </is>
       </c>
     </row>
@@ -4844,7 +4844,7 @@
       </c>
       <c r="B61" s="40" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>已处理</t>
         </is>
       </c>
       <c r="C61" s="40" t="inlineStr">
@@ -4870,14 +4870,22 @@
       <c r="H61" s="83" t="n">
         <v>46305</v>
       </c>
+      <c r="I61" s="83" t="n">
+        <v>46309</v>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>(push tip)</t>
+        </is>
+      </c>
       <c r="K61" s="40" t="inlineStr">
         <is>
-          <t>2026-10-10 一期冒烟记入二期池。</t>
+          <t>已关：wantsImageGeneration 加宽量词（只/条/匹等）与画只/画条；裸「画一只猫」可触发；闲聊不误触；失败仍 B-04d 人话。拟改 apps/server/src/services/imageGen.ts。</t>
         </is>
       </c>
       <c r="L61" s="40" t="inlineStr">
         <is>
-          <t>不适用</t>
+          <t>已 push</t>
         </is>
       </c>
     </row>
@@ -6122,7 +6130,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="41">
       <c r="A4" s="68" t="inlineStr">
         <is>
@@ -6315,7 +6322,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="41">
       <c r="A4" s="68" t="inlineStr">
         <is>
@@ -6383,7 +6389,6 @@
         <v/>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="15" customHeight="1" s="41">
       <c r="A11" s="72" t="inlineStr">
         <is>
@@ -6395,7 +6400,6 @@
         <v/>
       </c>
     </row>
-    <row r="12"/>
     <row r="13" ht="15" customHeight="1" s="41">
       <c r="A13" s="80" t="inlineStr">
         <is>
@@ -6527,7 +6531,7 @@
           <t>2026-10-13 补记：远程 tip（人工）=2332424；待明确：TTL 7天、静默 23:00–08:00、X-07 赞/评上限（及表上已有的 2静1开）；下一候选 M-05b；N-02/Gemini/X05 残债不动。</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="40" t="inlineStr">
         <is>
           <t>78d4e38</t>
         </is>

</xml_diff>

<commit_message>
docs: B-04c tip b1ad348
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -2396,7 +2396,7 @@
       </c>
       <c r="H17" s="44" t="inlineStr">
         <is>
-          <t>78d4e38</t>
+          <t>b1ad348</t>
         </is>
       </c>
       <c r="I17" s="82" t="n">
@@ -2738,7 +2738,7 @@
       </c>
       <c r="H23" s="44" t="inlineStr">
         <is>
-          <t>78d4e38</t>
+          <t>b1ad348</t>
         </is>
       </c>
       <c r="I23" s="82" t="n">
@@ -3863,7 +3863,7 @@
       </c>
       <c r="H43" s="62" t="inlineStr">
         <is>
-          <t>78d4e38</t>
+          <t>b1ad348</t>
         </is>
       </c>
       <c r="I43" s="65" t="n">
@@ -3881,7 +3881,7 @@
       </c>
       <c r="L43" s="40" t="inlineStr">
         <is>
-          <t>78d4e38</t>
+          <t>b1ad348</t>
         </is>
       </c>
     </row>
@@ -4322,7 +4322,7 @@
       </c>
       <c r="L51" s="40" t="inlineStr">
         <is>
-          <t>78d4e38</t>
+          <t>b1ad348</t>
         </is>
       </c>
     </row>
@@ -4716,7 +4716,7 @@
       </c>
       <c r="L58" s="40" t="inlineStr">
         <is>
-          <t>78d4e38</t>
+          <t>b1ad348</t>
         </is>
       </c>
     </row>
@@ -4873,9 +4873,9 @@
       <c r="I61" s="83" t="n">
         <v>46309</v>
       </c>
-      <c r="J61" t="inlineStr">
-        <is>
-          <t>(push tip)</t>
+      <c r="J61" s="40" t="inlineStr">
+        <is>
+          <t>b1ad348</t>
         </is>
       </c>
       <c r="K61" s="40" t="inlineStr">
@@ -6130,6 +6130,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="41">
       <c r="A4" s="68" t="inlineStr">
         <is>
@@ -6198,7 +6199,7 @@
       </c>
       <c r="B9" s="70" t="inlineStr">
         <is>
-          <t>78d4e38</t>
+          <t>b1ad348</t>
         </is>
       </c>
     </row>
@@ -6322,6 +6323,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="41">
       <c r="A4" s="68" t="inlineStr">
         <is>
@@ -6389,6 +6391,7 @@
         <v/>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="15" customHeight="1" s="41">
       <c r="A11" s="72" t="inlineStr">
         <is>
@@ -6400,6 +6403,7 @@
         <v/>
       </c>
     </row>
+    <row r="12"/>
     <row r="13" ht="15" customHeight="1" s="41">
       <c r="A13" s="80" t="inlineStr">
         <is>
@@ -6493,7 +6497,7 @@
       </c>
       <c r="B21" s="40" t="inlineStr">
         <is>
-          <t>78d4e38</t>
+          <t>b1ad348</t>
         </is>
       </c>
     </row>
@@ -6533,7 +6537,7 @@
       </c>
       <c r="B26" s="40" t="inlineStr">
         <is>
-          <t>78d4e38</t>
+          <t>b1ad348</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: 参数三条已定 — TTL7 / 静默23-08 / X-07赞2评1+2静1开
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -4428,7 +4428,7 @@
       </c>
       <c r="K53" s="40" t="inlineStr">
         <is>
-          <t>二期可选。 2026-10-13 关单。与 C-06/D-04 同组主动线；N-02/Gemini/X05-D3～D6 不动。 App.vue 仅模板+接线，逻辑在 useProactiveSettings。</t>
+          <t>二期可选。 2026-10-13 关单。与 C-06/D-04 同组主动线；N-02/Gemini/X05-D3～D6 不动。 App.vue 仅模板+接线，逻辑在 useProactiveSettings。；参数已定（2026-10-14）：MEMORY_PENDING_TTL_DAYS=7；静默 23:00–08:00；X-07 赞2/评1；群聊「2静1开」一并已定。已从表摘「待明确」。</t>
         </is>
       </c>
       <c r="L53" s="40" t="inlineStr">
@@ -4481,7 +4481,7 @@
       </c>
       <c r="K54" s="40" t="inlineStr">
         <is>
-          <t>已关 tip 3f9f54b；X-04 后 App.vue=1620 行。产品参数待用户明确：TTL 7 天、静默 23:00–08:00、2 静 1 开（硬编码可跑，改数另开刀）。</t>
+          <t>已关 tip 3f9f54b；X-04 后 App.vue=1620 行。产品参数已定：TTL 7 天、静默 23:00–08:00、2 静 1 开（硬编码可跑，改数另开刀）。；参数已定（2026-10-14）：MEMORY_PENDING_TTL_DAYS=7；静默 23:00–08:00；X-07 赞2/评1；群聊「2静1开」一并已定。已从表摘「待明确」。</t>
         </is>
       </c>
       <c r="L54" s="40" t="inlineStr">
@@ -4653,7 +4653,7 @@
       </c>
       <c r="K57" s="40" t="inlineStr">
         <is>
-          <t>功能已关 tip eb0bb54（feat 710bce9）；空间赞/评上限可调，不碰 daily_cap/总开关。参数待用户明确：赞/评上限数值（与 TTL/静默同挂）。</t>
+          <t>功能已关 tip eb0bb54（feat 710bce9）；空间赞/评上限可调，不碰 daily_cap/总开关。参数已定：赞/评上限数值（与 TTL/静默同挂）。；参数已定（2026-10-14）：MEMORY_PENDING_TTL_DAYS=7；静默 23:00–08:00；X-07 赞2/评1；群聊「2静1开」一并已定。已从表摘「待明确」。</t>
         </is>
       </c>
       <c r="L57" s="40" t="inlineStr">
@@ -5684,7 +5684,7 @@
       </c>
       <c r="K81" s="40" t="inlineStr">
         <is>
-          <t>来源 X-05。与 D5 同刀。D3/D4 延期；D6 维持 off。 TTL=7d 为 **agent 默认**（文档示例），**产品参数待用户明确**。</t>
+          <t>来源 X-05。与 D5 同刀。D3/D4 延期；D6 维持 off。 TTL=7d 为 **agent 默认**（文档示例），**产品参数已定**。</t>
         </is>
       </c>
       <c r="L81" s="40" t="inlineStr">
@@ -5954,7 +5954,7 @@
       </c>
       <c r="K86" s="40" t="inlineStr">
         <is>
-          <t>来源 ARCH-1 功能池 / C-06 遗留。N-02/Gemini/X05-D3～D6 不动。 备注：TTL 7d、静默 23:00–08:00 产品参数待明确；D-11 双机 .env、D-22 smoke_*.py 仍在 ARCH-1 池。</t>
+          <t>来源 ARCH-1 功能池 / C-06 遗留。N-02/Gemini/X05-D3～D6 不动。 备注：TTL 7d、静默 23:00–08:00 产品参数已定；D-11 双机 .env、D-22 smoke_*.py 仍在 ARCH-1 池。</t>
         </is>
       </c>
       <c r="L86" s="40" t="inlineStr">
@@ -6130,7 +6130,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="41">
       <c r="A4" s="68" t="inlineStr">
         <is>
@@ -6301,7 +6300,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="22" customWidth="1" style="40" min="1" max="1"/>
@@ -6323,7 +6322,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="41">
       <c r="A4" s="68" t="inlineStr">
         <is>
@@ -6391,7 +6389,6 @@
         <v/>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="15" customHeight="1" s="41">
       <c r="A11" s="72" t="inlineStr">
         <is>
@@ -6403,7 +6400,6 @@
         <v/>
       </c>
     </row>
-    <row r="12"/>
     <row r="13" ht="15" customHeight="1" s="41">
       <c r="A13" s="80" t="inlineStr">
         <is>
@@ -6538,6 +6534,13 @@
       <c r="B26" s="40" t="inlineStr">
         <is>
           <t>b1ad348</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-10-14 参数三条已定：TTL=7；静默23:00–08:00；X-07赞2评1 + 2静1开。docs-only，无功能刀。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: 第0步 — B-04c关、B-04d待实打、D-03/App.vue基线、EOD-10-14
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -4875,12 +4875,12 @@
       </c>
       <c r="J61" s="40" t="inlineStr">
         <is>
-          <t>b1ad348</t>
+          <t>af133b9</t>
         </is>
       </c>
       <c r="K61" s="40" t="inlineStr">
         <is>
-          <t>已关：wantsImageGeneration 加宽量词（只/条/匹等）与画只/画条；裸「画一只猫」可触发；闲聊不误触；失败仍 B-04d 人话。拟改 apps/server/src/services/imageGen.ts。</t>
+          <t>已关 tip af133b9（feat b1ad348）：wantsImageGeneration 加宽量词（只/条/匹等）；裸「画一只猫」可触发；闲聊不误触；云测过。失败仍 B-04d 人话路径。</t>
         </is>
       </c>
       <c r="L61" s="40" t="inlineStr">
@@ -4897,7 +4897,7 @@
       </c>
       <c r="B62" s="40" t="inlineStr">
         <is>
-          <t>已处理</t>
+          <t>待实打</t>
         </is>
       </c>
       <c r="C62" s="40" t="inlineStr">
@@ -4938,12 +4938,12 @@
       </c>
       <c r="K62" s="40" t="inlineStr">
         <is>
-          <t>挂 API/密钥试跑时顺带验。 2026-10-10：读图 VLM 债/B-04d 在 ARCH-2 试跑线里还（非独立刀）。 2026-10-10 试跑线观测：坏 IMAGE_GEN Key → 上游 HTTP 401 Token is invalid；产品侧失败回流人话路径未改代码实打，仍暂缓。 2026-10-11 收尾：Gemini TTS + 官方 VLM 仍挂债等 Key；排在 X05-D1 / D-02b 之后。 2026-10-13：DeepSeek 官方文本+识图已通，不再算试跑挂债；本条续挂 **Gemini TTS 等 Key** + 生图失败人话路径。 2026-10-13：B-04d 关单（验证失败路径+开发去 JSON）。Gemini TTS 仍等 Key，不在本条。 N-02 不动。生图 Key=IMAGE_GEN_*（硅基），非 DeepSeek 文本键。</t>
+          <t>挂 API/密钥试跑时顺带验。 2026-10-10：读图 VLM 债/B-04d 在 ARCH-2 试跑线里还（非独立刀）。 2026-10-10 试跑线观测：坏 IMAGE_GEN Key → 上游 HTTP 401 Token is invalid；产品侧失败回流人话路径未改代码实打，仍暂缓。 2026-10-11 收尾：Gemini TTS + 官方 VLM 仍挂债等 Key；排在 X05-D1 / D-02b 之后。 2026-10-13：DeepSeek 官方文本+识图已通，不再算试跑挂债；本条续挂 **Gemini TTS 等 Key** + 生图失败人话路径。 2026-10-13：B-04d 关单（验证失败路径+开发去 JSON）。Gemini TTS 仍等 Key，不在本条。 N-02 不动。生图 Key=IMAGE_GEN_*（硅基），非 DeepSeek 文本键。；2026-10-14：状态改为「待实打」——代码已合 tip 6263381（formatImageGenUserError 人话），非未做；待云侧坏 Key 实打验收（验完须恢复 .env）。</t>
         </is>
       </c>
       <c r="L62" s="40" t="inlineStr">
         <is>
-          <t>已 push（tip 6263381）</t>
+          <t>代码已合；待实打</t>
         </is>
       </c>
     </row>
@@ -5515,7 +5515,7 @@
       </c>
       <c r="K78" s="40" t="inlineStr">
         <is>
-          <t>2026-10-11 拍板关单：D-02 P0（useAppShell+useChatSession, 8606bbb）/P1（useProfileAppearance+useContactsImport, d6a00c5）/P2（useMemoryUi+useVoiceInput, bdca268）全部关单。App.vue 约 2446→1629（约−817）。状态部分已收；剩壳模板/胶水/status/展示辅助/emoji。拆出独立债 D-02b（壳层/辅助清理），不再继续抽 App.vue。 与状态债分离：壳层/辅助见 D-02b。 2026-10-13：D-02b 已处理（辅助清理）；D-02 仍部分收口。 2026-10-13 计分行（含 D-02b）：App.vue **2446 → 1527（−919 行）**。D-02 仍部分收口；D-02b 已关。 2026-10-13 计分行续：App.vue **2446 → 1527（D-02b）→ 1554（X05-D2+D5）**。D2+D5 +27=资料页丢弃模板+胶水；pending 状态在 useMemoryUi，非 App 新业务 ref。；App.vue 趋势：2446→1527（D-02b）→1554（D2+D5）→1590（X-03）→1620（X-04）→1655（X-02）；1527 后为功能 UI 模板抬回，非 D-02 回涨。现 tip App.vue=1655。</t>
+          <t>App.vue 趋势：2446→1527（D-02b）→1554（D2+D5）→1590（X-03）→1620（X-04）→1655（X-02）→1683（M-05b +28）；1527 后为功能 UI 模板抬回，非 D-02 回涨。现 tip App.vue=1683。</t>
         </is>
       </c>
       <c r="L78" s="40" t="inlineStr">
@@ -6130,6 +6130,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="41">
       <c r="A4" s="68" t="inlineStr">
         <is>
@@ -6300,7 +6301,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="22" customWidth="1" style="40" min="1" max="1"/>
@@ -6322,6 +6323,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="41">
       <c r="A4" s="68" t="inlineStr">
         <is>
@@ -6389,6 +6391,7 @@
         <v/>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="15" customHeight="1" s="41">
       <c r="A11" s="72" t="inlineStr">
         <is>
@@ -6400,6 +6403,7 @@
         <v/>
       </c>
     </row>
+    <row r="12"/>
     <row r="13" ht="15" customHeight="1" s="41">
       <c r="A13" s="80" t="inlineStr">
         <is>
@@ -6538,9 +6542,16 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="40" t="inlineStr">
         <is>
           <t>2026-10-14 参数三条已定：TTL=7；静默23:00–08:00；X-07赞2评1 + 2静1开。docs-only，无功能刀。</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-10-14 第0步：B-04c 关 af133b9；B-04d→待实打(6263381)；D-03 基线 864→1034；App.vue 1655→1683（M-05b+28）；见 EOD-2026-10-14.md</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(product): introduce W-series (world presence) design memo and re-scope proactive boundaries
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -1389,7 +1389,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L88"/>
+  <dimension ref="A1:L96"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="40" min="1" max="1"/>
@@ -6056,6 +6056,422 @@
       <c r="L88" s="40" t="inlineStr">
         <is>
           <t>已 push</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="86" t="inlineStr">
+        <is>
+          <t>W-01</t>
+        </is>
+      </c>
+      <c r="B89" s="86" t="inlineStr">
+        <is>
+          <t>暂缓</t>
+        </is>
+      </c>
+      <c r="C89" s="86" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D89" s="86" t="inlineStr">
+        <is>
+          <t>世界感</t>
+        </is>
+      </c>
+      <c r="E89" s="86" t="inlineStr">
+        <is>
+          <t>此刻上下文注入（时间+地点）</t>
+        </is>
+      </c>
+      <c r="F89" s="86" t="inlineStr">
+        <is>
+          <t>最小闭环：一行此刻上下文进 system prompt。</t>
+        </is>
+      </c>
+      <c r="G89" s="86" t="inlineStr">
+        <is>
+          <t>待排期；前置 D-25。见《真实世界感设计备忘》。</t>
+        </is>
+      </c>
+      <c r="H89" s="87" t="n">
+        <v>46310</v>
+      </c>
+      <c r="I89" s="86" t="n"/>
+      <c r="J89" s="86" t="n"/>
+      <c r="K89" s="86" t="inlineStr">
+        <is>
+          <t>二期新增；待用户排期；不插队下一刀</t>
+        </is>
+      </c>
+      <c r="L89" s="86" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="86" t="inlineStr">
+        <is>
+          <t>W-02</t>
+        </is>
+      </c>
+      <c r="B90" s="86" t="inlineStr">
+        <is>
+          <t>暂缓</t>
+        </is>
+      </c>
+      <c r="C90" s="86" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D90" s="86" t="inlineStr">
+        <is>
+          <t>世界感</t>
+        </is>
+      </c>
+      <c r="E90" s="86" t="inlineStr">
+        <is>
+          <t>角色 presence 惰性求值</t>
+        </is>
+      </c>
+      <c r="F90" s="86" t="inlineStr">
+        <is>
+          <t>位置状态机 + resolvePresence(now)；不跑全日定时器。</t>
+        </is>
+      </c>
+      <c r="G90" s="86" t="inlineStr">
+        <is>
+          <t>依赖 W-01。见备忘。</t>
+        </is>
+      </c>
+      <c r="H90" s="87" t="n">
+        <v>46310</v>
+      </c>
+      <c r="I90" s="86" t="n"/>
+      <c r="J90" s="86" t="n"/>
+      <c r="K90" s="86" t="inlineStr">
+        <is>
+          <t>二期新增；待用户排期</t>
+        </is>
+      </c>
+      <c r="L90" s="86" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="86" t="inlineStr">
+        <is>
+          <t>W-03</t>
+        </is>
+      </c>
+      <c r="B91" s="86" t="inlineStr">
+        <is>
+          <t>暂缓</t>
+        </is>
+      </c>
+      <c r="C91" s="86" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D91" s="86" t="inlineStr">
+        <is>
+          <t>世界感</t>
+        </is>
+      </c>
+      <c r="E91" s="86" t="inlineStr">
+        <is>
+          <t>生活事件流水 life_events</t>
+        </is>
+      </c>
+      <c r="F91" s="86" t="inlineStr">
+        <is>
+          <t>tick 推进世界状态并落流水；可召回。</t>
+        </is>
+      </c>
+      <c r="G91" s="86" t="inlineStr">
+        <is>
+          <t>依赖 W-02；推进分支不得调 LLM。跨重启依赖 D-15。</t>
+        </is>
+      </c>
+      <c r="H91" s="87" t="n">
+        <v>46310</v>
+      </c>
+      <c r="I91" s="86" t="n"/>
+      <c r="J91" s="86" t="n"/>
+      <c r="K91" s="86" t="inlineStr">
+        <is>
+          <t>二期新增；待用户排期</t>
+        </is>
+      </c>
+      <c r="L91" s="86" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="86" t="inlineStr">
+        <is>
+          <t>W-04</t>
+        </is>
+      </c>
+      <c r="B92" s="86" t="inlineStr">
+        <is>
+          <t>暂缓</t>
+        </is>
+      </c>
+      <c r="C92" s="86" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D92" s="86" t="inlineStr">
+        <is>
+          <t>世界感</t>
+        </is>
+      </c>
+      <c r="E92" s="86" t="inlineStr">
+        <is>
+          <t>跨重启流逝补偿</t>
+        </is>
+      </c>
+      <c r="F92" s="86" t="inlineStr">
+        <is>
+          <t>停机期间流逝按策略补算或作废。</t>
+        </is>
+      </c>
+      <c r="G92" s="86" t="inlineStr">
+        <is>
+          <t>打磨项；依赖 W-02/W-03 与 D-15。</t>
+        </is>
+      </c>
+      <c r="H92" s="87" t="n">
+        <v>46310</v>
+      </c>
+      <c r="I92" s="86" t="n"/>
+      <c r="J92" s="86" t="n"/>
+      <c r="K92" s="86" t="inlineStr">
+        <is>
+          <t>二期新增；不进最小闭环</t>
+        </is>
+      </c>
+      <c r="L92" s="86" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="86" t="inlineStr">
+        <is>
+          <t>W-05</t>
+        </is>
+      </c>
+      <c r="B93" s="86" t="inlineStr">
+        <is>
+          <t>暂缓</t>
+        </is>
+      </c>
+      <c r="C93" s="86" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D93" s="86" t="inlineStr">
+        <is>
+          <t>世界感</t>
+        </is>
+      </c>
+      <c r="E93" s="86" t="inlineStr">
+        <is>
+          <t>地图编辑器 / 全日作息引擎</t>
+        </is>
+      </c>
+      <c r="F93" s="86" t="inlineStr">
+        <is>
+          <t>nyairo 最重块；模拟经营向。**明确不做**。</t>
+        </is>
+      </c>
+      <c r="G93" s="86" t="inlineStr">
+        <is>
+          <t>明确不做。≠ W-03 生活痕迹。</t>
+        </is>
+      </c>
+      <c r="H93" s="87" t="n">
+        <v>46310</v>
+      </c>
+      <c r="I93" s="86" t="n"/>
+      <c r="J93" s="86" t="n"/>
+      <c r="K93" s="86" t="inlineStr">
+        <is>
+          <t>二期新增；产品已定明确不做（表无「不做」先例故暂缓+备注）</t>
+        </is>
+      </c>
+      <c r="L93" s="86" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="86" t="inlineStr">
+        <is>
+          <t>R-07</t>
+        </is>
+      </c>
+      <c r="B94" s="86" t="inlineStr">
+        <is>
+          <t>暂缓</t>
+        </is>
+      </c>
+      <c r="C94" s="86" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D94" s="86" t="inlineStr">
+        <is>
+          <t>角色</t>
+        </is>
+      </c>
+      <c r="E94" s="86" t="inlineStr">
+        <is>
+          <t>纠正后的历史复述污染</t>
+        </is>
+      </c>
+      <c r="F94" s="86" t="inlineStr">
+        <is>
+          <t>supersede 管行；messages 窗口仍可能复述旧事实。</t>
+        </is>
+      </c>
+      <c r="G94" s="86" t="inlineStr">
+        <is>
+          <t>记债不拆包；X-05 续债。见记忆备忘。</t>
+        </is>
+      </c>
+      <c r="H94" s="87" t="n">
+        <v>46310</v>
+      </c>
+      <c r="I94" s="86" t="n"/>
+      <c r="J94" s="86" t="n"/>
+      <c r="K94" s="86" t="inlineStr">
+        <is>
+          <t>二期新增；X-05 续债链</t>
+        </is>
+      </c>
+      <c r="L94" s="86" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="86" t="inlineStr">
+        <is>
+          <t>D-25</t>
+        </is>
+      </c>
+      <c r="B95" s="86" t="inlineStr">
+        <is>
+          <t>暂缓</t>
+        </is>
+      </c>
+      <c r="C95" s="86" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="D95" s="86" t="inlineStr">
+        <is>
+          <t>工程债</t>
+        </is>
+      </c>
+      <c r="E95" s="86" t="inlineStr">
+        <is>
+          <t>无 token 预算 / 注入硬截</t>
+        </is>
+      </c>
+      <c r="F95" s="86" t="inlineStr">
+        <is>
+          <t>conversations.ts LIMIT 40 等硬截；无 token 估算。</t>
+        </is>
+      </c>
+      <c r="G95" s="86" t="inlineStr">
+        <is>
+          <t>先补按 token 裁剪注入器，封在注入函数内。阻断 W-01。</t>
+        </is>
+      </c>
+      <c r="H95" s="87" t="n">
+        <v>46310</v>
+      </c>
+      <c r="I95" s="86" t="n"/>
+      <c r="J95" s="86" t="n"/>
+      <c r="K95" s="86" t="inlineStr">
+        <is>
+          <t>二期新增；W 前置；见 ARCH-1</t>
+        </is>
+      </c>
+      <c r="L95" s="86" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="86" t="inlineStr">
+        <is>
+          <t>D-26</t>
+        </is>
+      </c>
+      <c r="B96" s="86" t="inlineStr">
+        <is>
+          <t>暂缓</t>
+        </is>
+      </c>
+      <c r="C96" s="86" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="D96" s="86" t="inlineStr">
+        <is>
+          <t>工程债</t>
+        </is>
+      </c>
+      <c r="E96" s="86" t="inlineStr">
+        <is>
+          <t>created_at 双格式 + 存量归一化迁移</t>
+        </is>
+      </c>
+      <c r="F96" s="86" t="inlineStr">
+        <is>
+          <t>DEFAULT datetime(now) vs toISOString；流逝计算歧义。</t>
+        </is>
+      </c>
+      <c r="G96" s="86" t="inlineStr">
+        <is>
+          <t>统一单一 UTC；仿 moments__m06 建表回填改名迁存量。阻断 W-02/W-03。</t>
+        </is>
+      </c>
+      <c r="H96" s="87" t="n">
+        <v>46310</v>
+      </c>
+      <c r="I96" s="86" t="n"/>
+      <c r="J96" s="86" t="n"/>
+      <c r="K96" s="86" t="inlineStr">
+        <is>
+          <t>二期新增；W 前置；见 ARCH-1</t>
+        </is>
+      </c>
+      <c r="L96" s="86" t="inlineStr">
+        <is>
+          <t>不适用</t>
         </is>
       </c>
     </row>
@@ -6130,7 +6546,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="41">
       <c r="A4" s="68" t="inlineStr">
         <is>
@@ -6323,7 +6738,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="41">
       <c r="A4" s="68" t="inlineStr">
         <is>
@@ -6391,7 +6805,6 @@
         <v/>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="15" customHeight="1" s="41">
       <c r="A11" s="72" t="inlineStr">
         <is>
@@ -6403,7 +6816,6 @@
         <v/>
       </c>
     </row>
-    <row r="12"/>
     <row r="13" ht="15" customHeight="1" s="41">
       <c r="A13" s="80" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(product): close B-04c/B-04d after cloud verify
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -4867,20 +4867,25 @@
           <t>冒烟：「帮我画一只猫」可出图；裸「画一只猫」不触发 wantsImageGeneration。</t>
         </is>
       </c>
+      <c r="G61" s="40" t="inlineStr">
+        <is>
+          <t>触发词加宽已合；2026-10-15 云侧复验正负例均过。</t>
+        </is>
+      </c>
       <c r="H61" s="83" t="n">
         <v>46305</v>
       </c>
       <c r="I61" s="83" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="J61" s="40" t="inlineStr">
         <is>
-          <t>af133b9</t>
+          <t>af133b9 / 云验基 bff4424 / 表关 5c28fc1</t>
         </is>
       </c>
       <c r="K61" s="40" t="inlineStr">
         <is>
-          <t>已关 tip af133b9（feat b1ad348）：wantsImageGeneration 加宽量词（只/条/匹等）；裸「画一只猫」可触发；闲聊不误触；云测过。失败仍 B-04d 人话路径。</t>
+          <t>已关 tip af133b9（feat b1ad348）：wantsImageGeneration 加宽量词（只/条/匹等）；裸「画一只猫」可触发；闲聊不误触；云测过。失败仍 B-04d 人话路径。 2026-10-15 云侧复验：「画一只猫」「帮我画一只猫」出图；「天气怎么样」「你的画很好看」不误触；零功能 commit。表关见本 tip。</t>
         </is>
       </c>
       <c r="L61" s="40" t="inlineStr">
@@ -4897,7 +4902,7 @@
       </c>
       <c r="B62" s="40" t="inlineStr">
         <is>
-          <t>待实打</t>
+          <t>已处理</t>
         </is>
       </c>
       <c r="C62" s="40" t="inlineStr">
@@ -4922,28 +4927,28 @@
       </c>
       <c r="G62" s="40" t="inlineStr">
         <is>
-          <t>2026-10-13 BF 验证+小补：坏 IMAGE_GEN_API_KEY → 上游 401；用户气泡人话「这张图没画成：密钥无效或没有权限…」不再夹带上游 JSON。formatImageGenUserError + throw 仅保留状态码；服务端仍 log 截断 body。</t>
+          <t>2026-10-13 BF 验证+小补：坏 IMAGE_GEN_API_KEY → 上游 401；用户气泡人话「这张图没画成：密钥无效或没有权限…」不再夹带上游 JSON。formatImageGenUserError + throw 仅保留状态码；服务端仍 log 截断 body。 2026-10-15 云侧坏 Key 实打过：人话错误、无上游 JSON；.env 已恢复。待实打→已处理。</t>
         </is>
       </c>
       <c r="H62" s="83" t="n">
         <v>46305</v>
       </c>
       <c r="I62" s="88" t="n">
-        <v>46308</v>
+        <v>46310</v>
       </c>
       <c r="J62" s="40" t="inlineStr">
         <is>
-          <t>6263381</t>
+          <t>6263381 / 云验基 bff4424 / 表关 5c28fc1</t>
         </is>
       </c>
       <c r="K62" s="40" t="inlineStr">
         <is>
-          <t>挂 API/密钥试跑时顺带验。 2026-10-10：读图 VLM 债/B-04d 在 ARCH-2 试跑线里还（非独立刀）。 2026-10-10 试跑线观测：坏 IMAGE_GEN Key → 上游 HTTP 401 Token is invalid；产品侧失败回流人话路径未改代码实打，仍暂缓。 2026-10-11 收尾：Gemini TTS + 官方 VLM 仍挂债等 Key；排在 X05-D1 / D-02b 之后。 2026-10-13：DeepSeek 官方文本+识图已通，不再算试跑挂债；本条续挂 **Gemini TTS 等 Key** + 生图失败人话路径。 2026-10-13：B-04d 关单（验证失败路径+开发去 JSON）。Gemini TTS 仍等 Key，不在本条。 N-02 不动。生图 Key=IMAGE_GEN_*（硅基），非 DeepSeek 文本键。；2026-10-14：状态改为「待实打」——代码已合 tip 6263381（formatImageGenUserError 人话），非未做；待云侧坏 Key 实打验收（验完须恢复 .env）。</t>
+          <t>挂 API/密钥试跑时顺带验。 2026-10-10：读图 VLM 债/B-04d 在 ARCH-2 试跑线里还（非独立刀）。 2026-10-10 试跑线观测：坏 IMAGE_GEN Key → 上游 HTTP 401 Token is invalid；产品侧失败回流人话路径未改代码实打，仍暂缓。 2026-10-11 收尾：Gemini TTS + 官方 VLM 仍挂债等 Key；排在 X05-D1 / D-02b 之后。 2026-10-13：DeepSeek 官方文本+识图已通，不再算试跑挂债；本条续挂 **Gemini TTS 等 Key** + 生图失败人话路径。 2026-10-13：B-04d 关单（验证失败路径+开发去 JSON）。Gemini TTS 仍等 Key，不在本条。 N-02 不动。生图 Key=IMAGE_GEN_*（硅基），非 DeepSeek 文本键。；2026-10-14：状态改为「待实打」——代码已合 tip 6263381（formatImageGenUserError 人话），非未做；待云侧坏 Key 实打验收（验完须恢复 .env）。 2026-10-15 云侧坏 Key 验过：气泡含「密钥无效或没有权限，请检查本机 IMAGE_GEN_API_KEY」，无上游 JSON；.env 已恢复。表关见本 tip。</t>
         </is>
       </c>
       <c r="L62" s="40" t="inlineStr">
         <is>
-          <t>代码已合；待实打</t>
+          <t>已 push</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(product): backfill B-04c/B-04d close tip hash
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -4880,7 +4880,7 @@
       </c>
       <c r="J61" s="40" t="inlineStr">
         <is>
-          <t>af133b9 / 云验基 bff4424 / 表关 5c28fc1</t>
+          <t>af133b9 / 云验基 bff4424 / 表关 5fc84a7</t>
         </is>
       </c>
       <c r="K61" s="40" t="inlineStr">
@@ -4938,7 +4938,7 @@
       </c>
       <c r="J62" s="40" t="inlineStr">
         <is>
-          <t>6263381 / 云验基 bff4424 / 表关 5c28fc1</t>
+          <t>6263381 / 云验基 bff4424 / 表关 5fc84a7</t>
         </is>
       </c>
       <c r="K62" s="40" t="inlineStr">

</xml_diff>

<commit_message>
docs(product): record D-03-a chatTurn extract (tip 48cc22d)
ARCH-1 D-03 status, problem-table D-03-a row, EOD-10-15 line counts
conversations.ts 1034→651 / chatTurn.ts 426.
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -1389,7 +1389,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L96"/>
+  <dimension ref="A1:L97"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="40" min="1" max="1"/>
@@ -6477,6 +6477,64 @@
       <c r="L96" s="86" t="inlineStr">
         <is>
           <t>不适用</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="40" t="inlineStr">
+        <is>
+          <t>D-03-a</t>
+        </is>
+      </c>
+      <c r="B97" s="40" t="inlineStr">
+        <is>
+          <t>已处理</t>
+        </is>
+      </c>
+      <c r="C97" s="40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D97" s="40" t="inlineStr">
+        <is>
+          <t>后端</t>
+        </is>
+      </c>
+      <c r="E97" s="40" t="inlineStr">
+        <is>
+          <t>conversations handleUserMessage 下沉 chatTurn（D-03 第一刀）</t>
+        </is>
+      </c>
+      <c r="F97" s="40" t="inlineStr">
+        <is>
+          <t>ARCH-1 D-03：conversations.ts 路由上帝文件（~1034 行）承载 prompt/历史/LLM/落库/记忆/主动/群聊轮询。本刀只搬 handleUserMessage 主体+X-04 helper，不抽读图/语音独立服务。</t>
+        </is>
+      </c>
+      <c r="G97" s="40" t="inlineStr">
+        <is>
+          <t>2026-10-15 BF：新建 services/chatTurn.ts；conversations.ts 1034→651；tsc 过；API/行为零变化；生图分支随 handleUserMessage 搬入（未单拆）。读图 multipart / TTS 仍在路由。云侧冒烟由小助手。</t>
+        </is>
+      </c>
+      <c r="H97" s="83" t="n">
+        <v>46305</v>
+      </c>
+      <c r="I97" s="83" t="n">
+        <v>46310</v>
+      </c>
+      <c r="J97" s="40" t="inlineStr">
+        <is>
+          <t>48cc22d</t>
+        </is>
+      </c>
+      <c r="K97" s="40" t="inlineStr">
+        <is>
+          <t>基 tip ab4f4c6。D-03 其余：读图编排→D-03-b；语音/TTS→D-03-c/d。行数 651（非精确 400）因读图+TTS 路由仍在。 feat tip 48cc22d (48cc22d6108a…).</t>
+        </is>
+      </c>
+      <c r="L97" s="40" t="inlineStr">
+        <is>
+          <t>已 push</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(server): normalize created_at to UTC ISO with stock migration (D-26)
Unify DB timestamps on nowIso()/toUtcIso (utils/time.ts); change SQLite
DEFAULT from datetime('now') to strftime UTC ISO; rebuild tables with
moments__m06-style migration; characters INSERT writes created_at explicitly.
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -334,7 +334,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="89">
+  <cellXfs count="90">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -592,6 +592,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6436,7 +6439,7 @@
       </c>
       <c r="B96" s="86" t="inlineStr">
         <is>
-          <t>暂缓</t>
+          <t>已处理</t>
         </is>
       </c>
       <c r="C96" s="86" t="inlineStr">
@@ -6461,22 +6464,28 @@
       </c>
       <c r="G96" s="86" t="inlineStr">
         <is>
-          <t>统一单一 UTC；仿 moments__m06 建表回填改名迁存量。阻断 W-02/W-03。</t>
+          <t>2026-10-15 BF：统一 nowIso()/toUtcIso；DEFAULT 改 strftime UTC ISO；ensureUtcIsoTimestamps 仿 moments__m06 重建含 datetime('now') 的表并归一存量；characters INSERT 显式写 created_at。tsc 过。</t>
         </is>
       </c>
       <c r="H96" s="87" t="n">
         <v>46310</v>
       </c>
-      <c r="I96" s="86" t="n"/>
-      <c r="J96" s="86" t="n"/>
+      <c r="I96" s="89" t="n">
+        <v>46310</v>
+      </c>
+      <c r="J96" s="86" t="inlineStr">
+        <is>
+          <t>24ba36c</t>
+        </is>
+      </c>
       <c r="K96" s="86" t="inlineStr">
         <is>
-          <t>二期新增；W 前置；见 ARCH-1</t>
+          <t>写入统一 apps/server/src/utils/time.ts#nowIso；迁移表：characters/conversations/messages/moments/moment_likes/moment_comments/message_reactions/character_ref_images；in-place：user_profile/proactive_state/memories/memory_notices。 tip 24ba36c。</t>
         </is>
       </c>
       <c r="L96" s="86" t="inlineStr">
         <is>
-          <t>不适用</t>
+          <t>已 push</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(product): fill D-26 tip hash 5f31a5a
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -6475,12 +6475,12 @@
       </c>
       <c r="J96" s="86" t="inlineStr">
         <is>
-          <t>24ba36c</t>
+          <t>5f31a5a</t>
         </is>
       </c>
       <c r="K96" s="86" t="inlineStr">
         <is>
-          <t>写入统一 apps/server/src/utils/time.ts#nowIso；迁移表：characters/conversations/messages/moments/moment_likes/moment_comments/message_reactions/character_ref_images；in-place：user_profile/proactive_state/memories/memory_notices。 tip 24ba36c。</t>
+          <t>写入统一 apps/server/src/utils/time.ts#nowIso；迁移表：characters/conversations/messages/moments/moment_likes/moment_comments/message_reactions/character_ref_images；in-place：user_profile/proactive_state/memories/memory_notices。 tip 5f31a5a。</t>
         </is>
       </c>
       <c r="L96" s="86" t="inlineStr">

</xml_diff>

<commit_message>
docs(product): close D-25 tip 8d89f09
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -6387,7 +6387,7 @@
       </c>
       <c r="B95" s="86" t="inlineStr">
         <is>
-          <t>暂缓</t>
+          <t>已处理</t>
         </is>
       </c>
       <c r="C95" s="86" t="inlineStr">
@@ -6418,16 +6418,22 @@
       <c r="H95" s="87" t="n">
         <v>46310</v>
       </c>
-      <c r="I95" s="86" t="n"/>
-      <c r="J95" s="86" t="n"/>
+      <c r="I95" s="87" t="n">
+        <v>46310</v>
+      </c>
+      <c r="J95" s="86" t="inlineStr">
+        <is>
+          <t>8d89f09</t>
+        </is>
+      </c>
       <c r="K95" s="86" t="inlineStr">
         <is>
-          <t>二期新增；W 前置；见 ARCH-1</t>
+          <t>二期新增；W 前置；见 ARCH-1；promptInject + appendMemoryBlock 预算裁剪；调用方签名不变</t>
         </is>
       </c>
       <c r="L95" s="86" t="inlineStr">
         <is>
-          <t>不适用</t>
+          <t>已 push</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(product): close D-15 tip c41441e
Mark ARCH-1 D-15 / problem xlsx / EOD-10-15 closed with BF tip c41441e.
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -1392,7 +1392,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L97"/>
+  <dimension ref="A1:L98"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="40" min="1" max="1"/>
@@ -6548,6 +6548,64 @@
         </is>
       </c>
       <c r="L97" s="40" t="inlineStr">
+        <is>
+          <t>已 push</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="40" t="inlineStr">
+        <is>
+          <t>D-15</t>
+        </is>
+      </c>
+      <c r="B98" s="40" t="inlineStr">
+        <is>
+          <t>已处理</t>
+        </is>
+      </c>
+      <c r="C98" s="40" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="D98" s="40" t="inlineStr">
+        <is>
+          <t>工程债</t>
+        </is>
+      </c>
+      <c r="E98" s="40" t="inlineStr">
+        <is>
+          <t>空间赞评/作者回评内存定时器重启即丢</t>
+        </is>
+      </c>
+      <c r="F98" s="40" t="inlineStr">
+        <is>
+          <t>momentReactions pendingTimers/authorReplyTimers 仅内存；重启未结算任务丢失。</t>
+        </is>
+      </c>
+      <c r="G98" s="40" t="inlineStr">
+        <is>
+          <t>2026-10-15 BF：moment_reaction_due 落表；schedule 写 due+timer；启动 recoverMomentReactionJobs；过期立即跑；完成清行。tsc 过。proactive 语义不变。</t>
+        </is>
+      </c>
+      <c r="H98" s="83" t="n">
+        <v>46310</v>
+      </c>
+      <c r="I98" s="83" t="n">
+        <v>46310</v>
+      </c>
+      <c r="J98" s="40" t="inlineStr">
+        <is>
+          <t>c41441e</t>
+        </is>
+      </c>
+      <c r="K98" s="40" t="inlineStr">
+        <is>
+          <t>W-03/W-04 跨重启依赖；ARCH-1 D-15 关单。表 PK(kind,moment_id)。</t>
+        </is>
+      </c>
+      <c r="L98" s="40" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>

</xml_diff>

<commit_message>
docs(product): record Gemini TTS tryrun — geo block, not daily candidate
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -1392,7 +1392,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L98"/>
+  <dimension ref="A1:L99"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="40" min="1" max="1"/>
@@ -4772,7 +4772,7 @@
       </c>
       <c r="K59" s="40" t="inlineStr">
         <is>
-          <t>试跑主证据改为 HY 本地 VLM；硅基 Qwen3-VL 降为回落 2026-10-11 API 切换试跑线（HY）：DeepSeek 文本通（硅基 DeepSeek-V4-Flash，本机 DEEPSEEK_API_KEY 空）；读图：本地 Ollama qwen2.5vl:7b 通（官方/独立 VLM Key 未配）；Gemini TTS 缺 GEMINI_API_KEY → 挂债不阻塞（B-04d 续）。N-02 仍不动。 2026-10-11 收尾试跑线备注：DeepSeek 文本通（硅基 DeepSeek-V4-Flash，属 DeepSeek 系列）；本地 Ollama qwen2.5vl 读图通；Gemini TTS + 官方 VLM Key 挂债（不阻塞）。N-02 不动。 2026-10-13 BF 拍板：DeepSeek 官方试跑 **已通**（文本+识图均 api.deepseek.com / deepseek-flash；官方识图超出原仅文本计划）。Gemini TTS 仍等 GEMINI_API_KEY；N-02 不变。</t>
+          <t>试跑主证据改为 HY 本地 VLM；硅基 Qwen3-VL 降为回落 2026-10-11 API 切换试跑线（HY）：DeepSeek 文本通（硅基 DeepSeek-V4-Flash，本机 DEEPSEEK_API_KEY 空）；读图：本地 Ollama qwen2.5vl:7b 通（官方/独立 VLM Key 未配）；Gemini TTS 缺 GEMINI_API_KEY → 挂债不阻塞（B-04d 续）。N-02 仍不动。 2026-10-11 收尾试跑线备注：DeepSeek 文本通（硅基 DeepSeek-V4-Flash，属 DeepSeek 系列）；本地 Ollama qwen2.5vl 读图通；Gemini TTS + 官方 VLM Key 挂债（不阻塞）。N-02 不动。 2026-10-13 BF 拍板：DeepSeek 官方试跑 **已通**（文本+识图均 api.deepseek.com / deepseek-flash；官方识图超出原仅文本计划）。Gemini TTS 仍等 GEMINI_API_KEY；N-02 不变。 2026-10-16：Gemini TTS 试跑关 B-04e——官方未通（地域限制）+ 免费层 10RPD 不达日常；相对 CosyVoice2 无法对比；不列付费候选。</t>
         </is>
       </c>
       <c r="L59" s="40" t="inlineStr">
@@ -4946,7 +4946,7 @@
       </c>
       <c r="K62" s="40" t="inlineStr">
         <is>
-          <t>挂 API/密钥试跑时顺带验。 2026-10-10：读图 VLM 债/B-04d 在 ARCH-2 试跑线里还（非独立刀）。 2026-10-10 试跑线观测：坏 IMAGE_GEN Key → 上游 HTTP 401 Token is invalid；产品侧失败回流人话路径未改代码实打，仍暂缓。 2026-10-11 收尾：Gemini TTS + 官方 VLM 仍挂债等 Key；排在 X05-D1 / D-02b 之后。 2026-10-13：DeepSeek 官方文本+识图已通，不再算试跑挂债；本条续挂 **Gemini TTS 等 Key** + 生图失败人话路径。 2026-10-13：B-04d 关单（验证失败路径+开发去 JSON）。Gemini TTS 仍等 Key，不在本条。 N-02 不动。生图 Key=IMAGE_GEN_*（硅基），非 DeepSeek 文本键。；2026-10-14：状态改为「待实打」——代码已合 tip 6263381（formatImageGenUserError 人话），非未做；待云侧坏 Key 实打验收（验完须恢复 .env）。 2026-10-15 云侧坏 Key 验过：气泡含「密钥无效或没有权限，请检查本机 IMAGE_GEN_API_KEY」，无上游 JSON；.env 已恢复。表关见本 tip。</t>
+          <t>挂 API/密钥试跑时顺带验。 2026-10-10：读图 VLM 债/B-04d 在 ARCH-2 试跑线里还（非独立刀）。 2026-10-10 试跑线观测：坏 IMAGE_GEN Key → 上游 HTTP 401 Token is invalid；产品侧失败回流人话路径未改代码实打，仍暂缓。 2026-10-11 收尾：Gemini TTS + 官方 VLM 仍挂债等 Key；排在 X05-D1 / D-02b 之后。 2026-10-13：DeepSeek 官方文本+识图已通，不再算试跑挂债；本条续挂 **Gemini TTS 等 Key** + 生图失败人话路径。 2026-10-13：B-04d 关单（验证失败路径+开发去 JSON）。Gemini TTS 仍等 Key，不在本条。 N-02 不动。生图 Key=IMAGE_GEN_*（硅基），非 DeepSeek 文本键。；2026-10-14：状态改为「待实打」——代码已合 tip 6263381（formatImageGenUserError 人话），非未做；待云侧坏 Key 实打验收（验完须恢复 .env）。 2026-10-15 云侧坏 Key 验过：气泡含「密钥无效或没有权限，请检查本机 IMAGE_GEN_API_KEY」，无上游 JSON；.env 已恢复。表关见本 tip。 2026-10-16：Gemini TTS 已实跑见 B-04e（地域未通，非缺 Key）。</t>
         </is>
       </c>
       <c r="L62" s="40" t="inlineStr">
@@ -6606,6 +6606,60 @@
         </is>
       </c>
       <c r="L98" s="40" t="inlineStr">
+        <is>
+          <t>已 push</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="40" t="inlineStr">
+        <is>
+          <t>B-04e</t>
+        </is>
+      </c>
+      <c r="B99" s="40" t="inlineStr">
+        <is>
+          <t>已处理</t>
+        </is>
+      </c>
+      <c r="C99" s="40" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D99" s="40" t="inlineStr">
+        <is>
+          <t>消息</t>
+        </is>
+      </c>
+      <c r="E99" s="40" t="inlineStr">
+        <is>
+          <t>Gemini TTS 试跑</t>
+        </is>
+      </c>
+      <c r="F99" s="40" t="inlineStr">
+        <is>
+          <t>ARCH-2/API 试跑线续债：官方 Gemini TTS（Kore/Charon）与现网 CosyVoice2 同文 A/B。基 tip 5ea0ee6；仅配 GEMINI_API_KEY，不动生产 TTS_*；Gemini 调用≤2/3；wav 不入库。</t>
+        </is>
+      </c>
+      <c r="G99" s="40" t="inlineStr">
+        <is>
+          <t>官方未通（地域限制）+ 免费层 10RPD 不达日常；相对 CosyVoice2 无法对比音质；不备注付费候选。</t>
+        </is>
+      </c>
+      <c r="H99" s="88" t="n">
+        <v>46311</v>
+      </c>
+      <c r="I99" s="88" t="n">
+        <v>46311</v>
+      </c>
+      <c r="J99" s="40" t="n"/>
+      <c r="K99" s="40" t="inlineStr">
+        <is>
+          <t>2026-10-16 云验 tip 5ea0ee6：Gemini Kore/Charon 均 HTTP 400 FAILED_PRECONDITION User location is not supported for the API use.（云侧郑州出口）；无 gemini wav。CosyVoice2 anna 同文通 scripts/_tryrun_out/cosyvoice-anna.wav（Bearer 临时 IMAGE_GEN，未写 TTS_API_KEY）。听感无法 A/B。零功能 commit；本条仅文档关单。 docs tip 本关单。</t>
+        </is>
+      </c>
+      <c r="L99" s="40" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>

</xml_diff>

<commit_message>
docs(product): backfill B-04e tip 6a63f61
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -6653,15 +6653,19 @@
       <c r="I99" s="88" t="n">
         <v>46311</v>
       </c>
-      <c r="J99" s="40" t="n"/>
+      <c r="J99" s="40" t="inlineStr">
+        <is>
+          <t>6a63f61</t>
+        </is>
+      </c>
       <c r="K99" s="40" t="inlineStr">
         <is>
-          <t>2026-10-16 云验 tip 5ea0ee6：Gemini Kore/Charon 均 HTTP 400 FAILED_PRECONDITION User location is not supported for the API use.（云侧郑州出口）；无 gemini wav。CosyVoice2 anna 同文通 scripts/_tryrun_out/cosyvoice-anna.wav（Bearer 临时 IMAGE_GEN，未写 TTS_API_KEY）。听感无法 A/B。零功能 commit；本条仅文档关单。 docs tip 本关单。</t>
+          <t>2026-10-16 云验 tip 5ea0ee6：Gemini Kore/Charon 均 HTTP 400 FAILED_PRECONDITION User location is not supported for the API use.（云侧郑州出口）；无 gemini wav。CosyVoice2 anna 同文通 scripts/_tryrun_out/cosyvoice-anna.wav（Bearer 临时 IMAGE_GEN，未写 TTS_API_KEY）。听感无法 A/B。零功能 commit；本条仅文档关单。 docs tip 6a63f61。</t>
         </is>
       </c>
       <c r="L99" s="40" t="inlineStr">
         <is>
-          <t>已 push</t>
+          <t>已 push（tip 6a63f61）</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(product): W-01 tip 4ca8a9f; B-04e re-wording (overseas egress, not paid candidate)
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -6075,7 +6075,7 @@
       </c>
       <c r="B89" s="86" t="inlineStr">
         <is>
-          <t>暂缓</t>
+          <t>已处理</t>
         </is>
       </c>
       <c r="C89" s="86" t="inlineStr">
@@ -6100,22 +6100,28 @@
       </c>
       <c r="G89" s="86" t="inlineStr">
         <is>
-          <t>待排期；前置 D-25。见《真实世界感设计备忘》。</t>
+          <t>2026-10-16 BF：user_profile 加可空 location（幂等迁移，存量不动）；chatTurn 每轮 nowIso→Asia/Shanghai 常量，经 promptInject 装配注入一行「当前时间：…（周X 时段，北京时间）；用户所在地：…」，pinned 最高优先级不裁剪；location 空则不输出地点段。调用方签名不变；不改前端/X-07/主动/静默时段。tsc 过；本地注入行冒烟（有/无地点）过；私聊 LLM 冒烟由云电脑做。</t>
         </is>
       </c>
       <c r="H89" s="87" t="n">
         <v>46310</v>
       </c>
-      <c r="I89" s="86" t="n"/>
-      <c r="J89" s="86" t="n"/>
+      <c r="I89" s="89" t="n">
+        <v>46311</v>
+      </c>
+      <c r="J89" s="86" t="inlineStr">
+        <is>
+          <t>4ca8a9f</t>
+        </is>
+      </c>
       <c r="K89" s="86" t="inlineStr">
         <is>
-          <t>二期新增；待用户排期；不插队下一刀</t>
+          <t>feat 4ca8a9f；同刀 docs 并入 B-04e 改口径 + EOD-10-16。默认地点待用户明确；设置 UI 后置。下一刀 W-02 → W-03。</t>
         </is>
       </c>
       <c r="L89" s="86" t="inlineStr">
         <is>
-          <t>不适用</t>
+          <t>已 push</t>
         </is>
       </c>
     </row>
@@ -6644,7 +6650,7 @@
       </c>
       <c r="G99" s="40" t="inlineStr">
         <is>
-          <t>官方未通（地域限制）+ 免费层 10RPD 不达日常；相对 CosyVoice2 无法对比音质；不备注付费候选。</t>
+          <t>需境外出口才通（云电脑代理东京出口，200/2.4s，Kore）+ 试听不优于 CosyVoice2 → 不列付费候选，生产 TTS 继续硅基</t>
         </is>
       </c>
       <c r="H99" s="88" t="n">
@@ -6660,7 +6666,7 @@
       </c>
       <c r="K99" s="40" t="inlineStr">
         <is>
-          <t>2026-10-16 云验 tip 5ea0ee6：Gemini Kore/Charon 均 HTTP 400 FAILED_PRECONDITION User location is not supported for the API use.（云侧郑州出口）；无 gemini wav。CosyVoice2 anna 同文通 scripts/_tryrun_out/cosyvoice-anna.wav（Bearer 临时 IMAGE_GEN，未写 TTS_API_KEY）。听感无法 A/B。零功能 commit；本条仅文档关单。 docs tip 6a63f61。</t>
+          <t>需境外出口才通；Kore 听感正式中性，不贴产品默认音色；免费 10 RPD 不达日常；不列付费候选，生产沿用硅基流动。</t>
         </is>
       </c>
       <c r="L99" s="40" t="inlineStr">

</xml_diff>

<commit_message>
docs(product): W-01 hotfix tip 59073c1
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -6111,12 +6111,12 @@
       </c>
       <c r="J89" s="86" t="inlineStr">
         <is>
-          <t>4ca8a9f</t>
+          <t>59073c1</t>
         </is>
       </c>
       <c r="K89" s="86" t="inlineStr">
         <is>
-          <t>feat 4ca8a9f；同刀 docs 并入 B-04e 改口径 + EOD-10-16。默认地点待用户明确；设置 UI 后置。下一刀 W-02 → W-03。</t>
+          <t>feat 4ca8a9f；同刀 docs 并入 B-04e 改口径 + EOD-10-16。默认地点待用户明确；设置 UI 后置。下一刀 W-02 → W-03。a191d66 云验 500，迁移漏调用；修复 tip 59073c1</t>
         </is>
       </c>
       <c r="L89" s="86" t="inlineStr">

</xml_diff>

<commit_message>
docs(product): 10-16 multi-model tryrun appendix + pricing; B-04e/TTS note; W-01 close + r1/r2
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -1392,7 +1392,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L99"/>
+  <dimension ref="A1:L101"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="40" min="1" max="1"/>
@@ -4099,7 +4099,7 @@
       <c r="J47" s="86" t="n"/>
       <c r="K47" s="86" t="inlineStr">
         <is>
-          <t>来源：用户 2026-10-10 规划占位。触发：用户选定多模型供应商与路由规则后再开。 2026-10-10：提前至二期中后段；与 ARCH-2 共挂 API 试跑线（本地/硅基/官方；DeepSeek 文本、官方 VLM、Gemini TTS）。 2026-10-11 试跑线仍不动。 2026-10-13：仍暂缓，不发明工作。</t>
+          <t>来源：用户 2026-10-10 规划占位。触发：用户选定多模型供应商与路由规则后再开。 2026-10-10：提前至二期中后段；与 ARCH-2 共挂 API 试跑线（本地/硅基/官方；DeepSeek 文本、官方 VLM、Gemini TTS）。 2026-10-11 试跑线仍不动。 2026-10-13：仍暂缓，不发明工作。；触发条件追加：多模型成本策略成型中（10-16）；仍冻结</t>
         </is>
       </c>
       <c r="L47" s="86" t="inlineStr">
@@ -6111,12 +6111,12 @@
       </c>
       <c r="J89" s="86" t="inlineStr">
         <is>
-          <t>59073c1</t>
+          <t>cb22b74</t>
         </is>
       </c>
       <c r="K89" s="86" t="inlineStr">
         <is>
-          <t>feat 4ca8a9f；同刀 docs 并入 B-04e 改口径 + EOD-10-16。默认地点待用户明确；设置 UI 后置。下一刀 W-02 → W-03。a191d66 云验 500，迁移漏调用；修复 tip 59073c1</t>
+          <t>feat 4ca8a9f；同刀 docs 并入 B-04e 改口径 + EOD-10-16。默认地点待用户明确；设置 UI 后置。下一刀 W-02 → W-03。a191d66 云验 500，迁移漏调用；修复 tip 59073c1。已关（tip cb22b74，feat 4ca8a9f + fix 59073c1）；残项 W-01-r1/W-01-r2</t>
         </is>
       </c>
       <c r="L89" s="86" t="inlineStr">
@@ -6666,12 +6666,116 @@
       </c>
       <c r="K99" s="40" t="inlineStr">
         <is>
-          <t>需境外出口才通；Kore 听感正式中性，不贴产品默认音色；免费 10 RPD 不达日常；不列付费候选，生产沿用硅基流动。</t>
+          <t>付费层 100 次/日，需境外出口；作境外备用（备用型号 3.8-flash-lite-tts）。生产沿用硅基流动，默认音色仍是 CosyVoice2 anna。</t>
         </is>
       </c>
       <c r="L99" s="40" t="inlineStr">
         <is>
           <t>已 push（tip 6a63f61）</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="40" t="inlineStr">
+        <is>
+          <t>W-01-r1</t>
+        </is>
+      </c>
+      <c r="B100" s="40" t="inlineStr">
+        <is>
+          <t>待处理</t>
+        </is>
+      </c>
+      <c r="C100" s="40" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D100" s="40" t="inlineStr">
+        <is>
+          <t>世界感</t>
+        </is>
+      </c>
+      <c r="E100" s="40" t="inlineStr">
+        <is>
+          <t>地点感弱</t>
+        </is>
+      </c>
+      <c r="F100" s="40" t="inlineStr">
+        <is>
+          <t>地点注入已生效，但 9b 模型不会主动按所在地聊天气和吃的。</t>
+        </is>
+      </c>
+      <c r="G100" s="40" t="inlineStr">
+        <is>
+          <t>待默认地点或设置 UI 落地时补提示。</t>
+        </is>
+      </c>
+      <c r="H100" s="88" t="n">
+        <v>46311</v>
+      </c>
+      <c r="I100" s="88" t="n"/>
+      <c r="J100" s="40" t="n"/>
+      <c r="K100" s="40" t="inlineStr">
+        <is>
+          <t>W-01 云验残项（10-16）</t>
+        </is>
+      </c>
+      <c r="L100" s="40" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="40" t="inlineStr">
+        <is>
+          <t>W-01-r2</t>
+        </is>
+      </c>
+      <c r="B101" s="40" t="inlineStr">
+        <is>
+          <t>待处理</t>
+        </is>
+      </c>
+      <c r="C101" s="40" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D101" s="40" t="inlineStr">
+        <is>
+          <t>世界感</t>
+        </is>
+      </c>
+      <c r="E101" s="40" t="inlineStr">
+        <is>
+          <t>时段被历史带偏</t>
+        </is>
+      </c>
+      <c r="F101" s="40" t="inlineStr">
+        <is>
+          <t>注入当前时间后，回复仍随前一晚话题偏到夜里。</t>
+        </is>
+      </c>
+      <c r="G101" s="40" t="inlineStr">
+        <is>
+          <t>并入 W-02 评估。</t>
+        </is>
+      </c>
+      <c r="H101" s="88" t="n">
+        <v>46311</v>
+      </c>
+      <c r="I101" s="88" t="n"/>
+      <c r="J101" s="40" t="n"/>
+      <c r="K101" s="40" t="inlineStr">
+        <is>
+          <t>W-01 云验残项（10-16）</t>
+        </is>
+      </c>
+      <c r="L101" s="40" t="inlineStr">
+        <is>
+          <t>不适用</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(product): design calibration — L1/L2/L3 boundary, R-08, compression YAGNI, M-02 prereq W, reference registry
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -1392,7 +1392,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L101"/>
+  <dimension ref="A1:L102"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="40" min="1" max="1"/>
@@ -2466,7 +2466,7 @@
       <c r="J18" s="44" t="n"/>
       <c r="K18" s="46" t="inlineStr">
         <is>
-          <t>触发：好感度 R-03 立后，再做角色互评/图谱。 原待优化点第 5 条的大方案。</t>
+          <t>触发：好感度 R-03 立后，再做角色互评/图谱。 原待优化点第 5 条的大方案。；2026-10-16：前置 W 系列（角色要有共同时间线，互聊才有内容）</t>
         </is>
       </c>
       <c r="L18" s="40" t="inlineStr">
@@ -6774,6 +6774,58 @@
         </is>
       </c>
       <c r="L101" s="40" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="86" t="inlineStr">
+        <is>
+          <t>R-08</t>
+        </is>
+      </c>
+      <c r="B102" s="86" t="inlineStr">
+        <is>
+          <t>暂缓</t>
+        </is>
+      </c>
+      <c r="C102" s="86" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D102" s="86" t="inlineStr">
+        <is>
+          <t>记忆</t>
+        </is>
+      </c>
+      <c r="E102" s="86" t="inlineStr">
+        <is>
+          <t>中时段记忆</t>
+        </is>
+      </c>
+      <c r="F102" s="86" t="inlineStr">
+        <is>
+          <t>日程和会话摘要作为记忆行（走 L2，经注入统一出口）；与 R-07 同源（nyairo 参考评估）。</t>
+        </is>
+      </c>
+      <c r="G102" s="86" t="inlineStr">
+        <is>
+          <t>立账不拆包；触发：W-03 落地后真实使用中出现「角色记不住昨天」。与 W-01-r2 不合并。</t>
+        </is>
+      </c>
+      <c r="H102" s="87" t="n">
+        <v>46311</v>
+      </c>
+      <c r="I102" s="86" t="n"/>
+      <c r="J102" s="86" t="n"/>
+      <c r="K102" s="86" t="inlineStr">
+        <is>
+          <t>阶段归属：二期新增；暂缓</t>
+        </is>
+      </c>
+      <c r="L102" s="86" t="inlineStr">
         <is>
           <t>不适用</t>
         </is>

</xml_diff>

<commit_message>
docs(product): W-02 close-out — default location 上海, W-01-r2 evaluation, DS Bot/DSB split, R-08 P3, W-02-r1 tsconfig debt
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -1392,7 +1392,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L102"/>
+  <dimension ref="A1:L103"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="40" min="1" max="1"/>
@@ -6116,7 +6116,7 @@
       </c>
       <c r="K89" s="86" t="inlineStr">
         <is>
-          <t>feat 4ca8a9f；同刀 docs 并入 B-04e 改口径 + EOD-10-16。默认地点待用户明确；设置 UI 后置。下一刀 W-02 → W-03。a191d66 云验 500，迁移漏调用；修复 tip 59073c1。已关（tip cb22b74，feat 4ca8a9f + fix 59073c1）；残项 W-01-r1/W-01-r2</t>
+          <t>feat 4ca8a9f；同刀 docs 并入 B-04e 改口径 + EOD-10-16。默认地点待用户明确；设置 UI 后置。下一刀 W-02 → W-03。a191d66 云验 500，迁移漏调用；修复 tip 59073c1。已关（tip cb22b74，feat 4ca8a9f + fix 59073c1）；残项 W-01-r1/W-01-r2；默认地点 上海（用户 10-16 拍定，env DEFAULT_USER_LOCATION 可覆盖，W-02 刀落地）</t>
         </is>
       </c>
       <c r="L89" s="86" t="inlineStr">
@@ -6133,7 +6133,7 @@
       </c>
       <c r="B90" s="86" t="inlineStr">
         <is>
-          <t>暂缓</t>
+          <t>已处理</t>
         </is>
       </c>
       <c r="C90" s="86" t="inlineStr">
@@ -6148,7 +6148,7 @@
       </c>
       <c r="E90" s="86" t="inlineStr">
         <is>
-          <t>角色 presence 惰性求值</t>
+          <t>角色此刻状态 presence（惰性求值）</t>
         </is>
       </c>
       <c r="F90" s="86" t="inlineStr">
@@ -6158,22 +6158,28 @@
       </c>
       <c r="G90" s="86" t="inlineStr">
         <is>
-          <t>依赖 W-01。见备忘。</t>
+          <t>2026-10-16 BF：characters 加可空 JSON presence（幂等迁移，存量库副本连跑两次无错）；5 固定北京时段（深夜/早上/白天/傍晚/夜里，左闭右开）每段 {place, activity}；纯函数 resolvePresence，无 LLM/定时器/写库/随机；promptInject 注入 kind:'presence' 一行紧跟 W-01 时间行，非 pinned，预算不足整行裁；无配置/该段空不注入，行为零变化；调用方签名不变。单测 12 条、tsc server+web 过。云验待做。</t>
         </is>
       </c>
       <c r="H90" s="87" t="n">
         <v>46310</v>
       </c>
-      <c r="I90" s="86" t="n"/>
-      <c r="J90" s="86" t="n"/>
+      <c r="I90" s="89" t="n">
+        <v>46311</v>
+      </c>
+      <c r="J90" s="86" t="inlineStr">
+        <is>
+          <t>85d1392</t>
+        </is>
+      </c>
       <c r="K90" s="86" t="inlineStr">
         <is>
-          <t>二期新增；待用户排期</t>
+          <t>二期新增；用户 10-16 拍板开刀。同刀：默认地点上海、W-01-r2 评估、DeepSeek 拆两条、R-08→P3。待云验两轮。</t>
         </is>
       </c>
       <c r="L90" s="86" t="inlineStr">
         <is>
-          <t>不适用</t>
+          <t>已 push</t>
         </is>
       </c>
     </row>
@@ -6760,7 +6766,7 @@
       </c>
       <c r="G101" s="40" t="inlineStr">
         <is>
-          <t>并入 W-02 评估。</t>
+          <t>单次小样本（BF 本机 qwen2.5:7b；生产默认 qwen3.5:9b-nothink 本机未装），fixture=昨晚 21:30 火锅对话、now=15:00、问「现在该吃点啥？」：①历史行附相对时间 +24 tok，过 3072 闸，回复「热乎的粥还是炒点小菜」，不延续火锅也不提下午；②锚定句 +34 tok，过闸，回复仍建议火锅或汤面/粥，未体现下午；③两者 +58 tok，过闸，回复「清淡/重口/汤品」，未体现下午。三者均未出现「夜里」偏航，也都未明确对上下午；②不算通过，①③只是中性。结论：本刀不落地，另拆小刀用生产模型（qwen3.5:9b-nothink 或云端）复测后再定；①只动装配层（不动历史存储）。</t>
         </is>
       </c>
       <c r="H101" s="88" t="n">
@@ -6770,7 +6776,7 @@
       <c r="J101" s="40" t="n"/>
       <c r="K101" s="40" t="inlineStr">
         <is>
-          <t>W-01 云验残项（10-16）</t>
+          <t>W-01 云验残项（10-16）；W-02 刀评估完，未落地，待另拆小刀复测</t>
         </is>
       </c>
       <c r="L101" s="40" t="inlineStr">
@@ -6792,7 +6798,7 @@
       </c>
       <c r="C102" s="86" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="D102" s="86" t="inlineStr">
@@ -6822,10 +6828,62 @@
       <c r="J102" s="86" t="n"/>
       <c r="K102" s="86" t="inlineStr">
         <is>
-          <t>阶段归属：二期新增；暂缓</t>
+          <t>阶段归属：二期新增；暂缓；10-16 产品定 P2→P3</t>
         </is>
       </c>
       <c r="L102" s="86" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="86" t="inlineStr">
+        <is>
+          <t>W-02-r1</t>
+        </is>
+      </c>
+      <c r="B103" s="86" t="inlineStr">
+        <is>
+          <t>待处理</t>
+        </is>
+      </c>
+      <c r="C103" s="86" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D103" s="86" t="inlineStr">
+        <is>
+          <t>工程</t>
+        </is>
+      </c>
+      <c r="E103" s="86" t="inlineStr">
+        <is>
+          <t>server tsconfig 测试文件进 dist</t>
+        </is>
+      </c>
+      <c r="F103" s="86" t="inlineStr">
+        <is>
+          <t>apps/server tsconfig include src/**/*，*.test.ts 会被 build 进 dist（不执行，无功能影响）。</t>
+        </is>
+      </c>
+      <c r="G103" s="86" t="inlineStr">
+        <is>
+          <t>待统一测试目录时处理（exclude 或独立 tsconfig）。</t>
+        </is>
+      </c>
+      <c r="H103" s="87" t="n">
+        <v>46311</v>
+      </c>
+      <c r="I103" s="86" t="n"/>
+      <c r="J103" s="86" t="n"/>
+      <c r="K103" s="86" t="inlineStr">
+        <is>
+          <t>W-02 刀残债（10-16）</t>
+        </is>
+      </c>
+      <c r="L103" s="86" t="inlineStr">
         <is>
           <t>不适用</t>
         </is>

</xml_diff>

<commit_message>
fix(server): W residuals — unified 5-slot day period (W-02-r2), tests excluded from dist (W-02-r1), history breakpoint time anchors (W-01-r2) + docs
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -1392,7 +1392,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L103"/>
+  <dimension ref="A1:L104"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="40" min="1" max="1"/>
@@ -6174,7 +6174,7 @@
       </c>
       <c r="K90" s="86" t="inlineStr">
         <is>
-          <t>二期新增；用户 10-16 拍板开刀。同刀：默认地点上海、W-01-r2 评估、DeepSeek 拆两条、R-08→P3。待云验两轮。</t>
+          <t>二期新增；用户 10-16 拍板开刀。同刀：默认地点上海、W-01-r2 评估、DeepSeek 拆两条、R-08→P3。已关单 755a088，云验两轮通过。</t>
         </is>
       </c>
       <c r="L90" s="86" t="inlineStr">
@@ -6741,7 +6741,7 @@
       </c>
       <c r="B101" s="40" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>已处理</t>
         </is>
       </c>
       <c r="C101" s="40" t="inlineStr">
@@ -6766,22 +6766,28 @@
       </c>
       <c r="G101" s="40" t="inlineStr">
         <is>
-          <t>单次小样本（BF 本机 qwen2.5:7b；生产默认 qwen3.5:9b-nothink 本机未装），fixture=昨晚 21:30 火锅对话、now=15:00、问「现在该吃点啥？」：①历史行附相对时间 +24 tok，过 3072 闸，回复「热乎的粥还是炒点小菜」，不延续火锅也不提下午；②锚定句 +34 tok，过闸，回复仍建议火锅或汤面/粥，未体现下午；③两者 +58 tok，过闸，回复「清淡/重口/汤品」，未体现下午。三者均未出现「夜里」偏航，也都未明确对上下午；②不算通过，①③只是中性。结论：本刀不落地，另拆小刀用生产模型（qwen3.5:9b-nothink 或云端）复测后再定；①只动装配层（不动历史存储）。</t>
+          <t>BF 生产模型实测（qwen2.5:7b-fast，单次）：fixture=昨晚 21:30 火锅、now=15:00、问「现在该吃点啥？」。落地细粒度断点标注（只动装配层 historyAnchors + chatTurn，不动历史存储，调用方签名不变）：仅窗口内第一条用户消息、及与上一条间隔 ≥2h 的用户消息加前缀，今天「（今天 14:02）」、昨天「（昨天&lt;时段&gt; 21:30）」（时段用 presence 5 段，21:30 属傍晚）、更早「（10-14 20:00）」。fixture 新增 14 tok，历史合计 80 tok，过 3072 闸（超闸则整组标注不加）。回复「中午了，可以吃点米饭搭配红烧肉或者炖菜」：未当夜里、未延续火锅 → 通过（「中午」不准确但按口径不扣）。模型口径：qwen3.5:9b-nothink 为代码/示例默认占位值；BF 实机 = qwen2.5:7b-fast；开发期以 BF 实机为准，HY 上线后核（挂 D-11）。</t>
         </is>
       </c>
       <c r="H101" s="88" t="n">
         <v>46311</v>
       </c>
-      <c r="I101" s="88" t="n"/>
-      <c r="J101" s="40" t="n"/>
+      <c r="I101" s="88" t="n">
+        <v>46311</v>
+      </c>
+      <c r="J101" s="40" t="inlineStr">
+        <is>
+          <t>W 残项清理 commit（755a088 的下一个 commit，单 commit 无法自填 hash）</t>
+        </is>
+      </c>
       <c r="K101" s="40" t="inlineStr">
         <is>
-          <t>W-01 云验残项（10-16）；W-02 刀评估完，未落地，待另拆小刀复测</t>
+          <t>W-01 云验残项（10-16）；W-02 刀三候选中性未落地；W 残项刀 BF 生产模型实测通过并落地。开发期以 BF 实机为准，HY 上线后核（挂 D-11）</t>
         </is>
       </c>
       <c r="L101" s="40" t="inlineStr">
         <is>
-          <t>不适用</t>
+          <t>已 push</t>
         </is>
       </c>
     </row>
@@ -6845,7 +6851,7 @@
       </c>
       <c r="B103" s="86" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>已处理</t>
         </is>
       </c>
       <c r="C103" s="86" t="inlineStr">
@@ -6870,14 +6876,20 @@
       </c>
       <c r="G103" s="86" t="inlineStr">
         <is>
-          <t>待统一测试目录时处理（exclude 或独立 tsconfig）。</t>
+          <t>build 用 tsconfig.build.json exclude src/**/*.test.ts；npm run typecheck 用原 tsconfig 仍检查测试（故意类型错误能报出，已撤）。build 后 dist 无 *.test.js。</t>
         </is>
       </c>
       <c r="H103" s="87" t="n">
         <v>46311</v>
       </c>
-      <c r="I103" s="86" t="n"/>
-      <c r="J103" s="86" t="n"/>
+      <c r="I103" s="89" t="n">
+        <v>46311</v>
+      </c>
+      <c r="J103" s="86" t="inlineStr">
+        <is>
+          <t>W 残项清理 commit（755a088 的下一个 commit，单 commit 无法自填 hash）</t>
+        </is>
+      </c>
       <c r="K103" s="86" t="inlineStr">
         <is>
           <t>W-02 刀残债（10-16）</t>
@@ -6885,7 +6897,65 @@
       </c>
       <c r="L103" s="86" t="inlineStr">
         <is>
-          <t>不适用</t>
+          <t>已 push</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="86" t="inlineStr">
+        <is>
+          <t>W-02-r2</t>
+        </is>
+      </c>
+      <c r="B104" s="86" t="inlineStr">
+        <is>
+          <t>已处理</t>
+        </is>
+      </c>
+      <c r="C104" s="86" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D104" s="86" t="inlineStr">
+        <is>
+          <t>世界感</t>
+        </is>
+      </c>
+      <c r="E104" s="86" t="inlineStr">
+        <is>
+          <t>时段划分不统一（17:31 白天/傍晚）</t>
+        </is>
+      </c>
+      <c r="F104" s="86" t="inlineStr">
+        <is>
+          <t>W-01 时间行用 8 段 dayPeriod（含下午），presence 用 5 段，17:31 两行说法不一致。</t>
+        </is>
+      </c>
+      <c r="G104" s="86" t="inlineStr">
+        <is>
+          <t>presence 5 时段为唯一来源，W-01 buildNowContextLine 复用 presenceSlotForHour 与同一时区常量；17:31 统一「白天」，不留第二套边界。单测覆盖。</t>
+        </is>
+      </c>
+      <c r="H104" s="87" t="n">
+        <v>46311</v>
+      </c>
+      <c r="I104" s="89" t="n">
+        <v>46311</v>
+      </c>
+      <c r="J104" s="86" t="inlineStr">
+        <is>
+          <t>W 残项清理 commit（755a088 的下一个 commit，单 commit 无法自填 hash）</t>
+        </is>
+      </c>
+      <c r="K104" s="86" t="inlineStr">
+        <is>
+          <t>W-02 云验残项（10-16）</t>
+        </is>
+      </c>
+      <c r="L104" s="86" t="inlineStr">
+        <is>
+          <t>已 push</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(product): W-03 life_events landed (table, advance before gates, life inject); backfill r-items commit 0bcb5a9; EOD env note
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -6191,7 +6191,7 @@
       </c>
       <c r="B91" s="86" t="inlineStr">
         <is>
-          <t>暂缓</t>
+          <t>已处理</t>
         </is>
       </c>
       <c r="C91" s="86" t="inlineStr">
@@ -6216,22 +6216,28 @@
       </c>
       <c r="G91" s="86" t="inlineStr">
         <is>
-          <t>依赖 W-02；推进分支不得调 LLM。跨重启依赖 D-15。</t>
+          <t>2026-10-16 BF：life_events 表（local_date 唯一键 + occurred_at 索引，幂等迁移，副本两次无错）；advanceLifeEvents 挂主动 tick 入口、总开关前独立跑，纯计算不补记、清 7 天；注入 kind:'life' 一行跟 presence 后（24h、排除当前时段、≤3 条），非 pinned 整行裁。W-02 状态机推进本刀收。单测 30 条、typecheck server+web 过。</t>
         </is>
       </c>
       <c r="H91" s="87" t="n">
         <v>46310</v>
       </c>
-      <c r="I91" s="86" t="n"/>
-      <c r="J91" s="86" t="n"/>
+      <c r="I91" s="89" t="n">
+        <v>46311</v>
+      </c>
+      <c r="J91" s="86" t="inlineStr">
+        <is>
+          <t>259af7b</t>
+        </is>
+      </c>
       <c r="K91" s="86" t="inlineStr">
         <is>
-          <t>二期新增；待用户排期</t>
+          <t>二期新增；待云验</t>
         </is>
       </c>
       <c r="L91" s="86" t="inlineStr">
         <is>
-          <t>不适用</t>
+          <t>已 push</t>
         </is>
       </c>
     </row>
@@ -6777,7 +6783,7 @@
       </c>
       <c r="J101" s="40" t="inlineStr">
         <is>
-          <t>W 残项清理 commit（755a088 的下一个 commit，单 commit 无法自填 hash）</t>
+          <t>0bcb5a9</t>
         </is>
       </c>
       <c r="K101" s="40" t="inlineStr">
@@ -6887,7 +6893,7 @@
       </c>
       <c r="J103" s="86" t="inlineStr">
         <is>
-          <t>W 残项清理 commit（755a088 的下一个 commit，单 commit 无法自填 hash）</t>
+          <t>0bcb5a9</t>
         </is>
       </c>
       <c r="K103" s="86" t="inlineStr">
@@ -6945,7 +6951,7 @@
       </c>
       <c r="J104" s="86" t="inlineStr">
         <is>
-          <t>W 残项清理 commit（755a088 的下一个 commit，单 commit 无法自填 hash）</t>
+          <t>0bcb5a9</t>
         </is>
       </c>
       <c r="K104" s="86" t="inlineStr">

</xml_diff>

<commit_message>
docs(product): D-03-b close-out (7e6e22c), W-03-r1 row, W-03 closed note, EOD
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -1392,7 +1392,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L104"/>
+  <dimension ref="A1:L106"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="40" min="1" max="1"/>
@@ -6232,7 +6232,7 @@
       </c>
       <c r="K91" s="86" t="inlineStr">
         <is>
-          <t>二期新增；待云验</t>
+          <t>二期新增；已关单 122abc9</t>
         </is>
       </c>
       <c r="L91" s="86" t="inlineStr">
@@ -6960,6 +6960,122 @@
         </is>
       </c>
       <c r="L104" s="86" t="inlineStr">
+        <is>
+          <t>已 push</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="86" t="inlineStr">
+        <is>
+          <t>D-03-b</t>
+        </is>
+      </c>
+      <c r="B105" s="86" t="inlineStr">
+        <is>
+          <t>已处理</t>
+        </is>
+      </c>
+      <c r="C105" s="86" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D105" s="86" t="inlineStr">
+        <is>
+          <t>后端</t>
+        </is>
+      </c>
+      <c r="E105" s="86" t="inlineStr">
+        <is>
+          <t>读图编排下沉 chatImageTurn（D-03 第二刀）</t>
+        </is>
+      </c>
+      <c r="F105" s="86" t="inlineStr">
+        <is>
+          <t>conversations.ts 的 B-04A 私聊上传图片+视觉回复分支整体在路由里。</t>
+        </is>
+      </c>
+      <c r="G105" s="86" t="inlineStr">
+        <is>
+          <t>整段原样搬到 services/chatImageTurn.ts 的 handleImageMessage，路由只留会话校验与 multipart 读存图；markConversationRead 以参数传入。错误文案/日志 key/返回结构不变，仅代码移动+import 调整。conversations.ts 658→509 行（chatImageTurn.ts 178 行）；距 ~400 差约 109 行，主要是语音路由（D-03-c）与 TTS 路由（D-03-d）。BF 冒烟：文字私聊、画一只猫出图、坏 Key 人话、上传图走视觉失败人话（本机模型不支持多模态，环境既有）。</t>
+        </is>
+      </c>
+      <c r="H105" s="87" t="n">
+        <v>46311</v>
+      </c>
+      <c r="I105" s="89" t="n">
+        <v>46311</v>
+      </c>
+      <c r="J105" s="86" t="inlineStr">
+        <is>
+          <t>7e6e22c</t>
+        </is>
+      </c>
+      <c r="K105" s="86" t="inlineStr">
+        <is>
+          <t>用户 10-16 拍板 D-03-b；c/d 未做</t>
+        </is>
+      </c>
+      <c r="L105" s="86" t="inlineStr">
+        <is>
+          <t>已 push</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="86" t="inlineStr">
+        <is>
+          <t>W-03-r1</t>
+        </is>
+      </c>
+      <c r="B106" s="86" t="inlineStr">
+        <is>
+          <t>已处理</t>
+        </is>
+      </c>
+      <c r="C106" s="86" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D106" s="86" t="inlineStr">
+        <is>
+          <t>世界感</t>
+        </is>
+      </c>
+      <c r="E106" s="86" t="inlineStr">
+        <is>
+          <t>life 行首改「你最近：」</t>
+        </is>
+      </c>
+      <c r="F106" s="86" t="inlineStr">
+        <is>
+          <t>「你今天早些时候：」后面可能跟「昨天 夜里」，语义别扭。</t>
+        </is>
+      </c>
+      <c r="G106" s="86" t="inlineStr">
+        <is>
+          <t>行首改「你最近：」，单测同步。随 D-03-b feat commit。</t>
+        </is>
+      </c>
+      <c r="H106" s="87" t="n">
+        <v>46311</v>
+      </c>
+      <c r="I106" s="89" t="n">
+        <v>46311</v>
+      </c>
+      <c r="J106" s="86" t="inlineStr">
+        <is>
+          <t>7e6e22c</t>
+        </is>
+      </c>
+      <c r="K106" s="86" t="inlineStr">
+        <is>
+          <t>W-03 云验残项（10-16）</t>
+        </is>
+      </c>
+      <c r="L106" s="86" t="inlineStr">
         <is>
           <t>已 push</t>
         </is>

</xml_diff>

<commit_message>
docs(product): D-03 a/b/c/d close-out (mapping, 已收口), B-04f-r1 dc786bb, B-04f verdict in §五 + appendix, r2/r3 rows, EOD observations
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -1392,7 +1392,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L106"/>
+  <dimension ref="A1:L111"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="40" min="1" max="1"/>
@@ -6988,7 +6988,7 @@
       </c>
       <c r="E105" s="86" t="inlineStr">
         <is>
-          <t>读图编排下沉 chatImageTurn（D-03 第二刀）</t>
+          <t>读图编排下沉 chatVisionTurn（D-03 第二刀）</t>
         </is>
       </c>
       <c r="F105" s="86" t="inlineStr">
@@ -6998,7 +6998,7 @@
       </c>
       <c r="G105" s="86" t="inlineStr">
         <is>
-          <t>整段原样搬到 services/chatImageTurn.ts 的 handleImageMessage，路由只留会话校验与 multipart 读存图；markConversationRead 以参数传入。错误文案/日志 key/返回结构不变，仅代码移动+import 调整。conversations.ts 658→509 行（chatImageTurn.ts 178 行）；距 ~400 差约 109 行，主要是语音路由（D-03-c）与 TTS 路由（D-03-d）。BF 冒烟：文字私聊、画一只猫出图、坏 Key 人话、上传图走视觉失败人话（本机模型不支持多模态，环境既有）。</t>
+          <t>整段原样搬到 services/chatVisionTurn.ts 的 handleImageMessage，路由只留会话校验与 multipart 读存图；markConversationRead 以参数传入。错误文案/日志 key/返回结构不变，仅代码移动+import 调整。conversations.ts 658→509 行（chatVisionTurn.ts 178 行）；距 ~400 差约 109 行，主要是语音路由（D-03-c）与 TTS 路由（D-03-d）。BF 冒烟：文字私聊、画一只猫出图、坏 Key 人话、上传图走视觉失败人话（本机模型不支持多模态，环境既有）。（文件 becc7f8 由 chatImageTurn.ts 改名）</t>
         </is>
       </c>
       <c r="H105" s="87" t="n">
@@ -7014,7 +7014,7 @@
       </c>
       <c r="K105" s="86" t="inlineStr">
         <is>
-          <t>用户 10-16 拍板 D-03-b；c/d 未做</t>
+          <t>实际搬的是读图（生图在 D-03-a 已随 handleUserMessage 下沉 chatTurn）。对应：D-03-a 生图随 chatTurn；D-03-b 读图 chatVisionTurn；D-03-c 语音 STT voiceTurn；D-03-d TTS 缓存 ttsCache。D-03 收口口径：路由只剩校验和 I/O；残留 = 会话 CRUD 与路由 I/O，属正当边界。读图云验过（35fb80b）</t>
         </is>
       </c>
       <c r="L105" s="86" t="inlineStr">
@@ -7078,6 +7078,284 @@
       <c r="L106" s="86" t="inlineStr">
         <is>
           <t>已 push</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="86" t="inlineStr">
+        <is>
+          <t>D-03-c</t>
+        </is>
+      </c>
+      <c r="B107" s="86" t="inlineStr">
+        <is>
+          <t>已处理</t>
+        </is>
+      </c>
+      <c r="C107" s="86" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D107" s="86" t="inlineStr">
+        <is>
+          <t>后端</t>
+        </is>
+      </c>
+      <c r="E107" s="86" t="inlineStr">
+        <is>
+          <t>语音 STT 编排下沉 voiceTurn（D-03 第三刀）</t>
+        </is>
+      </c>
+      <c r="F107" s="86" t="inlineStr">
+        <is>
+          <t>conversations.ts 语音路由里「转写 → handleUserMessage」编排在路由。</t>
+        </is>
+      </c>
+      <c r="G107" s="86" t="inlineStr">
+        <is>
+          <t>原样搬到 services/voiceTurn.ts 的 handleVoiceMessage（27 行），multipart 解析与校验留路由；conversations.ts 509→500。BF 冒烟语音+纯文字过，云验过。</t>
+        </is>
+      </c>
+      <c r="H107" s="87" t="n">
+        <v>46311</v>
+      </c>
+      <c r="I107" s="89" t="n">
+        <v>46311</v>
+      </c>
+      <c r="J107" s="86" t="inlineStr">
+        <is>
+          <t>c08d5da</t>
+        </is>
+      </c>
+      <c r="K107" s="86" t="inlineStr">
+        <is>
+          <t>云验中 DeepSeek 偶发空 content 走降级，观察不挂残项</t>
+        </is>
+      </c>
+      <c r="L107" s="86" t="inlineStr">
+        <is>
+          <t>已 push</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="86" t="inlineStr">
+        <is>
+          <t>D-03-d</t>
+        </is>
+      </c>
+      <c r="B108" s="86" t="inlineStr">
+        <is>
+          <t>已处理</t>
+        </is>
+      </c>
+      <c r="C108" s="86" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D108" s="86" t="inlineStr">
+        <is>
+          <t>后端</t>
+        </is>
+      </c>
+      <c r="E108" s="86" t="inlineStr">
+        <is>
+          <t>TTS 缓存下沉 ttsCache（D-03 第四刀，D-03 收口）</t>
+        </is>
+      </c>
+      <c r="F108" s="86" t="inlineStr">
+        <is>
+          <t>/api/messages/:id/tts 的 voice 解析/缓存文件名/命中判定/缺了就合成在路由。</t>
+        </is>
+      </c>
+      <c r="G108" s="86" t="inlineStr">
+        <is>
+          <t>搬到 services/ttsCache.ts 的 ensureTtsCacheFile（39 行）；DB 查询与文件流留路由；conversations.ts 500→480。命中：再播 0.003s、哈希一致、mtime 不变；云端缺 Key 502 文案不变。D-03 已收口。</t>
+        </is>
+      </c>
+      <c r="H108" s="87" t="n">
+        <v>46311</v>
+      </c>
+      <c r="I108" s="89" t="n">
+        <v>46311</v>
+      </c>
+      <c r="J108" s="86" t="inlineStr">
+        <is>
+          <t>55bb600</t>
+        </is>
+      </c>
+      <c r="K108" s="86" t="inlineStr">
+        <is>
+          <t>原代码无 hit 日志，不另开残项（EOD 备注）</t>
+        </is>
+      </c>
+      <c r="L108" s="86" t="inlineStr">
+        <is>
+          <t>已 push</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="86" t="inlineStr">
+        <is>
+          <t>B-04f-r1</t>
+        </is>
+      </c>
+      <c r="B109" s="86" t="inlineStr">
+        <is>
+          <t>已处理</t>
+        </is>
+      </c>
+      <c r="C109" s="86" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D109" s="86" t="inlineStr">
+        <is>
+          <t>生图</t>
+        </is>
+      </c>
+      <c r="E109" s="86" t="inlineStr">
+        <is>
+          <t>删 imageGen.ts 已废弃 batch_size</t>
+        </is>
+      </c>
+      <c r="F109" s="86" t="inlineStr">
+        <is>
+          <t>硅基流动 2026-09-30 起 batch_size 废弃。</t>
+        </is>
+      </c>
+      <c r="G109" s="86" t="inlineStr">
+        <is>
+          <t>单独 commit 删除；私聊画猫 200 出图（Kolors 1024×1024），云验过。尺寸核对不挂（原图 1024，819 为查看缩放）。</t>
+        </is>
+      </c>
+      <c r="H109" s="87" t="n">
+        <v>46311</v>
+      </c>
+      <c r="I109" s="89" t="n">
+        <v>46311</v>
+      </c>
+      <c r="J109" s="86" t="inlineStr">
+        <is>
+          <t>dc786bb</t>
+        </is>
+      </c>
+      <c r="K109" s="86" t="inlineStr">
+        <is>
+          <t>B-04f 残项，提前到本轮</t>
+        </is>
+      </c>
+      <c r="L109" s="86" t="inlineStr">
+        <is>
+          <t>已 push</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="86" t="inlineStr">
+        <is>
+          <t>B-04f-r2</t>
+        </is>
+      </c>
+      <c r="B110" s="86" t="inlineStr">
+        <is>
+          <t>待处理</t>
+        </is>
+      </c>
+      <c r="C110" s="86" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D110" s="86" t="inlineStr">
+        <is>
+          <t>生图</t>
+        </is>
+      </c>
+      <c r="E110" s="86" t="inlineStr">
+        <is>
+          <t>验 BF 生产能否稳定走境外出口</t>
+        </is>
+      </c>
+      <c r="F110" s="86" t="inlineStr">
+        <is>
+          <t>NB2.1 动态配图立项的前置条件。</t>
+        </is>
+      </c>
+      <c r="G110" s="86" t="inlineStr">
+        <is>
+          <t>验过后再开「动态配图走 NB2.1，代理不可用/超时静默回落 Kolors，保住 moment_image_daily_cap」一刀。</t>
+        </is>
+      </c>
+      <c r="H110" s="87" t="n">
+        <v>46311</v>
+      </c>
+      <c r="I110" s="89" t="n"/>
+      <c r="J110" s="86" t="n"/>
+      <c r="K110" s="86" t="inlineStr">
+        <is>
+          <t>B-04f 用户拍板 10-16</t>
+        </is>
+      </c>
+      <c r="L110" s="86" t="inlineStr">
+        <is>
+          <t>未 push</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="86" t="inlineStr">
+        <is>
+          <t>B-04f-r3</t>
+        </is>
+      </c>
+      <c r="B111" s="86" t="inlineStr">
+        <is>
+          <t>暂缓</t>
+        </is>
+      </c>
+      <c r="C111" s="86" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D111" s="86" t="inlineStr">
+        <is>
+          <t>生图</t>
+        </is>
+      </c>
+      <c r="E111" s="86" t="inlineStr">
+        <is>
+          <t>候选：Kolors 关水印 + 自加 AI 标识</t>
+        </is>
+      </c>
+      <c r="F111" s="86" t="inlineStr">
+        <is>
+          <t>B-04f 参赛 Kolors 为关水印版（X-Enable-Watermark: 0）；关水印需自加可见 AI 标识。</t>
+        </is>
+      </c>
+      <c r="G111" s="86" t="inlineStr">
+        <is>
+          <t>生产维持默认水印；仅登记候选，未排期。</t>
+        </is>
+      </c>
+      <c r="H111" s="87" t="n">
+        <v>46311</v>
+      </c>
+      <c r="I111" s="89" t="n"/>
+      <c r="J111" s="86" t="n"/>
+      <c r="K111" s="86" t="inlineStr">
+        <is>
+          <t>B-04f 产品裁定 10-16</t>
+        </is>
+      </c>
+      <c r="L111" s="86" t="inlineStr">
+        <is>
+          <t>未 push</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(product): B-04f-r3 kept as pre-release compliance item (AI label + watermark-off, two steps); EOD smoke msgs deleted
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -7315,7 +7315,7 @@
       </c>
       <c r="B111" s="86" t="inlineStr">
         <is>
-          <t>暂缓</t>
+          <t>待处理</t>
         </is>
       </c>
       <c r="C111" s="86" t="inlineStr">
@@ -7330,17 +7330,17 @@
       </c>
       <c r="E111" s="86" t="inlineStr">
         <is>
-          <t>候选：Kolors 关水印 + 自加 AI 标识</t>
+          <t>对外发布前：自加 AI 标识 + 关水印（合规前置）</t>
         </is>
       </c>
       <c r="F111" s="86" t="inlineStr">
         <is>
-          <t>B-04f 参赛 Kolors 为关水印版（X-Enable-Watermark: 0）；关水印需自加可见 AI 标识。</t>
+          <t>对外发布时 AI 生成内容须带标识（国内生成式 AI / 深度合成标识要求）；Kolors 默认水印是已验证的体验问题，且与 DEFAULT_IMAGE_STYLE 的 no watermark 意图冲突。B-04f 参赛 Kolors 为关水印版（X-Enable-Watermark: 0）。</t>
         </is>
       </c>
       <c r="G111" s="86" t="inlineStr">
         <is>
-          <t>生产维持默认水印；仅登记候选，未排期。</t>
+          <t>拆两步：① 自加 AI 标识（合规必需，与去不去水印无关）；② 关水印（技术可行，生产默认关之前先确认供应商策略与许可）。</t>
         </is>
       </c>
       <c r="H111" s="87" t="n">
@@ -7350,7 +7350,7 @@
       <c r="J111" s="86" t="n"/>
       <c r="K111" s="86" t="inlineStr">
         <is>
-          <t>B-04f 产品裁定 10-16</t>
+          <t>触发条件：对外发布前（合规前置）｜阶段归属：发布准备，不是二期功能。用户 10-16 拍板保留</t>
         </is>
       </c>
       <c r="L111" s="86" t="inlineStr">

</xml_diff>

<commit_message>
docs(product): EOD-2026-10-17 wrap-up, issue table tips/parking, R-REL next
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -1392,7 +1392,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L111"/>
+  <dimension ref="A1:L113"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="40" min="1" max="1"/>
@@ -6557,7 +6557,7 @@
       </c>
       <c r="J97" s="40" t="inlineStr">
         <is>
-          <t>48cc22d / 表关 4e8d0db</t>
+          <t>feat 48cc22d / 表关 4e8d0db（回填 a527e44）</t>
         </is>
       </c>
       <c r="K97" s="40" t="inlineStr">
@@ -6695,7 +6695,7 @@
       </c>
       <c r="B100" s="40" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>暂缓</t>
         </is>
       </c>
       <c r="C100" s="40" t="inlineStr">
@@ -6730,7 +6730,7 @@
       <c r="J100" s="40" t="n"/>
       <c r="K100" s="40" t="inlineStr">
         <is>
-          <t>W-01 云验残项（10-16）</t>
+          <t>W-01 云验残项（10-16）｜挂账：等体感，并入「此刻感观察攒批」</t>
         </is>
       </c>
       <c r="L100" s="40" t="inlineStr">
@@ -6840,7 +6840,7 @@
       <c r="J102" s="86" t="n"/>
       <c r="K102" s="86" t="inlineStr">
         <is>
-          <t>阶段归属：二期新增；暂缓；10-16 产品定 P2→P3</t>
+          <t>阶段归属：二期新增；暂缓；10-16 产品定 P2→P3｜挂账：等体感，用户提出时再开（10-17 收尾）</t>
         </is>
       </c>
       <c r="L102" s="86" t="inlineStr">
@@ -7009,7 +7009,7 @@
       </c>
       <c r="J105" s="86" t="inlineStr">
         <is>
-          <t>7e6e22c</t>
+          <t>feat 7e6e22c / 表关 35fb80b（改名 becc7f8）</t>
         </is>
       </c>
       <c r="K105" s="86" t="inlineStr">
@@ -7067,7 +7067,7 @@
       </c>
       <c r="J106" s="86" t="inlineStr">
         <is>
-          <t>7e6e22c</t>
+          <t>feat 7e6e22c / 表关 35fb80b</t>
         </is>
       </c>
       <c r="K106" s="86" t="inlineStr">
@@ -7188,7 +7188,7 @@
       </c>
       <c r="K108" s="86" t="inlineStr">
         <is>
-          <t>D-03 收口刀（10-16）</t>
+          <t>D-03 收口刀（10-16）｜D-03 最终收口 tip 4f9b071；收口口径：路由只留校验与 I/O，conversations 480 行不再拆</t>
         </is>
       </c>
       <c r="L108" s="86" t="inlineStr">
@@ -7298,7 +7298,7 @@
       <c r="J110" s="86" t="n"/>
       <c r="K110" s="86" t="inlineStr">
         <is>
-          <t>B-04f 用户拍板 10-16</t>
+          <t>B-04f 用户拍板 10-16｜触发条件：动态配图真要切 NB2.1 前，先验 BF 生产境外出口</t>
         </is>
       </c>
       <c r="L110" s="86" t="inlineStr">
@@ -7350,12 +7350,116 @@
       <c r="J111" s="86" t="n"/>
       <c r="K111" s="86" t="inlineStr">
         <is>
-          <t>触发条件：对外发布前（合规前置）｜阶段归属：发布准备，不是二期功能。用户 10-16 拍板保留</t>
+          <t>触发条件：对外发布前（合规前置）｜阶段归属：发布准备，不是二期功能。用户 10-16 拍板保留｜发布准备：落在 R-REL 发布准备盘点</t>
         </is>
       </c>
       <c r="L111" s="86" t="inlineStr">
         <is>
           <t>未 push</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="86" t="inlineStr">
+        <is>
+          <t>OBS-01</t>
+        </is>
+      </c>
+      <c r="B112" s="86" t="inlineStr">
+        <is>
+          <t>暂缓</t>
+        </is>
+      </c>
+      <c r="C112" s="86" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D112" s="86" t="inlineStr">
+        <is>
+          <t>对话体感</t>
+        </is>
+      </c>
+      <c r="E112" s="86" t="inlineStr">
+        <is>
+          <t>此刻感观察攒批</t>
+        </is>
+      </c>
+      <c r="F112" s="86" t="inlineStr">
+        <is>
+          <t>此刻感相关体感问题攒批再评；W-01-r1「模型不主动用地点」并入本批。</t>
+        </is>
+      </c>
+      <c r="G112" s="86" t="inlineStr">
+        <is>
+          <t>攒够一批再评，不单开刀。</t>
+        </is>
+      </c>
+      <c r="H112" s="87" t="n">
+        <v>46312</v>
+      </c>
+      <c r="I112" s="89" t="n"/>
+      <c r="J112" s="86" t="n"/>
+      <c r="K112" s="86" t="inlineStr">
+        <is>
+          <t>挂账：等体感（10-17 收尾）</t>
+        </is>
+      </c>
+      <c r="L112" s="86" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="86" t="inlineStr">
+        <is>
+          <t>R-REL</t>
+        </is>
+      </c>
+      <c r="B113" s="86" t="inlineStr">
+        <is>
+          <t>待处理</t>
+        </is>
+      </c>
+      <c r="C113" s="86" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D113" s="86" t="inlineStr">
+        <is>
+          <t>发布准备</t>
+        </is>
+      </c>
+      <c r="E113" s="86" t="inlineStr">
+        <is>
+          <t>发布准备盘点（docs 规划刀）</t>
+        </is>
+      </c>
+      <c r="F113" s="86" t="inlineStr">
+        <is>
+          <t>盘点打包分发、首次启动、配置界面、数据目录与备份、合规、隐私口径、Ollama 模型引导，产出发布准备清单。</t>
+        </is>
+      </c>
+      <c r="G113" s="86" t="inlineStr">
+        <is>
+          <t>七个子项在盘点刀里再拆正式条目，各写触发条件与建议优先级；今晚不先编号。</t>
+        </is>
+      </c>
+      <c r="H113" s="87" t="n">
+        <v>46312</v>
+      </c>
+      <c r="I113" s="89" t="n"/>
+      <c r="J113" s="86" t="n"/>
+      <c r="K113" s="86" t="inlineStr">
+        <is>
+          <t>明日起点（10-17）。D-08（数据目录与备份）、B-04f-r3（合规，视觉Bot 出标识规格）落在这里</t>
+        </is>
+      </c>
+      <c r="L113" s="86" t="inlineStr">
+        <is>
+          <t>不适用</t>
         </is>
       </c>
     </row>
@@ -7498,7 +7602,7 @@
       </c>
       <c r="B9" s="70" t="inlineStr">
         <is>
-          <t>a2be134</t>
+          <t>2bc474b</t>
         </is>
       </c>
     </row>
@@ -7781,7 +7885,7 @@
       </c>
       <c r="B20" s="40" t="inlineStr">
         <is>
-          <t>X-07 已关（空间赞/评上限可调）。参数待明确：TTL 7d、静默默认。池：D-11 .env / D-22 smoke。挂：Gemini；X05-D3/D4；D6=off；N-02。X-02/X-04 未开。</t>
+          <t>R-REL 发布准备盘点（docs 规划刀，10-17 起点）。挂账：B-04f-r2 P3、B-04f-r3 发布准备、R-08 / 此刻感观察 OBS-01 等体感。</t>
         </is>
       </c>
     </row>
@@ -7793,7 +7897,7 @@
       </c>
       <c r="B21" s="40" t="inlineStr">
         <is>
-          <t>a2be134</t>
+          <t>2bc474b</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(product): REL-01 release-prep checklist (tier A), REL-02..04 rows, D-08 -> REL-03, BF .env vl record
</commit_message>
<xml_diff>
--- a/docs/product/AgentChat-问题记录.xlsx
+++ b/docs/product/AgentChat-问题记录.xlsx
@@ -1392,7 +1392,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L113"/>
+  <dimension ref="A1:L116"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="40" min="1" max="1"/>
@@ -6010,7 +6010,7 @@
       </c>
       <c r="K87" s="40" t="inlineStr">
         <is>
-          <t>全关 tip 0a153f5（表同步 3d18db9）：BF+HY 键名均入 D-11-env-key-diff.md，无密钥明文。｜BF 读图未就绪：缺 vl 模型（qwen2.5vl:7b 不在 BF，LLM_VISION_MODEL 指 7b-fast；读图验收在云端；拉不拉待三期与 kama 定，不另开单，10-17）｜10-17：BF 已拉 qwen2.5vl:7b，进程级 LLM_VISION_MODEL 实测通（21.5s），.env 未改，写不写入待 kama；.env.bak 已删，键名留档 D-11-env-key-diff.md</t>
+          <t>全关 tip 0a153f5（表同步 3d18db9）：BF+HY 键名均入 D-11-env-key-diff.md，无密钥明文。｜BF 读图：`qwen2.5vl:7b` 已拉，进程级实测通（10-17，单图约 21.5 秒）；kama 批准后已写入 BF `.env`：`LLM_VISION_MODEL=qwen2.5vl:7b`（只改这一行，其余 22 行和 TTS_*/LLM_* 未动；SHA256 改前 `5B48FB32…BD82A145`，改后 `97139408…EDC845228`；8790 临时起服 200，读到的 LLM_VISION_MODEL 正确）。.env 不入库，本条在 REL-01 docs commit 里落档。21.5 秒对陪聊偏慢，记观察不开单；云端 DeepSeek V4.1-Flash 直连作为候选留档（链路通，质量未测）。｜.env.bak 已删，键名留档 D-11-env-key-diff.md</t>
         </is>
       </c>
       <c r="L87" s="40" t="inlineStr">
@@ -7414,12 +7414,12 @@
     <row r="113">
       <c r="A113" s="86" t="inlineStr">
         <is>
-          <t>R-REL</t>
+          <t>REL-01</t>
         </is>
       </c>
       <c r="B113" s="86" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>已处理</t>
         </is>
       </c>
       <c r="C113" s="86" t="inlineStr">
@@ -7444,20 +7444,178 @@
       </c>
       <c r="G113" s="86" t="inlineStr">
         <is>
-          <t>七个子项在盘点刀里再拆正式条目，各写触发条件与建议优先级；今晚不先编号。</t>
+          <t>kama 10-17 定 A 档；产出 发布准备清单.md（A 内三项 + 明确不做项，八维度落位）；A 内三项开 REL-02/03/04。</t>
         </is>
       </c>
       <c r="H113" s="87" t="n">
         <v>46312</v>
       </c>
-      <c r="I113" s="89" t="n"/>
+      <c r="I113" s="89" t="n">
+        <v>46312</v>
+      </c>
       <c r="J113" s="86" t="n"/>
       <c r="K113" s="86" t="inlineStr">
         <is>
-          <t>明日起点（10-17）。D-08（数据目录与备份）、B-04f-r3（合规，视觉Bot 出标识规格）落在这里</t>
+          <t>R 前缀已被记忆线占用，R-REL 改名 REL-01（10-17）。D-08 落在 REL-03；B-04f-r3 合规登记在清单第 5 维（B 或 C 触发）</t>
         </is>
       </c>
       <c r="L113" s="86" t="inlineStr">
+        <is>
+          <t>已 push</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="86" t="inlineStr">
+        <is>
+          <t>REL-02</t>
+        </is>
+      </c>
+      <c r="B114" s="86" t="inlineStr">
+        <is>
+          <t>待处理</t>
+        </is>
+      </c>
+      <c r="C114" s="86" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D114" s="86" t="inlineStr">
+        <is>
+          <t>发布准备</t>
+        </is>
+      </c>
+      <c r="E114" s="86" t="inlineStr">
+        <is>
+          <t>一键启动（A①）</t>
+        </is>
+      </c>
+      <c r="F114" s="86" t="inlineStr">
+        <is>
+          <t>现状：根目录 npm run dev 起前后端（5173/8787），需开终端，Ollama 另行确保在跑，仓库没有启动脚本。</t>
+        </is>
+      </c>
+      <c r="G114" s="86" t="inlineStr">
+        <is>
+          <t>双击脚本起前后端，并检查 Ollama 在线、缺了给人话提示；脚本形态刀里定。</t>
+        </is>
+      </c>
+      <c r="H114" s="87" t="n">
+        <v>46312</v>
+      </c>
+      <c r="I114" s="89" t="n"/>
+      <c r="J114" s="86" t="n"/>
+      <c r="K114" s="86" t="inlineStr">
+        <is>
+          <t>触发：已触发（A 档第一刀）｜依赖：无</t>
+        </is>
+      </c>
+      <c r="L114" s="86" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="86" t="inlineStr">
+        <is>
+          <t>REL-03</t>
+        </is>
+      </c>
+      <c r="B115" s="86" t="inlineStr">
+        <is>
+          <t>待处理</t>
+        </is>
+      </c>
+      <c r="C115" s="86" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D115" s="86" t="inlineStr">
+        <is>
+          <t>发布准备</t>
+        </is>
+      </c>
+      <c r="E115" s="86" t="inlineStr">
+        <is>
+          <t>备份与可验证恢复（A②）</t>
+        </is>
+      </c>
+      <c r="F115" s="86" t="inlineStr">
+        <is>
+          <t>现状：data/agent-chat.db（含 WAL）与 uploads/ 无备份。</t>
+        </is>
+      </c>
+      <c r="G115" s="86" t="inlineStr">
+        <is>
+          <t>备份 db + uploads，并写实测过的恢复步骤；运行中 db 一致性做法刀里评估。</t>
+        </is>
+      </c>
+      <c r="H115" s="87" t="n">
+        <v>46312</v>
+      </c>
+      <c r="I115" s="89" t="n"/>
+      <c r="J115" s="86" t="n"/>
+      <c r="K115" s="86" t="inlineStr">
+        <is>
+          <t>D-08 落在这里，备份与可验证恢复是本刀主体；配额、TTL 和孤儿扫描开刀时再评估要不要一起做｜触发：REL-02 完成后｜依赖：建议在 REL-02 之后</t>
+        </is>
+      </c>
+      <c r="L115" s="86" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="86" t="inlineStr">
+        <is>
+          <t>REL-04</t>
+        </is>
+      </c>
+      <c r="B116" s="86" t="inlineStr">
+        <is>
+          <t>待处理</t>
+        </is>
+      </c>
+      <c r="C116" s="86" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D116" s="86" t="inlineStr">
+        <is>
+          <t>发布准备</t>
+        </is>
+      </c>
+      <c r="E116" s="86" t="inlineStr">
+        <is>
+          <t>A③（内部：云测环境恢复）系统层</t>
+        </is>
+      </c>
+      <c r="F116" s="86" t="inlineStr">
+        <is>
+          <t>restore-env.sh（云电脑，不入库）10-17 整套实跑通过，但系统包是在已装好的机器上重装的；上次事故恰恰是系统包丢失。</t>
+        </is>
+      </c>
+      <c r="G116" s="86" t="inlineStr">
+        <is>
+          <t>Docker 镜像 vs OS 前置清单，只比云测恢复，不当发布方案；Docker 待评估（云电脑当前未装 docker/podman）。</t>
+        </is>
+      </c>
+      <c r="H116" s="87" t="n">
+        <v>46312</v>
+      </c>
+      <c r="I116" s="89" t="n"/>
+      <c r="J116" s="86" t="n"/>
+      <c r="K116" s="86" t="inlineStr">
+        <is>
+          <t>内部项，不参与三档对照，不算用户机器需求｜触发：REL-03 完成后（A 档第三位）｜负责：云电脑运维</t>
+        </is>
+      </c>
+      <c r="L116" s="86" t="inlineStr">
         <is>
           <t>不适用</t>
         </is>
@@ -7602,7 +7760,7 @@
       </c>
       <c r="B9" s="70" t="inlineStr">
         <is>
-          <t>2bc474b</t>
+          <t>6085620</t>
         </is>
       </c>
     </row>
@@ -7885,7 +8043,7 @@
       </c>
       <c r="B20" s="40" t="inlineStr">
         <is>
-          <t>R-REL 发布准备盘点（docs 规划刀，10-17 起点）。挂账：B-04f-r2 P3、B-04f-r3 发布准备、R-08 / 此刻感观察 OBS-01 等体感。</t>
+          <t>REL-02 一键启动（A①），之后 REL-03 备份与可验证恢复（D-08）、REL-04 云测环境恢复系统层。挂账：B-04f-r2 P3、B-04f-r3、R-08 / OBS-01 等体感。</t>
         </is>
       </c>
     </row>
@@ -7897,7 +8055,7 @@
       </c>
       <c r="B21" s="40" t="inlineStr">
         <is>
-          <t>2bc474b</t>
+          <t>6085620</t>
         </is>
       </c>
     </row>

</xml_diff>